<commit_message>
Implement v2 methodology for the Fantasy Darkness Scale, introducing a new scoring system with integer criteria and interval-based tiering. Update the log with methodology changes, rescoring backlog, and theoretical constructs for each criterion. Preserve the original scoring data in a deprecated file for comparison. Add detailed scoring records for works rescored under the new methodology.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1874,17 +1874,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Harry Potter and the Chamber of Secrets</t>
+          <t>Legend</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Ridley Scott</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1907,22 +1907,22 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O13" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="P13" t="n">
-        <v>2.625</v>
+        <v>2.5125</v>
       </c>
       <c r="Q13" t="n">
         <v>2</v>
@@ -1939,17 +1939,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The Little Prince</t>
+          <t>Harry Potter and the Chamber of Secrets</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Book</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Antoine de Saint-Exupéry</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N14" t="n">
         <v>2</v>
@@ -1992,7 +1992,7 @@
       <c r="Q14" t="n">
         <v>2</v>
       </c>
-      <c r="R14" s="5" t="inlineStr"/>
+      <c r="R14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2005,17 +2005,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A Conspiracy of Truths</t>
+          <t>The Little Prince</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Book</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Alexandra Rowland</t>
+          <t>Antoine de Saint-Exupéry</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2038,7 +2038,7 @@
         <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -2047,13 +2047,13 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="P15" t="n">
-        <v>2.7375</v>
+        <v>2.625</v>
       </c>
       <c r="Q15" t="n">
         <v>2</v>
@@ -2071,17 +2071,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>The Chronicles of Narnia</t>
+          <t>A Conspiracy of Truths</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Novels / Films</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>C. S. Lewis</t>
+          <t>Alexandra Rowland</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -2101,25 +2101,25 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="P16" t="n">
-        <v>2.9625</v>
+        <v>2.7375</v>
       </c>
       <c r="Q16" t="n">
         <v>2</v>
@@ -2136,17 +2136,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The Legend of Zelda</t>
+          <t>Willow</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Nintendo</t>
+          <t>Ron Howard / George Lucas</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2160,10 +2160,10 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -2172,19 +2172,19 @@
         <v>1</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O17" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="P17" t="n">
-        <v>2.9625</v>
+        <v>2.85</v>
       </c>
       <c r="Q17" t="n">
         <v>2</v>
@@ -2193,26 +2193,26 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
+          <t>Resilient Cozy Fantasy, Fierce Hopepunk &amp; Heroic Fantasy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mushishi</t>
+          <t>The Chronicles of Narnia</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novels / Films</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Yuki Urushibara</t>
+          <t>C. S. Lewis</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2222,67 +2222,62 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H18" t="n">
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O18" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="P18" t="n">
-        <v>3.075</v>
+        <v>2.9625</v>
       </c>
       <c r="Q18" t="n">
-        <v>3</v>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Tier v1 era 2</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
+          <t>Resilient Cozy Fantasy, Fierce Hopepunk &amp; Heroic Fantasy</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>A Choir of Lies</t>
+          <t>The Legend of Zelda</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Alexandra Rowland</t>
+          <t>Nintendo</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2292,62 +2287,62 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H19" t="n">
         <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O19" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="P19" t="n">
-        <v>3.075</v>
+        <v>2.9625</v>
       </c>
       <c r="Q19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
+          <t>Resilient Cozy Fantasy, Fierce Hopepunk &amp; Heroic Fantasy</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The Hobbit</t>
+          <t>DanMachi</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Light Novels / Anime / Manga</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Fujino Ōmori</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2361,19 +2356,19 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M20" t="n">
         <v>0</v>
@@ -2382,13 +2377,13 @@
         <v>2</v>
       </c>
       <c r="O20" t="n">
-        <v>0.95</v>
+        <v>0.65</v>
       </c>
       <c r="P20" t="n">
-        <v>3.6375</v>
+        <v>2.9625</v>
       </c>
       <c r="Q20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R20" s="5" t="n"/>
     </row>
@@ -2403,17 +2398,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Spirited Away</t>
+          <t>Mushishi</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Yuki Urushibara</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2423,11 +2418,11 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
         <v>1</v>
@@ -2436,7 +2431,7 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2445,16 +2440,21 @@
         <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>0.95</v>
+        <v>0.7</v>
       </c>
       <c r="P21" t="n">
-        <v>3.6375</v>
+        <v>3.075</v>
       </c>
       <c r="Q21" t="n">
         <v>3</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Tier v1 era 2</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -2468,17 +2468,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Discworld</t>
+          <t>A Choir of Lies</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Novels / Games / Comics</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Terry Pratchett</t>
+          <t>Alexandra Rowland</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2495,7 +2495,7 @@
         <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
@@ -2507,25 +2507,21 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N22" t="n">
         <v>1</v>
       </c>
       <c r="O22" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="P22" t="n">
-        <v>3.75</v>
+        <v>3.075</v>
       </c>
       <c r="Q22" t="n">
         <v>3</v>
       </c>
-      <c r="R22" s="5" t="inlineStr">
-        <is>
-          <t>Tier v1 era 4</t>
-        </is>
-      </c>
+      <c r="R22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2538,17 +2534,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>The Lord of the Rings</t>
+          <t>Dungeon Meshi</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Novels / Films</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Ryoko Kui</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2562,7 +2558,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I23" t="n">
         <v>1</v>
@@ -2574,7 +2570,7 @@
         <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M23" t="n">
         <v>0</v>
@@ -2583,10 +2579,10 @@
         <v>2</v>
       </c>
       <c r="O23" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="P23" t="n">
-        <v>3.975</v>
+        <v>3.3</v>
       </c>
       <c r="Q23" t="n">
         <v>3</v>
@@ -2603,17 +2599,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Frieren: Beyond Journey's End</t>
+          <t>Final Fantasy IV</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Kanehito Yamada / Tsukasa Abe</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2623,35 +2619,35 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O24" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="P24" t="n">
-        <v>3.975</v>
+        <v>3.525</v>
       </c>
       <c r="Q24" t="n">
         <v>3</v>
@@ -2660,26 +2656,26 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Grimgar: Ashes and Illusions</t>
+          <t>The Hobbit</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Light Novels / Anime</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Ao Jyumonji</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2693,13 +2689,13 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
@@ -2708,48 +2704,44 @@
         <v>2</v>
       </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
         <v>2</v>
       </c>
       <c r="O25" t="n">
-        <v>1.4</v>
+        <v>0.95</v>
       </c>
       <c r="P25" t="n">
-        <v>4.65</v>
+        <v>3.6375</v>
       </c>
       <c r="Q25" t="n">
-        <v>4</v>
-      </c>
-      <c r="R25" s="5" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="R25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Avatar: The Last Airbender</t>
+          <t>Spirited Away</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2759,23 +2751,23 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M26" t="n">
         <v>1</v>
@@ -2784,42 +2776,37 @@
         <v>2</v>
       </c>
       <c r="O26" t="n">
-        <v>1.4</v>
+        <v>0.95</v>
       </c>
       <c r="P26" t="n">
-        <v>4.65</v>
+        <v>3.6375</v>
       </c>
       <c r="Q26" t="n">
-        <v>4</v>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>Tier v1 era 3</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist: Brotherhood</t>
+          <t>Howl's Moving Castle</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2839,52 +2826,52 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L27" t="n">
         <v>2</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O27" t="n">
-        <v>1.5</v>
+        <v>0.95</v>
       </c>
       <c r="P27" t="n">
-        <v>4.875</v>
+        <v>3.6375</v>
       </c>
       <c r="Q27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tales from Earthsea</t>
+          <t>Discworld</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Novels / Games / Comics</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Gorō Miyazaki</t>
+          <t>Terry Pratchett</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2894,11 +2881,11 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
         <v>1</v>
@@ -2910,51 +2897,51 @@
         <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O28" t="n">
-        <v>1.55</v>
+        <v>1</v>
       </c>
       <c r="P28" t="n">
-        <v>4.9875</v>
+        <v>3.75</v>
       </c>
       <c r="Q28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R28" s="5" t="inlineStr">
         <is>
-          <t>Tier v1 era 5</t>
+          <t>Tier v1 era 4</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V: Skyrim</t>
+          <t>The Lord of the Rings</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / Films</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Bethesda Game Studios</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2974,52 +2961,52 @@
         <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
         <v>2</v>
       </c>
       <c r="O29" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="P29" t="n">
-        <v>5.325</v>
+        <v>3.975</v>
       </c>
       <c r="Q29" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>Frieren: Beyond Journey's End</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Kanehito Yamada / Tsukasa Abe</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3029,23 +3016,23 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H30" t="n">
         <v>2</v>
       </c>
       <c r="I30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
         <v>2</v>
@@ -3054,37 +3041,37 @@
         <v>2</v>
       </c>
       <c r="O30" t="n">
-        <v>1.85</v>
+        <v>1.1</v>
       </c>
       <c r="P30" t="n">
-        <v>5.6625</v>
+        <v>3.975</v>
       </c>
       <c r="Q30" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>Black Clover</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Yūki Tabata</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3098,63 +3085,58 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O31" t="n">
-        <v>1.9</v>
+        <v>1.1</v>
       </c>
       <c r="P31" t="n">
-        <v>5.775</v>
+        <v>3.975</v>
       </c>
       <c r="Q31" t="n">
-        <v>5</v>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>Tier v1 era 6</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>The NeverEnding Story</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>Michael Ende</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3171,55 +3153,55 @@
         <v>2</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
         <v>2</v>
       </c>
       <c r="M32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
         <v>3</v>
       </c>
       <c r="O32" t="n">
-        <v>2.1</v>
+        <v>1.2</v>
       </c>
       <c r="P32" t="n">
-        <v>6.225</v>
+        <v>4.2</v>
       </c>
       <c r="Q32" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Harry Potter and the Prisoner of Azkaban</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3233,63 +3215,59 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M33" t="n">
         <v>2</v>
       </c>
       <c r="N33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O33" t="n">
-        <v>2.15</v>
+        <v>1.35</v>
       </c>
       <c r="P33" t="n">
-        <v>6.3375</v>
+        <v>4.5375</v>
       </c>
       <c r="Q33" t="n">
-        <v>6</v>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Grimgar: Ashes and Illusions</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Anime</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Ao Jyumonji</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3306,55 +3284,60 @@
         <v>2</v>
       </c>
       <c r="I34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L34" t="n">
         <v>2</v>
       </c>
       <c r="M34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N34" t="n">
+        <v>2</v>
+      </c>
+      <c r="O34" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="P34" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="Q34" t="n">
         <v>4</v>
       </c>
-      <c r="O34" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="P34" t="n">
-        <v>6.45</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>6</v>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Avatar: The Last Airbender</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3364,67 +3347,67 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L35" t="n">
         <v>2</v>
       </c>
       <c r="M35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O35" t="n">
-        <v>2.25</v>
+        <v>1.4</v>
       </c>
       <c r="P35" t="n">
-        <v>6.5625</v>
+        <v>4.65</v>
       </c>
       <c r="Q35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Tier v1 era 5</t>
+          <t>Tier v1 era 3</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist: Brotherhood</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3438,13 +3421,13 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K36" t="n">
         <v>2</v>
@@ -3453,48 +3436,43 @@
         <v>2</v>
       </c>
       <c r="M36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N36" t="n">
         <v>3</v>
       </c>
       <c r="O36" t="n">
-        <v>2.25</v>
+        <v>1.5</v>
       </c>
       <c r="P36" t="n">
-        <v>6.5625</v>
+        <v>4.875</v>
       </c>
       <c r="Q36" t="n">
-        <v>6</v>
-      </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>Tier v1 era 7</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Boy and the Heron</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3514,13 +3492,13 @@
         <v>2</v>
       </c>
       <c r="J37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M37" t="n">
         <v>2</v>
@@ -3529,27 +3507,27 @@
         <v>3</v>
       </c>
       <c r="O37" t="n">
-        <v>2.25</v>
+        <v>1.5</v>
       </c>
       <c r="P37" t="n">
-        <v>6.5625</v>
+        <v>4.875</v>
       </c>
       <c r="Q37" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Final Fantasy IX</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3559,7 +3537,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3573,16 +3551,16 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L38" t="n">
         <v>2</v>
@@ -3594,37 +3572,37 @@
         <v>3</v>
       </c>
       <c r="O38" t="n">
-        <v>2.25</v>
+        <v>1.5</v>
       </c>
       <c r="P38" t="n">
-        <v>6.5625</v>
+        <v>4.875</v>
       </c>
       <c r="Q38" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Tales from Earthsea</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Studio Ghibli / Gorō Miyazaki</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3638,63 +3616,63 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M39" t="n">
         <v>2</v>
       </c>
       <c r="N39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O39" t="n">
-        <v>2.4</v>
+        <v>1.55</v>
       </c>
       <c r="P39" t="n">
-        <v>6.9</v>
+        <v>4.9875</v>
       </c>
       <c r="Q39" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Tier v1 era 8</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>Dragonlance</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels / Games</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Margaret Weis / Tracy Hickman</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3708,58 +3686,58 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K40" t="n">
         <v>2</v>
       </c>
       <c r="L40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O40" t="n">
-        <v>2.65</v>
+        <v>1.65</v>
       </c>
       <c r="P40" t="n">
-        <v>7.4625</v>
+        <v>5.2125</v>
       </c>
       <c r="Q40" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>The Elder Scrolls V: Skyrim</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Bethesda Game Studios</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3773,58 +3751,58 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N41" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O41" t="n">
-        <v>3.1</v>
+        <v>1.7</v>
       </c>
       <c r="P41" t="n">
-        <v>8.475</v>
+        <v>5.325</v>
       </c>
       <c r="Q41" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3838,58 +3816,58 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O42" t="n">
-        <v>3.15</v>
+        <v>1.85</v>
       </c>
       <c r="P42" t="n">
-        <v>8.5875</v>
+        <v>5.6625</v>
       </c>
       <c r="Q42" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3903,58 +3881,63 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J43" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N43" t="n">
         <v>4</v>
       </c>
       <c r="O43" t="n">
-        <v>3.25</v>
+        <v>1.9</v>
       </c>
       <c r="P43" t="n">
-        <v>8.8125</v>
+        <v>5.775</v>
       </c>
       <c r="Q43" t="n">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3968,98 +3951,898 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O44" t="n">
-        <v>3.7</v>
+        <v>2.1</v>
       </c>
       <c r="P44" t="n">
-        <v>9.824999999999999</v>
+        <v>6.225</v>
       </c>
       <c r="Q44" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
+        <v>6</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Shin Sekai Yori (From the New World)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Novel / Anime</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Yusuke Kishi</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>2</v>
+      </c>
+      <c r="I45" t="n">
+        <v>2</v>
+      </c>
+      <c r="J45" t="n">
+        <v>2</v>
+      </c>
+      <c r="K45" t="n">
+        <v>3</v>
+      </c>
+      <c r="L45" t="n">
+        <v>2</v>
+      </c>
+      <c r="M45" t="n">
+        <v>2</v>
+      </c>
+      <c r="N45" t="n">
+        <v>2</v>
+      </c>
+      <c r="O45" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="P45" t="n">
+        <v>6.3375</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>6</v>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>6</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Made in Abyss</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Manga / Anime</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Akihito Tsukushi</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>2</v>
+      </c>
+      <c r="I46" t="n">
+        <v>2</v>
+      </c>
+      <c r="J46" t="n">
+        <v>2</v>
+      </c>
+      <c r="K46" t="n">
+        <v>2</v>
+      </c>
+      <c r="L46" t="n">
+        <v>2</v>
+      </c>
+      <c r="M46" t="n">
+        <v>2</v>
+      </c>
+      <c r="N46" t="n">
+        <v>4</v>
+      </c>
+      <c r="O46" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="P46" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>6</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Fullmetal Alchemist (2003)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Anime</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Hiromu Arakawa / Bones</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>3</v>
+      </c>
+      <c r="I47" t="n">
+        <v>2</v>
+      </c>
+      <c r="J47" t="n">
+        <v>2</v>
+      </c>
+      <c r="K47" t="n">
+        <v>2</v>
+      </c>
+      <c r="L47" t="n">
+        <v>2</v>
+      </c>
+      <c r="M47" t="n">
+        <v>2</v>
+      </c>
+      <c r="N47" t="n">
+        <v>3</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="P47" t="n">
+        <v>6.5625</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>6</v>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>6</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>The Saga of Tanya the Evil</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Light Novels / Manga / Anime / Film</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Carlo Zen</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>2</v>
+      </c>
+      <c r="I48" t="n">
+        <v>2</v>
+      </c>
+      <c r="J48" t="n">
+        <v>3</v>
+      </c>
+      <c r="K48" t="n">
+        <v>2</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2</v>
+      </c>
+      <c r="M48" t="n">
+        <v>2</v>
+      </c>
+      <c r="N48" t="n">
+        <v>3</v>
+      </c>
+      <c r="O48" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="P48" t="n">
+        <v>6.5625</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>6</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>6</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Claymore</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Manga / Anime</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Norihiro Yagi</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>2</v>
+      </c>
+      <c r="I49" t="n">
+        <v>2</v>
+      </c>
+      <c r="J49" t="n">
+        <v>2</v>
+      </c>
+      <c r="K49" t="n">
+        <v>3</v>
+      </c>
+      <c r="L49" t="n">
+        <v>2</v>
+      </c>
+      <c r="M49" t="n">
+        <v>2</v>
+      </c>
+      <c r="N49" t="n">
+        <v>3</v>
+      </c>
+      <c r="O49" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="P49" t="n">
+        <v>6.5625</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>6</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Final Fantasy XVI</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Video Game</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Square Enix</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>2</v>
+      </c>
+      <c r="I50" t="n">
+        <v>2</v>
+      </c>
+      <c r="J50" t="n">
+        <v>2</v>
+      </c>
+      <c r="K50" t="n">
+        <v>3</v>
+      </c>
+      <c r="L50" t="n">
+        <v>2</v>
+      </c>
+      <c r="M50" t="n">
+        <v>2</v>
+      </c>
+      <c r="N50" t="n">
+        <v>3</v>
+      </c>
+      <c r="O50" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="P50" t="n">
+        <v>6.5625</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>6</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Dark Souls I–III</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Video Games</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>3</v>
+      </c>
+      <c r="I51" t="n">
+        <v>2</v>
+      </c>
+      <c r="J51" t="n">
+        <v>2</v>
+      </c>
+      <c r="K51" t="n">
+        <v>2</v>
+      </c>
+      <c r="L51" t="n">
+        <v>3</v>
+      </c>
+      <c r="M51" t="n">
+        <v>2</v>
+      </c>
+      <c r="N51" t="n">
+        <v>3</v>
+      </c>
+      <c r="O51" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P51" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>6</v>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>7</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Extreme Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Berserk</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Manga / Anime / Films</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Kentaro Miura</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>3</v>
+      </c>
+      <c r="I52" t="n">
+        <v>2</v>
+      </c>
+      <c r="J52" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" t="n">
+        <v>2</v>
+      </c>
+      <c r="L52" t="n">
+        <v>3</v>
+      </c>
+      <c r="M52" t="n">
+        <v>2</v>
+      </c>
+      <c r="N52" t="n">
+        <v>4</v>
+      </c>
+      <c r="O52" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="P52" t="n">
+        <v>7.4625</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>8</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>A Song of Ice and Fire</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Novels / TV</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>George R. R. Martin</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>3</v>
+      </c>
+      <c r="I53" t="n">
+        <v>3</v>
+      </c>
+      <c r="J53" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" t="n">
+        <v>3</v>
+      </c>
+      <c r="L53" t="n">
+        <v>3</v>
+      </c>
+      <c r="M53" t="n">
+        <v>3</v>
+      </c>
+      <c r="N53" t="n">
+        <v>4</v>
+      </c>
+      <c r="O53" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="P53" t="n">
+        <v>8.475</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>8</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Elden Ring</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Video Game</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>4</v>
+      </c>
+      <c r="I54" t="n">
+        <v>3</v>
+      </c>
+      <c r="J54" t="n">
+        <v>3</v>
+      </c>
+      <c r="K54" t="n">
+        <v>3</v>
+      </c>
+      <c r="L54" t="n">
+        <v>3</v>
+      </c>
+      <c r="M54" t="n">
+        <v>3</v>
+      </c>
+      <c r="N54" t="n">
+        <v>3</v>
+      </c>
+      <c r="O54" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="P54" t="n">
+        <v>8.5875</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>8</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Fire Punch</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Tatsuki Fujimoto</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>3</v>
+      </c>
+      <c r="I55" t="n">
+        <v>3</v>
+      </c>
+      <c r="J55" t="n">
+        <v>4</v>
+      </c>
+      <c r="K55" t="n">
+        <v>3</v>
+      </c>
+      <c r="L55" t="n">
+        <v>3</v>
+      </c>
+      <c r="M55" t="n">
+        <v>3</v>
+      </c>
+      <c r="N55" t="n">
+        <v>4</v>
+      </c>
+      <c r="O55" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="P55" t="n">
+        <v>8.8125</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>9</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>The First Law</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Novels</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Joe Abercrombie</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>4</v>
+      </c>
+      <c r="I56" t="n">
+        <v>4</v>
+      </c>
+      <c r="J56" t="n">
+        <v>4</v>
+      </c>
+      <c r="K56" t="n">
+        <v>4</v>
+      </c>
+      <c r="L56" t="n">
+        <v>3</v>
+      </c>
+      <c r="M56" t="n">
+        <v>3</v>
+      </c>
+      <c r="N56" t="n">
+        <v>4</v>
+      </c>
+      <c r="O56" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P56" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
         <v>10</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>Very Extreme Grimdark</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>Warhammer 40,000</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>Tabletop / Novels / Games / Animation</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>Games Workshop</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H45" t="n">
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
         <v>4</v>
       </c>
-      <c r="I45" t="n">
+      <c r="I57" t="n">
         <v>4</v>
       </c>
-      <c r="J45" t="n">
+      <c r="J57" t="n">
         <v>4</v>
       </c>
-      <c r="K45" t="n">
+      <c r="K57" t="n">
         <v>4</v>
       </c>
-      <c r="L45" t="n">
+      <c r="L57" t="n">
         <v>4</v>
       </c>
-      <c r="M45" t="n">
+      <c r="M57" t="n">
         <v>4</v>
       </c>
-      <c r="N45" t="n">
+      <c r="N57" t="n">
         <v>4</v>
       </c>
-      <c r="O45" t="n">
+      <c r="O57" t="n">
         <v>4</v>
       </c>
-      <c r="P45" t="n">
+      <c r="P57" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q45" t="n">
+      <c r="Q57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4122,7 +4905,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -4135,7 +4918,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -4148,7 +4931,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -4161,7 +4944,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -4232,7 +5015,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 44 of 87 works in the full catalog (work in progress).</t>
+          <t>Total scored: 56 of 87 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ADDITIONS_LOG.md and SCORING_RECORD.md with detailed rescoring for multiple works, including Harry Potter and the Goblet of Fire, Earthsea, Witch Hat Atelier, Adventure Time, and Final Fantasy series. Adjust tiers based on new scoring criteria, reflecting thematic depth and content severity. Complete Tier 3 backlog and refine Tier 4 entries, ensuring accurate representation of narrative complexities and emotional weight.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1408,26 +1408,26 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Resilient Cozy Fantasy, Fierce Hopepunk &amp; Heroic Fantasy</t>
+          <t>Wholesome Cozy Fantasy, Gentle Hopepunk &amp; Very Bright Fantasy</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Harry Potter and the Philosopher's Stone</t>
+          <t>Final Fantasy I</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1450,7 +1450,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -1462,13 +1462,18 @@
         <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="P6" t="n">
-        <v>2.0625</v>
+        <v>1.725</v>
       </c>
       <c r="Q6" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1482,17 +1487,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The House in the Cerulean Sea</t>
+          <t>Harry Potter and the Philosopher's Stone</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>T. J. Klune</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1502,11 +1507,11 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1524,13 +1529,13 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="P7" t="n">
-        <v>2.175</v>
+        <v>2.0625</v>
       </c>
       <c r="Q7" t="n">
         <v>2</v>
@@ -1547,17 +1552,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Final Fantasy III &amp; V</t>
+          <t>The House in the Cerulean Sea</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>T. J. Klune</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1567,11 +1572,11 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -1580,7 +1585,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -1589,7 +1594,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
         <v>0.3</v>
@@ -1612,17 +1617,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Slayers</t>
+          <t>Final Fantasy III &amp; V</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Light Novels / Anime</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Hajime Kanzaka</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1677,17 +1682,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>The Nightmare Before Christmas</t>
+          <t>Slayers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Light Novels / Anime</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Tim Burton / Henry Selick</t>
+          <t>Hajime Kanzaka</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1713,19 +1718,19 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="P10" t="n">
-        <v>2.2875</v>
+        <v>2.175</v>
       </c>
       <c r="Q10" t="n">
         <v>2</v>
@@ -1743,7 +1748,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Castle in the Sky</t>
+          <t>The Nightmare Before Christmas</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1753,7 +1758,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Tim Burton / Henry Selick</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1776,10 +1781,10 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -1809,7 +1814,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dungeons &amp; Dragons: Honor Among Thieves</t>
+          <t>Castle in the Sky</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1819,7 +1824,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Jonathan Goldstein / John Francis Daley</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1839,7 +1844,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
         <v>1</v>
@@ -1851,13 +1856,13 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="P12" t="n">
-        <v>2.4</v>
+        <v>2.2875</v>
       </c>
       <c r="Q12" t="n">
         <v>2</v>
@@ -1874,7 +1879,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Dungeons &amp; Dragons: Honor Among Thieves</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1884,7 +1889,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ridley Scott</t>
+          <t>Jonathan Goldstein / John Francis Daley</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1904,25 +1909,25 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O13" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="P13" t="n">
-        <v>2.5125</v>
+        <v>2.4</v>
       </c>
       <c r="Q13" t="n">
         <v>2</v>
@@ -1939,17 +1944,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Harry Potter and the Chamber of Secrets</t>
+          <t>Legend</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Ridley Scott</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1972,22 +1977,22 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O14" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="P14" t="n">
-        <v>2.625</v>
+        <v>2.5125</v>
       </c>
       <c r="Q14" t="n">
         <v>2</v>
@@ -2005,17 +2010,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>The Little Prince</t>
+          <t>Harry Potter and the Chamber of Secrets</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Book</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Antoine de Saint-Exupéry</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2029,22 +2034,22 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15" t="n">
         <v>2</v>
@@ -2071,17 +2076,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A Conspiracy of Truths</t>
+          <t>The Little Prince</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Book</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Alexandra Rowland</t>
+          <t>Antoine de Saint-Exupéry</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2091,7 +2096,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -2104,7 +2109,7 @@
         <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -2113,13 +2118,13 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O16" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="P16" t="n">
-        <v>2.7375</v>
+        <v>2.625</v>
       </c>
       <c r="Q16" t="n">
         <v>2</v>
@@ -2136,17 +2141,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Willow</t>
+          <t>A Conspiracy of Truths</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ron Howard / George Lucas</t>
+          <t>Alexandra Rowland</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2156,35 +2161,35 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" t="n">
         <v>1</v>
       </c>
       <c r="L17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O17" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="P17" t="n">
-        <v>2.85</v>
+        <v>2.7375</v>
       </c>
       <c r="Q17" t="n">
         <v>2</v>
@@ -2202,17 +2207,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>The Chronicles of Narnia</t>
+          <t>Willow</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Novels / Films</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>C. S. Lewis</t>
+          <t>Ron Howard / George Lucas</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2226,7 +2231,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
@@ -2244,13 +2249,13 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O18" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="P18" t="n">
-        <v>2.9625</v>
+        <v>2.85</v>
       </c>
       <c r="Q18" t="n">
         <v>2</v>
@@ -2267,17 +2272,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The Legend of Zelda</t>
+          <t>The Chronicles of Narnia</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels / Films</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Nintendo</t>
+          <t>C. S. Lewis</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2294,7 +2299,7 @@
         <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -2303,7 +2308,7 @@
         <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19" t="n">
         <v>0</v>
@@ -2332,17 +2337,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DanMachi</t>
+          <t>The Legend of Zelda</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Light Novels / Anime / Manga</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fujino Ōmori</t>
+          <t>Nintendo</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2356,19 +2361,19 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
         <v>0</v>
@@ -2389,26 +2394,26 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
+          <t>Resilient Cozy Fantasy, Fierce Hopepunk &amp; Heroic Fantasy</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mushishi</t>
+          <t>DanMachi</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Anime / Manga</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Yuki Urushibara</t>
+          <t>Fujino Ōmori</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2418,43 +2423,38 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O21" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="P21" t="n">
-        <v>3.075</v>
+        <v>2.9625</v>
       </c>
       <c r="Q21" t="n">
-        <v>3</v>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Tier v1 era 2</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -2468,17 +2468,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>A Choir of Lies</t>
+          <t>Mushishi</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Alexandra Rowland</t>
+          <t>Yuki Urushibara</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2495,19 +2495,19 @@
         <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" t="n">
         <v>1</v>
@@ -2521,7 +2521,11 @@
       <c r="Q22" t="n">
         <v>3</v>
       </c>
-      <c r="R22" s="5" t="n"/>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>Tier v1 era 2</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2534,17 +2538,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dungeon Meshi</t>
+          <t>A Choir of Lies</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Ryoko Kui</t>
+          <t>Alexandra Rowland</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2554,17 +2558,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H23" t="n">
         <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>1</v>
@@ -2576,13 +2580,13 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O23" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="P23" t="n">
-        <v>3.3</v>
+        <v>3.075</v>
       </c>
       <c r="Q23" t="n">
         <v>3</v>
@@ -2599,17 +2603,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Final Fantasy IV</t>
+          <t>Dungeon Meshi</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Ryoko Kui</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2623,10 +2627,10 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -2635,19 +2639,19 @@
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O24" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="P24" t="n">
-        <v>3.525</v>
+        <v>3.3</v>
       </c>
       <c r="Q24" t="n">
         <v>3</v>
@@ -2665,17 +2669,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>The Hobbit</t>
+          <t>Cormyr</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Ed Greenwood / Jeff Grubb</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2695,13 +2699,13 @@
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
@@ -2710,10 +2714,10 @@
         <v>2</v>
       </c>
       <c r="O25" t="n">
-        <v>0.95</v>
+        <v>0.8</v>
       </c>
       <c r="P25" t="n">
-        <v>3.6375</v>
+        <v>3.3</v>
       </c>
       <c r="Q25" t="n">
         <v>3</v>
@@ -2731,17 +2735,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Spirited Away</t>
+          <t>Final Fantasy IV</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2758,28 +2762,28 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M26" t="n">
         <v>1</v>
       </c>
       <c r="N26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O26" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="P26" t="n">
-        <v>3.6375</v>
+        <v>3.525</v>
       </c>
       <c r="Q26" t="n">
         <v>3</v>
@@ -2796,17 +2800,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Howl's Moving Castle</t>
+          <t>The Hobbit</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2861,17 +2865,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Discworld</t>
+          <t>Spirited Away</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Novels / Games / Comics</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Terry Pratchett</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2881,20 +2885,20 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2903,22 +2907,18 @@
         <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O28" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="P28" t="n">
-        <v>3.75</v>
+        <v>3.6375</v>
       </c>
       <c r="Q28" t="n">
         <v>3</v>
       </c>
-      <c r="R28" s="5" t="inlineStr">
-        <is>
-          <t>Tier v1 era 4</t>
-        </is>
-      </c>
+      <c r="R28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2931,17 +2931,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>The Lord of the Rings</t>
+          <t>Howl's Moving Castle</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Novels / Films</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2955,7 +2955,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I29" t="n">
         <v>1</v>
@@ -2976,10 +2976,10 @@
         <v>2</v>
       </c>
       <c r="O29" t="n">
-        <v>1.1</v>
+        <v>0.95</v>
       </c>
       <c r="P29" t="n">
-        <v>3.975</v>
+        <v>3.6375</v>
       </c>
       <c r="Q29" t="n">
         <v>3</v>
@@ -2996,17 +2996,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Frieren: Beyond Journey's End</t>
+          <t>Discworld</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novels / Games / Comics</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Kanehito Yamada / Tsukasa Abe</t>
+          <t>Terry Pratchett</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3020,34 +3020,39 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O30" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="P30" t="n">
-        <v>3.975</v>
+        <v>3.75</v>
       </c>
       <c r="Q30" t="n">
         <v>3</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Tier v1 era 4</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -3061,17 +3066,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Black Clover</t>
+          <t>The Lord of the Rings</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Manga / Anime / Film</t>
+          <t>Novels / Films</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Yūki Tabata</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3085,7 +3090,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I31" t="n">
         <v>1</v>
@@ -3094,13 +3099,13 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>2</v>
@@ -3117,26 +3122,26 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>The NeverEnding Story</t>
+          <t>Frieren: Beyond Journey's End</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Michael Ende</t>
+          <t>Kanehito Yamada / Tsukasa Abe</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3146,7 +3151,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -3156,52 +3161,52 @@
         <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O32" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="P32" t="n">
-        <v>4.2</v>
+        <v>3.975</v>
       </c>
       <c r="Q32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Harry Potter and the Prisoner of Azkaban</t>
+          <t>Black Clover</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Yūki Tabata</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3221,53 +3226,52 @@
         <v>1</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
         <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O33" t="n">
-        <v>1.35</v>
+        <v>1.1</v>
       </c>
       <c r="P33" t="n">
-        <v>4.5375</v>
+        <v>3.975</v>
       </c>
       <c r="Q33" t="n">
-        <v>4</v>
-      </c>
-      <c r="R33" t="inlineStr"/>
+        <v>3</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Grimgar: Ashes and Illusions</t>
+          <t>Record of Lodoss War</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Light Novels / Anime</t>
+          <t>Novels / Anime</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Ao Jyumonji</t>
+          <t>Ryo Mizuno</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3281,7 +3285,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I34" t="n">
         <v>1</v>
@@ -3296,48 +3300,43 @@
         <v>2</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N34" t="n">
         <v>2</v>
       </c>
       <c r="O34" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="P34" t="n">
-        <v>4.65</v>
+        <v>3.975</v>
       </c>
       <c r="Q34" t="n">
-        <v>4</v>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Avatar: The Last Airbender</t>
+          <t>Final Fantasy II</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3347,11 +3346,11 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I35" t="n">
         <v>1</v>
@@ -3366,23 +3365,23 @@
         <v>2</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N35" t="n">
         <v>2</v>
       </c>
       <c r="O35" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="P35" t="n">
-        <v>4.65</v>
+        <v>3.975</v>
       </c>
       <c r="Q35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Tier v1 era 3</t>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
         </is>
       </c>
     </row>
@@ -3397,17 +3396,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist: Brotherhood</t>
+          <t>The NeverEnding Story</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa</t>
+          <t>Michael Ende</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3421,7 +3420,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I36" t="n">
         <v>1</v>
@@ -3430,22 +3429,22 @@
         <v>1</v>
       </c>
       <c r="K36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
         <v>2</v>
       </c>
       <c r="M36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N36" t="n">
         <v>3</v>
       </c>
       <c r="O36" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="P36" t="n">
-        <v>4.875</v>
+        <v>4.2</v>
       </c>
       <c r="Q36" t="n">
         <v>4</v>
@@ -3462,17 +3461,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>The Boy and the Heron</t>
+          <t>Witch Hat Atelier</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Kamome Shirahama</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3486,31 +3485,31 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O37" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="P37" t="n">
-        <v>4.875</v>
+        <v>4.3125</v>
       </c>
       <c r="Q37" t="n">
         <v>4</v>
@@ -3527,17 +3526,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Final Fantasy IX</t>
+          <t>Harry Potter and the Prisoner of Azkaban</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3557,13 +3556,13 @@
         <v>1</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K38" t="n">
         <v>2</v>
       </c>
       <c r="L38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
         <v>2</v>
@@ -3572,10 +3571,10 @@
         <v>3</v>
       </c>
       <c r="O38" t="n">
-        <v>1.5</v>
+        <v>1.35</v>
       </c>
       <c r="P38" t="n">
-        <v>4.875</v>
+        <v>4.5375</v>
       </c>
       <c r="Q38" t="n">
         <v>4</v>
@@ -3592,17 +3591,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Tales from Earthsea</t>
+          <t>Grimgar: Ashes and Illusions</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Light Novels / Anime</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Gorō Miyazaki</t>
+          <t>Ao Jyumonji</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3631,16 +3630,16 @@
         <v>2</v>
       </c>
       <c r="M39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N39" t="n">
         <v>2</v>
       </c>
       <c r="O39" t="n">
-        <v>1.55</v>
+        <v>1.4</v>
       </c>
       <c r="P39" t="n">
-        <v>4.9875</v>
+        <v>4.65</v>
       </c>
       <c r="Q39" t="n">
         <v>4</v>
@@ -3653,26 +3652,26 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Dragonlance</t>
+          <t>Avatar: The Last Airbender</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Novels / Games</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Margaret Weis / Tracy Hickman</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3682,7 +3681,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H40" t="n">
@@ -3695,7 +3694,7 @@
         <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L40" t="n">
         <v>2</v>
@@ -3704,40 +3703,45 @@
         <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O40" t="n">
-        <v>1.65</v>
+        <v>1.4</v>
       </c>
       <c r="P40" t="n">
-        <v>5.2125</v>
+        <v>4.65</v>
       </c>
       <c r="Q40" t="n">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Tier v1 era 3</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V: Skyrim</t>
+          <t>Earthsea</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Bethesda Game Studios</t>
+          <t>Ursula K. Le Guin</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3757,52 +3761,52 @@
         <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
         <v>2</v>
       </c>
       <c r="L41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N41" t="n">
         <v>2</v>
       </c>
       <c r="O41" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="P41" t="n">
-        <v>5.325</v>
+        <v>4.65</v>
       </c>
       <c r="Q41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>Final Fantasy XII</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3816,10 +3820,10 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J42" t="n">
         <v>1</v>
@@ -3828,7 +3832,7 @@
         <v>2</v>
       </c>
       <c r="L42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M42" t="n">
         <v>2</v>
@@ -3837,37 +3841,42 @@
         <v>2</v>
       </c>
       <c r="O42" t="n">
-        <v>1.85</v>
+        <v>1.4</v>
       </c>
       <c r="P42" t="n">
-        <v>5.6625</v>
+        <v>4.65</v>
       </c>
       <c r="Q42" t="n">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>Fullmetal Alchemist: Brotherhood</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Hiromu Arakawa</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3881,63 +3890,58 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N43" t="n">
+        <v>3</v>
+      </c>
+      <c r="O43" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P43" t="n">
+        <v>4.875</v>
+      </c>
+      <c r="Q43" t="n">
         <v>4</v>
-      </c>
-      <c r="O43" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="P43" t="n">
-        <v>5.775</v>
-      </c>
-      <c r="Q43" t="n">
-        <v>5</v>
-      </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Tier v1 era 6</t>
-        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>The Boy and the Heron</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3957,13 +3961,13 @@
         <v>2</v>
       </c>
       <c r="J44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M44" t="n">
         <v>2</v>
@@ -3972,37 +3976,37 @@
         <v>3</v>
       </c>
       <c r="O44" t="n">
-        <v>2.1</v>
+        <v>1.5</v>
       </c>
       <c r="P44" t="n">
-        <v>6.225</v>
+        <v>4.875</v>
       </c>
       <c r="Q44" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy IX</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4016,16 +4020,16 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L45" t="n">
         <v>2</v>
@@ -4034,45 +4038,40 @@
         <v>2</v>
       </c>
       <c r="N45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O45" t="n">
-        <v>2.15</v>
+        <v>1.5</v>
       </c>
       <c r="P45" t="n">
-        <v>6.3375</v>
+        <v>4.875</v>
       </c>
       <c r="Q45" t="n">
-        <v>6</v>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Tales from Earthsea</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Studio Ghibli / Gorō Miyazaki</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4089,13 +4088,13 @@
         <v>2</v>
       </c>
       <c r="I46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L46" t="n">
         <v>2</v>
@@ -4104,40 +4103,45 @@
         <v>2</v>
       </c>
       <c r="N46" t="n">
+        <v>2</v>
+      </c>
+      <c r="O46" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="P46" t="n">
+        <v>4.9875</v>
+      </c>
+      <c r="Q46" t="n">
         <v>4</v>
       </c>
-      <c r="O46" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="P46" t="n">
-        <v>6.45</v>
-      </c>
-      <c r="Q46" t="n">
-        <v>6</v>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Adventure Time</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>TV / Comics</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Pendleton Ward</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -4151,16 +4155,16 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L47" t="n">
         <v>2</v>
@@ -4169,45 +4173,40 @@
         <v>2</v>
       </c>
       <c r="N47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O47" t="n">
-        <v>2.25</v>
+        <v>1.55</v>
       </c>
       <c r="P47" t="n">
-        <v>6.5625</v>
+        <v>4.9875</v>
       </c>
       <c r="Q47" t="n">
-        <v>6</v>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Dragonlance</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Novels / Games</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Margaret Weis / Tracy Hickman</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4224,10 +4223,10 @@
         <v>2</v>
       </c>
       <c r="I48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K48" t="n">
         <v>2</v>
@@ -4236,48 +4235,43 @@
         <v>2</v>
       </c>
       <c r="M48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N48" t="n">
         <v>3</v>
       </c>
       <c r="O48" t="n">
-        <v>2.25</v>
+        <v>1.65</v>
       </c>
       <c r="P48" t="n">
-        <v>6.5625</v>
+        <v>5.2125</v>
       </c>
       <c r="Q48" t="n">
-        <v>6</v>
-      </c>
-      <c r="R48" t="inlineStr">
-        <is>
-          <t>Tier v1 era 7</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>Harry Potter and the Goblet of Fire</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -4291,19 +4285,19 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J49" t="n">
         <v>2</v>
       </c>
       <c r="K49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M49" t="n">
         <v>2</v>
@@ -4312,37 +4306,37 @@
         <v>3</v>
       </c>
       <c r="O49" t="n">
-        <v>2.25</v>
+        <v>1.65</v>
       </c>
       <c r="P49" t="n">
-        <v>6.5625</v>
+        <v>5.2125</v>
       </c>
       <c r="Q49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Elantris</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4359,55 +4353,55 @@
         <v>2</v>
       </c>
       <c r="I50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L50" t="n">
         <v>2</v>
       </c>
       <c r="M50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N50" t="n">
         <v>3</v>
       </c>
       <c r="O50" t="n">
-        <v>2.25</v>
+        <v>1.65</v>
       </c>
       <c r="P50" t="n">
-        <v>6.5625</v>
+        <v>5.2125</v>
       </c>
       <c r="Q50" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>The Elder Scrolls V: Skyrim</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Bethesda Game Studios</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4421,10 +4415,10 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J51" t="n">
         <v>2</v>
@@ -4433,51 +4427,46 @@
         <v>2</v>
       </c>
       <c r="L51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M51" t="n">
         <v>2</v>
       </c>
       <c r="N51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O51" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="P51" t="n">
-        <v>6.9</v>
+        <v>5.325</v>
       </c>
       <c r="Q51" t="n">
-        <v>6</v>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Silmarillion &amp; Great Tales</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Books</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4491,58 +4480,58 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" t="n">
         <v>2</v>
       </c>
       <c r="L52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O52" t="n">
-        <v>2.65</v>
+        <v>1.7</v>
       </c>
       <c r="P52" t="n">
-        <v>7.4625</v>
+        <v>5.325</v>
       </c>
       <c r="Q52" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4556,58 +4545,58 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O53" t="n">
-        <v>3.1</v>
+        <v>1.85</v>
       </c>
       <c r="P53" t="n">
-        <v>8.475</v>
+        <v>5.6625</v>
       </c>
       <c r="Q53" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4621,58 +4610,63 @@
         </is>
       </c>
       <c r="H54" t="n">
+        <v>2</v>
+      </c>
+      <c r="I54" t="n">
+        <v>2</v>
+      </c>
+      <c r="J54" t="n">
+        <v>2</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1</v>
+      </c>
+      <c r="L54" t="n">
+        <v>1</v>
+      </c>
+      <c r="M54" t="n">
+        <v>2</v>
+      </c>
+      <c r="N54" t="n">
         <v>4</v>
       </c>
-      <c r="I54" t="n">
-        <v>3</v>
-      </c>
-      <c r="J54" t="n">
-        <v>3</v>
-      </c>
-      <c r="K54" t="n">
-        <v>3</v>
-      </c>
-      <c r="L54" t="n">
-        <v>3</v>
-      </c>
-      <c r="M54" t="n">
-        <v>3</v>
-      </c>
-      <c r="N54" t="n">
-        <v>3</v>
-      </c>
       <c r="O54" t="n">
-        <v>3.15</v>
+        <v>1.9</v>
       </c>
       <c r="P54" t="n">
-        <v>8.5875</v>
+        <v>5.775</v>
       </c>
       <c r="Q54" t="n">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4686,58 +4680,58 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J55" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O55" t="n">
-        <v>3.25</v>
+        <v>2.1</v>
       </c>
       <c r="P55" t="n">
-        <v>8.8125</v>
+        <v>6.225</v>
       </c>
       <c r="Q55" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4751,98 +4745,964 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I56" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J56" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O56" t="n">
-        <v>3.7</v>
+        <v>2.1</v>
       </c>
       <c r="P56" t="n">
-        <v>9.824999999999999</v>
+        <v>6.225</v>
       </c>
       <c r="Q56" t="n">
-        <v>9</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="R56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
+        <v>6</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Shin Sekai Yori (From the New World)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Novel / Anime</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Yusuke Kishi</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>2</v>
+      </c>
+      <c r="I57" t="n">
+        <v>2</v>
+      </c>
+      <c r="J57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K57" t="n">
+        <v>3</v>
+      </c>
+      <c r="L57" t="n">
+        <v>2</v>
+      </c>
+      <c r="M57" t="n">
+        <v>2</v>
+      </c>
+      <c r="N57" t="n">
+        <v>2</v>
+      </c>
+      <c r="O57" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="P57" t="n">
+        <v>6.3375</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>6</v>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>6</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Made in Abyss</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Manga / Anime</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Akihito Tsukushi</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>2</v>
+      </c>
+      <c r="I58" t="n">
+        <v>2</v>
+      </c>
+      <c r="J58" t="n">
+        <v>2</v>
+      </c>
+      <c r="K58" t="n">
+        <v>2</v>
+      </c>
+      <c r="L58" t="n">
+        <v>2</v>
+      </c>
+      <c r="M58" t="n">
+        <v>2</v>
+      </c>
+      <c r="N58" t="n">
+        <v>4</v>
+      </c>
+      <c r="O58" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="P58" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>6</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Fullmetal Alchemist (2003)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Anime</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Hiromu Arakawa / Bones</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>3</v>
+      </c>
+      <c r="I59" t="n">
+        <v>2</v>
+      </c>
+      <c r="J59" t="n">
+        <v>2</v>
+      </c>
+      <c r="K59" t="n">
+        <v>2</v>
+      </c>
+      <c r="L59" t="n">
+        <v>2</v>
+      </c>
+      <c r="M59" t="n">
+        <v>2</v>
+      </c>
+      <c r="N59" t="n">
+        <v>3</v>
+      </c>
+      <c r="O59" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="P59" t="n">
+        <v>6.5625</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>6</v>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>6</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>The Saga of Tanya the Evil</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Light Novels / Manga / Anime / Film</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Carlo Zen</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>2</v>
+      </c>
+      <c r="I60" t="n">
+        <v>2</v>
+      </c>
+      <c r="J60" t="n">
+        <v>3</v>
+      </c>
+      <c r="K60" t="n">
+        <v>2</v>
+      </c>
+      <c r="L60" t="n">
+        <v>2</v>
+      </c>
+      <c r="M60" t="n">
+        <v>2</v>
+      </c>
+      <c r="N60" t="n">
+        <v>3</v>
+      </c>
+      <c r="O60" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="P60" t="n">
+        <v>6.5625</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>6</v>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Claymore</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Manga / Anime</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Norihiro Yagi</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>2</v>
+      </c>
+      <c r="I61" t="n">
+        <v>2</v>
+      </c>
+      <c r="J61" t="n">
+        <v>2</v>
+      </c>
+      <c r="K61" t="n">
+        <v>3</v>
+      </c>
+      <c r="L61" t="n">
+        <v>2</v>
+      </c>
+      <c r="M61" t="n">
+        <v>2</v>
+      </c>
+      <c r="N61" t="n">
+        <v>3</v>
+      </c>
+      <c r="O61" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="P61" t="n">
+        <v>6.5625</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>6</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Final Fantasy XVI</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Video Game</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Square Enix</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>2</v>
+      </c>
+      <c r="I62" t="n">
+        <v>2</v>
+      </c>
+      <c r="J62" t="n">
+        <v>2</v>
+      </c>
+      <c r="K62" t="n">
+        <v>3</v>
+      </c>
+      <c r="L62" t="n">
+        <v>2</v>
+      </c>
+      <c r="M62" t="n">
+        <v>2</v>
+      </c>
+      <c r="N62" t="n">
+        <v>3</v>
+      </c>
+      <c r="O62" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="P62" t="n">
+        <v>6.5625</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>6</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Dark Souls I–III</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Video Games</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>3</v>
+      </c>
+      <c r="I63" t="n">
+        <v>2</v>
+      </c>
+      <c r="J63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L63" t="n">
+        <v>3</v>
+      </c>
+      <c r="M63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N63" t="n">
+        <v>3</v>
+      </c>
+      <c r="O63" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P63" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>6</v>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>6</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>The Stormlight Archive</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Novels</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Brandon Sanderson</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>2</v>
+      </c>
+      <c r="I64" t="n">
+        <v>2</v>
+      </c>
+      <c r="J64" t="n">
+        <v>2</v>
+      </c>
+      <c r="K64" t="n">
+        <v>3</v>
+      </c>
+      <c r="L64" t="n">
+        <v>3</v>
+      </c>
+      <c r="M64" t="n">
+        <v>2</v>
+      </c>
+      <c r="N64" t="n">
+        <v>3</v>
+      </c>
+      <c r="O64" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P64" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>7</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Extreme Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Berserk</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Manga / Anime / Films</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Kentaro Miura</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>3</v>
+      </c>
+      <c r="I65" t="n">
+        <v>2</v>
+      </c>
+      <c r="J65" t="n">
+        <v>3</v>
+      </c>
+      <c r="K65" t="n">
+        <v>2</v>
+      </c>
+      <c r="L65" t="n">
+        <v>3</v>
+      </c>
+      <c r="M65" t="n">
+        <v>2</v>
+      </c>
+      <c r="N65" t="n">
+        <v>4</v>
+      </c>
+      <c r="O65" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="P65" t="n">
+        <v>7.4625</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>8</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>A Song of Ice and Fire</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Novels / TV</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>George R. R. Martin</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>3</v>
+      </c>
+      <c r="I66" t="n">
+        <v>3</v>
+      </c>
+      <c r="J66" t="n">
+        <v>3</v>
+      </c>
+      <c r="K66" t="n">
+        <v>3</v>
+      </c>
+      <c r="L66" t="n">
+        <v>3</v>
+      </c>
+      <c r="M66" t="n">
+        <v>3</v>
+      </c>
+      <c r="N66" t="n">
+        <v>4</v>
+      </c>
+      <c r="O66" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="P66" t="n">
+        <v>8.475</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>8</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Elden Ring</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Video Game</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>4</v>
+      </c>
+      <c r="I67" t="n">
+        <v>3</v>
+      </c>
+      <c r="J67" t="n">
+        <v>3</v>
+      </c>
+      <c r="K67" t="n">
+        <v>3</v>
+      </c>
+      <c r="L67" t="n">
+        <v>3</v>
+      </c>
+      <c r="M67" t="n">
+        <v>3</v>
+      </c>
+      <c r="N67" t="n">
+        <v>3</v>
+      </c>
+      <c r="O67" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="P67" t="n">
+        <v>8.5875</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>8</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Fire Punch</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Tatsuki Fujimoto</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>3</v>
+      </c>
+      <c r="I68" t="n">
+        <v>3</v>
+      </c>
+      <c r="J68" t="n">
+        <v>4</v>
+      </c>
+      <c r="K68" t="n">
+        <v>3</v>
+      </c>
+      <c r="L68" t="n">
+        <v>3</v>
+      </c>
+      <c r="M68" t="n">
+        <v>3</v>
+      </c>
+      <c r="N68" t="n">
+        <v>4</v>
+      </c>
+      <c r="O68" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="P68" t="n">
+        <v>8.8125</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>9</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>The First Law</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Novels</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Joe Abercrombie</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H69" t="n">
+        <v>4</v>
+      </c>
+      <c r="I69" t="n">
+        <v>4</v>
+      </c>
+      <c r="J69" t="n">
+        <v>4</v>
+      </c>
+      <c r="K69" t="n">
+        <v>4</v>
+      </c>
+      <c r="L69" t="n">
+        <v>3</v>
+      </c>
+      <c r="M69" t="n">
+        <v>3</v>
+      </c>
+      <c r="N69" t="n">
+        <v>4</v>
+      </c>
+      <c r="O69" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P69" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
         <v>10</v>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>Very Extreme Grimdark</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>Warhammer 40,000</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>Tabletop / Novels / Games / Animation</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>Games Workshop</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H57" t="n">
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
         <v>4</v>
       </c>
-      <c r="I57" t="n">
+      <c r="I70" t="n">
         <v>4</v>
       </c>
-      <c r="J57" t="n">
+      <c r="J70" t="n">
         <v>4</v>
       </c>
-      <c r="K57" t="n">
+      <c r="K70" t="n">
         <v>4</v>
       </c>
-      <c r="L57" t="n">
+      <c r="L70" t="n">
         <v>4</v>
       </c>
-      <c r="M57" t="n">
+      <c r="M70" t="n">
         <v>4</v>
       </c>
-      <c r="N57" t="n">
+      <c r="N70" t="n">
         <v>4</v>
       </c>
-      <c r="O57" t="n">
+      <c r="O70" t="n">
         <v>4</v>
       </c>
-      <c r="P57" t="n">
+      <c r="P70" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q57" t="n">
+      <c r="Q70" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4892,7 +5752,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -4918,7 +5778,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -4931,7 +5791,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -4944,7 +5804,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -4957,7 +5817,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -5015,7 +5875,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 56 of 87 works in the full catalog (work in progress).</t>
+          <t>Total scored: 69 of 89 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update scoring for Harry Potter and the Order of the Phoenix in SCORING_RECORD.md, reflecting a new tier 5 classification based on detailed analysis of structural despair, heroism, and corruption. Adjustments made to maintain thematic consistency with previous works, ensuring accurate representation of narrative complexities. Update ADDITIONS_LOG.md to reflect the new scoring outcome.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4647,26 +4647,26 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4692,7 +4692,7 @@
         <v>2</v>
       </c>
       <c r="L55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M55" t="n">
         <v>2</v>
@@ -4701,14 +4701,15 @@
         <v>3</v>
       </c>
       <c r="O55" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P55" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q55" t="n">
-        <v>6</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="R55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4721,17 +4722,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4745,16 +4746,16 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L56" t="n">
         <v>2</v>
@@ -4774,7 +4775,6 @@
       <c r="Q56" t="n">
         <v>6</v>
       </c>
-      <c r="R56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4787,17 +4787,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4811,13 +4811,13 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K57" t="n">
         <v>3</v>
@@ -4829,21 +4829,16 @@
         <v>2</v>
       </c>
       <c r="N57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O57" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P57" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q57" t="n">
         <v>6</v>
-      </c>
-      <c r="R57" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="58">
@@ -4857,17 +4852,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4890,7 +4885,7 @@
         <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L58" t="n">
         <v>2</v>
@@ -4899,16 +4894,21 @@
         <v>2</v>
       </c>
       <c r="N58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O58" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P58" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q58" t="n">
         <v>6</v>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -4922,17 +4922,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4946,7 +4946,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I59" t="n">
         <v>2</v>
@@ -4964,21 +4964,16 @@
         <v>2</v>
       </c>
       <c r="N59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O59" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P59" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q59" t="n">
         <v>6</v>
-      </c>
-      <c r="R59" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="60">
@@ -4992,17 +4987,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5016,13 +5011,13 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I60" t="n">
         <v>2</v>
       </c>
       <c r="J60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K60" t="n">
         <v>2</v>
@@ -5047,7 +5042,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -5062,17 +5057,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5092,10 +5087,10 @@
         <v>2</v>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L61" t="n">
         <v>2</v>
@@ -5114,6 +5109,11 @@
       </c>
       <c r="Q61" t="n">
         <v>6</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -5127,17 +5127,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5192,17 +5192,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5216,7 +5216,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I63" t="n">
         <v>2</v>
@@ -5225,10 +5225,10 @@
         <v>2</v>
       </c>
       <c r="K63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M63" t="n">
         <v>2</v>
@@ -5237,18 +5237,13 @@
         <v>3</v>
       </c>
       <c r="O63" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P63" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q63" t="n">
         <v>6</v>
-      </c>
-      <c r="R63" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="64">
@@ -5262,17 +5257,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5286,7 +5281,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I64" t="n">
         <v>2</v>
@@ -5295,7 +5290,7 @@
         <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L64" t="n">
         <v>3</v>
@@ -5315,29 +5310,34 @@
       <c r="Q64" t="n">
         <v>6</v>
       </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5351,16 +5351,16 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I65" t="n">
         <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L65" t="n">
         <v>3</v>
@@ -5369,40 +5369,40 @@
         <v>2</v>
       </c>
       <c r="N65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O65" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P65" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q65" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5419,31 +5419,31 @@
         <v>3</v>
       </c>
       <c r="I66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J66" t="n">
         <v>3</v>
       </c>
       <c r="K66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L66" t="n">
         <v>3</v>
       </c>
       <c r="M66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N66" t="n">
         <v>4</v>
       </c>
       <c r="O66" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P66" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q66" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="67">
@@ -5457,17 +5457,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5481,31 +5481,31 @@
         </is>
       </c>
       <c r="H67" t="n">
+        <v>3</v>
+      </c>
+      <c r="I67" t="n">
+        <v>3</v>
+      </c>
+      <c r="J67" t="n">
+        <v>3</v>
+      </c>
+      <c r="K67" t="n">
+        <v>3</v>
+      </c>
+      <c r="L67" t="n">
+        <v>3</v>
+      </c>
+      <c r="M67" t="n">
+        <v>3</v>
+      </c>
+      <c r="N67" t="n">
         <v>4</v>
       </c>
-      <c r="I67" t="n">
-        <v>3</v>
-      </c>
-      <c r="J67" t="n">
-        <v>3</v>
-      </c>
-      <c r="K67" t="n">
-        <v>3</v>
-      </c>
-      <c r="L67" t="n">
-        <v>3</v>
-      </c>
-      <c r="M67" t="n">
-        <v>3</v>
-      </c>
-      <c r="N67" t="n">
-        <v>3</v>
-      </c>
       <c r="O67" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P67" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q67" t="n">
         <v>8</v>
@@ -5522,17 +5522,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5546,13 +5546,13 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I68" t="n">
         <v>3</v>
       </c>
       <c r="J68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K68" t="n">
         <v>3</v>
@@ -5564,13 +5564,13 @@
         <v>3</v>
       </c>
       <c r="N68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O68" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P68" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q68" t="n">
         <v>8</v>
@@ -5578,26 +5578,26 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5611,16 +5611,16 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J69" t="n">
         <v>4</v>
       </c>
       <c r="K69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L69" t="n">
         <v>3</v>
@@ -5632,37 +5632,37 @@
         <v>4</v>
       </c>
       <c r="O69" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P69" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q69" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5688,21 +5688,86 @@
         <v>4</v>
       </c>
       <c r="L70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N70" t="n">
         <v>4</v>
       </c>
       <c r="O70" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P70" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>10</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H71" t="n">
         <v>4</v>
       </c>
-      <c r="P70" t="n">
+      <c r="I71" t="n">
+        <v>4</v>
+      </c>
+      <c r="J71" t="n">
+        <v>4</v>
+      </c>
+      <c r="K71" t="n">
+        <v>4</v>
+      </c>
+      <c r="L71" t="n">
+        <v>4</v>
+      </c>
+      <c r="M71" t="n">
+        <v>4</v>
+      </c>
+      <c r="N71" t="n">
+        <v>4</v>
+      </c>
+      <c r="O71" t="n">
+        <v>4</v>
+      </c>
+      <c r="P71" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q70" t="n">
+      <c r="Q71" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5804,7 +5869,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -5875,7 +5940,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 69 of 89 works in the full catalog (work in progress).</t>
+          <t>Total scored: 70 of 89 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update scoring for Harry Potter and the Half-Blood Prince in SCORING_RECORD.md, establishing a new tier 5 classification with a final score of 5.8875. Adjustments made to various criteria, including structural despair and moral cynicism, to accurately reflect the book's thematic complexities. Update ADDITIONS_LOG.md to include the new tier status and rationale for scoring decisions.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:R72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4709,30 +4709,29 @@
       <c r="Q55" t="n">
         <v>5</v>
       </c>
-      <c r="R55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4755,7 +4754,7 @@
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L56" t="n">
         <v>2</v>
@@ -4767,14 +4766,15 @@
         <v>3</v>
       </c>
       <c r="O56" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P56" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q56" t="n">
-        <v>6</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="R56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4787,17 +4787,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4811,16 +4811,16 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L57" t="n">
         <v>2</v>
@@ -4852,17 +4852,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4876,13 +4876,13 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K58" t="n">
         <v>3</v>
@@ -4894,21 +4894,16 @@
         <v>2</v>
       </c>
       <c r="N58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O58" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P58" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q58" t="n">
         <v>6</v>
-      </c>
-      <c r="R58" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="59">
@@ -4922,17 +4917,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4955,7 +4950,7 @@
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L59" t="n">
         <v>2</v>
@@ -4964,16 +4959,21 @@
         <v>2</v>
       </c>
       <c r="N59" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O59" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P59" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q59" t="n">
         <v>6</v>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -4987,17 +4987,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5011,7 +5011,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I60" t="n">
         <v>2</v>
@@ -5029,21 +5029,16 @@
         <v>2</v>
       </c>
       <c r="N60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O60" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P60" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q60" t="n">
         <v>6</v>
-      </c>
-      <c r="R60" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="61">
@@ -5057,17 +5052,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5081,13 +5076,13 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I61" t="n">
         <v>2</v>
       </c>
       <c r="J61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K61" t="n">
         <v>2</v>
@@ -5112,7 +5107,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -5127,17 +5122,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5157,10 +5152,10 @@
         <v>2</v>
       </c>
       <c r="J62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L62" t="n">
         <v>2</v>
@@ -5179,6 +5174,11 @@
       </c>
       <c r="Q62" t="n">
         <v>6</v>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -5192,17 +5192,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5257,17 +5257,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I64" t="n">
         <v>2</v>
@@ -5290,10 +5290,10 @@
         <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M64" t="n">
         <v>2</v>
@@ -5302,18 +5302,13 @@
         <v>3</v>
       </c>
       <c r="O64" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P64" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q64" t="n">
         <v>6</v>
-      </c>
-      <c r="R64" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="65">
@@ -5327,17 +5322,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5351,7 +5346,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I65" t="n">
         <v>2</v>
@@ -5360,7 +5355,7 @@
         <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L65" t="n">
         <v>3</v>
@@ -5380,29 +5375,34 @@
       <c r="Q65" t="n">
         <v>6</v>
       </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5416,16 +5416,16 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I66" t="n">
         <v>2</v>
       </c>
       <c r="J66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L66" t="n">
         <v>3</v>
@@ -5434,40 +5434,40 @@
         <v>2</v>
       </c>
       <c r="N66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O66" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P66" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q66" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5484,31 +5484,31 @@
         <v>3</v>
       </c>
       <c r="I67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J67" t="n">
         <v>3</v>
       </c>
       <c r="K67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L67" t="n">
         <v>3</v>
       </c>
       <c r="M67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N67" t="n">
         <v>4</v>
       </c>
       <c r="O67" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P67" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="68">
@@ -5522,17 +5522,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5546,31 +5546,31 @@
         </is>
       </c>
       <c r="H68" t="n">
+        <v>3</v>
+      </c>
+      <c r="I68" t="n">
+        <v>3</v>
+      </c>
+      <c r="J68" t="n">
+        <v>3</v>
+      </c>
+      <c r="K68" t="n">
+        <v>3</v>
+      </c>
+      <c r="L68" t="n">
+        <v>3</v>
+      </c>
+      <c r="M68" t="n">
+        <v>3</v>
+      </c>
+      <c r="N68" t="n">
         <v>4</v>
       </c>
-      <c r="I68" t="n">
-        <v>3</v>
-      </c>
-      <c r="J68" t="n">
-        <v>3</v>
-      </c>
-      <c r="K68" t="n">
-        <v>3</v>
-      </c>
-      <c r="L68" t="n">
-        <v>3</v>
-      </c>
-      <c r="M68" t="n">
-        <v>3</v>
-      </c>
-      <c r="N68" t="n">
-        <v>3</v>
-      </c>
       <c r="O68" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P68" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q68" t="n">
         <v>8</v>
@@ -5587,17 +5587,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5611,13 +5611,13 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I69" t="n">
         <v>3</v>
       </c>
       <c r="J69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K69" t="n">
         <v>3</v>
@@ -5629,13 +5629,13 @@
         <v>3</v>
       </c>
       <c r="N69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O69" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P69" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q69" t="n">
         <v>8</v>
@@ -5643,26 +5643,26 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5676,16 +5676,16 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J70" t="n">
         <v>4</v>
       </c>
       <c r="K70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L70" t="n">
         <v>3</v>
@@ -5697,37 +5697,37 @@
         <v>4</v>
       </c>
       <c r="O70" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P70" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q70" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5753,21 +5753,86 @@
         <v>4</v>
       </c>
       <c r="L71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N71" t="n">
         <v>4</v>
       </c>
       <c r="O71" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P71" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>10</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
         <v>4</v>
       </c>
-      <c r="P71" t="n">
+      <c r="I72" t="n">
+        <v>4</v>
+      </c>
+      <c r="J72" t="n">
+        <v>4</v>
+      </c>
+      <c r="K72" t="n">
+        <v>4</v>
+      </c>
+      <c r="L72" t="n">
+        <v>4</v>
+      </c>
+      <c r="M72" t="n">
+        <v>4</v>
+      </c>
+      <c r="N72" t="n">
+        <v>4</v>
+      </c>
+      <c r="O72" t="n">
+        <v>4</v>
+      </c>
+      <c r="P72" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q71" t="n">
+      <c r="Q72" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5869,7 +5934,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -5940,7 +6005,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 70 of 89 works in the full catalog (work in progress).</t>
+          <t>Total scored: 71 of 89 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ADDITIONS_LOG.md and SCORING_RECORD.md with detailed rescoring for multiple works, including Harry Potter and the Deathly Hallows, Mistborn, Nausicaä of the Valley of the Wind, and the Neverwinter Nights & Baldur's Gate series. Adjust tiers and scores based on new analyses, reflecting thematic depth and narrative complexities. Split Neverwinter Nights & Baldur's Gate into four separate entries for more accurate representation of their individual content severity. Add new entries for Dark Sun, Alice in Wonderland, The Wizard of Oz, and Wicked, expanding the catalog of works.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R72"/>
+  <dimension ref="A1:R80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2603,17 +2603,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dungeon Meshi</t>
+          <t>Neverwinter Nights</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Ryoko Kui</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2630,10 +2630,10 @@
         <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>1</v>
@@ -2645,18 +2645,22 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O24" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="P24" t="n">
-        <v>3.3</v>
+        <v>3.075</v>
       </c>
       <c r="Q24" t="n">
         <v>3</v>
       </c>
-      <c r="R24" s="5" t="n"/>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2669,17 +2673,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Cormyr</t>
+          <t>Dungeon Meshi</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Ed Greenwood / Jeff Grubb</t>
+          <t>Ryoko Kui</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2699,13 +2703,13 @@
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
@@ -2735,17 +2739,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Final Fantasy IV</t>
+          <t>Cormyr</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Ed Greenwood / Jeff Grubb</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2759,31 +2763,31 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K26" t="n">
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O26" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="P26" t="n">
-        <v>3.525</v>
+        <v>3.3</v>
       </c>
       <c r="Q26" t="n">
         <v>3</v>
@@ -2800,17 +2804,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>The Hobbit</t>
+          <t>Baldur's Gate I</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2830,28 +2834,33 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O27" t="n">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
       <c r="P27" t="n">
-        <v>3.6375</v>
+        <v>3.4125</v>
       </c>
       <c r="Q27" t="n">
         <v>3</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -2865,17 +2874,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Spirited Away</t>
+          <t>Final Fantasy IV</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2892,28 +2901,28 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M28" t="n">
         <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O28" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="P28" t="n">
-        <v>3.6375</v>
+        <v>3.525</v>
       </c>
       <c r="Q28" t="n">
         <v>3</v>
@@ -2931,17 +2940,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Howl's Moving Castle</t>
+          <t>The Hobbit</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2996,17 +3005,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Discworld</t>
+          <t>Spirited Away</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Novels / Games / Comics</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Terry Pratchett</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3016,20 +3025,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
@@ -3038,21 +3047,16 @@
         <v>1</v>
       </c>
       <c r="N30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O30" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="P30" t="n">
-        <v>3.75</v>
+        <v>3.6375</v>
       </c>
       <c r="Q30" t="n">
         <v>3</v>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>Tier v1 era 4</t>
-        </is>
       </c>
     </row>
     <row r="31">
@@ -3066,17 +3070,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>The Lord of the Rings</t>
+          <t>Howl's Moving Castle</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Novels / Films</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3090,7 +3094,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
         <v>1</v>
@@ -3111,10 +3115,10 @@
         <v>2</v>
       </c>
       <c r="O31" t="n">
-        <v>1.1</v>
+        <v>0.95</v>
       </c>
       <c r="P31" t="n">
-        <v>3.975</v>
+        <v>3.6375</v>
       </c>
       <c r="Q31" t="n">
         <v>3</v>
@@ -3131,17 +3135,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Frieren: Beyond Journey's End</t>
+          <t>Discworld</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novels / Games / Comics</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Kanehito Yamada / Tsukasa Abe</t>
+          <t>Terry Pratchett</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3155,34 +3159,39 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I32" t="n">
         <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O32" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="P32" t="n">
-        <v>3.975</v>
+        <v>3.75</v>
       </c>
       <c r="Q32" t="n">
         <v>3</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Tier v1 era 4</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -3196,17 +3205,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Black Clover</t>
+          <t>The Lord of the Rings</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Manga / Anime / Film</t>
+          <t>Novels / Films</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Yūki Tabata</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3220,7 +3229,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I33" t="n">
         <v>1</v>
@@ -3229,13 +3238,13 @@
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N33" t="n">
         <v>2</v>
@@ -3261,17 +3270,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Record of Lodoss War</t>
+          <t>Frieren: Beyond Journey's End</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Novels / Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Ryo Mizuno</t>
+          <t>Kanehito Yamada / Tsukasa Abe</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3281,26 +3290,26 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I34" t="n">
         <v>1</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N34" t="n">
         <v>2</v>
@@ -3326,17 +3335,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Final Fantasy II</t>
+          <t>Black Clover</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Yūki Tabata</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3356,16 +3365,16 @@
         <v>1</v>
       </c>
       <c r="J35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
         <v>2</v>
@@ -3379,34 +3388,29 @@
       <c r="Q35" t="n">
         <v>3</v>
       </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>The NeverEnding Story</t>
+          <t>Record of Lodoss War</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Novels / Anime</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Michael Ende</t>
+          <t>Ryo Mizuno</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3420,7 +3424,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I36" t="n">
         <v>1</v>
@@ -3429,7 +3433,7 @@
         <v>1</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L36" t="n">
         <v>2</v>
@@ -3438,40 +3442,40 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O36" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="P36" t="n">
-        <v>4.2</v>
+        <v>3.975</v>
       </c>
       <c r="Q36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Witch Hat Atelier</t>
+          <t>Final Fantasy II</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Kamome Shirahama</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3491,52 +3495,57 @@
         <v>1</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L37" t="n">
         <v>2</v>
       </c>
       <c r="M37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N37" t="n">
         <v>2</v>
       </c>
       <c r="O37" t="n">
-        <v>1.25</v>
+        <v>1.1</v>
       </c>
       <c r="P37" t="n">
-        <v>4.3125</v>
+        <v>3.975</v>
       </c>
       <c r="Q37" t="n">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Balanced, Bittersweet Hopepunk or Melancholic Fantasy</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Harry Potter and the Prisoner of Azkaban</t>
+          <t>Nausicaä of the Valley of the Wind</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3550,7 +3559,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I38" t="n">
         <v>1</v>
@@ -3559,25 +3568,25 @@
         <v>1</v>
       </c>
       <c r="K38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L38" t="n">
         <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O38" t="n">
-        <v>1.35</v>
+        <v>1.1</v>
       </c>
       <c r="P38" t="n">
-        <v>4.5375</v>
+        <v>3.975</v>
       </c>
       <c r="Q38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
@@ -3591,17 +3600,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Grimgar: Ashes and Illusions</t>
+          <t>The NeverEnding Story</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Light Novels / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Ao Jyumonji</t>
+          <t>Michael Ende</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3624,30 +3633,25 @@
         <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
         <v>2</v>
       </c>
       <c r="M39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O39" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="P39" t="n">
-        <v>4.65</v>
+        <v>4.2</v>
       </c>
       <c r="Q39" t="n">
         <v>4</v>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="40">
@@ -3661,17 +3665,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Avatar: The Last Airbender</t>
+          <t>Witch Hat Atelier</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>Kamome Shirahama</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3681,20 +3685,20 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I40" t="n">
         <v>1</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L40" t="n">
         <v>2</v>
@@ -3706,18 +3710,13 @@
         <v>2</v>
       </c>
       <c r="O40" t="n">
-        <v>1.4</v>
+        <v>1.25</v>
       </c>
       <c r="P40" t="n">
-        <v>4.65</v>
+        <v>4.3125</v>
       </c>
       <c r="Q40" t="n">
         <v>4</v>
-      </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>Tier v1 era 3</t>
-        </is>
       </c>
     </row>
     <row r="41">
@@ -3731,17 +3730,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Earthsea</t>
+          <t>Baldur's Gate II: Shadows of Amn</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Ursula K. Le Guin</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3755,19 +3754,19 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I41" t="n">
         <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" t="n">
         <v>2</v>
       </c>
       <c r="L41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M41" t="n">
         <v>1</v>
@@ -3776,13 +3775,18 @@
         <v>2</v>
       </c>
       <c r="O41" t="n">
-        <v>1.4</v>
+        <v>1.25</v>
       </c>
       <c r="P41" t="n">
-        <v>4.65</v>
+        <v>4.3125</v>
       </c>
       <c r="Q41" t="n">
         <v>4</v>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -3796,17 +3800,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Final Fantasy XII</t>
+          <t>Harry Potter and the Prisoner of Azkaban</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3832,27 +3836,22 @@
         <v>2</v>
       </c>
       <c r="L42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M42" t="n">
         <v>2</v>
       </c>
       <c r="N42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O42" t="n">
-        <v>1.4</v>
+        <v>1.35</v>
       </c>
       <c r="P42" t="n">
-        <v>4.65</v>
+        <v>4.5375</v>
       </c>
       <c r="Q42" t="n">
         <v>4</v>
-      </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
-        </is>
       </c>
     </row>
     <row r="43">
@@ -3866,17 +3865,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist: Brotherhood</t>
+          <t>Grimgar: Ashes and Illusions</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Anime</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa</t>
+          <t>Ao Jyumonji</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3890,7 +3889,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I43" t="n">
         <v>1</v>
@@ -3899,7 +3898,7 @@
         <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L43" t="n">
         <v>2</v>
@@ -3908,16 +3907,21 @@
         <v>1</v>
       </c>
       <c r="N43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O43" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="P43" t="n">
-        <v>4.875</v>
+        <v>4.65</v>
       </c>
       <c r="Q43" t="n">
         <v>4</v>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -3931,17 +3935,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>The Boy and the Heron</t>
+          <t>Avatar: The Last Airbender</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3951,38 +3955,43 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H44" t="n">
         <v>2</v>
       </c>
       <c r="I44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K44" t="n">
         <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O44" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="P44" t="n">
-        <v>4.875</v>
+        <v>4.65</v>
       </c>
       <c r="Q44" t="n">
         <v>4</v>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Tier v1 era 3</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -3996,17 +4005,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Final Fantasy IX</t>
+          <t>Earthsea</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Ursula K. Le Guin</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4020,7 +4029,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I45" t="n">
         <v>1</v>
@@ -4035,16 +4044,16 @@
         <v>2</v>
       </c>
       <c r="M45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O45" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="P45" t="n">
-        <v>4.875</v>
+        <v>4.65</v>
       </c>
       <c r="Q45" t="n">
         <v>4</v>
@@ -4061,17 +4070,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Tales from Earthsea</t>
+          <t>Final Fantasy XII</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Gorō Miyazaki</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4085,7 +4094,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I46" t="n">
         <v>1</v>
@@ -4094,10 +4103,10 @@
         <v>1</v>
       </c>
       <c r="K46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M46" t="n">
         <v>2</v>
@@ -4106,17 +4115,17 @@
         <v>2</v>
       </c>
       <c r="O46" t="n">
-        <v>1.55</v>
+        <v>1.4</v>
       </c>
       <c r="P46" t="n">
-        <v>4.9875</v>
+        <v>4.65</v>
       </c>
       <c r="Q46" t="n">
         <v>4</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Tier v1 era 5</t>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
         </is>
       </c>
     </row>
@@ -4131,17 +4140,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Adventure Time</t>
+          <t>Fullmetal Alchemist: Brotherhood</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>TV / Comics</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Pendleton Ward</t>
+          <t>Hiromu Arakawa</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -4155,7 +4164,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I47" t="n">
         <v>1</v>
@@ -4164,22 +4173,22 @@
         <v>1</v>
       </c>
       <c r="K47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L47" t="n">
         <v>2</v>
       </c>
       <c r="M47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O47" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="P47" t="n">
-        <v>4.9875</v>
+        <v>4.875</v>
       </c>
       <c r="Q47" t="n">
         <v>4</v>
@@ -4187,26 +4196,26 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Dragonlance</t>
+          <t>The Boy and the Heron</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Novels / Games</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Margaret Weis / Tracy Hickman</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4223,55 +4232,55 @@
         <v>2</v>
       </c>
       <c r="I48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N48" t="n">
         <v>3</v>
       </c>
       <c r="O48" t="n">
-        <v>1.65</v>
+        <v>1.5</v>
       </c>
       <c r="P48" t="n">
-        <v>5.2125</v>
+        <v>4.875</v>
       </c>
       <c r="Q48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Harry Potter and the Goblet of Fire</t>
+          <t>Final Fantasy IX</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -4291,13 +4300,13 @@
         <v>1</v>
       </c>
       <c r="J49" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K49" t="n">
         <v>2</v>
       </c>
       <c r="L49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M49" t="n">
         <v>2</v>
@@ -4306,37 +4315,37 @@
         <v>3</v>
       </c>
       <c r="O49" t="n">
-        <v>1.65</v>
+        <v>1.5</v>
       </c>
       <c r="P49" t="n">
-        <v>5.2125</v>
+        <v>4.875</v>
       </c>
       <c r="Q49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Elantris</t>
+          <t>Tales from Earthsea</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>Studio Ghibli / Gorō Miyazaki</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4359,49 +4368,54 @@
         <v>1</v>
       </c>
       <c r="K50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L50" t="n">
         <v>2</v>
       </c>
       <c r="M50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O50" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="P50" t="n">
-        <v>5.2125</v>
+        <v>4.9875</v>
       </c>
       <c r="Q50" t="n">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V: Skyrim</t>
+          <t>Adventure Time</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>TV / Comics</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bethesda Game Studios</t>
+          <t>Pendleton Ward</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4421,13 +4435,13 @@
         <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M51" t="n">
         <v>2</v>
@@ -4436,13 +4450,13 @@
         <v>2</v>
       </c>
       <c r="O51" t="n">
-        <v>1.7</v>
+        <v>1.55</v>
       </c>
       <c r="P51" t="n">
-        <v>5.325</v>
+        <v>4.9875</v>
       </c>
       <c r="Q51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -4456,17 +4470,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>The Silmarillion &amp; Great Tales</t>
+          <t>Dragonlance</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Books</t>
+          <t>Novels / Games</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Margaret Weis / Tracy Hickman</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4486,7 +4500,7 @@
         <v>1</v>
       </c>
       <c r="J52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K52" t="n">
         <v>2</v>
@@ -4498,13 +4512,13 @@
         <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O52" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="P52" t="n">
-        <v>5.325</v>
+        <v>5.2125</v>
       </c>
       <c r="Q52" t="n">
         <v>5</v>
@@ -4521,17 +4535,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>Harry Potter and the Goblet of Fire</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4545,31 +4559,31 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K53" t="n">
         <v>2</v>
       </c>
       <c r="L53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M53" t="n">
         <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O53" t="n">
-        <v>1.85</v>
+        <v>1.65</v>
       </c>
       <c r="P53" t="n">
-        <v>5.6625</v>
+        <v>5.2125</v>
       </c>
       <c r="Q53" t="n">
         <v>5</v>
@@ -4586,17 +4600,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>Elantris</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4613,36 +4627,31 @@
         <v>2</v>
       </c>
       <c r="I54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O54" t="n">
-        <v>1.9</v>
+        <v>1.65</v>
       </c>
       <c r="P54" t="n">
-        <v>5.775</v>
+        <v>5.2125</v>
       </c>
       <c r="Q54" t="n">
         <v>5</v>
-      </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>Tier v1 era 6</t>
-        </is>
       </c>
     </row>
     <row r="55">
@@ -4656,17 +4665,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Baldur's Gate III</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4680,10 +4689,10 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J55" t="n">
         <v>2</v>
@@ -4692,22 +4701,27 @@
         <v>2</v>
       </c>
       <c r="L55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N55" t="n">
         <v>3</v>
       </c>
       <c r="O55" t="n">
-        <v>1.95</v>
+        <v>1.65</v>
       </c>
       <c r="P55" t="n">
-        <v>5.8875</v>
+        <v>5.2125</v>
       </c>
       <c r="Q55" t="n">
         <v>5</v>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -4721,17 +4735,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>The Elder Scrolls V: Skyrim</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Bethesda Game Studios</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4748,56 +4762,55 @@
         <v>2</v>
       </c>
       <c r="I56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J56" t="n">
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M56" t="n">
         <v>2</v>
       </c>
       <c r="N56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O56" t="n">
-        <v>1.95</v>
+        <v>1.7</v>
       </c>
       <c r="P56" t="n">
-        <v>5.8875</v>
+        <v>5.325</v>
       </c>
       <c r="Q56" t="n">
         <v>5</v>
       </c>
-      <c r="R56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>The Silmarillion &amp; Great Tales</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Books</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4814,7 +4827,7 @@
         <v>2</v>
       </c>
       <c r="I57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J57" t="n">
         <v>2</v>
@@ -4826,43 +4839,43 @@
         <v>2</v>
       </c>
       <c r="M57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O57" t="n">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="P57" t="n">
-        <v>6.225</v>
+        <v>5.325</v>
       </c>
       <c r="Q57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>Ranking of Kings</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Sōsuke Tōka</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4876,19 +4889,19 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I58" t="n">
         <v>1</v>
       </c>
       <c r="J58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M58" t="n">
         <v>2</v>
@@ -4897,37 +4910,42 @@
         <v>3</v>
       </c>
       <c r="O58" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="P58" t="n">
-        <v>6.225</v>
+        <v>5.55</v>
       </c>
       <c r="Q58" t="n">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>rescored three times after user corrections on plot details</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4947,10 +4965,10 @@
         <v>2</v>
       </c>
       <c r="J59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L59" t="n">
         <v>2</v>
@@ -4962,42 +4980,37 @@
         <v>2</v>
       </c>
       <c r="O59" t="n">
-        <v>2.15</v>
+        <v>1.85</v>
       </c>
       <c r="P59" t="n">
-        <v>6.3375</v>
+        <v>5.6625</v>
       </c>
       <c r="Q59" t="n">
-        <v>6</v>
-      </c>
-      <c r="R59" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5020,10 +5033,10 @@
         <v>2</v>
       </c>
       <c r="K60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M60" t="n">
         <v>2</v>
@@ -5032,37 +5045,42 @@
         <v>4</v>
       </c>
       <c r="O60" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="P60" t="n">
-        <v>6.45</v>
+        <v>5.775</v>
       </c>
       <c r="Q60" t="n">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5076,7 +5094,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I61" t="n">
         <v>2</v>
@@ -5088,7 +5106,7 @@
         <v>2</v>
       </c>
       <c r="L61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M61" t="n">
         <v>2</v>
@@ -5097,42 +5115,37 @@
         <v>3</v>
       </c>
       <c r="O61" t="n">
-        <v>2.25</v>
+        <v>1.95</v>
       </c>
       <c r="P61" t="n">
-        <v>6.5625</v>
+        <v>5.8875</v>
       </c>
       <c r="Q61" t="n">
-        <v>6</v>
-      </c>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5152,10 +5165,10 @@
         <v>2</v>
       </c>
       <c r="J62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L62" t="n">
         <v>2</v>
@@ -5167,18 +5180,13 @@
         <v>3</v>
       </c>
       <c r="O62" t="n">
-        <v>2.25</v>
+        <v>1.95</v>
       </c>
       <c r="P62" t="n">
-        <v>6.5625</v>
+        <v>5.8875</v>
       </c>
       <c r="Q62" t="n">
-        <v>6</v>
-      </c>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>Tier v1 era 7</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="63">
@@ -5192,17 +5200,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5225,7 +5233,7 @@
         <v>2</v>
       </c>
       <c r="K63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L63" t="n">
         <v>2</v>
@@ -5237,10 +5245,10 @@
         <v>3</v>
       </c>
       <c r="O63" t="n">
-        <v>2.25</v>
+        <v>2.1</v>
       </c>
       <c r="P63" t="n">
-        <v>6.5625</v>
+        <v>6.225</v>
       </c>
       <c r="Q63" t="n">
         <v>6</v>
@@ -5257,12 +5265,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5281,13 +5289,13 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K64" t="n">
         <v>3</v>
@@ -5302,10 +5310,10 @@
         <v>3</v>
       </c>
       <c r="O64" t="n">
-        <v>2.25</v>
+        <v>2.1</v>
       </c>
       <c r="P64" t="n">
-        <v>6.5625</v>
+        <v>6.225</v>
       </c>
       <c r="Q64" t="n">
         <v>6</v>
@@ -5322,17 +5330,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5346,7 +5354,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I65" t="n">
         <v>2</v>
@@ -5355,22 +5363,22 @@
         <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M65" t="n">
         <v>2</v>
       </c>
       <c r="N65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O65" t="n">
-        <v>2.4</v>
+        <v>2.15</v>
       </c>
       <c r="P65" t="n">
-        <v>6.9</v>
+        <v>6.3375</v>
       </c>
       <c r="Q65" t="n">
         <v>6</v>
@@ -5392,17 +5400,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5425,22 +5433,22 @@
         <v>2</v>
       </c>
       <c r="K66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M66" t="n">
         <v>2</v>
       </c>
       <c r="N66" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O66" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="P66" t="n">
-        <v>6.9</v>
+        <v>6.45</v>
       </c>
       <c r="Q66" t="n">
         <v>6</v>
@@ -5448,26 +5456,26 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5487,52 +5495,57 @@
         <v>2</v>
       </c>
       <c r="J67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K67" t="n">
         <v>2</v>
       </c>
       <c r="L67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M67" t="n">
         <v>2</v>
       </c>
       <c r="N67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O67" t="n">
-        <v>2.65</v>
+        <v>2.25</v>
       </c>
       <c r="P67" t="n">
-        <v>7.4625</v>
+        <v>6.5625</v>
       </c>
       <c r="Q67" t="n">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5546,58 +5559,63 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J68" t="n">
         <v>3</v>
       </c>
       <c r="K68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O68" t="n">
-        <v>3.1</v>
+        <v>2.25</v>
       </c>
       <c r="P68" t="n">
-        <v>8.475</v>
+        <v>6.5625</v>
       </c>
       <c r="Q68" t="n">
-        <v>8</v>
+        <v>6</v>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5611,58 +5629,58 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K69" t="n">
         <v>3</v>
       </c>
       <c r="L69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N69" t="n">
         <v>3</v>
       </c>
       <c r="O69" t="n">
-        <v>3.15</v>
+        <v>2.25</v>
       </c>
       <c r="P69" t="n">
-        <v>8.5875</v>
+        <v>6.5625</v>
       </c>
       <c r="Q69" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5676,58 +5694,58 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K70" t="n">
         <v>3</v>
       </c>
       <c r="L70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O70" t="n">
-        <v>3.25</v>
+        <v>2.25</v>
       </c>
       <c r="P70" t="n">
-        <v>8.8125</v>
+        <v>6.5625</v>
       </c>
       <c r="Q70" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5741,98 +5759,623 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I71" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J71" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L71" t="n">
         <v>3</v>
       </c>
       <c r="M71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O71" t="n">
-        <v>3.7</v>
+        <v>2.25</v>
       </c>
       <c r="P71" t="n">
-        <v>9.824999999999999</v>
+        <v>6.5625</v>
       </c>
       <c r="Q71" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
+        <v>6</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Mistborn</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Novels</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Brandon Sanderson</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>3</v>
+      </c>
+      <c r="I72" t="n">
+        <v>1</v>
+      </c>
+      <c r="J72" t="n">
+        <v>2</v>
+      </c>
+      <c r="K72" t="n">
+        <v>3</v>
+      </c>
+      <c r="L72" t="n">
+        <v>2</v>
+      </c>
+      <c r="M72" t="n">
+        <v>2</v>
+      </c>
+      <c r="N72" t="n">
+        <v>3</v>
+      </c>
+      <c r="O72" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="P72" t="n">
+        <v>6.5625</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>6</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Dark Souls I–III</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Video Games</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H73" t="n">
+        <v>3</v>
+      </c>
+      <c r="I73" t="n">
+        <v>2</v>
+      </c>
+      <c r="J73" t="n">
+        <v>2</v>
+      </c>
+      <c r="K73" t="n">
+        <v>2</v>
+      </c>
+      <c r="L73" t="n">
+        <v>3</v>
+      </c>
+      <c r="M73" t="n">
+        <v>2</v>
+      </c>
+      <c r="N73" t="n">
+        <v>3</v>
+      </c>
+      <c r="O73" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P73" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>6</v>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>6</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>The Stormlight Archive</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Novels</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Brandon Sanderson</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H74" t="n">
+        <v>2</v>
+      </c>
+      <c r="I74" t="n">
+        <v>2</v>
+      </c>
+      <c r="J74" t="n">
+        <v>2</v>
+      </c>
+      <c r="K74" t="n">
+        <v>3</v>
+      </c>
+      <c r="L74" t="n">
+        <v>3</v>
+      </c>
+      <c r="M74" t="n">
+        <v>2</v>
+      </c>
+      <c r="N74" t="n">
+        <v>3</v>
+      </c>
+      <c r="O74" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P74" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>7</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Extreme Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Berserk</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Manga / Anime / Films</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Kentaro Miura</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H75" t="n">
+        <v>3</v>
+      </c>
+      <c r="I75" t="n">
+        <v>2</v>
+      </c>
+      <c r="J75" t="n">
+        <v>3</v>
+      </c>
+      <c r="K75" t="n">
+        <v>2</v>
+      </c>
+      <c r="L75" t="n">
+        <v>3</v>
+      </c>
+      <c r="M75" t="n">
+        <v>2</v>
+      </c>
+      <c r="N75" t="n">
+        <v>4</v>
+      </c>
+      <c r="O75" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="P75" t="n">
+        <v>7.4625</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>8</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>A Song of Ice and Fire</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Novels / TV</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>George R. R. Martin</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>3</v>
+      </c>
+      <c r="I76" t="n">
+        <v>3</v>
+      </c>
+      <c r="J76" t="n">
+        <v>3</v>
+      </c>
+      <c r="K76" t="n">
+        <v>3</v>
+      </c>
+      <c r="L76" t="n">
+        <v>3</v>
+      </c>
+      <c r="M76" t="n">
+        <v>3</v>
+      </c>
+      <c r="N76" t="n">
+        <v>4</v>
+      </c>
+      <c r="O76" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="P76" t="n">
+        <v>8.475</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>8</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Elden Ring</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Video Game</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>4</v>
+      </c>
+      <c r="I77" t="n">
+        <v>3</v>
+      </c>
+      <c r="J77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K77" t="n">
+        <v>3</v>
+      </c>
+      <c r="L77" t="n">
+        <v>3</v>
+      </c>
+      <c r="M77" t="n">
+        <v>3</v>
+      </c>
+      <c r="N77" t="n">
+        <v>3</v>
+      </c>
+      <c r="O77" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="P77" t="n">
+        <v>8.5875</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>8</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Fire Punch</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Tatsuki Fujimoto</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H78" t="n">
+        <v>3</v>
+      </c>
+      <c r="I78" t="n">
+        <v>3</v>
+      </c>
+      <c r="J78" t="n">
+        <v>4</v>
+      </c>
+      <c r="K78" t="n">
+        <v>3</v>
+      </c>
+      <c r="L78" t="n">
+        <v>3</v>
+      </c>
+      <c r="M78" t="n">
+        <v>3</v>
+      </c>
+      <c r="N78" t="n">
+        <v>4</v>
+      </c>
+      <c r="O78" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="P78" t="n">
+        <v>8.8125</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>9</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>The First Law</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Novels</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Joe Abercrombie</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H79" t="n">
+        <v>4</v>
+      </c>
+      <c r="I79" t="n">
+        <v>4</v>
+      </c>
+      <c r="J79" t="n">
+        <v>4</v>
+      </c>
+      <c r="K79" t="n">
+        <v>4</v>
+      </c>
+      <c r="L79" t="n">
+        <v>3</v>
+      </c>
+      <c r="M79" t="n">
+        <v>3</v>
+      </c>
+      <c r="N79" t="n">
+        <v>4</v>
+      </c>
+      <c r="O79" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P79" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
         <v>10</v>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>Very Extreme Grimdark</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>Warhammer 40,000</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>Tabletop / Novels / Games / Animation</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E80" t="inlineStr">
         <is>
           <t>Games Workshop</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H72" t="n">
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
         <v>4</v>
       </c>
-      <c r="I72" t="n">
+      <c r="I80" t="n">
         <v>4</v>
       </c>
-      <c r="J72" t="n">
+      <c r="J80" t="n">
         <v>4</v>
       </c>
-      <c r="K72" t="n">
+      <c r="K80" t="n">
         <v>4</v>
       </c>
-      <c r="L72" t="n">
+      <c r="L80" t="n">
         <v>4</v>
       </c>
-      <c r="M72" t="n">
+      <c r="M80" t="n">
         <v>4</v>
       </c>
-      <c r="N72" t="n">
+      <c r="N80" t="n">
         <v>4</v>
       </c>
-      <c r="O72" t="n">
+      <c r="O80" t="n">
         <v>4</v>
       </c>
-      <c r="P72" t="n">
+      <c r="P80" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q72" t="n">
+      <c r="Q80" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5908,7 +6451,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -5921,7 +6464,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -5934,7 +6477,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -5947,7 +6490,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -6005,7 +6548,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 71 of 89 works in the full catalog (work in progress).</t>
+          <t>Total scored: 79 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore The Dark Elf & Drizzt and The Legend of Korra to v2 methodology
Both move from v1 tier 4 to v2 tier 5 (Gloomy Fantasy), tied with Skyrim/
Silmarillion at 5.325. Drizzt's rise is driven by Menzoberranzan's institutional
corruption and inverted moral physics; Korra's is scored directly against
Avatar: The Last Airbender's already-rescored profile per the v1 note framing
it as heavier than its predecessor.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Methodology" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Evaluations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R80"/>
+  <dimension ref="A1:R82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4865,17 +4865,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Ranking of Kings</t>
+          <t>The Dark Elf / Drizzt</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Sōsuke Tōka</t>
+          <t>R. A. Salvatore</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4907,21 +4907,16 @@
         <v>2</v>
       </c>
       <c r="N58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O58" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="P58" t="n">
-        <v>5.55</v>
+        <v>5.325</v>
       </c>
       <c r="Q58" t="n">
         <v>5</v>
-      </c>
-      <c r="R58" t="inlineStr">
-        <is>
-          <t>rescored three times after user corrections on plot details</t>
-        </is>
       </c>
     </row>
     <row r="59">
@@ -4935,17 +4930,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>The Legend of Korra</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4955,7 +4950,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H59" t="n">
@@ -4974,16 +4969,16 @@
         <v>2</v>
       </c>
       <c r="M59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N59" t="n">
         <v>2</v>
       </c>
       <c r="O59" t="n">
-        <v>1.85</v>
+        <v>1.7</v>
       </c>
       <c r="P59" t="n">
-        <v>5.6625</v>
+        <v>5.325</v>
       </c>
       <c r="Q59" t="n">
         <v>5</v>
@@ -5000,17 +4995,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>Ranking of Kings</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Sōsuke Tōka</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5027,13 +5022,13 @@
         <v>2</v>
       </c>
       <c r="I60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J60" t="n">
         <v>2</v>
       </c>
       <c r="K60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L60" t="n">
         <v>1</v>
@@ -5042,20 +5037,20 @@
         <v>2</v>
       </c>
       <c r="N60" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O60" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="P60" t="n">
-        <v>5.775</v>
+        <v>5.55</v>
       </c>
       <c r="Q60" t="n">
         <v>5</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Tier v1 era 6</t>
+          <t>rescored three times after user corrections on plot details</t>
         </is>
       </c>
     </row>
@@ -5070,17 +5065,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5100,25 +5095,25 @@
         <v>2</v>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K61" t="n">
         <v>2</v>
       </c>
       <c r="L61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M61" t="n">
         <v>2</v>
       </c>
       <c r="N61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O61" t="n">
-        <v>1.95</v>
+        <v>1.85</v>
       </c>
       <c r="P61" t="n">
-        <v>5.8875</v>
+        <v>5.6625</v>
       </c>
       <c r="Q61" t="n">
         <v>5</v>
@@ -5135,17 +5130,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5171,46 +5166,51 @@
         <v>1</v>
       </c>
       <c r="L62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M62" t="n">
         <v>2</v>
       </c>
       <c r="N62" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O62" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="P62" t="n">
-        <v>5.8875</v>
+        <v>5.775</v>
       </c>
       <c r="Q62" t="n">
         <v>5</v>
       </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5236,7 +5236,7 @@
         <v>2</v>
       </c>
       <c r="L63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M63" t="n">
         <v>2</v>
@@ -5245,37 +5245,37 @@
         <v>3</v>
       </c>
       <c r="O63" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P63" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q63" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5289,16 +5289,16 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L64" t="n">
         <v>2</v>
@@ -5310,13 +5310,13 @@
         <v>3</v>
       </c>
       <c r="O64" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P64" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65">
@@ -5330,17 +5330,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5363,7 +5363,7 @@
         <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L65" t="n">
         <v>2</v>
@@ -5372,21 +5372,16 @@
         <v>2</v>
       </c>
       <c r="N65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O65" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P65" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q65" t="n">
         <v>6</v>
-      </c>
-      <c r="R65" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="66">
@@ -5400,17 +5395,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5424,16 +5419,16 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L66" t="n">
         <v>2</v>
@@ -5442,13 +5437,13 @@
         <v>2</v>
       </c>
       <c r="N66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O66" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="P66" t="n">
-        <v>6.45</v>
+        <v>6.225</v>
       </c>
       <c r="Q66" t="n">
         <v>6</v>
@@ -5465,17 +5460,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5489,7 +5484,7 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I67" t="n">
         <v>2</v>
@@ -5498,7 +5493,7 @@
         <v>2</v>
       </c>
       <c r="K67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L67" t="n">
         <v>2</v>
@@ -5507,20 +5502,20 @@
         <v>2</v>
       </c>
       <c r="N67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O67" t="n">
-        <v>2.25</v>
+        <v>2.15</v>
       </c>
       <c r="P67" t="n">
-        <v>6.5625</v>
+        <v>6.3375</v>
       </c>
       <c r="Q67" t="n">
         <v>6</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>Tier v1 era 5</t>
+          <t>Tier v1 era 8</t>
         </is>
       </c>
     </row>
@@ -5535,17 +5530,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5565,7 +5560,7 @@
         <v>2</v>
       </c>
       <c r="J68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K68" t="n">
         <v>2</v>
@@ -5577,21 +5572,16 @@
         <v>2</v>
       </c>
       <c r="N68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O68" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P68" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q68" t="n">
         <v>6</v>
-      </c>
-      <c r="R68" t="inlineStr">
-        <is>
-          <t>Tier v1 era 7</t>
-        </is>
       </c>
     </row>
     <row r="69">
@@ -5605,17 +5595,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5629,7 +5619,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I69" t="n">
         <v>2</v>
@@ -5638,7 +5628,7 @@
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L69" t="n">
         <v>2</v>
@@ -5657,6 +5647,11 @@
       </c>
       <c r="Q69" t="n">
         <v>6</v>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -5670,17 +5665,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5700,10 +5695,10 @@
         <v>2</v>
       </c>
       <c r="J70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L70" t="n">
         <v>2</v>
@@ -5722,6 +5717,11 @@
       </c>
       <c r="Q70" t="n">
         <v>6</v>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -5735,17 +5735,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5762,7 +5762,7 @@
         <v>2</v>
       </c>
       <c r="I71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J71" t="n">
         <v>2</v>
@@ -5771,7 +5771,7 @@
         <v>3</v>
       </c>
       <c r="L71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M71" t="n">
         <v>2</v>
@@ -5800,17 +5800,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5824,10 +5824,10 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J72" t="n">
         <v>2</v>
@@ -5865,17 +5865,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5889,16 +5889,16 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J73" t="n">
         <v>2</v>
       </c>
       <c r="K73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L73" t="n">
         <v>3</v>
@@ -5910,18 +5910,13 @@
         <v>3</v>
       </c>
       <c r="O73" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P73" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q73" t="n">
         <v>6</v>
-      </c>
-      <c r="R73" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="74">
@@ -5935,7 +5930,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -5959,10 +5954,10 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J74" t="n">
         <v>2</v>
@@ -5971,7 +5966,7 @@
         <v>3</v>
       </c>
       <c r="L74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M74" t="n">
         <v>2</v>
@@ -5980,10 +5975,10 @@
         <v>3</v>
       </c>
       <c r="O74" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P74" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q74" t="n">
         <v>6</v>
@@ -5991,26 +5986,26 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6030,7 +6025,7 @@
         <v>2</v>
       </c>
       <c r="J75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K75" t="n">
         <v>2</v>
@@ -6042,40 +6037,45 @@
         <v>2</v>
       </c>
       <c r="N75" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O75" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P75" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q75" t="n">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6089,13 +6089,13 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K76" t="n">
         <v>3</v>
@@ -6104,43 +6104,43 @@
         <v>3</v>
       </c>
       <c r="M76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O76" t="n">
-        <v>3.1</v>
+        <v>2.4</v>
       </c>
       <c r="P76" t="n">
-        <v>8.475</v>
+        <v>6.9</v>
       </c>
       <c r="Q76" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6154,34 +6154,34 @@
         </is>
       </c>
       <c r="H77" t="n">
+        <v>3</v>
+      </c>
+      <c r="I77" t="n">
+        <v>2</v>
+      </c>
+      <c r="J77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K77" t="n">
+        <v>2</v>
+      </c>
+      <c r="L77" t="n">
+        <v>3</v>
+      </c>
+      <c r="M77" t="n">
+        <v>2</v>
+      </c>
+      <c r="N77" t="n">
         <v>4</v>
       </c>
-      <c r="I77" t="n">
-        <v>3</v>
-      </c>
-      <c r="J77" t="n">
-        <v>3</v>
-      </c>
-      <c r="K77" t="n">
-        <v>3</v>
-      </c>
-      <c r="L77" t="n">
-        <v>3</v>
-      </c>
-      <c r="M77" t="n">
-        <v>3</v>
-      </c>
-      <c r="N77" t="n">
-        <v>3</v>
-      </c>
       <c r="O77" t="n">
-        <v>3.15</v>
+        <v>2.65</v>
       </c>
       <c r="P77" t="n">
-        <v>8.5875</v>
+        <v>7.4625</v>
       </c>
       <c r="Q77" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="78">
@@ -6195,17 +6195,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6225,7 +6225,7 @@
         <v>3</v>
       </c>
       <c r="J78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K78" t="n">
         <v>3</v>
@@ -6240,10 +6240,10 @@
         <v>4</v>
       </c>
       <c r="O78" t="n">
-        <v>3.25</v>
+        <v>3.1</v>
       </c>
       <c r="P78" t="n">
-        <v>8.8125</v>
+        <v>8.475</v>
       </c>
       <c r="Q78" t="n">
         <v>8</v>
@@ -6251,26 +6251,26 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6287,13 +6287,13 @@
         <v>4</v>
       </c>
       <c r="I79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L79" t="n">
         <v>3</v>
@@ -6302,40 +6302,40 @@
         <v>3</v>
       </c>
       <c r="N79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O79" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="P79" t="n">
-        <v>9.824999999999999</v>
+        <v>8.5875</v>
       </c>
       <c r="Q79" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6349,33 +6349,163 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J80" t="n">
         <v>4</v>
       </c>
       <c r="K80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N80" t="n">
         <v>4</v>
       </c>
       <c r="O80" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="P80" t="n">
+        <v>8.8125</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>9</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>The First Law</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Novels</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Joe Abercrombie</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H81" t="n">
         <v>4</v>
       </c>
-      <c r="P80" t="n">
+      <c r="I81" t="n">
+        <v>4</v>
+      </c>
+      <c r="J81" t="n">
+        <v>4</v>
+      </c>
+      <c r="K81" t="n">
+        <v>4</v>
+      </c>
+      <c r="L81" t="n">
+        <v>3</v>
+      </c>
+      <c r="M81" t="n">
+        <v>3</v>
+      </c>
+      <c r="N81" t="n">
+        <v>4</v>
+      </c>
+      <c r="O81" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P81" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>10</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H82" t="n">
+        <v>4</v>
+      </c>
+      <c r="I82" t="n">
+        <v>4</v>
+      </c>
+      <c r="J82" t="n">
+        <v>4</v>
+      </c>
+      <c r="K82" t="n">
+        <v>4</v>
+      </c>
+      <c r="L82" t="n">
+        <v>4</v>
+      </c>
+      <c r="M82" t="n">
+        <v>4</v>
+      </c>
+      <c r="N82" t="n">
+        <v>4</v>
+      </c>
+      <c r="O82" t="n">
+        <v>4</v>
+      </c>
+      <c r="P82" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q80" t="n">
+      <c r="Q82" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6477,7 +6607,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -6548,7 +6678,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 79 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 81 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore The Wheel of Time to v2 methodology
Moves from v1 tier 4 to v2 tier 5 (5.2125), tied with Dragonlance/Elantris.
Scored against both LOTR and Dragonlance as close genre neighbors — the
Seanchan a'dam slavery system and the sheer accumulated darkness across
fourteen books drive it above LOTR, while Rand's structural (not just
tactical) defeat of the Dark One keeps Limited Heroism as low as LOTR's.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R82"/>
+  <dimension ref="A1:R83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4665,17 +4665,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Baldur's Gate III</t>
+          <t>The Wheel of Time</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Robert Jordan / Brandon Sanderson</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4689,13 +4689,13 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I55" t="n">
         <v>1</v>
       </c>
       <c r="J55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K55" t="n">
         <v>2</v>
@@ -4717,11 +4717,6 @@
       </c>
       <c r="Q55" t="n">
         <v>5</v>
-      </c>
-      <c r="R55" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="56">
@@ -4735,17 +4730,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V: Skyrim</t>
+          <t>Baldur's Gate III</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Bethesda Game Studios</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4759,7 +4754,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I56" t="n">
         <v>1</v>
@@ -4771,22 +4766,27 @@
         <v>2</v>
       </c>
       <c r="L56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O56" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="P56" t="n">
-        <v>5.325</v>
+        <v>5.2125</v>
       </c>
       <c r="Q56" t="n">
         <v>5</v>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -4800,17 +4800,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>The Silmarillion &amp; Great Tales</t>
+          <t>The Elder Scrolls V: Skyrim</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Books</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Bethesda Game Studios</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4836,10 +4836,10 @@
         <v>2</v>
       </c>
       <c r="L57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N57" t="n">
         <v>2</v>
@@ -4865,17 +4865,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>The Dark Elf / Drizzt</t>
+          <t>The Silmarillion &amp; Great Tales</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Books</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>R. A. Salvatore</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4901,10 +4901,10 @@
         <v>2</v>
       </c>
       <c r="L58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N58" t="n">
         <v>2</v>
@@ -4930,17 +4930,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>The Legend of Korra</t>
+          <t>The Dark Elf / Drizzt</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>R. A. Salvatore</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4950,26 +4950,26 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H59" t="n">
         <v>2</v>
       </c>
       <c r="I59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K59" t="n">
         <v>2</v>
       </c>
       <c r="L59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N59" t="n">
         <v>2</v>
@@ -4995,17 +4995,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Ranking of Kings</t>
+          <t>The Legend of Korra</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Sōsuke Tōka</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5015,43 +5015,38 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H60" t="n">
         <v>2</v>
       </c>
       <c r="I60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K60" t="n">
         <v>2</v>
       </c>
       <c r="L60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O60" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="P60" t="n">
-        <v>5.55</v>
+        <v>5.325</v>
       </c>
       <c r="Q60" t="n">
         <v>5</v>
-      </c>
-      <c r="R60" t="inlineStr">
-        <is>
-          <t>rescored three times after user corrections on plot details</t>
-        </is>
       </c>
     </row>
     <row r="61">
@@ -5065,17 +5060,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>Ranking of Kings</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Sōsuke Tōka</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5092,31 +5087,36 @@
         <v>2</v>
       </c>
       <c r="I61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K61" t="n">
         <v>2</v>
       </c>
       <c r="L61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M61" t="n">
         <v>2</v>
       </c>
       <c r="N61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O61" t="n">
-        <v>1.85</v>
+        <v>1.8</v>
       </c>
       <c r="P61" t="n">
-        <v>5.6625</v>
+        <v>5.55</v>
       </c>
       <c r="Q61" t="n">
         <v>5</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>rescored three times after user corrections on plot details</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -5130,17 +5130,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5160,33 +5160,28 @@
         <v>2</v>
       </c>
       <c r="J62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M62" t="n">
         <v>2</v>
       </c>
       <c r="N62" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O62" t="n">
-        <v>1.9</v>
+        <v>1.85</v>
       </c>
       <c r="P62" t="n">
-        <v>5.775</v>
+        <v>5.6625</v>
       </c>
       <c r="Q62" t="n">
         <v>5</v>
-      </c>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>Tier v1 era 6</t>
-        </is>
       </c>
     </row>
     <row r="63">
@@ -5200,17 +5195,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5233,7 +5228,7 @@
         <v>2</v>
       </c>
       <c r="K63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L63" t="n">
         <v>1</v>
@@ -5242,16 +5237,21 @@
         <v>2</v>
       </c>
       <c r="N63" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O63" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="P63" t="n">
-        <v>5.8875</v>
+        <v>5.775</v>
       </c>
       <c r="Q63" t="n">
         <v>5</v>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -5298,10 +5298,10 @@
         <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M64" t="n">
         <v>2</v>
@@ -5321,26 +5321,26 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5363,7 +5363,7 @@
         <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L65" t="n">
         <v>2</v>
@@ -5375,13 +5375,13 @@
         <v>3</v>
       </c>
       <c r="O65" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P65" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66">
@@ -5395,17 +5395,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5419,16 +5419,16 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L66" t="n">
         <v>2</v>
@@ -5460,17 +5460,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5484,13 +5484,13 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K67" t="n">
         <v>3</v>
@@ -5502,21 +5502,16 @@
         <v>2</v>
       </c>
       <c r="N67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O67" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P67" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q67" t="n">
         <v>6</v>
-      </c>
-      <c r="R67" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="68">
@@ -5530,17 +5525,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5563,7 +5558,7 @@
         <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L68" t="n">
         <v>2</v>
@@ -5572,16 +5567,21 @@
         <v>2</v>
       </c>
       <c r="N68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O68" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P68" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q68" t="n">
         <v>6</v>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -5595,17 +5595,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5619,7 +5619,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I69" t="n">
         <v>2</v>
@@ -5637,21 +5637,16 @@
         <v>2</v>
       </c>
       <c r="N69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O69" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P69" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q69" t="n">
         <v>6</v>
-      </c>
-      <c r="R69" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="70">
@@ -5665,17 +5660,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5689,13 +5684,13 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I70" t="n">
         <v>2</v>
       </c>
       <c r="J70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K70" t="n">
         <v>2</v>
@@ -5720,7 +5715,7 @@
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -5735,17 +5730,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5765,10 +5760,10 @@
         <v>2</v>
       </c>
       <c r="J71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L71" t="n">
         <v>2</v>
@@ -5787,6 +5782,11 @@
       </c>
       <c r="Q71" t="n">
         <v>6</v>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -5800,17 +5800,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5865,17 +5865,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5892,7 +5892,7 @@
         <v>2</v>
       </c>
       <c r="I73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J73" t="n">
         <v>2</v>
@@ -5901,7 +5901,7 @@
         <v>3</v>
       </c>
       <c r="L73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M73" t="n">
         <v>2</v>
@@ -5930,17 +5930,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5954,7 +5954,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I74" t="n">
         <v>1</v>
@@ -5966,7 +5966,7 @@
         <v>3</v>
       </c>
       <c r="L74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M74" t="n">
         <v>2</v>
@@ -5995,17 +5995,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6022,16 +6022,16 @@
         <v>3</v>
       </c>
       <c r="I75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J75" t="n">
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M75" t="n">
         <v>2</v>
@@ -6040,18 +6040,13 @@
         <v>3</v>
       </c>
       <c r="O75" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P75" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q75" t="n">
         <v>6</v>
-      </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="76">
@@ -6065,17 +6060,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6089,7 +6084,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I76" t="n">
         <v>2</v>
@@ -6098,7 +6093,7 @@
         <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L76" t="n">
         <v>3</v>
@@ -6118,29 +6113,34 @@
       <c r="Q76" t="n">
         <v>6</v>
       </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6154,16 +6154,16 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I77" t="n">
         <v>2</v>
       </c>
       <c r="J77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L77" t="n">
         <v>3</v>
@@ -6172,40 +6172,40 @@
         <v>2</v>
       </c>
       <c r="N77" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O77" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P77" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q77" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6222,31 +6222,31 @@
         <v>3</v>
       </c>
       <c r="I78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J78" t="n">
         <v>3</v>
       </c>
       <c r="K78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L78" t="n">
         <v>3</v>
       </c>
       <c r="M78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N78" t="n">
         <v>4</v>
       </c>
       <c r="O78" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P78" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q78" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="79">
@@ -6260,17 +6260,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6284,31 +6284,31 @@
         </is>
       </c>
       <c r="H79" t="n">
+        <v>3</v>
+      </c>
+      <c r="I79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J79" t="n">
+        <v>3</v>
+      </c>
+      <c r="K79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L79" t="n">
+        <v>3</v>
+      </c>
+      <c r="M79" t="n">
+        <v>3</v>
+      </c>
+      <c r="N79" t="n">
         <v>4</v>
       </c>
-      <c r="I79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J79" t="n">
-        <v>3</v>
-      </c>
-      <c r="K79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L79" t="n">
-        <v>3</v>
-      </c>
-      <c r="M79" t="n">
-        <v>3</v>
-      </c>
-      <c r="N79" t="n">
-        <v>3</v>
-      </c>
       <c r="O79" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P79" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q79" t="n">
         <v>8</v>
@@ -6325,17 +6325,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6349,13 +6349,13 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I80" t="n">
         <v>3</v>
       </c>
       <c r="J80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K80" t="n">
         <v>3</v>
@@ -6367,13 +6367,13 @@
         <v>3</v>
       </c>
       <c r="N80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O80" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P80" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q80" t="n">
         <v>8</v>
@@ -6381,26 +6381,26 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6414,16 +6414,16 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J81" t="n">
         <v>4</v>
       </c>
       <c r="K81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L81" t="n">
         <v>3</v>
@@ -6435,37 +6435,37 @@
         <v>4</v>
       </c>
       <c r="O81" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P81" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q81" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6491,21 +6491,86 @@
         <v>4</v>
       </c>
       <c r="L82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N82" t="n">
         <v>4</v>
       </c>
       <c r="O82" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P82" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>10</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
         <v>4</v>
       </c>
-      <c r="P82" t="n">
+      <c r="I83" t="n">
+        <v>4</v>
+      </c>
+      <c r="J83" t="n">
+        <v>4</v>
+      </c>
+      <c r="K83" t="n">
+        <v>4</v>
+      </c>
+      <c r="L83" t="n">
+        <v>4</v>
+      </c>
+      <c r="M83" t="n">
+        <v>4</v>
+      </c>
+      <c r="N83" t="n">
+        <v>4</v>
+      </c>
+      <c r="O83" t="n">
+        <v>4</v>
+      </c>
+      <c r="P83" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q82" t="n">
+      <c r="Q83" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6607,7 +6672,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -6678,7 +6743,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 81 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 82 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore Princess Mononoke to v2 methodology
Moves from v1 tier 4 to v2 tier 5 (5.55), tied with Ranking of Kings. Scored
against the other already-rescored Ghibli films — clearly the most graphically
violent of the studio's works on the scale, and its refusal of a simple
virtue-is-rewarded framework pushes Moral Cynicism and Narrative Acceptance
of Injustice above its stablemates.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R83"/>
+  <dimension ref="A1:R84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5060,17 +5060,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Ranking of Kings</t>
+          <t>Princess Mononoke</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Sōsuke Tōka</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5087,13 +5087,13 @@
         <v>2</v>
       </c>
       <c r="I61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J61" t="n">
         <v>2</v>
       </c>
       <c r="K61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L61" t="n">
         <v>1</v>
@@ -5112,11 +5112,6 @@
       </c>
       <c r="Q61" t="n">
         <v>5</v>
-      </c>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>rescored three times after user corrections on plot details</t>
-        </is>
       </c>
     </row>
     <row r="62">
@@ -5130,17 +5125,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>Ranking of Kings</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Sōsuke Tōka</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5157,31 +5152,36 @@
         <v>2</v>
       </c>
       <c r="I62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K62" t="n">
         <v>2</v>
       </c>
       <c r="L62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M62" t="n">
         <v>2</v>
       </c>
       <c r="N62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O62" t="n">
-        <v>1.85</v>
+        <v>1.8</v>
       </c>
       <c r="P62" t="n">
-        <v>5.6625</v>
+        <v>5.55</v>
       </c>
       <c r="Q62" t="n">
         <v>5</v>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>rescored three times after user corrections on plot details</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -5195,17 +5195,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5225,33 +5225,28 @@
         <v>2</v>
       </c>
       <c r="J63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M63" t="n">
         <v>2</v>
       </c>
       <c r="N63" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O63" t="n">
-        <v>1.9</v>
+        <v>1.85</v>
       </c>
       <c r="P63" t="n">
-        <v>5.775</v>
+        <v>5.6625</v>
       </c>
       <c r="Q63" t="n">
         <v>5</v>
-      </c>
-      <c r="R63" t="inlineStr">
-        <is>
-          <t>Tier v1 era 6</t>
-        </is>
       </c>
     </row>
     <row r="64">
@@ -5265,17 +5260,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5298,7 +5293,7 @@
         <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L64" t="n">
         <v>1</v>
@@ -5307,16 +5302,21 @@
         <v>2</v>
       </c>
       <c r="N64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O64" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="P64" t="n">
-        <v>5.8875</v>
+        <v>5.775</v>
       </c>
       <c r="Q64" t="n">
         <v>5</v>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -5363,10 +5363,10 @@
         <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M65" t="n">
         <v>2</v>
@@ -5386,26 +5386,26 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5428,7 +5428,7 @@
         <v>2</v>
       </c>
       <c r="K66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L66" t="n">
         <v>2</v>
@@ -5440,13 +5440,13 @@
         <v>3</v>
       </c>
       <c r="O66" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P66" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q66" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67">
@@ -5460,17 +5460,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5484,16 +5484,16 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L67" t="n">
         <v>2</v>
@@ -5525,17 +5525,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5549,13 +5549,13 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K68" t="n">
         <v>3</v>
@@ -5567,21 +5567,16 @@
         <v>2</v>
       </c>
       <c r="N68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O68" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P68" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q68" t="n">
         <v>6</v>
-      </c>
-      <c r="R68" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="69">
@@ -5595,17 +5590,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5628,7 +5623,7 @@
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L69" t="n">
         <v>2</v>
@@ -5637,16 +5632,21 @@
         <v>2</v>
       </c>
       <c r="N69" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O69" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P69" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q69" t="n">
         <v>6</v>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -5660,17 +5660,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5684,7 +5684,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I70" t="n">
         <v>2</v>
@@ -5702,21 +5702,16 @@
         <v>2</v>
       </c>
       <c r="N70" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O70" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P70" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q70" t="n">
         <v>6</v>
-      </c>
-      <c r="R70" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="71">
@@ -5730,17 +5725,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5754,13 +5749,13 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I71" t="n">
         <v>2</v>
       </c>
       <c r="J71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K71" t="n">
         <v>2</v>
@@ -5785,7 +5780,7 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -5800,17 +5795,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5830,10 +5825,10 @@
         <v>2</v>
       </c>
       <c r="J72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L72" t="n">
         <v>2</v>
@@ -5852,6 +5847,11 @@
       </c>
       <c r="Q72" t="n">
         <v>6</v>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -5865,17 +5865,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5930,17 +5930,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5957,7 +5957,7 @@
         <v>2</v>
       </c>
       <c r="I74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J74" t="n">
         <v>2</v>
@@ -5966,7 +5966,7 @@
         <v>3</v>
       </c>
       <c r="L74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M74" t="n">
         <v>2</v>
@@ -5995,17 +5995,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6019,7 +6019,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I75" t="n">
         <v>1</v>
@@ -6031,7 +6031,7 @@
         <v>3</v>
       </c>
       <c r="L75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M75" t="n">
         <v>2</v>
@@ -6060,17 +6060,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6087,16 +6087,16 @@
         <v>3</v>
       </c>
       <c r="I76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J76" t="n">
         <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M76" t="n">
         <v>2</v>
@@ -6105,18 +6105,13 @@
         <v>3</v>
       </c>
       <c r="O76" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P76" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q76" t="n">
         <v>6</v>
-      </c>
-      <c r="R76" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="77">
@@ -6130,17 +6125,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6154,7 +6149,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I77" t="n">
         <v>2</v>
@@ -6163,7 +6158,7 @@
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L77" t="n">
         <v>3</v>
@@ -6183,29 +6178,34 @@
       <c r="Q77" t="n">
         <v>6</v>
       </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6219,16 +6219,16 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I78" t="n">
         <v>2</v>
       </c>
       <c r="J78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L78" t="n">
         <v>3</v>
@@ -6237,40 +6237,40 @@
         <v>2</v>
       </c>
       <c r="N78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O78" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P78" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q78" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6287,31 +6287,31 @@
         <v>3</v>
       </c>
       <c r="I79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J79" t="n">
         <v>3</v>
       </c>
       <c r="K79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L79" t="n">
         <v>3</v>
       </c>
       <c r="M79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N79" t="n">
         <v>4</v>
       </c>
       <c r="O79" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P79" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q79" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="80">
@@ -6325,17 +6325,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6349,31 +6349,31 @@
         </is>
       </c>
       <c r="H80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I80" t="n">
+        <v>3</v>
+      </c>
+      <c r="J80" t="n">
+        <v>3</v>
+      </c>
+      <c r="K80" t="n">
+        <v>3</v>
+      </c>
+      <c r="L80" t="n">
+        <v>3</v>
+      </c>
+      <c r="M80" t="n">
+        <v>3</v>
+      </c>
+      <c r="N80" t="n">
         <v>4</v>
       </c>
-      <c r="I80" t="n">
-        <v>3</v>
-      </c>
-      <c r="J80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K80" t="n">
-        <v>3</v>
-      </c>
-      <c r="L80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M80" t="n">
-        <v>3</v>
-      </c>
-      <c r="N80" t="n">
-        <v>3</v>
-      </c>
       <c r="O80" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P80" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q80" t="n">
         <v>8</v>
@@ -6390,17 +6390,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6414,13 +6414,13 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I81" t="n">
         <v>3</v>
       </c>
       <c r="J81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K81" t="n">
         <v>3</v>
@@ -6432,13 +6432,13 @@
         <v>3</v>
       </c>
       <c r="N81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O81" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P81" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q81" t="n">
         <v>8</v>
@@ -6446,26 +6446,26 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6479,16 +6479,16 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J82" t="n">
         <v>4</v>
       </c>
       <c r="K82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L82" t="n">
         <v>3</v>
@@ -6500,37 +6500,37 @@
         <v>4</v>
       </c>
       <c r="O82" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P82" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q82" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6556,21 +6556,86 @@
         <v>4</v>
       </c>
       <c r="L83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N83" t="n">
         <v>4</v>
       </c>
       <c r="O83" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P83" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>10</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H84" t="n">
         <v>4</v>
       </c>
-      <c r="P83" t="n">
+      <c r="I84" t="n">
+        <v>4</v>
+      </c>
+      <c r="J84" t="n">
+        <v>4</v>
+      </c>
+      <c r="K84" t="n">
+        <v>4</v>
+      </c>
+      <c r="L84" t="n">
+        <v>4</v>
+      </c>
+      <c r="M84" t="n">
+        <v>4</v>
+      </c>
+      <c r="N84" t="n">
+        <v>4</v>
+      </c>
+      <c r="O84" t="n">
+        <v>4</v>
+      </c>
+      <c r="P84" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q83" t="n">
+      <c r="Q84" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6672,7 +6737,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -6743,7 +6808,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 82 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 83 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore Star vs. the Forces of Evil to v2 methodology
Tier 4 -> tier 5 (score 5.6625, tied with The Kingkiller Chronicle), scored
directly against the already-rescored Avatar: The Last Airbender and Legend
of Korra profiles given the shared oppressed-group-plus-reconciliation shape.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R84"/>
+  <dimension ref="A1:R85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5260,17 +5260,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>Star vs. the Forces of Evil</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>TV, Comics</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Daron Nefcy</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5290,33 +5290,28 @@
         <v>2</v>
       </c>
       <c r="J64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M64" t="n">
         <v>2</v>
       </c>
       <c r="N64" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O64" t="n">
-        <v>1.9</v>
+        <v>1.85</v>
       </c>
       <c r="P64" t="n">
-        <v>5.775</v>
+        <v>5.6625</v>
       </c>
       <c r="Q64" t="n">
         <v>5</v>
-      </c>
-      <c r="R64" t="inlineStr">
-        <is>
-          <t>Tier v1 era 6</t>
-        </is>
       </c>
     </row>
     <row r="65">
@@ -5330,17 +5325,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5363,7 +5358,7 @@
         <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L65" t="n">
         <v>1</v>
@@ -5372,16 +5367,21 @@
         <v>2</v>
       </c>
       <c r="N65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O65" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="P65" t="n">
-        <v>5.8875</v>
+        <v>5.775</v>
       </c>
       <c r="Q65" t="n">
         <v>5</v>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -5428,10 +5428,10 @@
         <v>2</v>
       </c>
       <c r="K66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M66" t="n">
         <v>2</v>
@@ -5451,26 +5451,26 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5493,7 +5493,7 @@
         <v>2</v>
       </c>
       <c r="K67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L67" t="n">
         <v>2</v>
@@ -5505,13 +5505,13 @@
         <v>3</v>
       </c>
       <c r="O67" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P67" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q67" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68">
@@ -5525,17 +5525,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5549,16 +5549,16 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L68" t="n">
         <v>2</v>
@@ -5590,17 +5590,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5614,13 +5614,13 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K69" t="n">
         <v>3</v>
@@ -5632,21 +5632,16 @@
         <v>2</v>
       </c>
       <c r="N69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O69" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P69" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q69" t="n">
         <v>6</v>
-      </c>
-      <c r="R69" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="70">
@@ -5660,17 +5655,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5693,7 +5688,7 @@
         <v>2</v>
       </c>
       <c r="K70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L70" t="n">
         <v>2</v>
@@ -5702,16 +5697,21 @@
         <v>2</v>
       </c>
       <c r="N70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O70" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P70" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q70" t="n">
         <v>6</v>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -5725,17 +5725,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5749,7 +5749,7 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I71" t="n">
         <v>2</v>
@@ -5767,21 +5767,16 @@
         <v>2</v>
       </c>
       <c r="N71" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O71" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P71" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q71" t="n">
         <v>6</v>
-      </c>
-      <c r="R71" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="72">
@@ -5795,17 +5790,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5819,13 +5814,13 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I72" t="n">
         <v>2</v>
       </c>
       <c r="J72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K72" t="n">
         <v>2</v>
@@ -5850,7 +5845,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -5865,17 +5860,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5895,10 +5890,10 @@
         <v>2</v>
       </c>
       <c r="J73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L73" t="n">
         <v>2</v>
@@ -5917,6 +5912,11 @@
       </c>
       <c r="Q73" t="n">
         <v>6</v>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -5930,17 +5930,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5995,17 +5995,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6022,7 +6022,7 @@
         <v>2</v>
       </c>
       <c r="I75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J75" t="n">
         <v>2</v>
@@ -6031,7 +6031,7 @@
         <v>3</v>
       </c>
       <c r="L75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M75" t="n">
         <v>2</v>
@@ -6060,17 +6060,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6084,7 +6084,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I76" t="n">
         <v>1</v>
@@ -6096,7 +6096,7 @@
         <v>3</v>
       </c>
       <c r="L76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M76" t="n">
         <v>2</v>
@@ -6125,17 +6125,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6152,16 +6152,16 @@
         <v>3</v>
       </c>
       <c r="I77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J77" t="n">
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M77" t="n">
         <v>2</v>
@@ -6170,18 +6170,13 @@
         <v>3</v>
       </c>
       <c r="O77" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P77" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q77" t="n">
         <v>6</v>
-      </c>
-      <c r="R77" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="78">
@@ -6195,17 +6190,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6219,7 +6214,7 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I78" t="n">
         <v>2</v>
@@ -6228,7 +6223,7 @@
         <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L78" t="n">
         <v>3</v>
@@ -6248,29 +6243,34 @@
       <c r="Q78" t="n">
         <v>6</v>
       </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6284,16 +6284,16 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I79" t="n">
         <v>2</v>
       </c>
       <c r="J79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L79" t="n">
         <v>3</v>
@@ -6302,40 +6302,40 @@
         <v>2</v>
       </c>
       <c r="N79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O79" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P79" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q79" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6352,31 +6352,31 @@
         <v>3</v>
       </c>
       <c r="I80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J80" t="n">
         <v>3</v>
       </c>
       <c r="K80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L80" t="n">
         <v>3</v>
       </c>
       <c r="M80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N80" t="n">
         <v>4</v>
       </c>
       <c r="O80" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P80" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q80" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="81">
@@ -6390,17 +6390,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6414,31 +6414,31 @@
         </is>
       </c>
       <c r="H81" t="n">
+        <v>3</v>
+      </c>
+      <c r="I81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J81" t="n">
+        <v>3</v>
+      </c>
+      <c r="K81" t="n">
+        <v>3</v>
+      </c>
+      <c r="L81" t="n">
+        <v>3</v>
+      </c>
+      <c r="M81" t="n">
+        <v>3</v>
+      </c>
+      <c r="N81" t="n">
         <v>4</v>
       </c>
-      <c r="I81" t="n">
-        <v>3</v>
-      </c>
-      <c r="J81" t="n">
-        <v>3</v>
-      </c>
-      <c r="K81" t="n">
-        <v>3</v>
-      </c>
-      <c r="L81" t="n">
-        <v>3</v>
-      </c>
-      <c r="M81" t="n">
-        <v>3</v>
-      </c>
-      <c r="N81" t="n">
-        <v>3</v>
-      </c>
       <c r="O81" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P81" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q81" t="n">
         <v>8</v>
@@ -6455,17 +6455,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6479,13 +6479,13 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I82" t="n">
         <v>3</v>
       </c>
       <c r="J82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K82" t="n">
         <v>3</v>
@@ -6497,13 +6497,13 @@
         <v>3</v>
       </c>
       <c r="N82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O82" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P82" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q82" t="n">
         <v>8</v>
@@ -6511,26 +6511,26 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6544,16 +6544,16 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J83" t="n">
         <v>4</v>
       </c>
       <c r="K83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L83" t="n">
         <v>3</v>
@@ -6565,37 +6565,37 @@
         <v>4</v>
       </c>
       <c r="O83" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P83" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q83" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6621,21 +6621,86 @@
         <v>4</v>
       </c>
       <c r="L84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N84" t="n">
         <v>4</v>
       </c>
       <c r="O84" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P84" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>10</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
         <v>4</v>
       </c>
-      <c r="P84" t="n">
+      <c r="I85" t="n">
+        <v>4</v>
+      </c>
+      <c r="J85" t="n">
+        <v>4</v>
+      </c>
+      <c r="K85" t="n">
+        <v>4</v>
+      </c>
+      <c r="L85" t="n">
+        <v>4</v>
+      </c>
+      <c r="M85" t="n">
+        <v>4</v>
+      </c>
+      <c r="N85" t="n">
+        <v>4</v>
+      </c>
+      <c r="O85" t="n">
+        <v>4</v>
+      </c>
+      <c r="P85" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q84" t="n">
+      <c r="Q85" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6737,7 +6802,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -6808,7 +6873,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 83 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 84 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-audit tier-5 cluster: fix Ranking of Kings over-score
User flagged that 6 consecutive v2 rescores had all landed in tier 5.
Re-derived each axis of all six directly against the rubric anchor text
instead of copying values forward from the last-scored neighbor.

Ranking of Kings drops a full tier (5 -> 4, 5.55 -> 4.875): Moral Cynicism
and Redemption Difficulty were both one point too high against the actual
anchor text (and against evidence already documented in this log). Drizzt,
Korra, and Wheel of Time each got one or two axes corrected but stayed in
tier 5, converging at 5.55. Princess Mononoke and Star vs. the Forces of
Evil held unchanged after the same scrutiny.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -4335,17 +4335,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Tales from Earthsea</t>
+          <t>Ranking of Kings</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Gorō Miyazaki</t>
+          <t>Sōsuke Tōka</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4368,29 +4368,29 @@
         <v>1</v>
       </c>
       <c r="K50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L50" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M50" t="n">
         <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O50" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="P50" t="n">
-        <v>4.9875</v>
+        <v>4.875</v>
       </c>
       <c r="Q50" t="n">
         <v>4</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Tier v1 era 5</t>
+          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
         </is>
       </c>
     </row>
@@ -4405,17 +4405,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Adventure Time</t>
+          <t>Tales from Earthsea</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>TV / Comics</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Pendleton Ward</t>
+          <t>Studio Ghibli / Gorō Miyazaki</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4458,29 +4458,34 @@
       <c r="Q51" t="n">
         <v>4</v>
       </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Dragonlance</t>
+          <t>Adventure Time</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Novels / Games</t>
+          <t>TV / Comics</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Margaret Weis / Tracy Hickman</t>
+          <t>Pendleton Ward</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4503,25 +4508,25 @@
         <v>1</v>
       </c>
       <c r="K52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L52" t="n">
         <v>2</v>
       </c>
       <c r="M52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O52" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="P52" t="n">
-        <v>5.2125</v>
+        <v>4.9875</v>
       </c>
       <c r="Q52" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
@@ -4535,17 +4540,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Harry Potter and the Goblet of Fire</t>
+          <t>Dragonlance</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Novels / Games</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Margaret Weis / Tracy Hickman</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4559,22 +4564,22 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I53" t="n">
         <v>1</v>
       </c>
       <c r="J53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K53" t="n">
         <v>2</v>
       </c>
       <c r="L53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N53" t="n">
         <v>3</v>
@@ -4600,17 +4605,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Elantris</t>
+          <t>Harry Potter and the Goblet of Fire</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4624,22 +4629,22 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I54" t="n">
         <v>1</v>
       </c>
       <c r="J54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K54" t="n">
         <v>2</v>
       </c>
       <c r="L54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N54" t="n">
         <v>3</v>
@@ -4665,17 +4670,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>The Wheel of Time</t>
+          <t>Elantris</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Robert Jordan / Brandon Sanderson</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4930,17 +4935,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>The Dark Elf / Drizzt</t>
+          <t>Princess Mononoke</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>R. A. Salvatore</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4957,13 +4962,13 @@
         <v>2</v>
       </c>
       <c r="I59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J59" t="n">
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L59" t="n">
         <v>1</v>
@@ -4972,13 +4977,13 @@
         <v>2</v>
       </c>
       <c r="N59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O59" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="P59" t="n">
-        <v>5.325</v>
+        <v>5.55</v>
       </c>
       <c r="Q59" t="n">
         <v>5</v>
@@ -4995,17 +5000,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>The Legend of Korra</t>
+          <t>The Dark Elf / Drizzt</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>R. A. Salvatore</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5015,14 +5020,14 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H60" t="n">
         <v>2</v>
       </c>
       <c r="I60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J60" t="n">
         <v>1</v>
@@ -5034,19 +5039,24 @@
         <v>2</v>
       </c>
       <c r="M60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O60" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="P60" t="n">
-        <v>5.325</v>
+        <v>5.55</v>
       </c>
       <c r="Q60" t="n">
         <v>5</v>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -5060,17 +5070,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Princess Mononoke</t>
+          <t>The Legend of Korra</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5080,7 +5090,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H61" t="n">
@@ -5090,16 +5100,16 @@
         <v>2</v>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N61" t="n">
         <v>3</v>
@@ -5112,6 +5122,11 @@
       </c>
       <c r="Q61" t="n">
         <v>5</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -5125,17 +5140,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Ranking of Kings</t>
+          <t>The Wheel of Time</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Sōsuke Tōka</t>
+          <t>Robert Jordan / Brandon Sanderson</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5155,13 +5170,13 @@
         <v>1</v>
       </c>
       <c r="J62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K62" t="n">
         <v>2</v>
       </c>
       <c r="L62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M62" t="n">
         <v>2</v>
@@ -5180,7 +5195,7 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>rescored three times after user corrections on plot details</t>
+          <t>re-audited for v2 axis calibration</t>
         </is>
       </c>
     </row>
@@ -6789,7 +6804,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -6802,7 +6817,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Re-audit round 2: fix Star vs. the Forces of Evil, refine Korra
Extended the tier-5 audit to check each item against the entire tier
roster (not just neighbors) on both the old and new tier, plus a real
tier-label read, per user request.

Comparing against Fullmetal Alchemist: Brotherhood (a non-adjacent tier-4
item built on literal genocide) exposed that Korra and Star vs. the Forces
of Evil had each used one single fact to justify bumps across two or three
different constructs simultaneously -- the same double-counting failure
round 1 was meant to catch, missed because round 1 only checked neighbors.

Star vs. the Forces of Evil drops a full tier (5 -> 4, 5.6625 -> 4.9875),
back to its v1 tier, keeping only the one well-evidenced axis bump.
Korra keeps tier 5 (on independently-evidenced Limited Heroism) but drops
to 5.325 after its Explicit Darkness bump failed a frequency check against
true multi-volume sagas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -4531,26 +4531,26 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Dragonlance</t>
+          <t>Star vs. the Forces of Evil</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Novels / Games</t>
+          <t>TV, Comics</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Margaret Weis / Tracy Hickman</t>
+          <t>Daron Nefcy</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4564,7 +4564,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I53" t="n">
         <v>1</v>
@@ -4579,19 +4579,24 @@
         <v>2</v>
       </c>
       <c r="M53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O53" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="P53" t="n">
-        <v>5.2125</v>
+        <v>4.9875</v>
       </c>
       <c r="Q53" t="n">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -4605,17 +4610,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Harry Potter and the Goblet of Fire</t>
+          <t>Dragonlance</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Novels / Games</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Margaret Weis / Tracy Hickman</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4629,22 +4634,22 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I54" t="n">
         <v>1</v>
       </c>
       <c r="J54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K54" t="n">
         <v>2</v>
       </c>
       <c r="L54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N54" t="n">
         <v>3</v>
@@ -4670,17 +4675,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Elantris</t>
+          <t>Harry Potter and the Goblet of Fire</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4694,22 +4699,22 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I55" t="n">
         <v>1</v>
       </c>
       <c r="J55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K55" t="n">
         <v>2</v>
       </c>
       <c r="L55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N55" t="n">
         <v>3</v>
@@ -4735,17 +4740,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Baldur's Gate III</t>
+          <t>Elantris</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4759,13 +4764,13 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I56" t="n">
         <v>1</v>
       </c>
       <c r="J56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K56" t="n">
         <v>2</v>
@@ -4787,11 +4792,6 @@
       </c>
       <c r="Q56" t="n">
         <v>5</v>
-      </c>
-      <c r="R56" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="57">
@@ -4805,17 +4805,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V: Skyrim</t>
+          <t>Baldur's Gate III</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Bethesda Game Studios</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4829,7 +4829,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I57" t="n">
         <v>1</v>
@@ -4841,22 +4841,27 @@
         <v>2</v>
       </c>
       <c r="L57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O57" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="P57" t="n">
-        <v>5.325</v>
+        <v>5.2125</v>
       </c>
       <c r="Q57" t="n">
         <v>5</v>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -4870,17 +4875,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>The Silmarillion &amp; Great Tales</t>
+          <t>The Elder Scrolls V: Skyrim</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Books</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Bethesda Game Studios</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4906,10 +4911,10 @@
         <v>2</v>
       </c>
       <c r="L58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N58" t="n">
         <v>2</v>
@@ -4935,17 +4940,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Princess Mononoke</t>
+          <t>The Silmarillion &amp; Great Tales</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Books</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4962,28 +4967,28 @@
         <v>2</v>
       </c>
       <c r="I59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J59" t="n">
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O59" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="P59" t="n">
-        <v>5.55</v>
+        <v>5.325</v>
       </c>
       <c r="Q59" t="n">
         <v>5</v>
@@ -5000,17 +5005,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>The Dark Elf / Drizzt</t>
+          <t>The Legend of Korra</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>R. A. Salvatore</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5020,14 +5025,14 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H60" t="n">
         <v>2</v>
       </c>
       <c r="I60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J60" t="n">
         <v>1</v>
@@ -5039,23 +5044,23 @@
         <v>2</v>
       </c>
       <c r="M60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O60" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="P60" t="n">
-        <v>5.55</v>
+        <v>5.325</v>
       </c>
       <c r="Q60" t="n">
         <v>5</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>re-audited for v2 axis calibration</t>
+          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
         </is>
       </c>
     </row>
@@ -5070,17 +5075,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The Legend of Korra</t>
+          <t>Princess Mononoke</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5090,7 +5095,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H61" t="n">
@@ -5100,16 +5105,16 @@
         <v>2</v>
       </c>
       <c r="J61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N61" t="n">
         <v>3</v>
@@ -5122,11 +5127,6 @@
       </c>
       <c r="Q61" t="n">
         <v>5</v>
-      </c>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="62">
@@ -5140,17 +5140,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>The Wheel of Time</t>
+          <t>The Dark Elf / Drizzt</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Robert Jordan / Brandon Sanderson</t>
+          <t>R. A. Salvatore</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5210,17 +5210,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>The Wheel of Time</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Robert Jordan / Brandon Sanderson</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5237,7 +5237,7 @@
         <v>2</v>
       </c>
       <c r="I63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J63" t="n">
         <v>1</v>
@@ -5252,16 +5252,21 @@
         <v>2</v>
       </c>
       <c r="N63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O63" t="n">
-        <v>1.85</v>
+        <v>1.8</v>
       </c>
       <c r="P63" t="n">
-        <v>5.6625</v>
+        <v>5.55</v>
       </c>
       <c r="Q63" t="n">
         <v>5</v>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -5275,17 +5280,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Star vs. the Forces of Evil</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>TV, Comics</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Daron Nefcy</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -6804,7 +6809,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -6817,7 +6822,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Rescore The Legend of Vox Machina to v2 methodology
Tier 4 unchanged from v1 (score 4.8375), scored fresh against the rubric
anchors and checked against the full tier 4/5 rosters. TV-MA content
(confirmed gore, an on-screen torture scene) drives Explicit Darkness to 3,
offset by consistently effective heroism and a contained (not saga-wide)
institutional-evil arc.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R85"/>
+  <dimension ref="A1:R86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4140,17 +4140,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist: Brotherhood</t>
+          <t>The Legend of Vox Machina</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa</t>
+          <t>Critical Role</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -4173,7 +4173,7 @@
         <v>1</v>
       </c>
       <c r="K47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L47" t="n">
         <v>2</v>
@@ -4185,10 +4185,10 @@
         <v>3</v>
       </c>
       <c r="O47" t="n">
-        <v>1.5</v>
+        <v>1.35</v>
       </c>
       <c r="P47" t="n">
-        <v>4.875</v>
+        <v>4.8375</v>
       </c>
       <c r="Q47" t="n">
         <v>4</v>
@@ -4205,17 +4205,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>The Boy and the Heron</t>
+          <t>Fullmetal Alchemist: Brotherhood</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Hiromu Arakawa</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4229,22 +4229,22 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N48" t="n">
         <v>3</v>
@@ -4270,17 +4270,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Final Fantasy IX</t>
+          <t>The Boy and the Heron</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -4294,19 +4294,19 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
       </c>
       <c r="K49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M49" t="n">
         <v>2</v>
@@ -4335,17 +4335,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Ranking of Kings</t>
+          <t>Final Fantasy IX</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Sōsuke Tōka</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4359,19 +4359,19 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I50" t="n">
         <v>1</v>
       </c>
       <c r="J50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K50" t="n">
         <v>2</v>
       </c>
       <c r="L50" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M50" t="n">
         <v>2</v>
@@ -4387,11 +4387,6 @@
       </c>
       <c r="Q50" t="n">
         <v>4</v>
-      </c>
-      <c r="R50" t="inlineStr">
-        <is>
-          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="51">
@@ -4405,17 +4400,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Tales from Earthsea</t>
+          <t>Ranking of Kings</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Gorō Miyazaki</t>
+          <t>Sōsuke Tōka</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4438,29 +4433,29 @@
         <v>1</v>
       </c>
       <c r="K51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M51" t="n">
         <v>2</v>
       </c>
       <c r="N51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O51" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="P51" t="n">
-        <v>4.9875</v>
+        <v>4.875</v>
       </c>
       <c r="Q51" t="n">
         <v>4</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Tier v1 era 5</t>
+          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
         </is>
       </c>
     </row>
@@ -4475,17 +4470,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Adventure Time</t>
+          <t>Tales from Earthsea</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>TV / Comics</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Pendleton Ward</t>
+          <t>Studio Ghibli / Gorō Miyazaki</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4527,6 +4522,11 @@
       </c>
       <c r="Q52" t="n">
         <v>4</v>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -4540,17 +4540,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Star vs. the Forces of Evil</t>
+          <t>Adventure Time</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>TV, Comics</t>
+          <t>TV / Comics</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Daron Nefcy</t>
+          <t>Pendleton Ward</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4564,7 +4564,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I53" t="n">
         <v>1</v>
@@ -4573,7 +4573,7 @@
         <v>1</v>
       </c>
       <c r="K53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L53" t="n">
         <v>2</v>
@@ -4593,34 +4593,29 @@
       <c r="Q53" t="n">
         <v>4</v>
       </c>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Dragonlance</t>
+          <t>Star vs. the Forces of Evil</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Novels / Games</t>
+          <t>TV, Comics</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Margaret Weis / Tracy Hickman</t>
+          <t>Daron Nefcy</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4634,7 +4629,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I54" t="n">
         <v>1</v>
@@ -4649,19 +4644,24 @@
         <v>2</v>
       </c>
       <c r="M54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O54" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="P54" t="n">
-        <v>5.2125</v>
+        <v>4.9875</v>
       </c>
       <c r="Q54" t="n">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -4675,17 +4675,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Harry Potter and the Goblet of Fire</t>
+          <t>Dragonlance</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Novels / Games</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Margaret Weis / Tracy Hickman</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4699,22 +4699,22 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I55" t="n">
         <v>1</v>
       </c>
       <c r="J55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K55" t="n">
         <v>2</v>
       </c>
       <c r="L55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N55" t="n">
         <v>3</v>
@@ -4740,17 +4740,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Elantris</t>
+          <t>Harry Potter and the Goblet of Fire</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4764,22 +4764,22 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I56" t="n">
         <v>1</v>
       </c>
       <c r="J56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K56" t="n">
         <v>2</v>
       </c>
       <c r="L56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N56" t="n">
         <v>3</v>
@@ -4805,17 +4805,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Baldur's Gate III</t>
+          <t>Elantris</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4829,13 +4829,13 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I57" t="n">
         <v>1</v>
       </c>
       <c r="J57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K57" t="n">
         <v>2</v>
@@ -4857,11 +4857,6 @@
       </c>
       <c r="Q57" t="n">
         <v>5</v>
-      </c>
-      <c r="R57" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="58">
@@ -4875,17 +4870,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V: Skyrim</t>
+          <t>Baldur's Gate III</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Bethesda Game Studios</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4899,7 +4894,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I58" t="n">
         <v>1</v>
@@ -4911,22 +4906,27 @@
         <v>2</v>
       </c>
       <c r="L58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O58" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="P58" t="n">
-        <v>5.325</v>
+        <v>5.2125</v>
       </c>
       <c r="Q58" t="n">
         <v>5</v>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -4940,17 +4940,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>The Silmarillion &amp; Great Tales</t>
+          <t>The Elder Scrolls V: Skyrim</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Books</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Bethesda Game Studios</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4976,10 +4976,10 @@
         <v>2</v>
       </c>
       <c r="L59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N59" t="n">
         <v>2</v>
@@ -5005,17 +5005,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>The Legend of Korra</t>
+          <t>The Silmarillion &amp; Great Tales</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Books</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5025,17 +5025,17 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H60" t="n">
         <v>2</v>
       </c>
       <c r="I60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K60" t="n">
         <v>2</v>
@@ -5057,11 +5057,6 @@
       </c>
       <c r="Q60" t="n">
         <v>5</v>
-      </c>
-      <c r="R60" t="inlineStr">
-        <is>
-          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
-        </is>
       </c>
     </row>
     <row r="61">
@@ -5075,17 +5070,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Princess Mononoke</t>
+          <t>The Legend of Korra</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5095,7 +5090,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H61" t="n">
@@ -5105,28 +5100,33 @@
         <v>2</v>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O61" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="P61" t="n">
-        <v>5.55</v>
+        <v>5.325</v>
       </c>
       <c r="Q61" t="n">
         <v>5</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -5140,17 +5140,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>The Dark Elf / Drizzt</t>
+          <t>Princess Mononoke</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>R. A. Salvatore</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5167,16 +5167,16 @@
         <v>2</v>
       </c>
       <c r="I62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M62" t="n">
         <v>2</v>
@@ -5192,11 +5192,6 @@
       </c>
       <c r="Q62" t="n">
         <v>5</v>
-      </c>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="63">
@@ -5210,17 +5205,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The Wheel of Time</t>
+          <t>The Dark Elf / Drizzt</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Robert Jordan / Brandon Sanderson</t>
+          <t>R. A. Salvatore</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5280,17 +5275,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>The Wheel of Time</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Robert Jordan / Brandon Sanderson</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5307,7 +5302,7 @@
         <v>2</v>
       </c>
       <c r="I64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J64" t="n">
         <v>1</v>
@@ -5322,16 +5317,21 @@
         <v>2</v>
       </c>
       <c r="N64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O64" t="n">
-        <v>1.85</v>
+        <v>1.8</v>
       </c>
       <c r="P64" t="n">
-        <v>5.6625</v>
+        <v>5.55</v>
       </c>
       <c r="Q64" t="n">
         <v>5</v>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -5345,17 +5345,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5375,33 +5375,28 @@
         <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M65" t="n">
         <v>2</v>
       </c>
       <c r="N65" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O65" t="n">
-        <v>1.9</v>
+        <v>1.85</v>
       </c>
       <c r="P65" t="n">
-        <v>5.775</v>
+        <v>5.6625</v>
       </c>
       <c r="Q65" t="n">
         <v>5</v>
-      </c>
-      <c r="R65" t="inlineStr">
-        <is>
-          <t>Tier v1 era 6</t>
-        </is>
       </c>
     </row>
     <row r="66">
@@ -5415,17 +5410,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5448,7 +5443,7 @@
         <v>2</v>
       </c>
       <c r="K66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L66" t="n">
         <v>1</v>
@@ -5457,16 +5452,21 @@
         <v>2</v>
       </c>
       <c r="N66" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O66" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="P66" t="n">
-        <v>5.8875</v>
+        <v>5.775</v>
       </c>
       <c r="Q66" t="n">
         <v>5</v>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -5513,10 +5513,10 @@
         <v>2</v>
       </c>
       <c r="K67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M67" t="n">
         <v>2</v>
@@ -5536,26 +5536,26 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5578,7 +5578,7 @@
         <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L68" t="n">
         <v>2</v>
@@ -5590,13 +5590,13 @@
         <v>3</v>
       </c>
       <c r="O68" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P68" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q68" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69">
@@ -5610,17 +5610,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5634,16 +5634,16 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L69" t="n">
         <v>2</v>
@@ -5675,17 +5675,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5699,13 +5699,13 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K70" t="n">
         <v>3</v>
@@ -5717,21 +5717,16 @@
         <v>2</v>
       </c>
       <c r="N70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O70" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P70" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q70" t="n">
         <v>6</v>
-      </c>
-      <c r="R70" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="71">
@@ -5745,17 +5740,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5778,7 +5773,7 @@
         <v>2</v>
       </c>
       <c r="K71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L71" t="n">
         <v>2</v>
@@ -5787,16 +5782,21 @@
         <v>2</v>
       </c>
       <c r="N71" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O71" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P71" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q71" t="n">
         <v>6</v>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -5810,17 +5810,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5834,7 +5834,7 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I72" t="n">
         <v>2</v>
@@ -5852,21 +5852,16 @@
         <v>2</v>
       </c>
       <c r="N72" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O72" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P72" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q72" t="n">
         <v>6</v>
-      </c>
-      <c r="R72" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="73">
@@ -5880,17 +5875,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5904,13 +5899,13 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I73" t="n">
         <v>2</v>
       </c>
       <c r="J73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K73" t="n">
         <v>2</v>
@@ -5935,7 +5930,7 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -5950,17 +5945,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5980,10 +5975,10 @@
         <v>2</v>
       </c>
       <c r="J74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L74" t="n">
         <v>2</v>
@@ -6002,6 +5997,11 @@
       </c>
       <c r="Q74" t="n">
         <v>6</v>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -6015,17 +6015,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6080,17 +6080,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6107,7 +6107,7 @@
         <v>2</v>
       </c>
       <c r="I76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J76" t="n">
         <v>2</v>
@@ -6116,7 +6116,7 @@
         <v>3</v>
       </c>
       <c r="L76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M76" t="n">
         <v>2</v>
@@ -6145,17 +6145,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6169,7 +6169,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I77" t="n">
         <v>1</v>
@@ -6181,7 +6181,7 @@
         <v>3</v>
       </c>
       <c r="L77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M77" t="n">
         <v>2</v>
@@ -6210,17 +6210,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6237,16 +6237,16 @@
         <v>3</v>
       </c>
       <c r="I78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J78" t="n">
         <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M78" t="n">
         <v>2</v>
@@ -6255,18 +6255,13 @@
         <v>3</v>
       </c>
       <c r="O78" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P78" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q78" t="n">
         <v>6</v>
-      </c>
-      <c r="R78" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="79">
@@ -6280,17 +6275,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6304,7 +6299,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I79" t="n">
         <v>2</v>
@@ -6313,7 +6308,7 @@
         <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L79" t="n">
         <v>3</v>
@@ -6333,29 +6328,34 @@
       <c r="Q79" t="n">
         <v>6</v>
       </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6369,16 +6369,16 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I80" t="n">
         <v>2</v>
       </c>
       <c r="J80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L80" t="n">
         <v>3</v>
@@ -6387,40 +6387,40 @@
         <v>2</v>
       </c>
       <c r="N80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O80" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P80" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q80" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6437,31 +6437,31 @@
         <v>3</v>
       </c>
       <c r="I81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J81" t="n">
         <v>3</v>
       </c>
       <c r="K81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L81" t="n">
         <v>3</v>
       </c>
       <c r="M81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N81" t="n">
         <v>4</v>
       </c>
       <c r="O81" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P81" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q81" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="82">
@@ -6475,17 +6475,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6499,31 +6499,31 @@
         </is>
       </c>
       <c r="H82" t="n">
+        <v>3</v>
+      </c>
+      <c r="I82" t="n">
+        <v>3</v>
+      </c>
+      <c r="J82" t="n">
+        <v>3</v>
+      </c>
+      <c r="K82" t="n">
+        <v>3</v>
+      </c>
+      <c r="L82" t="n">
+        <v>3</v>
+      </c>
+      <c r="M82" t="n">
+        <v>3</v>
+      </c>
+      <c r="N82" t="n">
         <v>4</v>
       </c>
-      <c r="I82" t="n">
-        <v>3</v>
-      </c>
-      <c r="J82" t="n">
-        <v>3</v>
-      </c>
-      <c r="K82" t="n">
-        <v>3</v>
-      </c>
-      <c r="L82" t="n">
-        <v>3</v>
-      </c>
-      <c r="M82" t="n">
-        <v>3</v>
-      </c>
-      <c r="N82" t="n">
-        <v>3</v>
-      </c>
       <c r="O82" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P82" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q82" t="n">
         <v>8</v>
@@ -6540,17 +6540,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6564,13 +6564,13 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I83" t="n">
         <v>3</v>
       </c>
       <c r="J83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K83" t="n">
         <v>3</v>
@@ -6582,13 +6582,13 @@
         <v>3</v>
       </c>
       <c r="N83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O83" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P83" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q83" t="n">
         <v>8</v>
@@ -6596,26 +6596,26 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6629,16 +6629,16 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J84" t="n">
         <v>4</v>
       </c>
       <c r="K84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L84" t="n">
         <v>3</v>
@@ -6650,37 +6650,37 @@
         <v>4</v>
       </c>
       <c r="O84" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P84" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q84" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6706,21 +6706,86 @@
         <v>4</v>
       </c>
       <c r="L85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N85" t="n">
         <v>4</v>
       </c>
       <c r="O85" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P85" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>10</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
         <v>4</v>
       </c>
-      <c r="P85" t="n">
+      <c r="I86" t="n">
+        <v>4</v>
+      </c>
+      <c r="J86" t="n">
+        <v>4</v>
+      </c>
+      <c r="K86" t="n">
+        <v>4</v>
+      </c>
+      <c r="L86" t="n">
+        <v>4</v>
+      </c>
+      <c r="M86" t="n">
+        <v>4</v>
+      </c>
+      <c r="N86" t="n">
+        <v>4</v>
+      </c>
+      <c r="O86" t="n">
+        <v>4</v>
+      </c>
+      <c r="P86" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q85" t="n">
+      <c r="Q86" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6809,7 +6874,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -6893,7 +6958,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 84 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 85 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore Final Fantasy VI to v2 methodology
Tier 5 unchanged from v1 (score 5.6625, tied with The Kingkiller Chronicle).
The game's completed mid-story apocalypse drives Structural Despair to 3,
offset by a fully decisive final battle and a plot that actively resolves
its injustices -- deliberately avoiding double-counting the apocalypse fact
across Limited Heroism and Narrative Acceptance of Injustice, the same
failure mode caught in the earlier Korra/Star vs. the Forces of Evil audit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R86"/>
+  <dimension ref="A1:R87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5345,17 +5345,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>Final Fantasy VI</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5369,13 +5369,13 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K65" t="n">
         <v>2</v>
@@ -5384,7 +5384,7 @@
         <v>2</v>
       </c>
       <c r="M65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N65" t="n">
         <v>2</v>
@@ -5410,17 +5410,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5440,33 +5440,28 @@
         <v>2</v>
       </c>
       <c r="J66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M66" t="n">
         <v>2</v>
       </c>
       <c r="N66" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O66" t="n">
-        <v>1.9</v>
+        <v>1.85</v>
       </c>
       <c r="P66" t="n">
-        <v>5.775</v>
+        <v>5.6625</v>
       </c>
       <c r="Q66" t="n">
         <v>5</v>
-      </c>
-      <c r="R66" t="inlineStr">
-        <is>
-          <t>Tier v1 era 6</t>
-        </is>
       </c>
     </row>
     <row r="67">
@@ -5480,17 +5475,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5513,7 +5508,7 @@
         <v>2</v>
       </c>
       <c r="K67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L67" t="n">
         <v>1</v>
@@ -5522,16 +5517,21 @@
         <v>2</v>
       </c>
       <c r="N67" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O67" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="P67" t="n">
-        <v>5.8875</v>
+        <v>5.775</v>
       </c>
       <c r="Q67" t="n">
         <v>5</v>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -5578,10 +5578,10 @@
         <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M68" t="n">
         <v>2</v>
@@ -5601,26 +5601,26 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5643,7 +5643,7 @@
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L69" t="n">
         <v>2</v>
@@ -5655,13 +5655,13 @@
         <v>3</v>
       </c>
       <c r="O69" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P69" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q69" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70">
@@ -5675,17 +5675,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5699,16 +5699,16 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L70" t="n">
         <v>2</v>
@@ -5740,17 +5740,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5764,13 +5764,13 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K71" t="n">
         <v>3</v>
@@ -5782,21 +5782,16 @@
         <v>2</v>
       </c>
       <c r="N71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O71" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P71" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q71" t="n">
         <v>6</v>
-      </c>
-      <c r="R71" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="72">
@@ -5810,17 +5805,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5843,7 +5838,7 @@
         <v>2</v>
       </c>
       <c r="K72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L72" t="n">
         <v>2</v>
@@ -5852,16 +5847,21 @@
         <v>2</v>
       </c>
       <c r="N72" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O72" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P72" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q72" t="n">
         <v>6</v>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -5875,17 +5875,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5899,7 +5899,7 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I73" t="n">
         <v>2</v>
@@ -5917,21 +5917,16 @@
         <v>2</v>
       </c>
       <c r="N73" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O73" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P73" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q73" t="n">
         <v>6</v>
-      </c>
-      <c r="R73" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="74">
@@ -5945,17 +5940,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5969,13 +5964,13 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I74" t="n">
         <v>2</v>
       </c>
       <c r="J74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K74" t="n">
         <v>2</v>
@@ -6000,7 +5995,7 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6015,17 +6010,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6045,10 +6040,10 @@
         <v>2</v>
       </c>
       <c r="J75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L75" t="n">
         <v>2</v>
@@ -6067,6 +6062,11 @@
       </c>
       <c r="Q75" t="n">
         <v>6</v>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -6080,17 +6080,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6145,17 +6145,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6172,7 +6172,7 @@
         <v>2</v>
       </c>
       <c r="I77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J77" t="n">
         <v>2</v>
@@ -6181,7 +6181,7 @@
         <v>3</v>
       </c>
       <c r="L77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M77" t="n">
         <v>2</v>
@@ -6210,17 +6210,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6234,7 +6234,7 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I78" t="n">
         <v>1</v>
@@ -6246,7 +6246,7 @@
         <v>3</v>
       </c>
       <c r="L78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M78" t="n">
         <v>2</v>
@@ -6275,17 +6275,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6302,16 +6302,16 @@
         <v>3</v>
       </c>
       <c r="I79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J79" t="n">
         <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M79" t="n">
         <v>2</v>
@@ -6320,18 +6320,13 @@
         <v>3</v>
       </c>
       <c r="O79" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P79" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q79" t="n">
         <v>6</v>
-      </c>
-      <c r="R79" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="80">
@@ -6345,17 +6340,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6369,7 +6364,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I80" t="n">
         <v>2</v>
@@ -6378,7 +6373,7 @@
         <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L80" t="n">
         <v>3</v>
@@ -6398,29 +6393,34 @@
       <c r="Q80" t="n">
         <v>6</v>
       </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6434,16 +6434,16 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I81" t="n">
         <v>2</v>
       </c>
       <c r="J81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L81" t="n">
         <v>3</v>
@@ -6452,40 +6452,40 @@
         <v>2</v>
       </c>
       <c r="N81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O81" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P81" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q81" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6502,31 +6502,31 @@
         <v>3</v>
       </c>
       <c r="I82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J82" t="n">
         <v>3</v>
       </c>
       <c r="K82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L82" t="n">
         <v>3</v>
       </c>
       <c r="M82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N82" t="n">
         <v>4</v>
       </c>
       <c r="O82" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P82" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q82" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="83">
@@ -6540,17 +6540,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6564,31 +6564,31 @@
         </is>
       </c>
       <c r="H83" t="n">
+        <v>3</v>
+      </c>
+      <c r="I83" t="n">
+        <v>3</v>
+      </c>
+      <c r="J83" t="n">
+        <v>3</v>
+      </c>
+      <c r="K83" t="n">
+        <v>3</v>
+      </c>
+      <c r="L83" t="n">
+        <v>3</v>
+      </c>
+      <c r="M83" t="n">
+        <v>3</v>
+      </c>
+      <c r="N83" t="n">
         <v>4</v>
       </c>
-      <c r="I83" t="n">
-        <v>3</v>
-      </c>
-      <c r="J83" t="n">
-        <v>3</v>
-      </c>
-      <c r="K83" t="n">
-        <v>3</v>
-      </c>
-      <c r="L83" t="n">
-        <v>3</v>
-      </c>
-      <c r="M83" t="n">
-        <v>3</v>
-      </c>
-      <c r="N83" t="n">
-        <v>3</v>
-      </c>
       <c r="O83" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P83" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q83" t="n">
         <v>8</v>
@@ -6605,17 +6605,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6629,13 +6629,13 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I84" t="n">
         <v>3</v>
       </c>
       <c r="J84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K84" t="n">
         <v>3</v>
@@ -6647,13 +6647,13 @@
         <v>3</v>
       </c>
       <c r="N84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O84" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P84" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q84" t="n">
         <v>8</v>
@@ -6661,26 +6661,26 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6694,16 +6694,16 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J85" t="n">
         <v>4</v>
       </c>
       <c r="K85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L85" t="n">
         <v>3</v>
@@ -6715,37 +6715,37 @@
         <v>4</v>
       </c>
       <c r="O85" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P85" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q85" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6771,21 +6771,86 @@
         <v>4</v>
       </c>
       <c r="L86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N86" t="n">
         <v>4</v>
       </c>
       <c r="O86" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P86" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>10</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H87" t="n">
         <v>4</v>
       </c>
-      <c r="P86" t="n">
+      <c r="I87" t="n">
+        <v>4</v>
+      </c>
+      <c r="J87" t="n">
+        <v>4</v>
+      </c>
+      <c r="K87" t="n">
+        <v>4</v>
+      </c>
+      <c r="L87" t="n">
+        <v>4</v>
+      </c>
+      <c r="M87" t="n">
+        <v>4</v>
+      </c>
+      <c r="N87" t="n">
+        <v>4</v>
+      </c>
+      <c r="O87" t="n">
+        <v>4</v>
+      </c>
+      <c r="P87" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q86" t="n">
+      <c r="Q87" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6887,7 +6952,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -6958,7 +7023,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 85 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 86 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore Final Fantasy VII to v2 methodology
Tier 5 unchanged from v1 (score 5.8875, tied with HP Order of the
Phoenix/Half-Blood Prince). Shinra's planet-wide extraction business model
drives Structural Corruption to 3. Cross-checked against HP Deathly Hallows
(tier 6): identical profile except Redemption Difficulty, a well-justified
single-axis gap that accounts for the whole tier difference.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R87"/>
+  <dimension ref="A1:R88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5545,17 +5545,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Final Fantasy VII</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Games / Remake Project</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5572,13 +5572,13 @@
         <v>2</v>
       </c>
       <c r="I68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J68" t="n">
         <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L68" t="n">
         <v>1</v>
@@ -5610,7 +5610,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -5643,10 +5643,10 @@
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M69" t="n">
         <v>2</v>
@@ -5666,26 +5666,26 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5708,7 +5708,7 @@
         <v>2</v>
       </c>
       <c r="K70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L70" t="n">
         <v>2</v>
@@ -5720,13 +5720,13 @@
         <v>3</v>
       </c>
       <c r="O70" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P70" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q70" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
@@ -5740,17 +5740,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5764,16 +5764,16 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L71" t="n">
         <v>2</v>
@@ -5805,17 +5805,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5829,13 +5829,13 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K72" t="n">
         <v>3</v>
@@ -5847,21 +5847,16 @@
         <v>2</v>
       </c>
       <c r="N72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O72" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P72" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q72" t="n">
         <v>6</v>
-      </c>
-      <c r="R72" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="73">
@@ -5875,17 +5870,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5908,7 +5903,7 @@
         <v>2</v>
       </c>
       <c r="K73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L73" t="n">
         <v>2</v>
@@ -5917,16 +5912,21 @@
         <v>2</v>
       </c>
       <c r="N73" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O73" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P73" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q73" t="n">
         <v>6</v>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -5940,17 +5940,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5964,7 +5964,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I74" t="n">
         <v>2</v>
@@ -5982,21 +5982,16 @@
         <v>2</v>
       </c>
       <c r="N74" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O74" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P74" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q74" t="n">
         <v>6</v>
-      </c>
-      <c r="R74" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="75">
@@ -6010,17 +6005,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6034,13 +6029,13 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I75" t="n">
         <v>2</v>
       </c>
       <c r="J75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K75" t="n">
         <v>2</v>
@@ -6065,7 +6060,7 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6080,17 +6075,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6110,10 +6105,10 @@
         <v>2</v>
       </c>
       <c r="J76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L76" t="n">
         <v>2</v>
@@ -6132,6 +6127,11 @@
       </c>
       <c r="Q76" t="n">
         <v>6</v>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -6145,17 +6145,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6210,17 +6210,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6237,7 +6237,7 @@
         <v>2</v>
       </c>
       <c r="I78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J78" t="n">
         <v>2</v>
@@ -6246,7 +6246,7 @@
         <v>3</v>
       </c>
       <c r="L78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M78" t="n">
         <v>2</v>
@@ -6275,17 +6275,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6299,7 +6299,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I79" t="n">
         <v>1</v>
@@ -6311,7 +6311,7 @@
         <v>3</v>
       </c>
       <c r="L79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M79" t="n">
         <v>2</v>
@@ -6340,17 +6340,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6367,16 +6367,16 @@
         <v>3</v>
       </c>
       <c r="I80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J80" t="n">
         <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M80" t="n">
         <v>2</v>
@@ -6385,18 +6385,13 @@
         <v>3</v>
       </c>
       <c r="O80" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P80" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q80" t="n">
         <v>6</v>
-      </c>
-      <c r="R80" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="81">
@@ -6410,17 +6405,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6434,7 +6429,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I81" t="n">
         <v>2</v>
@@ -6443,7 +6438,7 @@
         <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L81" t="n">
         <v>3</v>
@@ -6463,29 +6458,34 @@
       <c r="Q81" t="n">
         <v>6</v>
       </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6499,16 +6499,16 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I82" t="n">
         <v>2</v>
       </c>
       <c r="J82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L82" t="n">
         <v>3</v>
@@ -6517,40 +6517,40 @@
         <v>2</v>
       </c>
       <c r="N82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O82" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P82" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q82" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6567,31 +6567,31 @@
         <v>3</v>
       </c>
       <c r="I83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J83" t="n">
         <v>3</v>
       </c>
       <c r="K83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L83" t="n">
         <v>3</v>
       </c>
       <c r="M83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N83" t="n">
         <v>4</v>
       </c>
       <c r="O83" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P83" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q83" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="84">
@@ -6605,17 +6605,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6629,31 +6629,31 @@
         </is>
       </c>
       <c r="H84" t="n">
+        <v>3</v>
+      </c>
+      <c r="I84" t="n">
+        <v>3</v>
+      </c>
+      <c r="J84" t="n">
+        <v>3</v>
+      </c>
+      <c r="K84" t="n">
+        <v>3</v>
+      </c>
+      <c r="L84" t="n">
+        <v>3</v>
+      </c>
+      <c r="M84" t="n">
+        <v>3</v>
+      </c>
+      <c r="N84" t="n">
         <v>4</v>
       </c>
-      <c r="I84" t="n">
-        <v>3</v>
-      </c>
-      <c r="J84" t="n">
-        <v>3</v>
-      </c>
-      <c r="K84" t="n">
-        <v>3</v>
-      </c>
-      <c r="L84" t="n">
-        <v>3</v>
-      </c>
-      <c r="M84" t="n">
-        <v>3</v>
-      </c>
-      <c r="N84" t="n">
-        <v>3</v>
-      </c>
       <c r="O84" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P84" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q84" t="n">
         <v>8</v>
@@ -6670,17 +6670,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6694,13 +6694,13 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I85" t="n">
         <v>3</v>
       </c>
       <c r="J85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K85" t="n">
         <v>3</v>
@@ -6712,13 +6712,13 @@
         <v>3</v>
       </c>
       <c r="N85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O85" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P85" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q85" t="n">
         <v>8</v>
@@ -6726,26 +6726,26 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6759,16 +6759,16 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J86" t="n">
         <v>4</v>
       </c>
       <c r="K86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L86" t="n">
         <v>3</v>
@@ -6780,37 +6780,37 @@
         <v>4</v>
       </c>
       <c r="O86" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P86" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q86" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6836,21 +6836,86 @@
         <v>4</v>
       </c>
       <c r="L87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N87" t="n">
         <v>4</v>
       </c>
       <c r="O87" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P87" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>10</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
         <v>4</v>
       </c>
-      <c r="P87" t="n">
+      <c r="I88" t="n">
+        <v>4</v>
+      </c>
+      <c r="J88" t="n">
+        <v>4</v>
+      </c>
+      <c r="K88" t="n">
+        <v>4</v>
+      </c>
+      <c r="L88" t="n">
+        <v>4</v>
+      </c>
+      <c r="M88" t="n">
+        <v>4</v>
+      </c>
+      <c r="N88" t="n">
+        <v>4</v>
+      </c>
+      <c r="O88" t="n">
+        <v>4</v>
+      </c>
+      <c r="P88" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q87" t="n">
+      <c r="Q88" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6952,7 +7017,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -7023,7 +7088,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 86 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 87 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore Final Fantasy X to v2 methodology
Tier 5 unchanged from v1 (score 5.8875, tied with Final Fantasy
VII/HP Order of the Phoenix/Half-Blood Prince). Sin's thousand-year
repeating destruction cycle drives Structural Despair to 3; Yevon's
church-and-state fusion, founded on a lie to sustain its own power, drives
Structural Corruption to 3. Kept Limited Heroism low since the party's
victory is unusually complete -- unlike every prior summoner's temporary
fix, this one permanently ends the cycle.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R88"/>
+  <dimension ref="A1:R89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5545,17 +5545,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Final Fantasy VII</t>
+          <t>Final Fantasy X</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Video Games / Remake Project</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5569,7 +5569,7 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I68" t="n">
         <v>1</v>
@@ -5584,7 +5584,7 @@
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N68" t="n">
         <v>3</v>
@@ -5610,17 +5610,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Final Fantasy VII</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Games / Remake Project</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5637,13 +5637,13 @@
         <v>2</v>
       </c>
       <c r="I69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J69" t="n">
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L69" t="n">
         <v>1</v>
@@ -5675,7 +5675,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -5708,10 +5708,10 @@
         <v>2</v>
       </c>
       <c r="K70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M70" t="n">
         <v>2</v>
@@ -5731,26 +5731,26 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5773,7 +5773,7 @@
         <v>2</v>
       </c>
       <c r="K71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L71" t="n">
         <v>2</v>
@@ -5785,13 +5785,13 @@
         <v>3</v>
       </c>
       <c r="O71" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P71" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q71" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="72">
@@ -5805,17 +5805,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5829,16 +5829,16 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L72" t="n">
         <v>2</v>
@@ -5870,17 +5870,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5894,13 +5894,13 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K73" t="n">
         <v>3</v>
@@ -5912,21 +5912,16 @@
         <v>2</v>
       </c>
       <c r="N73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O73" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P73" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q73" t="n">
         <v>6</v>
-      </c>
-      <c r="R73" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="74">
@@ -5940,17 +5935,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5973,7 +5968,7 @@
         <v>2</v>
       </c>
       <c r="K74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L74" t="n">
         <v>2</v>
@@ -5982,16 +5977,21 @@
         <v>2</v>
       </c>
       <c r="N74" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O74" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P74" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q74" t="n">
         <v>6</v>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -6005,17 +6005,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I75" t="n">
         <v>2</v>
@@ -6047,21 +6047,16 @@
         <v>2</v>
       </c>
       <c r="N75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O75" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P75" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q75" t="n">
         <v>6</v>
-      </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="76">
@@ -6075,17 +6070,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6099,13 +6094,13 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I76" t="n">
         <v>2</v>
       </c>
       <c r="J76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K76" t="n">
         <v>2</v>
@@ -6130,7 +6125,7 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6145,17 +6140,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6175,10 +6170,10 @@
         <v>2</v>
       </c>
       <c r="J77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L77" t="n">
         <v>2</v>
@@ -6197,6 +6192,11 @@
       </c>
       <c r="Q77" t="n">
         <v>6</v>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -6210,17 +6210,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6275,17 +6275,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6302,7 +6302,7 @@
         <v>2</v>
       </c>
       <c r="I79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J79" t="n">
         <v>2</v>
@@ -6311,7 +6311,7 @@
         <v>3</v>
       </c>
       <c r="L79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M79" t="n">
         <v>2</v>
@@ -6340,17 +6340,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6364,7 +6364,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I80" t="n">
         <v>1</v>
@@ -6376,7 +6376,7 @@
         <v>3</v>
       </c>
       <c r="L80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M80" t="n">
         <v>2</v>
@@ -6405,17 +6405,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6432,16 +6432,16 @@
         <v>3</v>
       </c>
       <c r="I81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J81" t="n">
         <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M81" t="n">
         <v>2</v>
@@ -6450,18 +6450,13 @@
         <v>3</v>
       </c>
       <c r="O81" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P81" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q81" t="n">
         <v>6</v>
-      </c>
-      <c r="R81" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="82">
@@ -6475,17 +6470,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6499,7 +6494,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I82" t="n">
         <v>2</v>
@@ -6508,7 +6503,7 @@
         <v>2</v>
       </c>
       <c r="K82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L82" t="n">
         <v>3</v>
@@ -6528,29 +6523,34 @@
       <c r="Q82" t="n">
         <v>6</v>
       </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6564,16 +6564,16 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I83" t="n">
         <v>2</v>
       </c>
       <c r="J83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L83" t="n">
         <v>3</v>
@@ -6582,40 +6582,40 @@
         <v>2</v>
       </c>
       <c r="N83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O83" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P83" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q83" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6632,31 +6632,31 @@
         <v>3</v>
       </c>
       <c r="I84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J84" t="n">
         <v>3</v>
       </c>
       <c r="K84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L84" t="n">
         <v>3</v>
       </c>
       <c r="M84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N84" t="n">
         <v>4</v>
       </c>
       <c r="O84" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P84" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q84" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="85">
@@ -6670,17 +6670,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6694,31 +6694,31 @@
         </is>
       </c>
       <c r="H85" t="n">
+        <v>3</v>
+      </c>
+      <c r="I85" t="n">
+        <v>3</v>
+      </c>
+      <c r="J85" t="n">
+        <v>3</v>
+      </c>
+      <c r="K85" t="n">
+        <v>3</v>
+      </c>
+      <c r="L85" t="n">
+        <v>3</v>
+      </c>
+      <c r="M85" t="n">
+        <v>3</v>
+      </c>
+      <c r="N85" t="n">
         <v>4</v>
       </c>
-      <c r="I85" t="n">
-        <v>3</v>
-      </c>
-      <c r="J85" t="n">
-        <v>3</v>
-      </c>
-      <c r="K85" t="n">
-        <v>3</v>
-      </c>
-      <c r="L85" t="n">
-        <v>3</v>
-      </c>
-      <c r="M85" t="n">
-        <v>3</v>
-      </c>
-      <c r="N85" t="n">
-        <v>3</v>
-      </c>
       <c r="O85" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P85" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q85" t="n">
         <v>8</v>
@@ -6735,17 +6735,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6759,13 +6759,13 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I86" t="n">
         <v>3</v>
       </c>
       <c r="J86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K86" t="n">
         <v>3</v>
@@ -6777,13 +6777,13 @@
         <v>3</v>
       </c>
       <c r="N86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O86" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P86" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q86" t="n">
         <v>8</v>
@@ -6791,26 +6791,26 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6824,16 +6824,16 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J87" t="n">
         <v>4</v>
       </c>
       <c r="K87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L87" t="n">
         <v>3</v>
@@ -6845,37 +6845,37 @@
         <v>4</v>
       </c>
       <c r="O87" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P87" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q87" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6901,21 +6901,86 @@
         <v>4</v>
       </c>
       <c r="L88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N88" t="n">
         <v>4</v>
       </c>
       <c r="O88" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P88" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>10</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H89" t="n">
         <v>4</v>
       </c>
-      <c r="P88" t="n">
+      <c r="I89" t="n">
+        <v>4</v>
+      </c>
+      <c r="J89" t="n">
+        <v>4</v>
+      </c>
+      <c r="K89" t="n">
+        <v>4</v>
+      </c>
+      <c r="L89" t="n">
+        <v>4</v>
+      </c>
+      <c r="M89" t="n">
+        <v>4</v>
+      </c>
+      <c r="N89" t="n">
+        <v>4</v>
+      </c>
+      <c r="O89" t="n">
+        <v>4</v>
+      </c>
+      <c r="P89" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q88" t="n">
+      <c r="Q89" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7017,7 +7082,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -7088,7 +7153,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 87 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 88 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore Final Fantasy XV to v2 methodology, complete tier 5 backlog
Tier 5 unchanged from v1 (score 5.8875, tied with FFVII/FFX/HP Order of
the Phoenix/Half-Blood Prince). First pass landed tier 6 by letting
Ardyn's tragic backstory inflate both Moral Cynicism and Narrative
Acceptance of Injustice toward the same conclusion; corrected by keeping
NAI low since the story's own central conflicts are all fully resolved,
unlike Ardyn's untouched ancient grievance. The ten-year Long Night drives
Structural Despair to 3.

This completes the tier-5 v2 rescoring backlog (4/4).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R89"/>
+  <dimension ref="A1:R90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5796,26 +5796,26 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Final Fantasy XV</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5829,10 +5829,10 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J72" t="n">
         <v>2</v>
@@ -5844,19 +5844,19 @@
         <v>2</v>
       </c>
       <c r="M72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N72" t="n">
         <v>3</v>
       </c>
       <c r="O72" t="n">
-        <v>2.1</v>
+        <v>1.95</v>
       </c>
       <c r="P72" t="n">
-        <v>6.225</v>
+        <v>5.8875</v>
       </c>
       <c r="Q72" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="73">
@@ -5870,17 +5870,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5894,16 +5894,16 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L73" t="n">
         <v>2</v>
@@ -5935,17 +5935,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5959,13 +5959,13 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K74" t="n">
         <v>3</v>
@@ -5977,21 +5977,16 @@
         <v>2</v>
       </c>
       <c r="N74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O74" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P74" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q74" t="n">
         <v>6</v>
-      </c>
-      <c r="R74" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="75">
@@ -6005,17 +6000,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6038,7 +6033,7 @@
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L75" t="n">
         <v>2</v>
@@ -6047,16 +6042,21 @@
         <v>2</v>
       </c>
       <c r="N75" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O75" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P75" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q75" t="n">
         <v>6</v>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -6070,17 +6070,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6094,7 +6094,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I76" t="n">
         <v>2</v>
@@ -6112,21 +6112,16 @@
         <v>2</v>
       </c>
       <c r="N76" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O76" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P76" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q76" t="n">
         <v>6</v>
-      </c>
-      <c r="R76" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="77">
@@ -6140,17 +6135,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6164,13 +6159,13 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I77" t="n">
         <v>2</v>
       </c>
       <c r="J77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K77" t="n">
         <v>2</v>
@@ -6195,7 +6190,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6210,17 +6205,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6240,10 +6235,10 @@
         <v>2</v>
       </c>
       <c r="J78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L78" t="n">
         <v>2</v>
@@ -6262,6 +6257,11 @@
       </c>
       <c r="Q78" t="n">
         <v>6</v>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -6275,17 +6275,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6340,17 +6340,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6367,7 +6367,7 @@
         <v>2</v>
       </c>
       <c r="I80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J80" t="n">
         <v>2</v>
@@ -6376,7 +6376,7 @@
         <v>3</v>
       </c>
       <c r="L80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M80" t="n">
         <v>2</v>
@@ -6405,17 +6405,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6429,7 +6429,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I81" t="n">
         <v>1</v>
@@ -6441,7 +6441,7 @@
         <v>3</v>
       </c>
       <c r="L81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M81" t="n">
         <v>2</v>
@@ -6470,17 +6470,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6497,16 +6497,16 @@
         <v>3</v>
       </c>
       <c r="I82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J82" t="n">
         <v>2</v>
       </c>
       <c r="K82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M82" t="n">
         <v>2</v>
@@ -6515,18 +6515,13 @@
         <v>3</v>
       </c>
       <c r="O82" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P82" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q82" t="n">
         <v>6</v>
-      </c>
-      <c r="R82" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="83">
@@ -6540,17 +6535,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6564,7 +6559,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I83" t="n">
         <v>2</v>
@@ -6573,7 +6568,7 @@
         <v>2</v>
       </c>
       <c r="K83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L83" t="n">
         <v>3</v>
@@ -6593,29 +6588,34 @@
       <c r="Q83" t="n">
         <v>6</v>
       </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6629,16 +6629,16 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I84" t="n">
         <v>2</v>
       </c>
       <c r="J84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L84" t="n">
         <v>3</v>
@@ -6647,40 +6647,40 @@
         <v>2</v>
       </c>
       <c r="N84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O84" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P84" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q84" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6697,31 +6697,31 @@
         <v>3</v>
       </c>
       <c r="I85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J85" t="n">
         <v>3</v>
       </c>
       <c r="K85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L85" t="n">
         <v>3</v>
       </c>
       <c r="M85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N85" t="n">
         <v>4</v>
       </c>
       <c r="O85" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P85" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q85" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="86">
@@ -6735,17 +6735,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6759,31 +6759,31 @@
         </is>
       </c>
       <c r="H86" t="n">
+        <v>3</v>
+      </c>
+      <c r="I86" t="n">
+        <v>3</v>
+      </c>
+      <c r="J86" t="n">
+        <v>3</v>
+      </c>
+      <c r="K86" t="n">
+        <v>3</v>
+      </c>
+      <c r="L86" t="n">
+        <v>3</v>
+      </c>
+      <c r="M86" t="n">
+        <v>3</v>
+      </c>
+      <c r="N86" t="n">
         <v>4</v>
       </c>
-      <c r="I86" t="n">
-        <v>3</v>
-      </c>
-      <c r="J86" t="n">
-        <v>3</v>
-      </c>
-      <c r="K86" t="n">
-        <v>3</v>
-      </c>
-      <c r="L86" t="n">
-        <v>3</v>
-      </c>
-      <c r="M86" t="n">
-        <v>3</v>
-      </c>
-      <c r="N86" t="n">
-        <v>3</v>
-      </c>
       <c r="O86" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P86" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q86" t="n">
         <v>8</v>
@@ -6800,17 +6800,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6824,13 +6824,13 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I87" t="n">
         <v>3</v>
       </c>
       <c r="J87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K87" t="n">
         <v>3</v>
@@ -6842,13 +6842,13 @@
         <v>3</v>
       </c>
       <c r="N87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O87" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P87" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q87" t="n">
         <v>8</v>
@@ -6856,26 +6856,26 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6889,16 +6889,16 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J88" t="n">
         <v>4</v>
       </c>
       <c r="K88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L88" t="n">
         <v>3</v>
@@ -6910,37 +6910,37 @@
         <v>4</v>
       </c>
       <c r="O88" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P88" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q88" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6966,21 +6966,86 @@
         <v>4</v>
       </c>
       <c r="L89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N89" t="n">
         <v>4</v>
       </c>
       <c r="O89" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P89" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>10</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
         <v>4</v>
       </c>
-      <c r="P89" t="n">
+      <c r="I90" t="n">
+        <v>4</v>
+      </c>
+      <c r="J90" t="n">
+        <v>4</v>
+      </c>
+      <c r="K90" t="n">
+        <v>4</v>
+      </c>
+      <c r="L90" t="n">
+        <v>4</v>
+      </c>
+      <c r="M90" t="n">
+        <v>4</v>
+      </c>
+      <c r="N90" t="n">
+        <v>4</v>
+      </c>
+      <c r="O90" t="n">
+        <v>4</v>
+      </c>
+      <c r="P90" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q89" t="n">
+      <c r="Q90" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7082,7 +7147,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -7153,7 +7218,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 88 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 89 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore Clevatess to v2 methodology
Tier 6 unchanged from v1 (score 6.1125). Lower-confidence entry than the
recent mainstream franchises -- scored partly from the existing summary
already in this log rather than fresh primary-source detail. Explicit
Darkness at 4 (an official content warning for sustained abuse, plus
infant trafficking) is the standout axis; Structural Corruption
reconsidered down to 2, flagged as the most uncertain call.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R90"/>
+  <dimension ref="A1:R91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5870,17 +5870,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Clevatess</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>Yūji Iwahara</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5906,22 +5906,27 @@
         <v>2</v>
       </c>
       <c r="L73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M73" t="n">
         <v>2</v>
       </c>
       <c r="N73" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O73" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="P73" t="n">
-        <v>6.225</v>
+        <v>6.1125</v>
       </c>
       <c r="Q73" t="n">
         <v>6</v>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>scored against the story as currently published/aired; ongoing/unresolved, later arcs may shift this</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -5935,17 +5940,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5959,16 +5964,16 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L74" t="n">
         <v>2</v>
@@ -6000,17 +6005,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6024,13 +6029,13 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K75" t="n">
         <v>3</v>
@@ -6042,21 +6047,16 @@
         <v>2</v>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O75" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P75" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q75" t="n">
         <v>6</v>
-      </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="76">
@@ -6070,17 +6070,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6103,7 +6103,7 @@
         <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L76" t="n">
         <v>2</v>
@@ -6112,16 +6112,21 @@
         <v>2</v>
       </c>
       <c r="N76" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O76" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P76" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q76" t="n">
         <v>6</v>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -6135,17 +6140,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6159,7 +6164,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I77" t="n">
         <v>2</v>
@@ -6177,21 +6182,16 @@
         <v>2</v>
       </c>
       <c r="N77" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O77" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P77" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q77" t="n">
         <v>6</v>
-      </c>
-      <c r="R77" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="78">
@@ -6205,17 +6205,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6229,13 +6229,13 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I78" t="n">
         <v>2</v>
       </c>
       <c r="J78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K78" t="n">
         <v>2</v>
@@ -6260,7 +6260,7 @@
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6275,17 +6275,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6305,10 +6305,10 @@
         <v>2</v>
       </c>
       <c r="J79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L79" t="n">
         <v>2</v>
@@ -6327,6 +6327,11 @@
       </c>
       <c r="Q79" t="n">
         <v>6</v>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -6340,17 +6345,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6405,17 +6410,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6432,7 +6437,7 @@
         <v>2</v>
       </c>
       <c r="I81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J81" t="n">
         <v>2</v>
@@ -6441,7 +6446,7 @@
         <v>3</v>
       </c>
       <c r="L81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M81" t="n">
         <v>2</v>
@@ -6470,17 +6475,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6494,7 +6499,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I82" t="n">
         <v>1</v>
@@ -6506,7 +6511,7 @@
         <v>3</v>
       </c>
       <c r="L82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M82" t="n">
         <v>2</v>
@@ -6535,17 +6540,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6562,16 +6567,16 @@
         <v>3</v>
       </c>
       <c r="I83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J83" t="n">
         <v>2</v>
       </c>
       <c r="K83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M83" t="n">
         <v>2</v>
@@ -6580,18 +6585,13 @@
         <v>3</v>
       </c>
       <c r="O83" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P83" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q83" t="n">
         <v>6</v>
-      </c>
-      <c r="R83" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="84">
@@ -6605,17 +6605,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6629,7 +6629,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I84" t="n">
         <v>2</v>
@@ -6638,7 +6638,7 @@
         <v>2</v>
       </c>
       <c r="K84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L84" t="n">
         <v>3</v>
@@ -6658,29 +6658,34 @@
       <c r="Q84" t="n">
         <v>6</v>
       </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6694,16 +6699,16 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I85" t="n">
         <v>2</v>
       </c>
       <c r="J85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L85" t="n">
         <v>3</v>
@@ -6712,40 +6717,40 @@
         <v>2</v>
       </c>
       <c r="N85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O85" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P85" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6762,31 +6767,31 @@
         <v>3</v>
       </c>
       <c r="I86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J86" t="n">
         <v>3</v>
       </c>
       <c r="K86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L86" t="n">
         <v>3</v>
       </c>
       <c r="M86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N86" t="n">
         <v>4</v>
       </c>
       <c r="O86" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P86" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q86" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="87">
@@ -6800,17 +6805,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6824,31 +6829,31 @@
         </is>
       </c>
       <c r="H87" t="n">
+        <v>3</v>
+      </c>
+      <c r="I87" t="n">
+        <v>3</v>
+      </c>
+      <c r="J87" t="n">
+        <v>3</v>
+      </c>
+      <c r="K87" t="n">
+        <v>3</v>
+      </c>
+      <c r="L87" t="n">
+        <v>3</v>
+      </c>
+      <c r="M87" t="n">
+        <v>3</v>
+      </c>
+      <c r="N87" t="n">
         <v>4</v>
       </c>
-      <c r="I87" t="n">
-        <v>3</v>
-      </c>
-      <c r="J87" t="n">
-        <v>3</v>
-      </c>
-      <c r="K87" t="n">
-        <v>3</v>
-      </c>
-      <c r="L87" t="n">
-        <v>3</v>
-      </c>
-      <c r="M87" t="n">
-        <v>3</v>
-      </c>
-      <c r="N87" t="n">
-        <v>3</v>
-      </c>
       <c r="O87" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P87" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q87" t="n">
         <v>8</v>
@@ -6865,17 +6870,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6889,13 +6894,13 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I88" t="n">
         <v>3</v>
       </c>
       <c r="J88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K88" t="n">
         <v>3</v>
@@ -6907,13 +6912,13 @@
         <v>3</v>
       </c>
       <c r="N88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O88" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P88" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q88" t="n">
         <v>8</v>
@@ -6921,26 +6926,26 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6954,16 +6959,16 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J89" t="n">
         <v>4</v>
       </c>
       <c r="K89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L89" t="n">
         <v>3</v>
@@ -6975,37 +6980,37 @@
         <v>4</v>
       </c>
       <c r="O89" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P89" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q89" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -7031,21 +7036,86 @@
         <v>4</v>
       </c>
       <c r="L90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N90" t="n">
         <v>4</v>
       </c>
       <c r="O90" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P90" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>10</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H91" t="n">
         <v>4</v>
       </c>
-      <c r="P90" t="n">
+      <c r="I91" t="n">
+        <v>4</v>
+      </c>
+      <c r="J91" t="n">
+        <v>4</v>
+      </c>
+      <c r="K91" t="n">
+        <v>4</v>
+      </c>
+      <c r="L91" t="n">
+        <v>4</v>
+      </c>
+      <c r="M91" t="n">
+        <v>4</v>
+      </c>
+      <c r="N91" t="n">
+        <v>4</v>
+      </c>
+      <c r="O91" t="n">
+        <v>4</v>
+      </c>
+      <c r="P91" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q90" t="n">
+      <c r="Q91" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7160,7 +7230,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -7218,7 +7288,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 89 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 90 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore Re:Zero to v2 methodology, complete v2 backlog except Marchen Crown
Tier 6 unchanged from v1 (score 6.1125, tied exactly with Clevatess).
Return by Death's genuinely graphic, repeated on-screen deaths are a
central, recurring narrative feature (Explicit Darkness 4). Limited
Heroism stays low since the loop mechanic lets Subaru genuinely undo
failures, unlike Made in Abyss's permanent, irreversible Curse of the
Abyss -- a specific reason for the gap between two otherwise similar
ED4 entries.

This completes the tier-6 v2 rescoring backlog (2/2) and, with it, the
entire v2 rescoring backlog: 91 of 92 catalog works are now scored under
v2. Only Marchen Crown remains, parked earlier for low confidence.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R91"/>
+  <dimension ref="A1:R92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5940,17 +5940,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Re:Zero − Starting Life in Another World</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Light Novels, Manga, Anime</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>Tappei Nagatsuki</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5967,7 +5967,7 @@
         <v>2</v>
       </c>
       <c r="I74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J74" t="n">
         <v>2</v>
@@ -5982,16 +5982,21 @@
         <v>2</v>
       </c>
       <c r="N74" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O74" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="P74" t="n">
-        <v>6.225</v>
+        <v>6.1125</v>
       </c>
       <c r="Q74" t="n">
         <v>6</v>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>scored against the arcs most widely adapted/translated (roughly Arcs 1-6); later arcs may shift this</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -6005,17 +6010,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6029,16 +6034,16 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L75" t="n">
         <v>2</v>
@@ -6070,17 +6075,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6094,13 +6099,13 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K76" t="n">
         <v>3</v>
@@ -6112,21 +6117,16 @@
         <v>2</v>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O76" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P76" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q76" t="n">
         <v>6</v>
-      </c>
-      <c r="R76" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="77">
@@ -6140,17 +6140,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6173,7 +6173,7 @@
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L77" t="n">
         <v>2</v>
@@ -6182,16 +6182,21 @@
         <v>2</v>
       </c>
       <c r="N77" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O77" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P77" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q77" t="n">
         <v>6</v>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -6205,17 +6210,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6229,7 +6234,7 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I78" t="n">
         <v>2</v>
@@ -6247,21 +6252,16 @@
         <v>2</v>
       </c>
       <c r="N78" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O78" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P78" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q78" t="n">
         <v>6</v>
-      </c>
-      <c r="R78" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="79">
@@ -6275,17 +6275,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6299,13 +6299,13 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I79" t="n">
         <v>2</v>
       </c>
       <c r="J79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K79" t="n">
         <v>2</v>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6345,17 +6345,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6375,10 +6375,10 @@
         <v>2</v>
       </c>
       <c r="J80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L80" t="n">
         <v>2</v>
@@ -6397,6 +6397,11 @@
       </c>
       <c r="Q80" t="n">
         <v>6</v>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -6410,17 +6415,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6475,17 +6480,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6502,7 +6507,7 @@
         <v>2</v>
       </c>
       <c r="I82" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J82" t="n">
         <v>2</v>
@@ -6511,7 +6516,7 @@
         <v>3</v>
       </c>
       <c r="L82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M82" t="n">
         <v>2</v>
@@ -6540,17 +6545,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6564,7 +6569,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I83" t="n">
         <v>1</v>
@@ -6576,7 +6581,7 @@
         <v>3</v>
       </c>
       <c r="L83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M83" t="n">
         <v>2</v>
@@ -6605,17 +6610,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6632,16 +6637,16 @@
         <v>3</v>
       </c>
       <c r="I84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J84" t="n">
         <v>2</v>
       </c>
       <c r="K84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M84" t="n">
         <v>2</v>
@@ -6650,18 +6655,13 @@
         <v>3</v>
       </c>
       <c r="O84" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="P84" t="n">
-        <v>6.9</v>
+        <v>6.5625</v>
       </c>
       <c r="Q84" t="n">
         <v>6</v>
-      </c>
-      <c r="R84" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="85">
@@ -6675,17 +6675,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6699,7 +6699,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I85" t="n">
         <v>2</v>
@@ -6708,7 +6708,7 @@
         <v>2</v>
       </c>
       <c r="K85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L85" t="n">
         <v>3</v>
@@ -6728,29 +6728,34 @@
       <c r="Q85" t="n">
         <v>6</v>
       </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6764,16 +6769,16 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I86" t="n">
         <v>2</v>
       </c>
       <c r="J86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K86" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L86" t="n">
         <v>3</v>
@@ -6782,40 +6787,40 @@
         <v>2</v>
       </c>
       <c r="N86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O86" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P86" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q86" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6832,31 +6837,31 @@
         <v>3</v>
       </c>
       <c r="I87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J87" t="n">
         <v>3</v>
       </c>
       <c r="K87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L87" t="n">
         <v>3</v>
       </c>
       <c r="M87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N87" t="n">
         <v>4</v>
       </c>
       <c r="O87" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P87" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q87" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="88">
@@ -6870,17 +6875,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6894,31 +6899,31 @@
         </is>
       </c>
       <c r="H88" t="n">
+        <v>3</v>
+      </c>
+      <c r="I88" t="n">
+        <v>3</v>
+      </c>
+      <c r="J88" t="n">
+        <v>3</v>
+      </c>
+      <c r="K88" t="n">
+        <v>3</v>
+      </c>
+      <c r="L88" t="n">
+        <v>3</v>
+      </c>
+      <c r="M88" t="n">
+        <v>3</v>
+      </c>
+      <c r="N88" t="n">
         <v>4</v>
       </c>
-      <c r="I88" t="n">
-        <v>3</v>
-      </c>
-      <c r="J88" t="n">
-        <v>3</v>
-      </c>
-      <c r="K88" t="n">
-        <v>3</v>
-      </c>
-      <c r="L88" t="n">
-        <v>3</v>
-      </c>
-      <c r="M88" t="n">
-        <v>3</v>
-      </c>
-      <c r="N88" t="n">
-        <v>3</v>
-      </c>
       <c r="O88" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P88" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q88" t="n">
         <v>8</v>
@@ -6935,17 +6940,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6959,13 +6964,13 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I89" t="n">
         <v>3</v>
       </c>
       <c r="J89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K89" t="n">
         <v>3</v>
@@ -6977,13 +6982,13 @@
         <v>3</v>
       </c>
       <c r="N89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O89" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P89" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q89" t="n">
         <v>8</v>
@@ -6991,26 +6996,26 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -7024,16 +7029,16 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J90" t="n">
         <v>4</v>
       </c>
       <c r="K90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L90" t="n">
         <v>3</v>
@@ -7045,37 +7050,37 @@
         <v>4</v>
       </c>
       <c r="O90" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P90" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q90" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -7101,21 +7106,86 @@
         <v>4</v>
       </c>
       <c r="L91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N91" t="n">
         <v>4</v>
       </c>
       <c r="O91" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P91" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>10</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H92" t="n">
         <v>4</v>
       </c>
-      <c r="P91" t="n">
+      <c r="I92" t="n">
+        <v>4</v>
+      </c>
+      <c r="J92" t="n">
+        <v>4</v>
+      </c>
+      <c r="K92" t="n">
+        <v>4</v>
+      </c>
+      <c r="L92" t="n">
+        <v>4</v>
+      </c>
+      <c r="M92" t="n">
+        <v>4</v>
+      </c>
+      <c r="N92" t="n">
+        <v>4</v>
+      </c>
+      <c r="O92" t="n">
+        <v>4</v>
+      </c>
+      <c r="P92" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q91" t="n">
+      <c r="Q92" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7230,7 +7300,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -7288,7 +7358,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 90 of 92 works in the full catalog (work in progress).</t>
+          <t>Total scored: 91 of 92 works in the full catalog (work in progress).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix underscored The Nightmare Before Christmas entry
User flagged this as underscored on the live site (2.29, tier 2). It was
one of the first entries scored under v2, before the more disciplined
process used throughout the rest of this backlog -- Explicit Darkness was
capped at 2 despite this exact entry's own documented content list
(Sally's recurring self-dismemberment, Oogie Boogie's sadism, the
shooting-down sequence) already establishing frequent, genuinely macabre
content when the v1 tier-1-to-tier-2 correction was made.

Revised Explicit Darkness to 3, landing at 2.5125 -- tier unchanged, but
now tied exactly with Legend, a strong precedent match (same profile,
same "atmospheric horror-villain content, story resolves cleanly" shape).
Updated the xlsx, scoring record, and live site.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1748,7 +1748,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>The Nightmare Before Christmas</t>
+          <t>Castle in the Sky</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tim Burton / Henry Selick</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1781,10 +1781,10 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -1801,7 +1801,6 @@
       <c r="Q11" t="n">
         <v>2</v>
       </c>
-      <c r="R11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1814,7 +1813,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Castle in the Sky</t>
+          <t>Dungeons &amp; Dragons: Honor Among Thieves</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1824,7 +1823,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Jonathan Goldstein / John Francis Daley</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1844,7 +1843,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
         <v>1</v>
@@ -1856,13 +1855,13 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O12" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="P12" t="n">
-        <v>2.2875</v>
+        <v>2.4</v>
       </c>
       <c r="Q12" t="n">
         <v>2</v>
@@ -1879,7 +1878,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dungeons &amp; Dragons: Honor Among Thieves</t>
+          <t>Legend</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1889,7 +1888,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Jonathan Goldstein / John Francis Daley</t>
+          <t>Ridley Scott</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1909,29 +1908,30 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O13" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="P13" t="n">
-        <v>2.4</v>
+        <v>2.5125</v>
       </c>
       <c r="Q13" t="n">
         <v>2</v>
       </c>
+      <c r="R13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>The Nightmare Before Christmas</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ridley Scott</t>
+          <t>Tim Burton / Henry Selick</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1997,7 +1997,6 @@
       <c r="Q14" t="n">
         <v>2</v>
       </c>
-      <c r="R14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="n">

</xml_diff>

<commit_message>
Add Labyrinth (1986) to tier 2
Tier 2 (Bright Fantasy), score 2.2875, tied exactly with Castle in the
Sky. A contained, personal coming-of-age quest -- Sarah's defiance of
Jareth fully resolves the threat to Toby, and her own arc working
through real selfishness is the story's only real cost. Explicit
Darkness carries the film's real weight (the Bog of Eternal Stench,
Jareth's often-noted uncomfortable dynamic with a teenage Sarah), kept
at 2 rather than 3 since the register stays dreamlike/surreal rather
than genuinely graphic.

First queue addition scored directly under v2 methodology (no v1
predecessor). Updated xlsx, scoring record, and both language pages;
catalog now stands at 93 works.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -466,7 +466,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="40" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -474,7 +473,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -503,7 +501,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -511,7 +508,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -914,7 +910,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -1036,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R93"/>
+  <dimension ref="A1:R94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1818,7 +1813,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dungeons &amp; Dragons: Honor Among Thieves</t>
+          <t>Labyrinth</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1828,7 +1823,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Jonathan Goldstein / John Francis Daley</t>
+          <t>Jim Henson</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1848,25 +1843,25 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="P12" t="n">
-        <v>2.4</v>
+        <v>2.2875</v>
       </c>
       <c r="Q12" t="n">
         <v>2</v>
@@ -1883,7 +1878,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>Dungeons &amp; Dragons: Honor Among Thieves</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1893,7 +1888,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ridley Scott</t>
+          <t>Jonathan Goldstein / John Francis Daley</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1913,30 +1908,29 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O13" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="P13" t="n">
-        <v>2.5125</v>
+        <v>2.4</v>
       </c>
       <c r="Q13" t="n">
         <v>2</v>
       </c>
-      <c r="R13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1949,7 +1943,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The Nightmare Before Christmas</t>
+          <t>Legend</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1959,7 +1953,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Tim Burton / Henry Selick</t>
+          <t>Ridley Scott</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2002,6 +1996,7 @@
       <c r="Q14" t="n">
         <v>2</v>
       </c>
+      <c r="R14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2014,17 +2009,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Harry Potter and the Chamber of Secrets</t>
+          <t>The Nightmare Before Christmas</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Tim Burton / Henry Selick</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2047,27 +2042,26 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O15" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="P15" t="n">
-        <v>2.625</v>
+        <v>2.5125</v>
       </c>
       <c r="Q15" t="n">
         <v>2</v>
       </c>
-      <c r="R15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2080,17 +2074,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>The Little Prince</t>
+          <t>Harry Potter and the Chamber of Secrets</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Book</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Antoine de Saint-Exupéry</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2104,22 +2098,22 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N16" t="n">
         <v>2</v>
@@ -2133,6 +2127,7 @@
       <c r="Q16" t="n">
         <v>2</v>
       </c>
+      <c r="R16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2145,17 +2140,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A Conspiracy of Truths</t>
+          <t>The Little Prince</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Book</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Alexandra Rowland</t>
+          <t>Antoine de Saint-Exupéry</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2165,7 +2160,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -2178,7 +2173,7 @@
         <v>1</v>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -2187,18 +2182,17 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O17" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="P17" t="n">
-        <v>2.7375</v>
+        <v>2.625</v>
       </c>
       <c r="Q17" t="n">
         <v>2</v>
       </c>
-      <c r="R17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2211,17 +2205,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Willow</t>
+          <t>A Conspiracy of Truths</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ron Howard / George Lucas</t>
+          <t>Alexandra Rowland</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2231,39 +2225,40 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O18" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="P18" t="n">
-        <v>2.85</v>
+        <v>2.7375</v>
       </c>
       <c r="Q18" t="n">
         <v>2</v>
       </c>
+      <c r="R18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2276,17 +2271,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The Chronicles of Narnia</t>
+          <t>Willow</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Novels / Films</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>C. S. Lewis</t>
+          <t>Ron Howard / George Lucas</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2300,7 +2295,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -2318,13 +2313,13 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="P19" t="n">
-        <v>2.9625</v>
+        <v>2.85</v>
       </c>
       <c r="Q19" t="n">
         <v>2</v>
@@ -2341,17 +2336,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The Legend of Zelda</t>
+          <t>The Chronicles of Narnia</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels / Films</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Nintendo</t>
+          <t>C. S. Lewis</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2368,7 +2363,7 @@
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -2377,7 +2372,7 @@
         <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" t="n">
         <v>0</v>
@@ -2394,7 +2389,6 @@
       <c r="Q20" t="n">
         <v>2</v>
       </c>
-      <c r="R20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2407,17 +2401,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DanMachi</t>
+          <t>The Legend of Zelda</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Light Novels / Anime / Manga</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fujino Ōmori</t>
+          <t>Nintendo</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2431,19 +2425,19 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
@@ -2460,29 +2454,30 @@
       <c r="Q21" t="n">
         <v>2</v>
       </c>
+      <c r="R21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Moderately Bright Fantasy</t>
+          <t>Bright Fantasy</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mushishi</t>
+          <t>DanMachi</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Anime / Manga</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Yuki Urushibara</t>
+          <t>Fujino Ōmori</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2492,43 +2487,38 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O22" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="P22" t="n">
-        <v>3.075</v>
+        <v>2.9625</v>
       </c>
       <c r="Q22" t="n">
-        <v>3</v>
-      </c>
-      <c r="R22" s="5" t="inlineStr">
-        <is>
-          <t>Tier v1 era 2</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -2542,17 +2532,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>A Choir of Lies</t>
+          <t>Mushishi</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Alexandra Rowland</t>
+          <t>Yuki Urushibara</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2569,19 +2559,19 @@
         <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N23" t="n">
         <v>1</v>
@@ -2595,6 +2585,11 @@
       <c r="Q23" t="n">
         <v>3</v>
       </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Tier v1 era 2</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2607,17 +2602,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Neverwinter Nights</t>
+          <t>A Choir of Lies</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Alexandra Rowland</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2627,7 +2622,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -2660,11 +2655,6 @@
       <c r="Q24" t="n">
         <v>3</v>
       </c>
-      <c r="R24" s="5" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2677,17 +2667,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dungeon Meshi</t>
+          <t>Neverwinter Nights</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Ryoko Kui</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2704,10 +2694,10 @@
         <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
@@ -2719,18 +2709,22 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O25" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="P25" t="n">
-        <v>3.3</v>
+        <v>3.075</v>
       </c>
       <c r="Q25" t="n">
         <v>3</v>
       </c>
-      <c r="R25" s="5" t="n"/>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2743,17 +2737,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Cormyr</t>
+          <t>Dungeon Meshi</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Ed Greenwood / Jeff Grubb</t>
+          <t>Ryoko Kui</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2773,13 +2767,13 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
@@ -2796,6 +2790,7 @@
       <c r="Q26" t="n">
         <v>3</v>
       </c>
+      <c r="R26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2808,17 +2803,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Baldur's Gate I</t>
+          <t>Cormyr</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Ed Greenwood / Jeff Grubb</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2844,27 +2839,22 @@
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O27" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="P27" t="n">
-        <v>3.4125</v>
+        <v>3.3</v>
       </c>
       <c r="Q27" t="n">
         <v>3</v>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="28">
@@ -2878,17 +2868,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Final Fantasy IV</t>
+          <t>Baldur's Gate I</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2902,36 +2892,40 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
         <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O28" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="P28" t="n">
-        <v>3.525</v>
+        <v>3.4125</v>
       </c>
       <c r="Q28" t="n">
         <v>3</v>
       </c>
-      <c r="R28" s="5" t="n"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2944,17 +2938,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>The Hobbit</t>
+          <t>Final Fantasy IV</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2968,10 +2962,10 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -2983,20 +2977,21 @@
         <v>2</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O29" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="P29" t="n">
-        <v>3.6375</v>
+        <v>3.525</v>
       </c>
       <c r="Q29" t="n">
         <v>3</v>
       </c>
+      <c r="R29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3009,17 +3004,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Spirited Away</t>
+          <t>The Hobbit</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3033,7 +3028,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
         <v>1</v>
@@ -3042,13 +3037,13 @@
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>2</v>
@@ -3074,7 +3069,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Howl's Moving Castle</t>
+          <t>Spirited Away</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3098,7 +3093,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
         <v>1</v>
@@ -3107,13 +3102,13 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N31" t="n">
         <v>2</v>
@@ -3139,17 +3134,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Discworld</t>
+          <t>Howl's Moving Castle</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Novels / Games / Comics</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Terry Pratchett</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3159,7 +3154,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -3169,33 +3164,28 @@
         <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
         <v>1</v>
       </c>
       <c r="L32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O32" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="P32" t="n">
-        <v>3.75</v>
+        <v>3.6375</v>
       </c>
       <c r="Q32" t="n">
         <v>3</v>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>Tier v1 era 4</t>
-        </is>
       </c>
     </row>
     <row r="33">
@@ -3209,17 +3199,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>The Lord of the Rings</t>
+          <t>Discworld</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Novels / Films</t>
+          <t>Novels / Games / Comics</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Terry Pratchett</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3229,38 +3219,43 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I33" t="n">
         <v>1</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" t="n">
         <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O33" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="P33" t="n">
-        <v>3.975</v>
+        <v>3.75</v>
       </c>
       <c r="Q33" t="n">
         <v>3</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Tier v1 era 4</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -3274,17 +3269,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Frieren: Beyond Journey's End</t>
+          <t>The Lord of the Rings</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novels / Films</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Kanehito Yamada / Tsukasa Abe</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3294,7 +3289,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H34" t="n">
@@ -3307,13 +3302,13 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N34" t="n">
         <v>2</v>
@@ -3339,17 +3334,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Black Clover</t>
+          <t>Frieren: Beyond Journey's End</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Manga / Anime / Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Yūki Tabata</t>
+          <t>Kanehito Yamada / Tsukasa Abe</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3359,11 +3354,11 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I35" t="n">
         <v>1</v>
@@ -3372,13 +3367,13 @@
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N35" t="n">
         <v>2</v>
@@ -3404,17 +3399,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Record of Lodoss War</t>
+          <t>Black Clover</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Novels / Anime</t>
+          <t>Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Ryo Mizuno</t>
+          <t>Yūki Tabata</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3434,16 +3429,16 @@
         <v>1</v>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N36" t="n">
         <v>2</v>
@@ -3469,17 +3464,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Final Fantasy II</t>
+          <t>Record of Lodoss War</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels / Anime</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Ryo Mizuno</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3522,11 +3517,6 @@
       <c r="Q37" t="n">
         <v>3</v>
       </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3539,17 +3529,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Nausicaä of the Valley of the Wind</t>
+          <t>Final Fantasy II</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3563,7 +3553,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I38" t="n">
         <v>1</v>
@@ -3575,10 +3565,10 @@
         <v>1</v>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N38" t="n">
         <v>2</v>
@@ -3592,29 +3582,34 @@
       <c r="Q38" t="n">
         <v>3</v>
       </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Moderately Bright Fantasy</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>The NeverEnding Story</t>
+          <t>Nausicaä of the Valley of the Wind</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Michael Ende</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3637,25 +3632,25 @@
         <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O39" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="P39" t="n">
-        <v>4.2</v>
+        <v>3.975</v>
       </c>
       <c r="Q39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -3669,17 +3664,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Witch Hat Atelier</t>
+          <t>The NeverEnding Story</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Kamome Shirahama</t>
+          <t>Michael Ende</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3693,31 +3688,31 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I40" t="n">
         <v>1</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L40" t="n">
         <v>2</v>
       </c>
       <c r="M40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O40" t="n">
-        <v>1.25</v>
+        <v>1.2</v>
       </c>
       <c r="P40" t="n">
-        <v>4.3125</v>
+        <v>4.2</v>
       </c>
       <c r="Q40" t="n">
         <v>4</v>
@@ -3734,17 +3729,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Baldur's Gate II: Shadows of Amn</t>
+          <t>Witch Hat Atelier</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Kamome Shirahama</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3764,13 +3759,13 @@
         <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
         <v>2</v>
       </c>
       <c r="L41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M41" t="n">
         <v>1</v>
@@ -3786,11 +3781,6 @@
       </c>
       <c r="Q41" t="n">
         <v>4</v>
-      </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="42">
@@ -3804,17 +3794,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Harry Potter and the Prisoner of Azkaban</t>
+          <t>Baldur's Gate II: Shadows of Amn</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3840,22 +3830,27 @@
         <v>2</v>
       </c>
       <c r="L42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O42" t="n">
-        <v>1.35</v>
+        <v>1.25</v>
       </c>
       <c r="P42" t="n">
-        <v>4.5375</v>
+        <v>4.3125</v>
       </c>
       <c r="Q42" t="n">
         <v>4</v>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -3869,17 +3864,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Grimgar: Ashes and Illusions</t>
+          <t>Harry Potter and the Prisoner of Azkaban</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Light Novels / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Ao Jyumonji</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3893,7 +3888,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I43" t="n">
         <v>1</v>
@@ -3902,30 +3897,25 @@
         <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O43" t="n">
-        <v>1.4</v>
+        <v>1.35</v>
       </c>
       <c r="P43" t="n">
-        <v>4.65</v>
+        <v>4.5375</v>
       </c>
       <c r="Q43" t="n">
         <v>4</v>
-      </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="44">
@@ -3939,17 +3929,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Avatar: The Last Airbender</t>
+          <t>Grimgar: Ashes and Illusions</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Light Novels / Anime</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>Ao Jyumonji</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3959,7 +3949,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H44" t="n">
@@ -3994,7 +3984,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Tier v1 era 3</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -4009,17 +3999,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Earthsea</t>
+          <t>Avatar: The Last Airbender</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Ursula K. Le Guin</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4029,7 +4019,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -4039,10 +4029,10 @@
         <v>1</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L45" t="n">
         <v>2</v>
@@ -4061,6 +4051,11 @@
       </c>
       <c r="Q45" t="n">
         <v>4</v>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Tier v1 era 3</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -4074,17 +4069,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Final Fantasy XII</t>
+          <t>Earthsea</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Ursula K. Le Guin</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4098,22 +4093,22 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I46" t="n">
         <v>1</v>
       </c>
       <c r="J46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K46" t="n">
         <v>2</v>
       </c>
       <c r="L46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N46" t="n">
         <v>2</v>
@@ -4126,11 +4121,6 @@
       </c>
       <c r="Q46" t="n">
         <v>4</v>
-      </c>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
-        </is>
       </c>
     </row>
     <row r="47">
@@ -4144,17 +4134,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>The Legend of Vox Machina</t>
+          <t>Final Fantasy XII</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Critical Role</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -4177,25 +4167,30 @@
         <v>1</v>
       </c>
       <c r="K47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O47" t="n">
-        <v>1.35</v>
+        <v>1.4</v>
       </c>
       <c r="P47" t="n">
-        <v>4.8375</v>
+        <v>4.65</v>
       </c>
       <c r="Q47" t="n">
         <v>4</v>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -4209,17 +4204,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist: Brotherhood</t>
+          <t>The Legend of Vox Machina</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa</t>
+          <t>Critical Role</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4242,7 +4237,7 @@
         <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L48" t="n">
         <v>2</v>
@@ -4254,10 +4249,10 @@
         <v>3</v>
       </c>
       <c r="O48" t="n">
-        <v>1.5</v>
+        <v>1.35</v>
       </c>
       <c r="P48" t="n">
-        <v>4.875</v>
+        <v>4.8375</v>
       </c>
       <c r="Q48" t="n">
         <v>4</v>
@@ -4274,17 +4269,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>The Boy and the Heron</t>
+          <t>Fullmetal Alchemist: Brotherhood</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Hiromu Arakawa</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -4298,22 +4293,22 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N49" t="n">
         <v>3</v>
@@ -4339,17 +4334,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Final Fantasy IX</t>
+          <t>The Boy and the Heron</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4363,19 +4358,19 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
       </c>
       <c r="K50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M50" t="n">
         <v>2</v>
@@ -4404,17 +4399,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Ranking of Kings</t>
+          <t>Final Fantasy IX</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Sōsuke Tōka</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4428,19 +4423,19 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I51" t="n">
         <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K51" t="n">
         <v>2</v>
       </c>
       <c r="L51" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M51" t="n">
         <v>2</v>
@@ -4456,11 +4451,6 @@
       </c>
       <c r="Q51" t="n">
         <v>4</v>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="52">
@@ -4474,17 +4464,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Tales from Earthsea</t>
+          <t>Ranking of Kings</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Gorō Miyazaki</t>
+          <t>Sōsuke Tōka</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4507,29 +4497,29 @@
         <v>1</v>
       </c>
       <c r="K52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L52" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M52" t="n">
         <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O52" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="P52" t="n">
-        <v>4.9875</v>
+        <v>4.875</v>
       </c>
       <c r="Q52" t="n">
         <v>4</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Tier v1 era 5</t>
+          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
         </is>
       </c>
     </row>
@@ -4544,17 +4534,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Adventure Time</t>
+          <t>Tales from Earthsea</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>TV / Comics</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Pendleton Ward</t>
+          <t>Studio Ghibli / Gorō Miyazaki</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4596,6 +4586,11 @@
       </c>
       <c r="Q53" t="n">
         <v>4</v>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Tier v1 era 5</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -4609,17 +4604,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Star vs. the Forces of Evil</t>
+          <t>Adventure Time</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>TV, Comics</t>
+          <t>TV / Comics</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Daron Nefcy</t>
+          <t>Pendleton Ward</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4633,7 +4628,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I54" t="n">
         <v>1</v>
@@ -4642,7 +4637,7 @@
         <v>1</v>
       </c>
       <c r="K54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L54" t="n">
         <v>2</v>
@@ -4662,34 +4657,29 @@
       <c r="Q54" t="n">
         <v>4</v>
       </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Dragonlance</t>
+          <t>Star vs. the Forces of Evil</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Novels / Games</t>
+          <t>TV, Comics</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Margaret Weis / Tracy Hickman</t>
+          <t>Daron Nefcy</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4703,7 +4693,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I55" t="n">
         <v>1</v>
@@ -4718,19 +4708,24 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O55" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="P55" t="n">
-        <v>5.2125</v>
+        <v>4.9875</v>
       </c>
       <c r="Q55" t="n">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -4744,17 +4739,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Harry Potter and the Goblet of Fire</t>
+          <t>Dragonlance</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Novels / Games</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Margaret Weis / Tracy Hickman</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4768,22 +4763,22 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I56" t="n">
         <v>1</v>
       </c>
       <c r="J56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K56" t="n">
         <v>2</v>
       </c>
       <c r="L56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N56" t="n">
         <v>3</v>
@@ -4809,17 +4804,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Elantris</t>
+          <t>Harry Potter and the Goblet of Fire</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4833,22 +4828,22 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I57" t="n">
         <v>1</v>
       </c>
       <c r="J57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K57" t="n">
         <v>2</v>
       </c>
       <c r="L57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N57" t="n">
         <v>3</v>
@@ -4874,17 +4869,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Baldur's Gate III</t>
+          <t>Elantris</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4898,13 +4893,13 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I58" t="n">
         <v>1</v>
       </c>
       <c r="J58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K58" t="n">
         <v>2</v>
@@ -4926,11 +4921,6 @@
       </c>
       <c r="Q58" t="n">
         <v>5</v>
-      </c>
-      <c r="R58" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="59">
@@ -4944,17 +4934,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V: Skyrim</t>
+          <t>Baldur's Gate III</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Bethesda Game Studios</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4968,7 +4958,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
@@ -4980,22 +4970,27 @@
         <v>2</v>
       </c>
       <c r="L59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O59" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="P59" t="n">
-        <v>5.325</v>
+        <v>5.2125</v>
       </c>
       <c r="Q59" t="n">
         <v>5</v>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -5009,17 +5004,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>The Silmarillion &amp; Great Tales</t>
+          <t>The Elder Scrolls V: Skyrim</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Books</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Bethesda Game Studios</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5045,10 +5040,10 @@
         <v>2</v>
       </c>
       <c r="L60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N60" t="n">
         <v>2</v>
@@ -5074,17 +5069,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The Legend of Korra</t>
+          <t>The Silmarillion &amp; Great Tales</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Books</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5094,17 +5089,17 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H61" t="n">
         <v>2</v>
       </c>
       <c r="I61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K61" t="n">
         <v>2</v>
@@ -5126,11 +5121,6 @@
       </c>
       <c r="Q61" t="n">
         <v>5</v>
-      </c>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
-        </is>
       </c>
     </row>
     <row r="62">
@@ -5144,17 +5134,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Princess Mononoke</t>
+          <t>The Legend of Korra</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5164,7 +5154,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H62" t="n">
@@ -5174,28 +5164,33 @@
         <v>2</v>
       </c>
       <c r="J62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O62" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="P62" t="n">
-        <v>5.55</v>
+        <v>5.325</v>
       </c>
       <c r="Q62" t="n">
         <v>5</v>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -5209,17 +5204,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The Dark Elf / Drizzt</t>
+          <t>Princess Mononoke</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>R. A. Salvatore</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5236,16 +5231,16 @@
         <v>2</v>
       </c>
       <c r="I63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M63" t="n">
         <v>2</v>
@@ -5261,11 +5256,6 @@
       </c>
       <c r="Q63" t="n">
         <v>5</v>
-      </c>
-      <c r="R63" t="inlineStr">
-        <is>
-          <t>re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="64">
@@ -5279,17 +5269,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The Wheel of Time</t>
+          <t>The Dark Elf / Drizzt</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Robert Jordan / Brandon Sanderson</t>
+          <t>R. A. Salvatore</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5349,17 +5339,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Final Fantasy VI</t>
+          <t>The Wheel of Time</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Robert Jordan / Brandon Sanderson</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5373,13 +5363,13 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I65" t="n">
         <v>1</v>
       </c>
       <c r="J65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K65" t="n">
         <v>2</v>
@@ -5388,19 +5378,24 @@
         <v>2</v>
       </c>
       <c r="M65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O65" t="n">
-        <v>1.85</v>
+        <v>1.8</v>
       </c>
       <c r="P65" t="n">
-        <v>5.6625</v>
+        <v>5.55</v>
       </c>
       <c r="Q65" t="n">
         <v>5</v>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -5414,17 +5409,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>Final Fantasy VI</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5438,13 +5433,13 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K66" t="n">
         <v>2</v>
@@ -5453,7 +5448,7 @@
         <v>2</v>
       </c>
       <c r="M66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N66" t="n">
         <v>2</v>
@@ -5479,17 +5474,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5509,33 +5504,28 @@
         <v>2</v>
       </c>
       <c r="J67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M67" t="n">
         <v>2</v>
       </c>
       <c r="N67" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O67" t="n">
-        <v>1.9</v>
+        <v>1.85</v>
       </c>
       <c r="P67" t="n">
-        <v>5.775</v>
+        <v>5.6625</v>
       </c>
       <c r="Q67" t="n">
         <v>5</v>
-      </c>
-      <c r="R67" t="inlineStr">
-        <is>
-          <t>Tier v1 era 6</t>
-        </is>
       </c>
     </row>
     <row r="68">
@@ -5549,17 +5539,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Final Fantasy X</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5573,34 +5563,39 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J68" t="n">
         <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L68" t="n">
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O68" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="P68" t="n">
-        <v>5.8875</v>
+        <v>5.775</v>
       </c>
       <c r="Q68" t="n">
         <v>5</v>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -5614,17 +5609,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Final Fantasy VII</t>
+          <t>Final Fantasy X</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Video Games / Remake Project</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5638,7 +5633,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I69" t="n">
         <v>1</v>
@@ -5653,7 +5648,7 @@
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N69" t="n">
         <v>3</v>
@@ -5679,17 +5674,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Final Fantasy VII</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Games / Remake Project</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5706,13 +5701,13 @@
         <v>2</v>
       </c>
       <c r="I70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J70" t="n">
         <v>2</v>
       </c>
       <c r="K70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L70" t="n">
         <v>1</v>
@@ -5744,7 +5739,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -5777,10 +5772,10 @@
         <v>2</v>
       </c>
       <c r="K71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M71" t="n">
         <v>2</v>
@@ -5809,17 +5804,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Final Fantasy XV</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5833,22 +5828,22 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J72" t="n">
         <v>2</v>
       </c>
       <c r="K72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L72" t="n">
         <v>2</v>
       </c>
       <c r="M72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N72" t="n">
         <v>3</v>
@@ -5865,26 +5860,26 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Clevatess</t>
+          <t>Final Fantasy XV</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Yūji Iwahara</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5898,10 +5893,10 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J73" t="n">
         <v>2</v>
@@ -5910,27 +5905,22 @@
         <v>2</v>
       </c>
       <c r="L73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N73" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O73" t="n">
-        <v>2.05</v>
+        <v>1.95</v>
       </c>
       <c r="P73" t="n">
-        <v>6.1125</v>
+        <v>5.8875</v>
       </c>
       <c r="Q73" t="n">
-        <v>6</v>
-      </c>
-      <c r="R73" t="inlineStr">
-        <is>
-          <t>scored against the story as currently published/aired; ongoing/unresolved, later arcs may shift this</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="74">
@@ -5944,17 +5934,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Re:Zero − Starting Life in Another World</t>
+          <t>Clevatess</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Light Novels, Manga, Anime</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Tappei Nagatsuki</t>
+          <t>Yūji Iwahara</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5971,7 +5961,7 @@
         <v>2</v>
       </c>
       <c r="I74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J74" t="n">
         <v>2</v>
@@ -5980,7 +5970,7 @@
         <v>2</v>
       </c>
       <c r="L74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M74" t="n">
         <v>2</v>
@@ -5999,7 +5989,7 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>scored against the arcs most widely adapted/translated (roughly Arcs 1-6); later arcs may shift this</t>
+          <t>scored against the story as currently published/aired; ongoing/unresolved, later arcs may shift this</t>
         </is>
       </c>
     </row>
@@ -6014,17 +6004,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Re:Zero − Starting Life in Another World</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Light Novels, Manga, Anime</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>Tappei Nagatsuki</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6041,7 +6031,7 @@
         <v>2</v>
       </c>
       <c r="I75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J75" t="n">
         <v>2</v>
@@ -6056,16 +6046,21 @@
         <v>2</v>
       </c>
       <c r="N75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O75" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="P75" t="n">
-        <v>6.225</v>
+        <v>6.1125</v>
       </c>
       <c r="Q75" t="n">
         <v>6</v>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>scored against the arcs most widely adapted/translated (roughly Arcs 1-6); later arcs may shift this</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -6079,17 +6074,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6103,16 +6098,16 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L76" t="n">
         <v>2</v>
@@ -6144,17 +6139,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6168,13 +6163,13 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K77" t="n">
         <v>3</v>
@@ -6186,21 +6181,16 @@
         <v>2</v>
       </c>
       <c r="N77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O77" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P77" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q77" t="n">
         <v>6</v>
-      </c>
-      <c r="R77" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="78">
@@ -6214,17 +6204,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6247,7 +6237,7 @@
         <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L78" t="n">
         <v>2</v>
@@ -6256,16 +6246,21 @@
         <v>2</v>
       </c>
       <c r="N78" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O78" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P78" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q78" t="n">
         <v>6</v>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -6279,17 +6274,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6303,7 +6298,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I79" t="n">
         <v>2</v>
@@ -6321,21 +6316,16 @@
         <v>2</v>
       </c>
       <c r="N79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O79" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P79" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q79" t="n">
         <v>6</v>
-      </c>
-      <c r="R79" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="80">
@@ -6349,17 +6339,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6373,13 +6363,13 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I80" t="n">
         <v>2</v>
       </c>
       <c r="J80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K80" t="n">
         <v>2</v>
@@ -6404,7 +6394,7 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6419,17 +6409,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6449,10 +6439,10 @@
         <v>2</v>
       </c>
       <c r="J81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L81" t="n">
         <v>2</v>
@@ -6471,6 +6461,11 @@
       </c>
       <c r="Q81" t="n">
         <v>6</v>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -6484,17 +6479,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6549,17 +6544,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6576,7 +6571,7 @@
         <v>2</v>
       </c>
       <c r="I83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J83" t="n">
         <v>2</v>
@@ -6585,7 +6580,7 @@
         <v>3</v>
       </c>
       <c r="L83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M83" t="n">
         <v>2</v>
@@ -6614,17 +6609,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6638,7 +6633,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I84" t="n">
         <v>1</v>
@@ -6650,7 +6645,7 @@
         <v>3</v>
       </c>
       <c r="L84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M84" t="n">
         <v>2</v>
@@ -6679,17 +6674,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Märchen Crown</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Aka Akasaka / Aoi Kujira / Azychika</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6703,10 +6698,10 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J85" t="n">
         <v>2</v>
@@ -6721,21 +6716,16 @@
         <v>2</v>
       </c>
       <c r="N85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O85" t="n">
-        <v>2.35</v>
+        <v>2.25</v>
       </c>
       <c r="P85" t="n">
-        <v>6.7875</v>
+        <v>6.5625</v>
       </c>
       <c r="Q85" t="n">
         <v>6</v>
-      </c>
-      <c r="R85" t="inlineStr">
-        <is>
-          <t>ongoing/unresolved as of ch. 47 (Jul 2026); low-mid confidence given thin reception in most languages researched</t>
-        </is>
       </c>
     </row>
     <row r="86">
@@ -6749,17 +6739,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Märchen Crown</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Aka Akasaka / Aoi Kujira / Azychika</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6773,7 +6763,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I86" t="n">
         <v>2</v>
@@ -6782,29 +6772,29 @@
         <v>2</v>
       </c>
       <c r="K86" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M86" t="n">
         <v>2</v>
       </c>
       <c r="N86" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O86" t="n">
-        <v>2.4</v>
+        <v>2.35</v>
       </c>
       <c r="P86" t="n">
-        <v>6.9</v>
+        <v>6.7875</v>
       </c>
       <c r="Q86" t="n">
         <v>6</v>
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>Tier v1 era 8</t>
+          <t>ongoing/unresolved as of ch. 47 (Jul 2026); low-mid confidence given thin reception in most languages researched</t>
         </is>
       </c>
     </row>
@@ -6819,17 +6809,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6843,7 +6833,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I87" t="n">
         <v>2</v>
@@ -6852,7 +6842,7 @@
         <v>2</v>
       </c>
       <c r="K87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L87" t="n">
         <v>3</v>
@@ -6872,29 +6862,34 @@
       <c r="Q87" t="n">
         <v>6</v>
       </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6908,16 +6903,16 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I88" t="n">
         <v>2</v>
       </c>
       <c r="J88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K88" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L88" t="n">
         <v>3</v>
@@ -6926,40 +6921,40 @@
         <v>2</v>
       </c>
       <c r="N88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O88" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P88" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q88" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6976,31 +6971,31 @@
         <v>3</v>
       </c>
       <c r="I89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J89" t="n">
         <v>3</v>
       </c>
       <c r="K89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L89" t="n">
         <v>3</v>
       </c>
       <c r="M89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N89" t="n">
         <v>4</v>
       </c>
       <c r="O89" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P89" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q89" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="90">
@@ -7014,17 +7009,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -7038,31 +7033,31 @@
         </is>
       </c>
       <c r="H90" t="n">
+        <v>3</v>
+      </c>
+      <c r="I90" t="n">
+        <v>3</v>
+      </c>
+      <c r="J90" t="n">
+        <v>3</v>
+      </c>
+      <c r="K90" t="n">
+        <v>3</v>
+      </c>
+      <c r="L90" t="n">
+        <v>3</v>
+      </c>
+      <c r="M90" t="n">
+        <v>3</v>
+      </c>
+      <c r="N90" t="n">
         <v>4</v>
       </c>
-      <c r="I90" t="n">
-        <v>3</v>
-      </c>
-      <c r="J90" t="n">
-        <v>3</v>
-      </c>
-      <c r="K90" t="n">
-        <v>3</v>
-      </c>
-      <c r="L90" t="n">
-        <v>3</v>
-      </c>
-      <c r="M90" t="n">
-        <v>3</v>
-      </c>
-      <c r="N90" t="n">
-        <v>3</v>
-      </c>
       <c r="O90" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P90" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q90" t="n">
         <v>8</v>
@@ -7079,17 +7074,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -7103,13 +7098,13 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I91" t="n">
         <v>3</v>
       </c>
       <c r="J91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K91" t="n">
         <v>3</v>
@@ -7121,13 +7116,13 @@
         <v>3</v>
       </c>
       <c r="N91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O91" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P91" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q91" t="n">
         <v>8</v>
@@ -7135,26 +7130,26 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -7168,16 +7163,16 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J92" t="n">
         <v>4</v>
       </c>
       <c r="K92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L92" t="n">
         <v>3</v>
@@ -7189,37 +7184,37 @@
         <v>4</v>
       </c>
       <c r="O92" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P92" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q92" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -7245,21 +7240,86 @@
         <v>4</v>
       </c>
       <c r="L93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N93" t="n">
         <v>4</v>
       </c>
       <c r="O93" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P93" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>10</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H94" t="n">
         <v>4</v>
       </c>
-      <c r="P93" t="n">
+      <c r="I94" t="n">
+        <v>4</v>
+      </c>
+      <c r="J94" t="n">
+        <v>4</v>
+      </c>
+      <c r="K94" t="n">
+        <v>4</v>
+      </c>
+      <c r="L94" t="n">
+        <v>4</v>
+      </c>
+      <c r="M94" t="n">
+        <v>4</v>
+      </c>
+      <c r="N94" t="n">
+        <v>4</v>
+      </c>
+      <c r="O94" t="n">
+        <v>4</v>
+      </c>
+      <c r="P94" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q93" t="n">
+      <c r="Q94" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7322,7 +7382,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -7429,11 +7489,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 92 of 92 works in the full catalog.</t>
+          <t>Total scored: 93 of 93 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Pan's Labyrinth (2006) to tier 6
Tier 6 (Dark Fantasy), score 6.45, tied exactly with Made in Abyss.
Captain Vidal's Francoist military apparatus is thoroughly corrupt
(torture, extrajudicial killing of innocents), and the film is among the
most graphically intense in the catalog (Explicit Darkness 4). Against
that, Ofelia's moral integrity -- refusing to harm her infant brother
even under lethal threat -- is the film's real thematic center, and the
story deliberately keeps Moral Cynicism ambiguous rather than fully
cynical. Checked against Berserk (Tier 7): lower Moral Cynicism and
Redemption Difficulty keep this a full tier below, appropriately, for a
tightly-constructed single film rather than an open-ended chronicle of
escalating despair.

Catalog now stands at 94 works.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R94"/>
+  <dimension ref="A1:R95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6339,17 +6339,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Pan's Labyrinth</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Guillermo del Toro</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6363,7 +6363,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I80" t="n">
         <v>2</v>
@@ -6372,30 +6372,25 @@
         <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L80" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O80" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P80" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q80" t="n">
         <v>6</v>
-      </c>
-      <c r="R80" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="81">
@@ -6409,17 +6404,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6433,13 +6428,13 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I81" t="n">
         <v>2</v>
       </c>
       <c r="J81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K81" t="n">
         <v>2</v>
@@ -6464,7 +6459,7 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6479,17 +6474,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6509,10 +6504,10 @@
         <v>2</v>
       </c>
       <c r="J82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L82" t="n">
         <v>2</v>
@@ -6531,6 +6526,11 @@
       </c>
       <c r="Q82" t="n">
         <v>6</v>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -6544,17 +6544,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6609,17 +6609,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6636,7 +6636,7 @@
         <v>2</v>
       </c>
       <c r="I84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J84" t="n">
         <v>2</v>
@@ -6645,7 +6645,7 @@
         <v>3</v>
       </c>
       <c r="L84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M84" t="n">
         <v>2</v>
@@ -6674,17 +6674,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6698,7 +6698,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I85" t="n">
         <v>1</v>
@@ -6710,7 +6710,7 @@
         <v>3</v>
       </c>
       <c r="L85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M85" t="n">
         <v>2</v>
@@ -6739,17 +6739,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Märchen Crown</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Aka Akasaka / Aoi Kujira / Azychika</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6763,10 +6763,10 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J86" t="n">
         <v>2</v>
@@ -6781,21 +6781,16 @@
         <v>2</v>
       </c>
       <c r="N86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O86" t="n">
-        <v>2.35</v>
+        <v>2.25</v>
       </c>
       <c r="P86" t="n">
-        <v>6.7875</v>
+        <v>6.5625</v>
       </c>
       <c r="Q86" t="n">
         <v>6</v>
-      </c>
-      <c r="R86" t="inlineStr">
-        <is>
-          <t>ongoing/unresolved as of ch. 47 (Jul 2026); low-mid confidence given thin reception in most languages researched</t>
-        </is>
       </c>
     </row>
     <row r="87">
@@ -6809,17 +6804,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Märchen Crown</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Aka Akasaka / Aoi Kujira / Azychika</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6833,7 +6828,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I87" t="n">
         <v>2</v>
@@ -6842,29 +6837,29 @@
         <v>2</v>
       </c>
       <c r="K87" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M87" t="n">
         <v>2</v>
       </c>
       <c r="N87" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O87" t="n">
-        <v>2.4</v>
+        <v>2.35</v>
       </c>
       <c r="P87" t="n">
-        <v>6.9</v>
+        <v>6.7875</v>
       </c>
       <c r="Q87" t="n">
         <v>6</v>
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>Tier v1 era 8</t>
+          <t>ongoing/unresolved as of ch. 47 (Jul 2026); low-mid confidence given thin reception in most languages researched</t>
         </is>
       </c>
     </row>
@@ -6879,17 +6874,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6903,7 +6898,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I88" t="n">
         <v>2</v>
@@ -6912,7 +6907,7 @@
         <v>2</v>
       </c>
       <c r="K88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L88" t="n">
         <v>3</v>
@@ -6932,29 +6927,34 @@
       <c r="Q88" t="n">
         <v>6</v>
       </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Manga / Anime / Films</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6968,16 +6968,16 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I89" t="n">
         <v>2</v>
       </c>
       <c r="J89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K89" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L89" t="n">
         <v>3</v>
@@ -6986,40 +6986,40 @@
         <v>2</v>
       </c>
       <c r="N89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O89" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
       <c r="P89" t="n">
-        <v>7.4625</v>
+        <v>6.9</v>
       </c>
       <c r="Q89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga / Anime / Films</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -7036,31 +7036,31 @@
         <v>3</v>
       </c>
       <c r="I90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J90" t="n">
         <v>3</v>
       </c>
       <c r="K90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L90" t="n">
         <v>3</v>
       </c>
       <c r="M90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N90" t="n">
         <v>4</v>
       </c>
       <c r="O90" t="n">
-        <v>3.1</v>
+        <v>2.65</v>
       </c>
       <c r="P90" t="n">
-        <v>8.475</v>
+        <v>7.4625</v>
       </c>
       <c r="Q90" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="91">
@@ -7074,17 +7074,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -7098,31 +7098,31 @@
         </is>
       </c>
       <c r="H91" t="n">
+        <v>3</v>
+      </c>
+      <c r="I91" t="n">
+        <v>3</v>
+      </c>
+      <c r="J91" t="n">
+        <v>3</v>
+      </c>
+      <c r="K91" t="n">
+        <v>3</v>
+      </c>
+      <c r="L91" t="n">
+        <v>3</v>
+      </c>
+      <c r="M91" t="n">
+        <v>3</v>
+      </c>
+      <c r="N91" t="n">
         <v>4</v>
       </c>
-      <c r="I91" t="n">
-        <v>3</v>
-      </c>
-      <c r="J91" t="n">
-        <v>3</v>
-      </c>
-      <c r="K91" t="n">
-        <v>3</v>
-      </c>
-      <c r="L91" t="n">
-        <v>3</v>
-      </c>
-      <c r="M91" t="n">
-        <v>3</v>
-      </c>
-      <c r="N91" t="n">
-        <v>3</v>
-      </c>
       <c r="O91" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P91" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q91" t="n">
         <v>8</v>
@@ -7139,17 +7139,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -7163,13 +7163,13 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I92" t="n">
         <v>3</v>
       </c>
       <c r="J92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K92" t="n">
         <v>3</v>
@@ -7181,13 +7181,13 @@
         <v>3</v>
       </c>
       <c r="N92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O92" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P92" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q92" t="n">
         <v>8</v>
@@ -7195,26 +7195,26 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -7228,16 +7228,16 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J93" t="n">
         <v>4</v>
       </c>
       <c r="K93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L93" t="n">
         <v>3</v>
@@ -7249,37 +7249,37 @@
         <v>4</v>
       </c>
       <c r="O93" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P93" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q93" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -7305,21 +7305,86 @@
         <v>4</v>
       </c>
       <c r="L94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N94" t="n">
         <v>4</v>
       </c>
       <c r="O94" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P94" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>10</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H95" t="n">
         <v>4</v>
       </c>
-      <c r="P94" t="n">
+      <c r="I95" t="n">
+        <v>4</v>
+      </c>
+      <c r="J95" t="n">
+        <v>4</v>
+      </c>
+      <c r="K95" t="n">
+        <v>4</v>
+      </c>
+      <c r="L95" t="n">
+        <v>4</v>
+      </c>
+      <c r="M95" t="n">
+        <v>4</v>
+      </c>
+      <c r="N95" t="n">
+        <v>4</v>
+      </c>
+      <c r="O95" t="n">
+        <v>4</v>
+      </c>
+      <c r="P95" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q94" t="n">
+      <c r="Q95" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7434,7 +7499,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -7492,7 +7557,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 93 of 93 works in the full catalog.</t>
+          <t>Total scored: 94 of 94 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Attack on Titan to tier 7
Tier 7 (Extreme Dark Fantasy), score 7.8, joining Berserk (which returns
tier 7 to the standard grid layout). First pass landed tier 8 -- an exact
profile match for A Song of Ice and Fire -- by defaulting to maximum
severity across every axis, the same trap caught before in Marchen
Crown. Corrected by checking each axis against real tier 6-8 precedent:
Limited Heroism and Narrative Acceptance of Injustice both pulled back
from 3 to 2, since the ending achieves a genuine, hard-won structural
peace rather than "even the biggest wins are insufficient." Structural
Corruption 3 (two distinct, thoroughly corrupt institutions) is
specifically what pushes this above Berserk, whose evil is more
cosmic/personal than institutional -- the two profiles are otherwise
identical.

Catalog now stands at 95 works.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R95"/>
+  <dimension ref="A1:R96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7065,26 +7065,26 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Attack on Titan</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>Hajime Isayama</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -7101,7 +7101,7 @@
         <v>3</v>
       </c>
       <c r="I91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J91" t="n">
         <v>3</v>
@@ -7113,19 +7113,19 @@
         <v>3</v>
       </c>
       <c r="M91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N91" t="n">
         <v>4</v>
       </c>
       <c r="O91" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
       <c r="P91" t="n">
-        <v>8.475</v>
+        <v>7.8</v>
       </c>
       <c r="Q91" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="92">
@@ -7139,17 +7139,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -7163,31 +7163,31 @@
         </is>
       </c>
       <c r="H92" t="n">
+        <v>3</v>
+      </c>
+      <c r="I92" t="n">
+        <v>3</v>
+      </c>
+      <c r="J92" t="n">
+        <v>3</v>
+      </c>
+      <c r="K92" t="n">
+        <v>3</v>
+      </c>
+      <c r="L92" t="n">
+        <v>3</v>
+      </c>
+      <c r="M92" t="n">
+        <v>3</v>
+      </c>
+      <c r="N92" t="n">
         <v>4</v>
       </c>
-      <c r="I92" t="n">
-        <v>3</v>
-      </c>
-      <c r="J92" t="n">
-        <v>3</v>
-      </c>
-      <c r="K92" t="n">
-        <v>3</v>
-      </c>
-      <c r="L92" t="n">
-        <v>3</v>
-      </c>
-      <c r="M92" t="n">
-        <v>3</v>
-      </c>
-      <c r="N92" t="n">
-        <v>3</v>
-      </c>
       <c r="O92" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P92" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q92" t="n">
         <v>8</v>
@@ -7204,17 +7204,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -7228,13 +7228,13 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I93" t="n">
         <v>3</v>
       </c>
       <c r="J93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K93" t="n">
         <v>3</v>
@@ -7246,13 +7246,13 @@
         <v>3</v>
       </c>
       <c r="N93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O93" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P93" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q93" t="n">
         <v>8</v>
@@ -7260,26 +7260,26 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -7293,16 +7293,16 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J94" t="n">
         <v>4</v>
       </c>
       <c r="K94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L94" t="n">
         <v>3</v>
@@ -7314,37 +7314,37 @@
         <v>4</v>
       </c>
       <c r="O94" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P94" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q94" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -7370,21 +7370,86 @@
         <v>4</v>
       </c>
       <c r="L95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N95" t="n">
         <v>4</v>
       </c>
       <c r="O95" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P95" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>10</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H96" t="n">
         <v>4</v>
       </c>
-      <c r="P95" t="n">
+      <c r="I96" t="n">
+        <v>4</v>
+      </c>
+      <c r="J96" t="n">
+        <v>4</v>
+      </c>
+      <c r="K96" t="n">
+        <v>4</v>
+      </c>
+      <c r="L96" t="n">
+        <v>4</v>
+      </c>
+      <c r="M96" t="n">
+        <v>4</v>
+      </c>
+      <c r="N96" t="n">
+        <v>4</v>
+      </c>
+      <c r="O96" t="n">
+        <v>4</v>
+      </c>
+      <c r="P96" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q95" t="n">
+      <c r="Q96" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7512,7 +7577,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -7557,7 +7622,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 94 of 94 works in the full catalog.</t>
+          <t>Total scored: 95 of 95 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Maleficent (2014) to tier 3; document remaining bare entries
Maleficent: Tier 3 (Moderately Bright Fantasy), score 3.3, matching
Cormyr/Dungeon Meshi. A contained personal betrayal/revenge/redemption
story -- the resolution is genuinely complete (the two kingdoms unite
under Aurora's rule). The wing-mutilation scene carries real thematic
weight but stays within Disney/PG depiction restraint.

Also added full documented reasoning to Kiki's Delivery Service, Ponyo,
and Warhammer 40,000 -- the three bare-number entries from the earlier
sweep that were confirmed not miscalibrated, but still deserved proper
reasoning instead of an unexplained score. No SCORING_RECORD.md entry is
now undocumented.

Catalog now stands at 96 works.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R96"/>
+  <dimension ref="A1:R97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2868,17 +2868,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Baldur's Gate I</t>
+          <t>Maleficent</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Robert Stromberg</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2892,10 +2892,10 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
         <v>1</v>
@@ -2907,24 +2907,19 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O28" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="P28" t="n">
-        <v>3.4125</v>
+        <v>3.3</v>
       </c>
       <c r="Q28" t="n">
         <v>3</v>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="29">
@@ -2938,17 +2933,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Final Fantasy IV</t>
+          <t>Baldur's Gate I</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2962,36 +2957,40 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" t="n">
         <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O29" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="P29" t="n">
-        <v>3.525</v>
+        <v>3.4125</v>
       </c>
       <c r="Q29" t="n">
         <v>3</v>
       </c>
-      <c r="R29" s="5" t="n"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3004,17 +3003,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>The Hobbit</t>
+          <t>Final Fantasy IV</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3028,10 +3027,10 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -3043,20 +3042,21 @@
         <v>2</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O30" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="P30" t="n">
-        <v>3.6375</v>
+        <v>3.525</v>
       </c>
       <c r="Q30" t="n">
         <v>3</v>
       </c>
+      <c r="R30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3069,17 +3069,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Spirited Away</t>
+          <t>The Hobbit</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3093,7 +3093,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
         <v>1</v>
@@ -3102,13 +3102,13 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>2</v>
@@ -3134,7 +3134,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Howl's Moving Castle</t>
+          <t>Spirited Away</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
         <v>1</v>
@@ -3167,13 +3167,13 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N32" t="n">
         <v>2</v>
@@ -3199,17 +3199,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Discworld</t>
+          <t>Howl's Moving Castle</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Novels / Games / Comics</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Terry Pratchett</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -3229,33 +3229,28 @@
         <v>1</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
         <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O33" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="P33" t="n">
-        <v>3.75</v>
+        <v>3.6375</v>
       </c>
       <c r="Q33" t="n">
         <v>3</v>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Tier v1 era 4</t>
-        </is>
       </c>
     </row>
     <row r="34">
@@ -3269,17 +3264,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>The Lord of the Rings</t>
+          <t>Discworld</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Novels / Films</t>
+          <t>Novels / Games / Comics</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Terry Pratchett</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3289,38 +3284,43 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I34" t="n">
         <v>1</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K34" t="n">
         <v>1</v>
       </c>
       <c r="L34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O34" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="P34" t="n">
-        <v>3.975</v>
+        <v>3.75</v>
       </c>
       <c r="Q34" t="n">
         <v>3</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Tier v1 era 4</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -3334,17 +3334,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Frieren: Beyond Journey's End</t>
+          <t>The Lord of the Rings</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novels / Films</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Kanehito Yamada / Tsukasa Abe</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H35" t="n">
@@ -3367,13 +3367,13 @@
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N35" t="n">
         <v>2</v>
@@ -3399,17 +3399,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Black Clover</t>
+          <t>Frieren: Beyond Journey's End</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Manga / Anime / Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Yūki Tabata</t>
+          <t>Kanehito Yamada / Tsukasa Abe</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3419,11 +3419,11 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I36" t="n">
         <v>1</v>
@@ -3432,13 +3432,13 @@
         <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N36" t="n">
         <v>2</v>
@@ -3464,17 +3464,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Record of Lodoss War</t>
+          <t>Black Clover</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Novels / Anime</t>
+          <t>Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Ryo Mizuno</t>
+          <t>Yūki Tabata</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3494,16 +3494,16 @@
         <v>1</v>
       </c>
       <c r="J37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N37" t="n">
         <v>2</v>
@@ -3529,17 +3529,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Final Fantasy II</t>
+          <t>Record of Lodoss War</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels / Anime</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Ryo Mizuno</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3582,11 +3582,6 @@
       <c r="Q38" t="n">
         <v>3</v>
       </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3599,17 +3594,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Nausicaä of the Valley of the Wind</t>
+          <t>Final Fantasy II</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3623,7 +3618,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I39" t="n">
         <v>1</v>
@@ -3635,10 +3630,10 @@
         <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
         <v>2</v>
@@ -3652,29 +3647,34 @@
       <c r="Q39" t="n">
         <v>3</v>
       </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Moderately Bright Fantasy</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>The NeverEnding Story</t>
+          <t>Nausicaä of the Valley of the Wind</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Michael Ende</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3697,25 +3697,25 @@
         <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L40" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O40" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="P40" t="n">
-        <v>4.2</v>
+        <v>3.975</v>
       </c>
       <c r="Q40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
@@ -3729,17 +3729,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Witch Hat Atelier</t>
+          <t>The NeverEnding Story</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Kamome Shirahama</t>
+          <t>Michael Ende</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3753,31 +3753,31 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I41" t="n">
         <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L41" t="n">
         <v>2</v>
       </c>
       <c r="M41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O41" t="n">
-        <v>1.25</v>
+        <v>1.2</v>
       </c>
       <c r="P41" t="n">
-        <v>4.3125</v>
+        <v>4.2</v>
       </c>
       <c r="Q41" t="n">
         <v>4</v>
@@ -3794,17 +3794,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Baldur's Gate II: Shadows of Amn</t>
+          <t>Witch Hat Atelier</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Kamome Shirahama</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3824,13 +3824,13 @@
         <v>1</v>
       </c>
       <c r="J42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K42" t="n">
         <v>2</v>
       </c>
       <c r="L42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M42" t="n">
         <v>1</v>
@@ -3846,11 +3846,6 @@
       </c>
       <c r="Q42" t="n">
         <v>4</v>
-      </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="43">
@@ -3864,17 +3859,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Harry Potter and the Prisoner of Azkaban</t>
+          <t>Baldur's Gate II: Shadows of Amn</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3900,22 +3895,27 @@
         <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O43" t="n">
-        <v>1.35</v>
+        <v>1.25</v>
       </c>
       <c r="P43" t="n">
-        <v>4.5375</v>
+        <v>4.3125</v>
       </c>
       <c r="Q43" t="n">
         <v>4</v>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -3929,17 +3929,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Grimgar: Ashes and Illusions</t>
+          <t>Harry Potter and the Prisoner of Azkaban</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Light Novels / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Ao Jyumonji</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3953,7 +3953,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I44" t="n">
         <v>1</v>
@@ -3962,30 +3962,25 @@
         <v>1</v>
       </c>
       <c r="K44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O44" t="n">
-        <v>1.4</v>
+        <v>1.35</v>
       </c>
       <c r="P44" t="n">
-        <v>4.65</v>
+        <v>4.5375</v>
       </c>
       <c r="Q44" t="n">
         <v>4</v>
-      </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>re-audited: held after a Narrative Acceptance of Injustice / Redemption Difficulty trade that cancelled out</t>
-        </is>
       </c>
     </row>
     <row r="45">
@@ -3999,17 +3994,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Avatar: The Last Airbender</t>
+          <t>Grimgar: Ashes and Illusions</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Light Novels / Anime</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>Ao Jyumonji</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4019,7 +4014,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -4054,7 +4049,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Tier v1 era 3</t>
+          <t>re-audited: held after a Narrative Acceptance of Injustice / Redemption Difficulty trade that cancelled out</t>
         </is>
       </c>
     </row>
@@ -4069,17 +4064,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Earthsea</t>
+          <t>Avatar: The Last Airbender</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Ursula K. Le Guin</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4089,7 +4084,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -4099,10 +4094,10 @@
         <v>1</v>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L46" t="n">
         <v>2</v>
@@ -4121,6 +4116,11 @@
       </c>
       <c r="Q46" t="n">
         <v>4</v>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Tier v1 era 3</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -4134,17 +4134,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Final Fantasy XII</t>
+          <t>Earthsea</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Ursula K. Le Guin</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -4158,22 +4158,22 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I47" t="n">
         <v>1</v>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K47" t="n">
         <v>2</v>
       </c>
       <c r="L47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N47" t="n">
         <v>2</v>
@@ -4186,11 +4186,6 @@
       </c>
       <c r="Q47" t="n">
         <v>4</v>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
-        </is>
       </c>
     </row>
     <row r="48">
@@ -4204,17 +4199,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>The Legend of Vox Machina</t>
+          <t>Final Fantasy XII</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Critical Role</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4237,25 +4232,30 @@
         <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O48" t="n">
-        <v>1.35</v>
+        <v>1.4</v>
       </c>
       <c r="P48" t="n">
-        <v>4.8375</v>
+        <v>4.65</v>
       </c>
       <c r="Q48" t="n">
         <v>4</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -4269,17 +4269,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist: Brotherhood</t>
+          <t>The Legend of Vox Machina</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa</t>
+          <t>Critical Role</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -4302,7 +4302,7 @@
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L49" t="n">
         <v>2</v>
@@ -4314,10 +4314,10 @@
         <v>3</v>
       </c>
       <c r="O49" t="n">
-        <v>1.5</v>
+        <v>1.35</v>
       </c>
       <c r="P49" t="n">
-        <v>4.875</v>
+        <v>4.8375</v>
       </c>
       <c r="Q49" t="n">
         <v>4</v>
@@ -4334,17 +4334,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>The Boy and the Heron</t>
+          <t>Fullmetal Alchemist: Brotherhood</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Hiromu Arakawa</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4358,22 +4358,22 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N50" t="n">
         <v>3</v>
@@ -4399,17 +4399,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Final Fantasy IX</t>
+          <t>The Boy and the Heron</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4423,19 +4423,19 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M51" t="n">
         <v>2</v>
@@ -4464,17 +4464,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Ranking of Kings</t>
+          <t>Final Fantasy IX</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Sōsuke Tōka</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4488,19 +4488,19 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I52" t="n">
         <v>1</v>
       </c>
       <c r="J52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" t="n">
         <v>2</v>
       </c>
       <c r="L52" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M52" t="n">
         <v>2</v>
@@ -4516,11 +4516,6 @@
       </c>
       <c r="Q52" t="n">
         <v>4</v>
-      </c>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="53">
@@ -4534,17 +4529,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Adventure Time</t>
+          <t>Ranking of Kings</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>TV / Comics</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Pendleton Ward</t>
+          <t>Sōsuke Tōka</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4567,25 +4562,30 @@
         <v>1</v>
       </c>
       <c r="K53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L53" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M53" t="n">
         <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O53" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="P53" t="n">
-        <v>4.9875</v>
+        <v>4.875</v>
       </c>
       <c r="Q53" t="n">
         <v>4</v>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -4599,17 +4599,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Star vs. the Forces of Evil</t>
+          <t>Adventure Time</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>TV, Comics</t>
+          <t>TV / Comics</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Daron Nefcy</t>
+          <t>Pendleton Ward</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4623,7 +4623,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I54" t="n">
         <v>1</v>
@@ -4632,7 +4632,7 @@
         <v>1</v>
       </c>
       <c r="K54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L54" t="n">
         <v>2</v>
@@ -4652,34 +4652,29 @@
       <c r="Q54" t="n">
         <v>4</v>
       </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Tales from Earthsea</t>
+          <t>Star vs. the Forces of Evil</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV, Comics</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Gorō Miyazaki</t>
+          <t>Daron Nefcy</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4693,7 +4688,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I55" t="n">
         <v>1</v>
@@ -4702,7 +4697,7 @@
         <v>1</v>
       </c>
       <c r="K55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L55" t="n">
         <v>2</v>
@@ -4711,20 +4706,20 @@
         <v>2</v>
       </c>
       <c r="N55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O55" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="P55" t="n">
-        <v>5.2125</v>
+        <v>4.9875</v>
       </c>
       <c r="Q55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>re-audited: Explicit Darkness raised for the patricide opening and Therru's sustained visible abuse scarring</t>
+          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
         </is>
       </c>
     </row>
@@ -4739,17 +4734,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Dragonlance</t>
+          <t>Tales from Earthsea</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Novels / Games</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Margaret Weis / Tracy Hickman</t>
+          <t>Studio Ghibli / Gorō Miyazaki</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4772,13 +4767,13 @@
         <v>1</v>
       </c>
       <c r="K56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L56" t="n">
         <v>2</v>
       </c>
       <c r="M56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N56" t="n">
         <v>3</v>
@@ -4791,6 +4786,11 @@
       </c>
       <c r="Q56" t="n">
         <v>5</v>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>re-audited: Explicit Darkness raised for the patricide opening and Therru's sustained visible abuse scarring</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -4804,17 +4804,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Harry Potter and the Goblet of Fire</t>
+          <t>Dragonlance</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Novels / Games</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Margaret Weis / Tracy Hickman</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4828,22 +4828,22 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I57" t="n">
         <v>1</v>
       </c>
       <c r="J57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K57" t="n">
         <v>2</v>
       </c>
       <c r="L57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N57" t="n">
         <v>3</v>
@@ -4869,17 +4869,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Elantris</t>
+          <t>Harry Potter and the Goblet of Fire</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4893,22 +4893,22 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I58" t="n">
         <v>1</v>
       </c>
       <c r="J58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K58" t="n">
         <v>2</v>
       </c>
       <c r="L58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N58" t="n">
         <v>3</v>
@@ -4934,17 +4934,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Baldur's Gate III</t>
+          <t>Elantris</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4958,13 +4958,13 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
       </c>
       <c r="J59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K59" t="n">
         <v>2</v>
@@ -4986,11 +4986,6 @@
       </c>
       <c r="Q59" t="n">
         <v>5</v>
-      </c>
-      <c r="R59" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="60">
@@ -5004,17 +4999,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V: Skyrim</t>
+          <t>Baldur's Gate III</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Bethesda Game Studios</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5028,7 +5023,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I60" t="n">
         <v>1</v>
@@ -5040,22 +5035,27 @@
         <v>2</v>
       </c>
       <c r="L60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O60" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="P60" t="n">
-        <v>5.325</v>
+        <v>5.2125</v>
       </c>
       <c r="Q60" t="n">
         <v>5</v>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -5069,17 +5069,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The Silmarillion &amp; Great Tales</t>
+          <t>The Elder Scrolls V: Skyrim</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Books</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Bethesda Game Studios</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5105,10 +5105,10 @@
         <v>2</v>
       </c>
       <c r="L61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N61" t="n">
         <v>2</v>
@@ -5134,17 +5134,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>The Legend of Korra</t>
+          <t>The Silmarillion &amp; Great Tales</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Books</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5154,17 +5154,17 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H62" t="n">
         <v>2</v>
       </c>
       <c r="I62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K62" t="n">
         <v>2</v>
@@ -5186,11 +5186,6 @@
       </c>
       <c r="Q62" t="n">
         <v>5</v>
-      </c>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
-        </is>
       </c>
     </row>
     <row r="63">
@@ -5204,17 +5199,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Princess Mononoke</t>
+          <t>The Legend of Korra</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5224,7 +5219,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H63" t="n">
@@ -5234,28 +5229,33 @@
         <v>2</v>
       </c>
       <c r="J63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O63" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="P63" t="n">
-        <v>5.55</v>
+        <v>5.325</v>
       </c>
       <c r="Q63" t="n">
         <v>5</v>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -5269,17 +5269,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The Dark Elf / Drizzt</t>
+          <t>Princess Mononoke</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>R. A. Salvatore</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5296,16 +5296,16 @@
         <v>2</v>
       </c>
       <c r="I64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M64" t="n">
         <v>2</v>
@@ -5321,11 +5321,6 @@
       </c>
       <c r="Q64" t="n">
         <v>5</v>
-      </c>
-      <c r="R64" t="inlineStr">
-        <is>
-          <t>re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="65">
@@ -5339,17 +5334,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The Wheel of Time</t>
+          <t>The Dark Elf / Drizzt</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Robert Jordan / Brandon Sanderson</t>
+          <t>R. A. Salvatore</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5409,17 +5404,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Final Fantasy VI</t>
+          <t>The Wheel of Time</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Robert Jordan / Brandon Sanderson</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5433,13 +5428,13 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I66" t="n">
         <v>1</v>
       </c>
       <c r="J66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K66" t="n">
         <v>2</v>
@@ -5448,19 +5443,24 @@
         <v>2</v>
       </c>
       <c r="M66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O66" t="n">
-        <v>1.85</v>
+        <v>1.8</v>
       </c>
       <c r="P66" t="n">
-        <v>5.6625</v>
+        <v>5.55</v>
       </c>
       <c r="Q66" t="n">
         <v>5</v>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -5474,17 +5474,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>Final Fantasy VI</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5498,13 +5498,13 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K67" t="n">
         <v>2</v>
@@ -5513,7 +5513,7 @@
         <v>2</v>
       </c>
       <c r="M67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N67" t="n">
         <v>2</v>
@@ -5526,11 +5526,6 @@
       </c>
       <c r="Q67" t="n">
         <v>5</v>
-      </c>
-      <c r="R67" t="inlineStr">
-        <is>
-          <t>re-audited: held after testing Moral Cynicism and Limited Heroism revisions, both rejected on discipline grounds</t>
-        </is>
       </c>
     </row>
     <row r="68">
@@ -5544,17 +5539,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5574,32 +5569,32 @@
         <v>2</v>
       </c>
       <c r="J68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M68" t="n">
         <v>2</v>
       </c>
       <c r="N68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O68" t="n">
-        <v>1.9</v>
+        <v>1.85</v>
       </c>
       <c r="P68" t="n">
-        <v>5.775</v>
+        <v>5.6625</v>
       </c>
       <c r="Q68" t="n">
         <v>5</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Tier v1 era 6</t>
+          <t>re-audited: held after testing Moral Cynicism and Limited Heroism revisions, both rejected on discipline grounds</t>
         </is>
       </c>
     </row>
@@ -5614,17 +5609,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Final Fantasy X</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5638,34 +5633,39 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J69" t="n">
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L69" t="n">
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O69" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="P69" t="n">
-        <v>5.8875</v>
+        <v>5.775</v>
       </c>
       <c r="Q69" t="n">
         <v>5</v>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -5679,17 +5679,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Final Fantasy VII</t>
+          <t>Final Fantasy X</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Video Games / Remake Project</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5703,7 +5703,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I70" t="n">
         <v>1</v>
@@ -5718,7 +5718,7 @@
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N70" t="n">
         <v>3</v>
@@ -5744,17 +5744,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Final Fantasy VII</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Games / Remake Project</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5771,13 +5771,13 @@
         <v>2</v>
       </c>
       <c r="I71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J71" t="n">
         <v>2</v>
       </c>
       <c r="K71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L71" t="n">
         <v>1</v>
@@ -5809,7 +5809,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -5842,10 +5842,10 @@
         <v>2</v>
       </c>
       <c r="K72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M72" t="n">
         <v>2</v>
@@ -5874,17 +5874,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Final Fantasy XV</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5898,22 +5898,22 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J73" t="n">
         <v>2</v>
       </c>
       <c r="K73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L73" t="n">
         <v>2</v>
       </c>
       <c r="M73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N73" t="n">
         <v>3</v>
@@ -5930,26 +5930,26 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Clevatess</t>
+          <t>Final Fantasy XV</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Yūji Iwahara</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5963,10 +5963,10 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J74" t="n">
         <v>2</v>
@@ -5975,27 +5975,22 @@
         <v>2</v>
       </c>
       <c r="L74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O74" t="n">
-        <v>2.05</v>
+        <v>1.95</v>
       </c>
       <c r="P74" t="n">
-        <v>6.1125</v>
+        <v>5.8875</v>
       </c>
       <c r="Q74" t="n">
-        <v>6</v>
-      </c>
-      <c r="R74" t="inlineStr">
-        <is>
-          <t>scored against the story as currently published/aired; ongoing/unresolved, later arcs may shift this</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="75">
@@ -6009,17 +6004,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Re:Zero − Starting Life in Another World</t>
+          <t>Clevatess</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Light Novels, Manga, Anime</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Tappei Nagatsuki</t>
+          <t>Yūji Iwahara</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6036,7 +6031,7 @@
         <v>2</v>
       </c>
       <c r="I75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J75" t="n">
         <v>2</v>
@@ -6045,7 +6040,7 @@
         <v>2</v>
       </c>
       <c r="L75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M75" t="n">
         <v>2</v>
@@ -6064,7 +6059,7 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>scored against the arcs most widely adapted/translated (roughly Arcs 1-6); later arcs may shift this</t>
+          <t>scored against the story as currently published/aired; ongoing/unresolved, later arcs may shift this</t>
         </is>
       </c>
     </row>
@@ -6079,17 +6074,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Re:Zero − Starting Life in Another World</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Light Novels, Manga, Anime</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>Tappei Nagatsuki</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6106,7 +6101,7 @@
         <v>2</v>
       </c>
       <c r="I76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J76" t="n">
         <v>2</v>
@@ -6121,16 +6116,21 @@
         <v>2</v>
       </c>
       <c r="N76" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O76" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="P76" t="n">
-        <v>6.225</v>
+        <v>6.1125</v>
       </c>
       <c r="Q76" t="n">
         <v>6</v>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>scored against the arcs most widely adapted/translated (roughly Arcs 1-6); later arcs may shift this</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -6144,17 +6144,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6168,16 +6168,16 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L77" t="n">
         <v>2</v>
@@ -6209,17 +6209,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6233,13 +6233,13 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K78" t="n">
         <v>3</v>
@@ -6251,21 +6251,16 @@
         <v>2</v>
       </c>
       <c r="N78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O78" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P78" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q78" t="n">
         <v>6</v>
-      </c>
-      <c r="R78" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="79">
@@ -6279,17 +6274,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6312,7 +6307,7 @@
         <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L79" t="n">
         <v>2</v>
@@ -6321,16 +6316,21 @@
         <v>2</v>
       </c>
       <c r="N79" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O79" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P79" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q79" t="n">
         <v>6</v>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -6344,17 +6344,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Pan's Labyrinth</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Guillermo del Toro</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6377,13 +6377,13 @@
         <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L80" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N80" t="n">
         <v>4</v>
@@ -6409,17 +6409,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Pan's Labyrinth</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Guillermo del Toro</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6433,7 +6433,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I81" t="n">
         <v>2</v>
@@ -6442,30 +6442,25 @@
         <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L81" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O81" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P81" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q81" t="n">
         <v>6</v>
-      </c>
-      <c r="R81" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="82">
@@ -6479,17 +6474,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6503,13 +6498,13 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I82" t="n">
         <v>2</v>
       </c>
       <c r="J82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K82" t="n">
         <v>2</v>
@@ -6534,7 +6529,7 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6549,17 +6544,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6579,10 +6574,10 @@
         <v>2</v>
       </c>
       <c r="J83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L83" t="n">
         <v>2</v>
@@ -6601,6 +6596,11 @@
       </c>
       <c r="Q83" t="n">
         <v>6</v>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -6614,17 +6614,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6679,17 +6679,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6706,7 +6706,7 @@
         <v>2</v>
       </c>
       <c r="I85" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J85" t="n">
         <v>2</v>
@@ -6715,7 +6715,7 @@
         <v>3</v>
       </c>
       <c r="L85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M85" t="n">
         <v>2</v>
@@ -6744,17 +6744,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6768,7 +6768,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I86" t="n">
         <v>1</v>
@@ -6780,7 +6780,7 @@
         <v>3</v>
       </c>
       <c r="L86" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M86" t="n">
         <v>2</v>
@@ -6809,17 +6809,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Märchen Crown</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Aka Akasaka / Aoi Kujira / Azychika</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6833,10 +6833,10 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J87" t="n">
         <v>2</v>
@@ -6851,21 +6851,16 @@
         <v>2</v>
       </c>
       <c r="N87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O87" t="n">
-        <v>2.35</v>
+        <v>2.25</v>
       </c>
       <c r="P87" t="n">
-        <v>6.7875</v>
+        <v>6.5625</v>
       </c>
       <c r="Q87" t="n">
         <v>6</v>
-      </c>
-      <c r="R87" t="inlineStr">
-        <is>
-          <t>ongoing/unresolved as of ch. 47 (Jul 2026); low-mid confidence given thin reception in most languages researched</t>
-        </is>
       </c>
     </row>
     <row r="88">
@@ -6879,17 +6874,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Märchen Crown</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>Aka Akasaka / Aoi Kujira / Azychika</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6915,46 +6910,51 @@
         <v>3</v>
       </c>
       <c r="L88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M88" t="n">
         <v>2</v>
       </c>
       <c r="N88" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O88" t="n">
-        <v>2.4</v>
+        <v>2.35</v>
       </c>
       <c r="P88" t="n">
-        <v>6.9</v>
+        <v>6.7875</v>
       </c>
       <c r="Q88" t="n">
         <v>6</v>
       </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>ongoing/unresolved as of ch. 47 (Jul 2026); low-mid confidence given thin reception in most languages researched</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Attack on Titan</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Hajime Isayama</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6968,13 +6968,13 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I89" t="n">
         <v>2</v>
       </c>
       <c r="J89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K89" t="n">
         <v>3</v>
@@ -6986,40 +6986,40 @@
         <v>2</v>
       </c>
       <c r="N89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O89" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="P89" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="Q89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>Attack on Titan</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Manga, Anime, Films</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Hajime Isayama</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -7036,36 +7036,31 @@
         <v>3</v>
       </c>
       <c r="I90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J90" t="n">
         <v>3</v>
       </c>
       <c r="K90" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L90" t="n">
         <v>3</v>
       </c>
       <c r="M90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N90" t="n">
         <v>4</v>
       </c>
       <c r="O90" t="n">
-        <v>2.95</v>
+        <v>2.8</v>
       </c>
       <c r="P90" t="n">
-        <v>8.137499999999999</v>
+        <v>7.8</v>
       </c>
       <c r="Q90" t="n">
-        <v>8</v>
-      </c>
-      <c r="R90" t="inlineStr">
-        <is>
-          <t>re-audited: no documented reasoning survived from the original score; Limited Heroism and Narrative Acceptance of Injustice revised up on distinct evidence, Structural Corruption held at 2 after checking against A Song of Ice and Fire's multi-institutional bar</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="91">
@@ -7079,17 +7074,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Manga, Anime, Films</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -7112,7 +7107,7 @@
         <v>3</v>
       </c>
       <c r="K91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L91" t="n">
         <v>3</v>
@@ -7121,20 +7116,20 @@
         <v>3</v>
       </c>
       <c r="N91" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O91" t="n">
-        <v>3</v>
+        <v>2.95</v>
       </c>
       <c r="P91" t="n">
-        <v>8.25</v>
+        <v>8.137499999999999</v>
       </c>
       <c r="Q91" t="n">
         <v>8</v>
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>re-audited: previously flagged inconsistency vs. Elden Ring, resolved</t>
+          <t>re-audited: no documented reasoning survived from the original score; Limited Heroism and Narrative Acceptance of Injustice revised up on distinct evidence, Structural Corruption held at 2 after checking against A Song of Ice and Fire's multi-institutional bar</t>
         </is>
       </c>
     </row>
@@ -7149,17 +7144,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -7191,16 +7186,21 @@
         <v>3</v>
       </c>
       <c r="N92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O92" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="P92" t="n">
-        <v>8.475</v>
+        <v>8.25</v>
       </c>
       <c r="Q92" t="n">
         <v>8</v>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>re-audited: previously flagged inconsistency vs. Elden Ring, resolved</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -7214,17 +7214,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -7238,31 +7238,31 @@
         </is>
       </c>
       <c r="H93" t="n">
+        <v>3</v>
+      </c>
+      <c r="I93" t="n">
+        <v>3</v>
+      </c>
+      <c r="J93" t="n">
+        <v>3</v>
+      </c>
+      <c r="K93" t="n">
+        <v>3</v>
+      </c>
+      <c r="L93" t="n">
+        <v>3</v>
+      </c>
+      <c r="M93" t="n">
+        <v>3</v>
+      </c>
+      <c r="N93" t="n">
         <v>4</v>
       </c>
-      <c r="I93" t="n">
-        <v>3</v>
-      </c>
-      <c r="J93" t="n">
-        <v>3</v>
-      </c>
-      <c r="K93" t="n">
-        <v>3</v>
-      </c>
-      <c r="L93" t="n">
-        <v>3</v>
-      </c>
-      <c r="M93" t="n">
-        <v>3</v>
-      </c>
-      <c r="N93" t="n">
-        <v>3</v>
-      </c>
       <c r="O93" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P93" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q93" t="n">
         <v>8</v>
@@ -7279,17 +7279,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -7303,13 +7303,13 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I94" t="n">
         <v>3</v>
       </c>
       <c r="J94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K94" t="n">
         <v>3</v>
@@ -7321,13 +7321,13 @@
         <v>3</v>
       </c>
       <c r="N94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O94" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P94" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q94" t="n">
         <v>8</v>
@@ -7335,26 +7335,26 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -7368,16 +7368,16 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J95" t="n">
         <v>4</v>
       </c>
       <c r="K95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L95" t="n">
         <v>3</v>
@@ -7389,37 +7389,37 @@
         <v>4</v>
       </c>
       <c r="O95" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P95" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q95" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -7445,21 +7445,86 @@
         <v>4</v>
       </c>
       <c r="L96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N96" t="n">
         <v>4</v>
       </c>
       <c r="O96" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P96" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>10</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H97" t="n">
         <v>4</v>
       </c>
-      <c r="P96" t="n">
+      <c r="I97" t="n">
+        <v>4</v>
+      </c>
+      <c r="J97" t="n">
+        <v>4</v>
+      </c>
+      <c r="K97" t="n">
+        <v>4</v>
+      </c>
+      <c r="L97" t="n">
+        <v>4</v>
+      </c>
+      <c r="M97" t="n">
+        <v>4</v>
+      </c>
+      <c r="N97" t="n">
+        <v>4</v>
+      </c>
+      <c r="O97" t="n">
+        <v>4</v>
+      </c>
+      <c r="P97" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q96" t="n">
+      <c r="Q97" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7535,7 +7600,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -7632,7 +7697,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 95 of 95 works in the full catalog.</t>
+          <t>Total scored: 96 of 96 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Disenchantment (2018) to tier 4
Tier 4 (Fantasy in Gray Tones), score 4.3125, matching Witch Hat
Atelier/Baldur's Gate II. Real institutional darkness (Zog's cruel,
incompetent monarchy; Dagmar's manipulative secret society) and genuine
dark content (Elfo's on-screen death, elf-blood-harvesting for
immortality potions), softened by Groening's fundamentally comedic,
satirical register and exaggerated animation style.

Catalog now stands at 97 works.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R97"/>
+  <dimension ref="A1:R98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3929,17 +3929,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Harry Potter and the Prisoner of Azkaban</t>
+          <t>Disenchantment</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Matt Groening</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3965,19 +3965,19 @@
         <v>2</v>
       </c>
       <c r="L44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O44" t="n">
-        <v>1.35</v>
+        <v>1.25</v>
       </c>
       <c r="P44" t="n">
-        <v>4.5375</v>
+        <v>4.3125</v>
       </c>
       <c r="Q44" t="n">
         <v>4</v>
@@ -3994,17 +3994,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Grimgar: Ashes and Illusions</t>
+          <t>Harry Potter and the Prisoner of Azkaban</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Light Novels / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Ao Jyumonji</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4018,7 +4018,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I45" t="n">
         <v>1</v>
@@ -4027,30 +4027,25 @@
         <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O45" t="n">
-        <v>1.4</v>
+        <v>1.35</v>
       </c>
       <c r="P45" t="n">
-        <v>4.65</v>
+        <v>4.5375</v>
       </c>
       <c r="Q45" t="n">
         <v>4</v>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>re-audited: held after a Narrative Acceptance of Injustice / Redemption Difficulty trade that cancelled out</t>
-        </is>
       </c>
     </row>
     <row r="46">
@@ -4064,17 +4059,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Avatar: The Last Airbender</t>
+          <t>Grimgar: Ashes and Illusions</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Light Novels / Anime</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>Ao Jyumonji</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4084,7 +4079,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -4119,7 +4114,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Tier v1 era 3</t>
+          <t>re-audited: held after a Narrative Acceptance of Injustice / Redemption Difficulty trade that cancelled out</t>
         </is>
       </c>
     </row>
@@ -4134,17 +4129,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Earthsea</t>
+          <t>Avatar: The Last Airbender</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Ursula K. Le Guin</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -4154,7 +4149,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H47" t="n">
@@ -4164,10 +4159,10 @@
         <v>1</v>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L47" t="n">
         <v>2</v>
@@ -4186,6 +4181,11 @@
       </c>
       <c r="Q47" t="n">
         <v>4</v>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Tier v1 era 3</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -4199,17 +4199,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Final Fantasy XII</t>
+          <t>Earthsea</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Ursula K. Le Guin</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4223,22 +4223,22 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I48" t="n">
         <v>1</v>
       </c>
       <c r="J48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K48" t="n">
         <v>2</v>
       </c>
       <c r="L48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N48" t="n">
         <v>2</v>
@@ -4251,11 +4251,6 @@
       </c>
       <c r="Q48" t="n">
         <v>4</v>
-      </c>
-      <c r="R48" t="inlineStr">
-        <is>
-          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
-        </is>
       </c>
     </row>
     <row r="49">
@@ -4269,17 +4264,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>The Legend of Vox Machina</t>
+          <t>Final Fantasy XII</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Critical Role</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -4302,25 +4297,30 @@
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O49" t="n">
-        <v>1.35</v>
+        <v>1.4</v>
       </c>
       <c r="P49" t="n">
-        <v>4.8375</v>
+        <v>4.65</v>
       </c>
       <c r="Q49" t="n">
         <v>4</v>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -4334,17 +4334,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist: Brotherhood</t>
+          <t>The Legend of Vox Machina</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa</t>
+          <t>Critical Role</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4367,7 +4367,7 @@
         <v>1</v>
       </c>
       <c r="K50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L50" t="n">
         <v>2</v>
@@ -4379,10 +4379,10 @@
         <v>3</v>
       </c>
       <c r="O50" t="n">
-        <v>1.5</v>
+        <v>1.35</v>
       </c>
       <c r="P50" t="n">
-        <v>4.875</v>
+        <v>4.8375</v>
       </c>
       <c r="Q50" t="n">
         <v>4</v>
@@ -4399,17 +4399,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>The Boy and the Heron</t>
+          <t>Fullmetal Alchemist: Brotherhood</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Hiromu Arakawa</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4423,22 +4423,22 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N51" t="n">
         <v>3</v>
@@ -4464,17 +4464,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Final Fantasy IX</t>
+          <t>The Boy and the Heron</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4488,19 +4488,19 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M52" t="n">
         <v>2</v>
@@ -4529,17 +4529,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Ranking of Kings</t>
+          <t>Final Fantasy IX</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Sōsuke Tōka</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4553,19 +4553,19 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I53" t="n">
         <v>1</v>
       </c>
       <c r="J53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K53" t="n">
         <v>2</v>
       </c>
       <c r="L53" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M53" t="n">
         <v>2</v>
@@ -4581,11 +4581,6 @@
       </c>
       <c r="Q53" t="n">
         <v>4</v>
-      </c>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="54">
@@ -4599,17 +4594,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Adventure Time</t>
+          <t>Ranking of Kings</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>TV / Comics</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Pendleton Ward</t>
+          <t>Sōsuke Tōka</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4632,25 +4627,30 @@
         <v>1</v>
       </c>
       <c r="K54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L54" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M54" t="n">
         <v>2</v>
       </c>
       <c r="N54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O54" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="P54" t="n">
-        <v>4.9875</v>
+        <v>4.875</v>
       </c>
       <c r="Q54" t="n">
         <v>4</v>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -4664,17 +4664,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Star vs. the Forces of Evil</t>
+          <t>Adventure Time</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>TV, Comics</t>
+          <t>TV / Comics</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Daron Nefcy</t>
+          <t>Pendleton Ward</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4688,7 +4688,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I55" t="n">
         <v>1</v>
@@ -4697,7 +4697,7 @@
         <v>1</v>
       </c>
       <c r="K55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L55" t="n">
         <v>2</v>
@@ -4717,34 +4717,29 @@
       <c r="Q55" t="n">
         <v>4</v>
       </c>
-      <c r="R55" t="inlineStr">
-        <is>
-          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Tales from Earthsea</t>
+          <t>Star vs. the Forces of Evil</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV, Comics</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Gorō Miyazaki</t>
+          <t>Daron Nefcy</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4758,7 +4753,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I56" t="n">
         <v>1</v>
@@ -4767,7 +4762,7 @@
         <v>1</v>
       </c>
       <c r="K56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L56" t="n">
         <v>2</v>
@@ -4776,20 +4771,20 @@
         <v>2</v>
       </c>
       <c r="N56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O56" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="P56" t="n">
-        <v>5.2125</v>
+        <v>4.9875</v>
       </c>
       <c r="Q56" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>re-audited: Explicit Darkness raised for the patricide opening and Therru's sustained visible abuse scarring</t>
+          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
         </is>
       </c>
     </row>
@@ -4804,17 +4799,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Dragonlance</t>
+          <t>Tales from Earthsea</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Novels / Games</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Margaret Weis / Tracy Hickman</t>
+          <t>Studio Ghibli / Gorō Miyazaki</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4837,13 +4832,13 @@
         <v>1</v>
       </c>
       <c r="K57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L57" t="n">
         <v>2</v>
       </c>
       <c r="M57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N57" t="n">
         <v>3</v>
@@ -4856,6 +4851,11 @@
       </c>
       <c r="Q57" t="n">
         <v>5</v>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>re-audited: Explicit Darkness raised for the patricide opening and Therru's sustained visible abuse scarring</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -4869,17 +4869,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Harry Potter and the Goblet of Fire</t>
+          <t>Dragonlance</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Novels / Games</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Margaret Weis / Tracy Hickman</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4893,22 +4893,22 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I58" t="n">
         <v>1</v>
       </c>
       <c r="J58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K58" t="n">
         <v>2</v>
       </c>
       <c r="L58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N58" t="n">
         <v>3</v>
@@ -4934,17 +4934,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Elantris</t>
+          <t>Harry Potter and the Goblet of Fire</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4958,22 +4958,22 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
       </c>
       <c r="J59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K59" t="n">
         <v>2</v>
       </c>
       <c r="L59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N59" t="n">
         <v>3</v>
@@ -4999,17 +4999,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Baldur's Gate III</t>
+          <t>Elantris</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5023,13 +5023,13 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I60" t="n">
         <v>1</v>
       </c>
       <c r="J60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K60" t="n">
         <v>2</v>
@@ -5051,11 +5051,6 @@
       </c>
       <c r="Q60" t="n">
         <v>5</v>
-      </c>
-      <c r="R60" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="61">
@@ -5069,17 +5064,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V: Skyrim</t>
+          <t>Baldur's Gate III</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Bethesda Game Studios</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5093,7 +5088,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I61" t="n">
         <v>1</v>
@@ -5105,22 +5100,27 @@
         <v>2</v>
       </c>
       <c r="L61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O61" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="P61" t="n">
-        <v>5.325</v>
+        <v>5.2125</v>
       </c>
       <c r="Q61" t="n">
         <v>5</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -5134,17 +5134,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>The Silmarillion &amp; Great Tales</t>
+          <t>The Elder Scrolls V: Skyrim</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Books</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Bethesda Game Studios</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5170,10 +5170,10 @@
         <v>2</v>
       </c>
       <c r="L62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N62" t="n">
         <v>2</v>
@@ -5199,17 +5199,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The Legend of Korra</t>
+          <t>The Silmarillion &amp; Great Tales</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Books</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5219,17 +5219,17 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H63" t="n">
         <v>2</v>
       </c>
       <c r="I63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K63" t="n">
         <v>2</v>
@@ -5251,11 +5251,6 @@
       </c>
       <c r="Q63" t="n">
         <v>5</v>
-      </c>
-      <c r="R63" t="inlineStr">
-        <is>
-          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
-        </is>
       </c>
     </row>
     <row r="64">
@@ -5269,17 +5264,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Princess Mononoke</t>
+          <t>The Legend of Korra</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5289,7 +5284,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H64" t="n">
@@ -5299,28 +5294,33 @@
         <v>2</v>
       </c>
       <c r="J64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O64" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="P64" t="n">
-        <v>5.55</v>
+        <v>5.325</v>
       </c>
       <c r="Q64" t="n">
         <v>5</v>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -5334,17 +5334,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The Dark Elf / Drizzt</t>
+          <t>Princess Mononoke</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>R. A. Salvatore</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5361,16 +5361,16 @@
         <v>2</v>
       </c>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M65" t="n">
         <v>2</v>
@@ -5386,11 +5386,6 @@
       </c>
       <c r="Q65" t="n">
         <v>5</v>
-      </c>
-      <c r="R65" t="inlineStr">
-        <is>
-          <t>re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="66">
@@ -5404,17 +5399,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Wheel of Time</t>
+          <t>The Dark Elf / Drizzt</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Robert Jordan / Brandon Sanderson</t>
+          <t>R. A. Salvatore</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5474,17 +5469,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Final Fantasy VI</t>
+          <t>The Wheel of Time</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Robert Jordan / Brandon Sanderson</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5498,13 +5493,13 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I67" t="n">
         <v>1</v>
       </c>
       <c r="J67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K67" t="n">
         <v>2</v>
@@ -5513,19 +5508,24 @@
         <v>2</v>
       </c>
       <c r="M67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O67" t="n">
-        <v>1.85</v>
+        <v>1.8</v>
       </c>
       <c r="P67" t="n">
-        <v>5.6625</v>
+        <v>5.55</v>
       </c>
       <c r="Q67" t="n">
         <v>5</v>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -5539,17 +5539,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>Final Fantasy VI</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5563,13 +5563,13 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K68" t="n">
         <v>2</v>
@@ -5578,7 +5578,7 @@
         <v>2</v>
       </c>
       <c r="M68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N68" t="n">
         <v>2</v>
@@ -5591,11 +5591,6 @@
       </c>
       <c r="Q68" t="n">
         <v>5</v>
-      </c>
-      <c r="R68" t="inlineStr">
-        <is>
-          <t>re-audited: held after testing Moral Cynicism and Limited Heroism revisions, both rejected on discipline grounds</t>
-        </is>
       </c>
     </row>
     <row r="69">
@@ -5609,17 +5604,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5639,32 +5634,32 @@
         <v>2</v>
       </c>
       <c r="J69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M69" t="n">
         <v>2</v>
       </c>
       <c r="N69" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O69" t="n">
-        <v>1.9</v>
+        <v>1.85</v>
       </c>
       <c r="P69" t="n">
-        <v>5.775</v>
+        <v>5.6625</v>
       </c>
       <c r="Q69" t="n">
         <v>5</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>Tier v1 era 6</t>
+          <t>re-audited: held after testing Moral Cynicism and Limited Heroism revisions, both rejected on discipline grounds</t>
         </is>
       </c>
     </row>
@@ -5679,17 +5674,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Final Fantasy X</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5703,34 +5698,39 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J70" t="n">
         <v>2</v>
       </c>
       <c r="K70" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L70" t="n">
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N70" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O70" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="P70" t="n">
-        <v>5.8875</v>
+        <v>5.775</v>
       </c>
       <c r="Q70" t="n">
         <v>5</v>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -5744,17 +5744,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Final Fantasy VII</t>
+          <t>Final Fantasy X</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Video Games / Remake Project</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5768,7 +5768,7 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I71" t="n">
         <v>1</v>
@@ -5783,7 +5783,7 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N71" t="n">
         <v>3</v>
@@ -5809,17 +5809,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Final Fantasy VII</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Games / Remake Project</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5836,13 +5836,13 @@
         <v>2</v>
       </c>
       <c r="I72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J72" t="n">
         <v>2</v>
       </c>
       <c r="K72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L72" t="n">
         <v>1</v>
@@ -5874,7 +5874,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -5907,10 +5907,10 @@
         <v>2</v>
       </c>
       <c r="K73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M73" t="n">
         <v>2</v>
@@ -5939,17 +5939,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Final Fantasy XV</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5963,22 +5963,22 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J74" t="n">
         <v>2</v>
       </c>
       <c r="K74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L74" t="n">
         <v>2</v>
       </c>
       <c r="M74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N74" t="n">
         <v>3</v>
@@ -5995,26 +5995,26 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Clevatess</t>
+          <t>Final Fantasy XV</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Yūji Iwahara</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6028,10 +6028,10 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J75" t="n">
         <v>2</v>
@@ -6040,27 +6040,22 @@
         <v>2</v>
       </c>
       <c r="L75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N75" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O75" t="n">
-        <v>2.05</v>
+        <v>1.95</v>
       </c>
       <c r="P75" t="n">
-        <v>6.1125</v>
+        <v>5.8875</v>
       </c>
       <c r="Q75" t="n">
-        <v>6</v>
-      </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>scored against the story as currently published/aired; ongoing/unresolved, later arcs may shift this</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="76">
@@ -6074,17 +6069,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Re:Zero − Starting Life in Another World</t>
+          <t>Clevatess</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Light Novels, Manga, Anime</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Tappei Nagatsuki</t>
+          <t>Yūji Iwahara</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6101,7 +6096,7 @@
         <v>2</v>
       </c>
       <c r="I76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J76" t="n">
         <v>2</v>
@@ -6110,7 +6105,7 @@
         <v>2</v>
       </c>
       <c r="L76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M76" t="n">
         <v>2</v>
@@ -6129,7 +6124,7 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>scored against the arcs most widely adapted/translated (roughly Arcs 1-6); later arcs may shift this</t>
+          <t>scored against the story as currently published/aired; ongoing/unresolved, later arcs may shift this</t>
         </is>
       </c>
     </row>
@@ -6144,17 +6139,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Re:Zero − Starting Life in Another World</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Light Novels, Manga, Anime</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>Tappei Nagatsuki</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6171,7 +6166,7 @@
         <v>2</v>
       </c>
       <c r="I77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J77" t="n">
         <v>2</v>
@@ -6186,16 +6181,21 @@
         <v>2</v>
       </c>
       <c r="N77" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O77" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="P77" t="n">
-        <v>6.225</v>
+        <v>6.1125</v>
       </c>
       <c r="Q77" t="n">
         <v>6</v>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>scored against the arcs most widely adapted/translated (roughly Arcs 1-6); later arcs may shift this</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -6209,17 +6209,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6233,16 +6233,16 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L78" t="n">
         <v>2</v>
@@ -6274,17 +6274,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6298,13 +6298,13 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K79" t="n">
         <v>3</v>
@@ -6316,21 +6316,16 @@
         <v>2</v>
       </c>
       <c r="N79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O79" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P79" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q79" t="n">
         <v>6</v>
-      </c>
-      <c r="R79" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="80">
@@ -6344,17 +6339,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6377,7 +6372,7 @@
         <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L80" t="n">
         <v>2</v>
@@ -6386,16 +6381,21 @@
         <v>2</v>
       </c>
       <c r="N80" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O80" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P80" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q80" t="n">
         <v>6</v>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -6409,17 +6409,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Pan's Labyrinth</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Guillermo del Toro</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6442,13 +6442,13 @@
         <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L81" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N81" t="n">
         <v>4</v>
@@ -6474,17 +6474,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Pan's Labyrinth</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Guillermo del Toro</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6498,7 +6498,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I82" t="n">
         <v>2</v>
@@ -6507,30 +6507,25 @@
         <v>2</v>
       </c>
       <c r="K82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L82" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N82" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O82" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P82" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q82" t="n">
         <v>6</v>
-      </c>
-      <c r="R82" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="83">
@@ -6544,17 +6539,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6568,13 +6563,13 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I83" t="n">
         <v>2</v>
       </c>
       <c r="J83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K83" t="n">
         <v>2</v>
@@ -6599,7 +6594,7 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6614,17 +6609,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6644,10 +6639,10 @@
         <v>2</v>
       </c>
       <c r="J84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L84" t="n">
         <v>2</v>
@@ -6666,6 +6661,11 @@
       </c>
       <c r="Q84" t="n">
         <v>6</v>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -6679,17 +6679,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6744,17 +6744,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6771,7 +6771,7 @@
         <v>2</v>
       </c>
       <c r="I86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J86" t="n">
         <v>2</v>
@@ -6780,7 +6780,7 @@
         <v>3</v>
       </c>
       <c r="L86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M86" t="n">
         <v>2</v>
@@ -6809,17 +6809,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6833,7 +6833,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I87" t="n">
         <v>1</v>
@@ -6845,7 +6845,7 @@
         <v>3</v>
       </c>
       <c r="L87" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M87" t="n">
         <v>2</v>
@@ -6874,17 +6874,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Märchen Crown</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Aka Akasaka / Aoi Kujira / Azychika</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6898,10 +6898,10 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J88" t="n">
         <v>2</v>
@@ -6916,21 +6916,16 @@
         <v>2</v>
       </c>
       <c r="N88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O88" t="n">
-        <v>2.35</v>
+        <v>2.25</v>
       </c>
       <c r="P88" t="n">
-        <v>6.7875</v>
+        <v>6.5625</v>
       </c>
       <c r="Q88" t="n">
         <v>6</v>
-      </c>
-      <c r="R88" t="inlineStr">
-        <is>
-          <t>ongoing/unresolved as of ch. 47 (Jul 2026); low-mid confidence given thin reception in most languages researched</t>
-        </is>
       </c>
     </row>
     <row r="89">
@@ -6944,17 +6939,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Märchen Crown</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>Aka Akasaka / Aoi Kujira / Azychika</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6980,46 +6975,51 @@
         <v>3</v>
       </c>
       <c r="L89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M89" t="n">
         <v>2</v>
       </c>
       <c r="N89" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O89" t="n">
-        <v>2.4</v>
+        <v>2.35</v>
       </c>
       <c r="P89" t="n">
-        <v>6.9</v>
+        <v>6.7875</v>
       </c>
       <c r="Q89" t="n">
         <v>6</v>
       </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>ongoing/unresolved as of ch. 47 (Jul 2026); low-mid confidence given thin reception in most languages researched</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Attack on Titan</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Hajime Isayama</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -7033,13 +7033,13 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I90" t="n">
         <v>2</v>
       </c>
       <c r="J90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K90" t="n">
         <v>3</v>
@@ -7051,40 +7051,40 @@
         <v>2</v>
       </c>
       <c r="N90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O90" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="P90" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="Q90" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>Attack on Titan</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Manga, Anime, Films</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Hajime Isayama</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -7101,36 +7101,31 @@
         <v>3</v>
       </c>
       <c r="I91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J91" t="n">
         <v>3</v>
       </c>
       <c r="K91" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L91" t="n">
         <v>3</v>
       </c>
       <c r="M91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N91" t="n">
         <v>4</v>
       </c>
       <c r="O91" t="n">
-        <v>2.95</v>
+        <v>2.8</v>
       </c>
       <c r="P91" t="n">
-        <v>8.137499999999999</v>
+        <v>7.8</v>
       </c>
       <c r="Q91" t="n">
-        <v>8</v>
-      </c>
-      <c r="R91" t="inlineStr">
-        <is>
-          <t>re-audited: no documented reasoning survived from the original score; Limited Heroism and Narrative Acceptance of Injustice revised up on distinct evidence, Structural Corruption held at 2 after checking against A Song of Ice and Fire's multi-institutional bar</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="92">
@@ -7144,17 +7139,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Manga, Anime, Films</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -7177,7 +7172,7 @@
         <v>3</v>
       </c>
       <c r="K92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L92" t="n">
         <v>3</v>
@@ -7186,20 +7181,20 @@
         <v>3</v>
       </c>
       <c r="N92" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O92" t="n">
-        <v>3</v>
+        <v>2.95</v>
       </c>
       <c r="P92" t="n">
-        <v>8.25</v>
+        <v>8.137499999999999</v>
       </c>
       <c r="Q92" t="n">
         <v>8</v>
       </c>
       <c r="R92" t="inlineStr">
         <is>
-          <t>re-audited: previously flagged inconsistency vs. Elden Ring, resolved</t>
+          <t>re-audited: no documented reasoning survived from the original score; Limited Heroism and Narrative Acceptance of Injustice revised up on distinct evidence, Structural Corruption held at 2 after checking against A Song of Ice and Fire's multi-institutional bar</t>
         </is>
       </c>
     </row>
@@ -7214,17 +7209,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -7256,16 +7251,21 @@
         <v>3</v>
       </c>
       <c r="N93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O93" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="P93" t="n">
-        <v>8.475</v>
+        <v>8.25</v>
       </c>
       <c r="Q93" t="n">
         <v>8</v>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>re-audited: previously flagged inconsistency vs. Elden Ring, resolved</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -7279,17 +7279,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -7303,31 +7303,31 @@
         </is>
       </c>
       <c r="H94" t="n">
+        <v>3</v>
+      </c>
+      <c r="I94" t="n">
+        <v>3</v>
+      </c>
+      <c r="J94" t="n">
+        <v>3</v>
+      </c>
+      <c r="K94" t="n">
+        <v>3</v>
+      </c>
+      <c r="L94" t="n">
+        <v>3</v>
+      </c>
+      <c r="M94" t="n">
+        <v>3</v>
+      </c>
+      <c r="N94" t="n">
         <v>4</v>
       </c>
-      <c r="I94" t="n">
-        <v>3</v>
-      </c>
-      <c r="J94" t="n">
-        <v>3</v>
-      </c>
-      <c r="K94" t="n">
-        <v>3</v>
-      </c>
-      <c r="L94" t="n">
-        <v>3</v>
-      </c>
-      <c r="M94" t="n">
-        <v>3</v>
-      </c>
-      <c r="N94" t="n">
-        <v>3</v>
-      </c>
       <c r="O94" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P94" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q94" t="n">
         <v>8</v>
@@ -7344,17 +7344,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -7368,13 +7368,13 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I95" t="n">
         <v>3</v>
       </c>
       <c r="J95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K95" t="n">
         <v>3</v>
@@ -7386,13 +7386,13 @@
         <v>3</v>
       </c>
       <c r="N95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O95" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P95" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q95" t="n">
         <v>8</v>
@@ -7400,26 +7400,26 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -7433,16 +7433,16 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J96" t="n">
         <v>4</v>
       </c>
       <c r="K96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L96" t="n">
         <v>3</v>
@@ -7454,37 +7454,37 @@
         <v>4</v>
       </c>
       <c r="O96" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P96" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q96" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -7510,21 +7510,86 @@
         <v>4</v>
       </c>
       <c r="L97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N97" t="n">
         <v>4</v>
       </c>
       <c r="O97" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P97" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>10</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H98" t="n">
         <v>4</v>
       </c>
-      <c r="P97" t="n">
+      <c r="I98" t="n">
+        <v>4</v>
+      </c>
+      <c r="J98" t="n">
+        <v>4</v>
+      </c>
+      <c r="K98" t="n">
+        <v>4</v>
+      </c>
+      <c r="L98" t="n">
+        <v>4</v>
+      </c>
+      <c r="M98" t="n">
+        <v>4</v>
+      </c>
+      <c r="N98" t="n">
+        <v>4</v>
+      </c>
+      <c r="O98" t="n">
+        <v>4</v>
+      </c>
+      <c r="P98" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q97" t="n">
+      <c r="Q98" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7613,7 +7678,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -7697,7 +7762,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 96 of 96 works in the full catalog.</t>
+          <t>Total scored: 97 of 97 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Dungeons & Dragons (1983) to tier 2
Tier 2 (Bright Fantasy), score 2.7375, matching A Conspiracy of Truths.
Classic, restrained Saturday-morning-cartoon content on every axis
except one: the show's central promise (getting the six kids home) is
never fulfilled, since the series was cancelled before a planned
resolution could air. Episode-level conflicts against Venger resolve
cleanly each time, but that core injustice never does, driving Narrative
Acceptance of Injustice to 2 while every other axis stays low. Title
carries a "(1983)" suffix to distinguish it from the 2023 film already
in the catalog.

Catalog now stands at 98 works.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R98"/>
+  <dimension ref="A1:R99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2271,17 +2271,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Willow</t>
+          <t>Dungeons &amp; Dragons (1983)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ron Howard / George Lucas</t>
+          <t>Marvel Productions / TSR</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2298,31 +2298,36 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O19" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="P19" t="n">
-        <v>2.85</v>
+        <v>2.7375</v>
       </c>
       <c r="Q19" t="n">
         <v>2</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1983 animated series</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -2336,17 +2341,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The Chronicles of Narnia</t>
+          <t>Willow</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Novels / Films</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>C. S. Lewis</t>
+          <t>Ron Howard / George Lucas</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2360,7 +2365,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -2378,13 +2383,13 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="P20" t="n">
-        <v>2.9625</v>
+        <v>2.85</v>
       </c>
       <c r="Q20" t="n">
         <v>2</v>
@@ -2401,17 +2406,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>The Legend of Zelda</t>
+          <t>The Chronicles of Narnia</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels / Films</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Nintendo</t>
+          <t>C. S. Lewis</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2428,7 +2433,7 @@
         <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -2437,7 +2442,7 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
@@ -2454,7 +2459,6 @@
       <c r="Q21" t="n">
         <v>2</v>
       </c>
-      <c r="R21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2467,17 +2471,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DanMachi</t>
+          <t>The Legend of Zelda</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Light Novels / Anime / Manga</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fujino Ōmori</t>
+          <t>Nintendo</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2491,19 +2495,19 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
         <v>0</v>
@@ -2520,29 +2524,30 @@
       <c r="Q22" t="n">
         <v>2</v>
       </c>
+      <c r="R22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Moderately Bright Fantasy</t>
+          <t>Bright Fantasy</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mushishi</t>
+          <t>DanMachi</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Anime / Manga</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Yuki Urushibara</t>
+          <t>Fujino Ōmori</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2552,43 +2557,38 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O23" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="P23" t="n">
-        <v>3.075</v>
+        <v>2.9625</v>
       </c>
       <c r="Q23" t="n">
-        <v>3</v>
-      </c>
-      <c r="R23" s="5" t="inlineStr">
-        <is>
-          <t>Tier v1 era 2</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -2602,17 +2602,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A Choir of Lies</t>
+          <t>Mushishi</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Alexandra Rowland</t>
+          <t>Yuki Urushibara</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2629,19 +2629,19 @@
         <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N24" t="n">
         <v>1</v>
@@ -2655,6 +2655,11 @@
       <c r="Q24" t="n">
         <v>3</v>
       </c>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>Tier v1 era 2</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2667,17 +2672,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Neverwinter Nights</t>
+          <t>A Choir of Lies</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Alexandra Rowland</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2687,7 +2692,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -2720,11 +2725,6 @@
       <c r="Q25" t="n">
         <v>3</v>
       </c>
-      <c r="R25" s="5" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2737,17 +2737,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dungeon Meshi</t>
+          <t>Neverwinter Nights</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Ryoko Kui</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2764,10 +2764,10 @@
         <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K26" t="n">
         <v>1</v>
@@ -2779,18 +2779,22 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O26" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="P26" t="n">
-        <v>3.3</v>
+        <v>3.075</v>
       </c>
       <c r="Q26" t="n">
         <v>3</v>
       </c>
-      <c r="R26" s="5" t="n"/>
+      <c r="R26" s="5" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2803,17 +2807,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Cormyr</t>
+          <t>Dungeon Meshi</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ed Greenwood / Jeff Grubb</t>
+          <t>Ryoko Kui</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2833,13 +2837,13 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
@@ -2856,6 +2860,7 @@
       <c r="Q27" t="n">
         <v>3</v>
       </c>
+      <c r="R27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2868,17 +2873,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Maleficent</t>
+          <t>Cormyr</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Robert Stromberg</t>
+          <t>Ed Greenwood / Jeff Grubb</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2892,10 +2897,10 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="n">
         <v>1</v>
@@ -2904,10 +2909,10 @@
         <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N28" t="n">
         <v>2</v>
@@ -2933,17 +2938,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Baldur's Gate I</t>
+          <t>Maleficent</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Robert Stromberg</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2957,10 +2962,10 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
         <v>1</v>
@@ -2972,24 +2977,19 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O29" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="P29" t="n">
-        <v>3.4125</v>
+        <v>3.3</v>
       </c>
       <c r="Q29" t="n">
         <v>3</v>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="30">
@@ -3003,17 +3003,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Final Fantasy IV</t>
+          <t>Baldur's Gate I</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3027,36 +3027,40 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K30" t="n">
         <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O30" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="P30" t="n">
-        <v>3.525</v>
+        <v>3.4125</v>
       </c>
       <c r="Q30" t="n">
         <v>3</v>
       </c>
-      <c r="R30" s="5" t="n"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3069,17 +3073,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>The Hobbit</t>
+          <t>Final Fantasy IV</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3093,10 +3097,10 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -3108,20 +3112,21 @@
         <v>2</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O31" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="P31" t="n">
-        <v>3.6375</v>
+        <v>3.525</v>
       </c>
       <c r="Q31" t="n">
         <v>3</v>
       </c>
+      <c r="R31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -3134,17 +3139,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Spirited Away</t>
+          <t>The Hobbit</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3158,7 +3163,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" t="n">
         <v>1</v>
@@ -3167,13 +3172,13 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
         <v>2</v>
@@ -3199,7 +3204,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Howl's Moving Castle</t>
+          <t>Spirited Away</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3223,7 +3228,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
         <v>1</v>
@@ -3232,13 +3237,13 @@
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N33" t="n">
         <v>2</v>
@@ -3264,17 +3269,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Discworld</t>
+          <t>Howl's Moving Castle</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Novels / Games / Comics</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Terry Pratchett</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3284,7 +3289,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H34" t="n">
@@ -3294,33 +3299,28 @@
         <v>1</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
         <v>1</v>
       </c>
       <c r="L34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O34" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="P34" t="n">
-        <v>3.75</v>
+        <v>3.6375</v>
       </c>
       <c r="Q34" t="n">
         <v>3</v>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>Tier v1 era 4</t>
-        </is>
       </c>
     </row>
     <row r="35">
@@ -3334,17 +3334,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>The Lord of the Rings</t>
+          <t>Discworld</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Novels / Films</t>
+          <t>Novels / Games / Comics</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Terry Pratchett</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3354,38 +3354,43 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I35" t="n">
         <v>1</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K35" t="n">
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O35" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="P35" t="n">
-        <v>3.975</v>
+        <v>3.75</v>
       </c>
       <c r="Q35" t="n">
         <v>3</v>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Tier v1 era 4</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -3399,17 +3404,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Frieren: Beyond Journey's End</t>
+          <t>The Lord of the Rings</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novels / Films</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Kanehito Yamada / Tsukasa Abe</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3419,7 +3424,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H36" t="n">
@@ -3432,13 +3437,13 @@
         <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N36" t="n">
         <v>2</v>
@@ -3464,17 +3469,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Black Clover</t>
+          <t>Frieren: Beyond Journey's End</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Manga / Anime / Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Yūki Tabata</t>
+          <t>Kanehito Yamada / Tsukasa Abe</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3484,11 +3489,11 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I37" t="n">
         <v>1</v>
@@ -3497,13 +3502,13 @@
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N37" t="n">
         <v>2</v>
@@ -3529,17 +3534,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Record of Lodoss War</t>
+          <t>Black Clover</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Novels / Anime</t>
+          <t>Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Ryo Mizuno</t>
+          <t>Yūki Tabata</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3559,16 +3564,16 @@
         <v>1</v>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N38" t="n">
         <v>2</v>
@@ -3594,17 +3599,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Final Fantasy II</t>
+          <t>Record of Lodoss War</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels / Anime</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Ryo Mizuno</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3647,11 +3652,6 @@
       <c r="Q39" t="n">
         <v>3</v>
       </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3664,17 +3664,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Nausicaä of the Valley of the Wind</t>
+          <t>Final Fantasy II</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3688,7 +3688,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I40" t="n">
         <v>1</v>
@@ -3700,10 +3700,10 @@
         <v>1</v>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N40" t="n">
         <v>2</v>
@@ -3717,29 +3717,34 @@
       <c r="Q40" t="n">
         <v>3</v>
       </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Fantasy in Gray Tones</t>
+          <t>Moderately Bright Fantasy</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>The NeverEnding Story</t>
+          <t>Nausicaä of the Valley of the Wind</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Michael Ende</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3762,25 +3767,25 @@
         <v>1</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O41" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="P41" t="n">
-        <v>4.2</v>
+        <v>3.975</v>
       </c>
       <c r="Q41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
@@ -3794,17 +3799,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Witch Hat Atelier</t>
+          <t>The NeverEnding Story</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Kamome Shirahama</t>
+          <t>Michael Ende</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3818,31 +3823,31 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I42" t="n">
         <v>1</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
         <v>2</v>
       </c>
       <c r="M42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O42" t="n">
-        <v>1.25</v>
+        <v>1.2</v>
       </c>
       <c r="P42" t="n">
-        <v>4.3125</v>
+        <v>4.2</v>
       </c>
       <c r="Q42" t="n">
         <v>4</v>
@@ -3859,17 +3864,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Baldur's Gate II: Shadows of Amn</t>
+          <t>Witch Hat Atelier</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Kamome Shirahama</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3889,13 +3894,13 @@
         <v>1</v>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K43" t="n">
         <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M43" t="n">
         <v>1</v>
@@ -3911,11 +3916,6 @@
       </c>
       <c r="Q43" t="n">
         <v>4</v>
-      </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="44">
@@ -3929,17 +3929,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Disenchantment</t>
+          <t>Baldur's Gate II: Shadows of Amn</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Matt Groening</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3981,6 +3981,11 @@
       </c>
       <c r="Q44" t="n">
         <v>4</v>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -3994,17 +3999,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Harry Potter and the Prisoner of Azkaban</t>
+          <t>Disenchantment</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Matt Groening</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4030,19 +4035,19 @@
         <v>2</v>
       </c>
       <c r="L45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O45" t="n">
-        <v>1.35</v>
+        <v>1.25</v>
       </c>
       <c r="P45" t="n">
-        <v>4.5375</v>
+        <v>4.3125</v>
       </c>
       <c r="Q45" t="n">
         <v>4</v>
@@ -4059,17 +4064,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Grimgar: Ashes and Illusions</t>
+          <t>Harry Potter and the Prisoner of Azkaban</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Light Novels / Anime</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Ao Jyumonji</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4083,7 +4088,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I46" t="n">
         <v>1</v>
@@ -4092,30 +4097,25 @@
         <v>1</v>
       </c>
       <c r="K46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L46" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O46" t="n">
-        <v>1.4</v>
+        <v>1.35</v>
       </c>
       <c r="P46" t="n">
-        <v>4.65</v>
+        <v>4.5375</v>
       </c>
       <c r="Q46" t="n">
         <v>4</v>
-      </c>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>re-audited: held after a Narrative Acceptance of Injustice / Redemption Difficulty trade that cancelled out</t>
-        </is>
       </c>
     </row>
     <row r="47">
@@ -4129,17 +4129,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Avatar: The Last Airbender</t>
+          <t>Grimgar: Ashes and Illusions</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Light Novels / Anime</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>Ao Jyumonji</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -4149,7 +4149,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H47" t="n">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>Tier v1 era 3</t>
+          <t>re-audited: held after a Narrative Acceptance of Injustice / Redemption Difficulty trade that cancelled out</t>
         </is>
       </c>
     </row>
@@ -4199,17 +4199,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Earthsea</t>
+          <t>Avatar: The Last Airbender</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Ursula K. Le Guin</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H48" t="n">
@@ -4229,10 +4229,10 @@
         <v>1</v>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L48" t="n">
         <v>2</v>
@@ -4251,6 +4251,11 @@
       </c>
       <c r="Q48" t="n">
         <v>4</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Tier v1 era 3</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -4264,17 +4269,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Final Fantasy XII</t>
+          <t>Earthsea</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Ursula K. Le Guin</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -4288,22 +4293,22 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I49" t="n">
         <v>1</v>
       </c>
       <c r="J49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K49" t="n">
         <v>2</v>
       </c>
       <c r="L49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N49" t="n">
         <v>2</v>
@@ -4316,11 +4321,6 @@
       </c>
       <c r="Q49" t="n">
         <v>4</v>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
-        </is>
       </c>
     </row>
     <row r="50">
@@ -4334,17 +4334,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>The Legend of Vox Machina</t>
+          <t>Final Fantasy XII</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Critical Role</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4367,25 +4367,30 @@
         <v>1</v>
       </c>
       <c r="K50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O50" t="n">
-        <v>1.35</v>
+        <v>1.4</v>
       </c>
       <c r="P50" t="n">
-        <v>4.8375</v>
+        <v>4.65</v>
       </c>
       <c r="Q50" t="n">
         <v>4</v>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>split from bundled 'Final Fantasy I, II &amp; XII'</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -4399,17 +4404,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist: Brotherhood</t>
+          <t>The Legend of Vox Machina</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa</t>
+          <t>Critical Role</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4432,7 +4437,7 @@
         <v>1</v>
       </c>
       <c r="K51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L51" t="n">
         <v>2</v>
@@ -4444,10 +4449,10 @@
         <v>3</v>
       </c>
       <c r="O51" t="n">
-        <v>1.5</v>
+        <v>1.35</v>
       </c>
       <c r="P51" t="n">
-        <v>4.875</v>
+        <v>4.8375</v>
       </c>
       <c r="Q51" t="n">
         <v>4</v>
@@ -4464,17 +4469,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>The Boy and the Heron</t>
+          <t>Fullmetal Alchemist: Brotherhood</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Hiromu Arakawa</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4488,22 +4493,22 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N52" t="n">
         <v>3</v>
@@ -4529,17 +4534,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Final Fantasy IX</t>
+          <t>The Boy and the Heron</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4553,19 +4558,19 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
       </c>
       <c r="K53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M53" t="n">
         <v>2</v>
@@ -4594,17 +4599,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Ranking of Kings</t>
+          <t>Final Fantasy IX</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Sōsuke Tōka</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4618,19 +4623,19 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I54" t="n">
         <v>1</v>
       </c>
       <c r="J54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K54" t="n">
         <v>2</v>
       </c>
       <c r="L54" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M54" t="n">
         <v>2</v>
@@ -4646,11 +4651,6 @@
       </c>
       <c r="Q54" t="n">
         <v>4</v>
-      </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="55">
@@ -4664,17 +4664,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Adventure Time</t>
+          <t>Ranking of Kings</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>TV / Comics</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Pendleton Ward</t>
+          <t>Sōsuke Tōka</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4697,25 +4697,30 @@
         <v>1</v>
       </c>
       <c r="K55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L55" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M55" t="n">
         <v>2</v>
       </c>
       <c r="N55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O55" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="P55" t="n">
-        <v>4.9875</v>
+        <v>4.875</v>
       </c>
       <c r="Q55" t="n">
         <v>4</v>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>rescored three times after user corrections on plot details; re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -4729,17 +4734,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Star vs. the Forces of Evil</t>
+          <t>Adventure Time</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>TV, Comics</t>
+          <t>TV / Comics</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Daron Nefcy</t>
+          <t>Pendleton Ward</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4753,7 +4758,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I56" t="n">
         <v>1</v>
@@ -4762,7 +4767,7 @@
         <v>1</v>
       </c>
       <c r="K56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L56" t="n">
         <v>2</v>
@@ -4782,34 +4787,29 @@
       <c r="Q56" t="n">
         <v>4</v>
       </c>
-      <c r="R56" t="inlineStr">
-        <is>
-          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Gloomy Fantasy</t>
+          <t>Fantasy in Gray Tones</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Tales from Earthsea</t>
+          <t>Star vs. the Forces of Evil</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV, Comics</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Gorō Miyazaki</t>
+          <t>Daron Nefcy</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4823,7 +4823,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I57" t="n">
         <v>1</v>
@@ -4832,7 +4832,7 @@
         <v>1</v>
       </c>
       <c r="K57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L57" t="n">
         <v>2</v>
@@ -4841,20 +4841,20 @@
         <v>2</v>
       </c>
       <c r="N57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O57" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="P57" t="n">
-        <v>5.2125</v>
+        <v>4.9875</v>
       </c>
       <c r="Q57" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>re-audited: Explicit Darkness raised for the patricide opening and Therru's sustained visible abuse scarring</t>
+          <t>re-audited: SD/LH had been inflated from the same single finale fact as NAI</t>
         </is>
       </c>
     </row>
@@ -4869,17 +4869,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Dragonlance</t>
+          <t>Tales from Earthsea</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Novels / Games</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Margaret Weis / Tracy Hickman</t>
+          <t>Studio Ghibli / Gorō Miyazaki</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4902,13 +4902,13 @@
         <v>1</v>
       </c>
       <c r="K58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L58" t="n">
         <v>2</v>
       </c>
       <c r="M58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N58" t="n">
         <v>3</v>
@@ -4921,6 +4921,11 @@
       </c>
       <c r="Q58" t="n">
         <v>5</v>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>re-audited: Explicit Darkness raised for the patricide opening and Therru's sustained visible abuse scarring</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -4934,17 +4939,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Harry Potter and the Goblet of Fire</t>
+          <t>Dragonlance</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Novels / Games</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Margaret Weis / Tracy Hickman</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4958,22 +4963,22 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
       </c>
       <c r="J59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K59" t="n">
         <v>2</v>
       </c>
       <c r="L59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N59" t="n">
         <v>3</v>
@@ -4999,17 +5004,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Elantris</t>
+          <t>Harry Potter and the Goblet of Fire</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5023,22 +5028,22 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I60" t="n">
         <v>1</v>
       </c>
       <c r="J60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K60" t="n">
         <v>2</v>
       </c>
       <c r="L60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N60" t="n">
         <v>3</v>
@@ -5064,17 +5069,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Baldur's Gate III</t>
+          <t>Elantris</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>BioWare / Black Isle / Larian</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5088,13 +5093,13 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I61" t="n">
         <v>1</v>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K61" t="n">
         <v>2</v>
@@ -5116,11 +5121,6 @@
       </c>
       <c r="Q61" t="n">
         <v>5</v>
-      </c>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
-        </is>
       </c>
     </row>
     <row r="62">
@@ -5134,17 +5134,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V: Skyrim</t>
+          <t>Baldur's Gate III</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Bethesda Game Studios</t>
+          <t>BioWare / Black Isle / Larian</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5158,7 +5158,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I62" t="n">
         <v>1</v>
@@ -5170,22 +5170,27 @@
         <v>2</v>
       </c>
       <c r="L62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O62" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="P62" t="n">
-        <v>5.325</v>
+        <v>5.2125</v>
       </c>
       <c r="Q62" t="n">
         <v>5</v>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>split from bundled 'Neverwinter Nights &amp; Baldur's Gate I-III'</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -5199,17 +5204,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The Silmarillion &amp; Great Tales</t>
+          <t>The Elder Scrolls V: Skyrim</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Books</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>J. R. R. Tolkien</t>
+          <t>Bethesda Game Studios</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5235,10 +5240,10 @@
         <v>2</v>
       </c>
       <c r="L63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N63" t="n">
         <v>2</v>
@@ -5264,17 +5269,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The Legend of Korra</t>
+          <t>The Silmarillion &amp; Great Tales</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>TV / Novels / Comics</t>
+          <t>Books</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Michael Dante DiMartino / Bryan Konietzko</t>
+          <t>J. R. R. Tolkien</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5284,17 +5289,17 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H64" t="n">
         <v>2</v>
       </c>
       <c r="I64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K64" t="n">
         <v>2</v>
@@ -5316,11 +5321,6 @@
       </c>
       <c r="Q64" t="n">
         <v>5</v>
-      </c>
-      <c r="R64" t="inlineStr">
-        <is>
-          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
-        </is>
       </c>
     </row>
     <row r="65">
@@ -5334,17 +5334,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Princess Mononoke</t>
+          <t>The Legend of Korra</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>TV / Novels / Comics</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Studio Ghibli / Hayao Miyazaki</t>
+          <t>Michael Dante DiMartino / Bryan Konietzko</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H65" t="n">
@@ -5364,28 +5364,33 @@
         <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O65" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="P65" t="n">
-        <v>5.55</v>
+        <v>5.325</v>
       </c>
       <c r="Q65" t="n">
         <v>5</v>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>re-audited: Explicit Darkness reverted to Avatar-level (2) — dark content is concentrated in a few arc-climax beats across 4 books, not frequent the way tier-5 multi-volume sagas are</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -5399,17 +5404,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Dark Elf / Drizzt</t>
+          <t>Princess Mononoke</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>R. A. Salvatore</t>
+          <t>Studio Ghibli / Hayao Miyazaki</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5426,16 +5431,16 @@
         <v>2</v>
       </c>
       <c r="I66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M66" t="n">
         <v>2</v>
@@ -5451,11 +5456,6 @@
       </c>
       <c r="Q66" t="n">
         <v>5</v>
-      </c>
-      <c r="R66" t="inlineStr">
-        <is>
-          <t>re-audited for v2 axis calibration</t>
-        </is>
       </c>
     </row>
     <row r="67">
@@ -5469,17 +5469,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The Wheel of Time</t>
+          <t>The Dark Elf / Drizzt</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Robert Jordan / Brandon Sanderson</t>
+          <t>R. A. Salvatore</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5539,17 +5539,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Final Fantasy VI</t>
+          <t>The Wheel of Time</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Robert Jordan / Brandon Sanderson</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5563,13 +5563,13 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I68" t="n">
         <v>1</v>
       </c>
       <c r="J68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K68" t="n">
         <v>2</v>
@@ -5578,19 +5578,24 @@
         <v>2</v>
       </c>
       <c r="M68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O68" t="n">
-        <v>1.85</v>
+        <v>1.8</v>
       </c>
       <c r="P68" t="n">
-        <v>5.6625</v>
+        <v>5.55</v>
       </c>
       <c r="Q68" t="n">
         <v>5</v>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>re-audited for v2 axis calibration</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -5604,17 +5609,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The Kingkiller Chronicle</t>
+          <t>Final Fantasy VI</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Patrick Rothfuss</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5628,13 +5633,13 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K69" t="n">
         <v>2</v>
@@ -5643,7 +5648,7 @@
         <v>2</v>
       </c>
       <c r="M69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N69" t="n">
         <v>2</v>
@@ -5656,11 +5661,6 @@
       </c>
       <c r="Q69" t="n">
         <v>5</v>
-      </c>
-      <c r="R69" t="inlineStr">
-        <is>
-          <t>re-audited: held after testing Moral Cynicism and Limited Heroism revisions, both rejected on discipline grounds</t>
-        </is>
       </c>
     </row>
     <row r="70">
@@ -5674,17 +5674,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Goblin Slayer</t>
+          <t>The Kingkiller Chronicle</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Kumo Kagyu</t>
+          <t>Patrick Rothfuss</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5704,32 +5704,32 @@
         <v>2</v>
       </c>
       <c r="J70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M70" t="n">
         <v>2</v>
       </c>
       <c r="N70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O70" t="n">
-        <v>1.9</v>
+        <v>1.85</v>
       </c>
       <c r="P70" t="n">
-        <v>5.775</v>
+        <v>5.6625</v>
       </c>
       <c r="Q70" t="n">
         <v>5</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Tier v1 era 6</t>
+          <t>re-audited: held after testing Moral Cynicism and Limited Heroism revisions, both rejected on discipline grounds</t>
         </is>
       </c>
     </row>
@@ -5744,17 +5744,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Final Fantasy X</t>
+          <t>Goblin Slayer</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Light Novels / Manga / Anime</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Square</t>
+          <t>Kumo Kagyu</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5768,34 +5768,39 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J71" t="n">
         <v>2</v>
       </c>
       <c r="K71" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L71" t="n">
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N71" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O71" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="P71" t="n">
-        <v>5.8875</v>
+        <v>5.775</v>
       </c>
       <c r="Q71" t="n">
         <v>5</v>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Tier v1 era 6</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -5809,17 +5814,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Final Fantasy VII</t>
+          <t>Final Fantasy X</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Video Games / Remake Project</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Square / Square Enix</t>
+          <t>Square</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5833,7 +5838,7 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I72" t="n">
         <v>1</v>
@@ -5848,7 +5853,7 @@
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N72" t="n">
         <v>3</v>
@@ -5874,17 +5879,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Harry Potter and the Order of the Phoenix</t>
+          <t>Final Fantasy VII</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Video Games / Remake Project</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square / Square Enix</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5901,13 +5906,13 @@
         <v>2</v>
       </c>
       <c r="I73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J73" t="n">
         <v>2</v>
       </c>
       <c r="K73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L73" t="n">
         <v>1</v>
@@ -5939,7 +5944,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Harry Potter and the Half-Blood Prince</t>
+          <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -5972,10 +5977,10 @@
         <v>2</v>
       </c>
       <c r="K74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M74" t="n">
         <v>2</v>
@@ -6004,17 +6009,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Final Fantasy XV</t>
+          <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6028,22 +6033,22 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J75" t="n">
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L75" t="n">
         <v>2</v>
       </c>
       <c r="M75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N75" t="n">
         <v>3</v>
@@ -6060,26 +6065,26 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Dark Fantasy</t>
+          <t>Gloomy Fantasy</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Clevatess</t>
+          <t>Final Fantasy XV</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Yūji Iwahara</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6093,10 +6098,10 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J76" t="n">
         <v>2</v>
@@ -6105,27 +6110,22 @@
         <v>2</v>
       </c>
       <c r="L76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O76" t="n">
-        <v>2.05</v>
+        <v>1.95</v>
       </c>
       <c r="P76" t="n">
-        <v>6.1125</v>
+        <v>5.8875</v>
       </c>
       <c r="Q76" t="n">
-        <v>6</v>
-      </c>
-      <c r="R76" t="inlineStr">
-        <is>
-          <t>scored against the story as currently published/aired; ongoing/unresolved, later arcs may shift this</t>
-        </is>
+        <v>5</v>
       </c>
     </row>
     <row r="77">
@@ -6139,17 +6139,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Re:Zero − Starting Life in Another World</t>
+          <t>Clevatess</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Light Novels, Manga, Anime</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Tappei Nagatsuki</t>
+          <t>Yūji Iwahara</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6166,7 +6166,7 @@
         <v>2</v>
       </c>
       <c r="I77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J77" t="n">
         <v>2</v>
@@ -6175,7 +6175,7 @@
         <v>2</v>
       </c>
       <c r="L77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M77" t="n">
         <v>2</v>
@@ -6194,7 +6194,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>scored against the arcs most widely adapted/translated (roughly Arcs 1-6); later arcs may shift this</t>
+          <t>scored against the story as currently published/aired; ongoing/unresolved, later arcs may shift this</t>
         </is>
       </c>
     </row>
@@ -6209,17 +6209,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>The Witcher</t>
+          <t>Re:Zero − Starting Life in Another World</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Novels / Games / TV</t>
+          <t>Light Novels, Manga, Anime</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Andrzej Sapkowski</t>
+          <t>Tappei Nagatsuki</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -6236,7 +6236,7 @@
         <v>2</v>
       </c>
       <c r="I78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J78" t="n">
         <v>2</v>
@@ -6251,16 +6251,21 @@
         <v>2</v>
       </c>
       <c r="N78" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O78" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="P78" t="n">
-        <v>6.225</v>
+        <v>6.1125</v>
       </c>
       <c r="Q78" t="n">
         <v>6</v>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>scored against the arcs most widely adapted/translated (roughly Arcs 1-6); later arcs may shift this</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -6274,17 +6279,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Final Fantasy XIV</t>
+          <t>The Witcher</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>MMORPG</t>
+          <t>Novels / Games / TV</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Andrzej Sapkowski</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -6298,16 +6303,16 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L79" t="n">
         <v>2</v>
@@ -6339,17 +6344,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Shin Sekai Yori (From the New World)</t>
+          <t>Final Fantasy XIV</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Novel / Anime</t>
+          <t>MMORPG</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Yusuke Kishi</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6363,13 +6368,13 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K80" t="n">
         <v>3</v>
@@ -6381,21 +6386,16 @@
         <v>2</v>
       </c>
       <c r="N80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O80" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="P80" t="n">
-        <v>6.3375</v>
+        <v>6.225</v>
       </c>
       <c r="Q80" t="n">
         <v>6</v>
-      </c>
-      <c r="R80" t="inlineStr">
-        <is>
-          <t>Tier v1 era 8</t>
-        </is>
       </c>
     </row>
     <row r="81">
@@ -6409,17 +6409,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Shin Sekai Yori (From the New World)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Novel / Anime</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Akihito Tsukushi</t>
+          <t>Yusuke Kishi</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -6442,7 +6442,7 @@
         <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L81" t="n">
         <v>2</v>
@@ -6451,16 +6451,21 @@
         <v>2</v>
       </c>
       <c r="N81" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O81" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="P81" t="n">
-        <v>6.45</v>
+        <v>6.3375</v>
       </c>
       <c r="Q81" t="n">
         <v>6</v>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Tier v1 era 8</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -6474,17 +6479,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Pan's Labyrinth</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Guillermo del Toro</t>
+          <t>Akihito Tsukushi</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -6507,13 +6512,13 @@
         <v>2</v>
       </c>
       <c r="K82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L82" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N82" t="n">
         <v>4</v>
@@ -6539,17 +6544,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist (2003)</t>
+          <t>Pan's Labyrinth</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Anime</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Hiromu Arakawa / Bones</t>
+          <t>Guillermo del Toro</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -6563,7 +6568,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I83" t="n">
         <v>2</v>
@@ -6572,30 +6577,25 @@
         <v>2</v>
       </c>
       <c r="K83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L83" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N83" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O83" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="P83" t="n">
-        <v>6.5625</v>
+        <v>6.45</v>
       </c>
       <c r="Q83" t="n">
         <v>6</v>
-      </c>
-      <c r="R83" t="inlineStr">
-        <is>
-          <t>Tier v1 era 5</t>
-        </is>
       </c>
     </row>
     <row r="84">
@@ -6609,17 +6609,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The Saga of Tanya the Evil</t>
+          <t>Fullmetal Alchemist (2003)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Light Novels / Manga / Anime / Film</t>
+          <t>Anime</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Carlo Zen</t>
+          <t>Hiromu Arakawa / Bones</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -6633,13 +6633,13 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I84" t="n">
         <v>2</v>
       </c>
       <c r="J84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K84" t="n">
         <v>2</v>
@@ -6664,7 +6664,7 @@
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t>Tier v1 era 7</t>
+          <t>Tier v1 era 5</t>
         </is>
       </c>
     </row>
@@ -6679,17 +6679,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Claymore</t>
+          <t>The Saga of Tanya the Evil</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Manga / Anime</t>
+          <t>Light Novels / Manga / Anime / Film</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Norihiro Yagi</t>
+          <t>Carlo Zen</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6709,10 +6709,10 @@
         <v>2</v>
       </c>
       <c r="J85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L85" t="n">
         <v>2</v>
@@ -6731,6 +6731,11 @@
       </c>
       <c r="Q85" t="n">
         <v>6</v>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Tier v1 era 7</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -6744,17 +6749,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Final Fantasy XVI</t>
+          <t>Claymore</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Manga / Anime</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Square Enix</t>
+          <t>Norihiro Yagi</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -6809,17 +6814,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Harry Potter and the Deathly Hallows</t>
+          <t>Final Fantasy XVI</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Novel / Films</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Square Enix</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -6836,7 +6841,7 @@
         <v>2</v>
       </c>
       <c r="I87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J87" t="n">
         <v>2</v>
@@ -6845,7 +6850,7 @@
         <v>3</v>
       </c>
       <c r="L87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M87" t="n">
         <v>2</v>
@@ -6874,17 +6879,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Mistborn</t>
+          <t>Harry Potter and the Deathly Hallows</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Novel / Films</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6898,7 +6903,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I88" t="n">
         <v>1</v>
@@ -6910,7 +6915,7 @@
         <v>3</v>
       </c>
       <c r="L88" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M88" t="n">
         <v>2</v>
@@ -6939,17 +6944,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Märchen Crown</t>
+          <t>Mistborn</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Aka Akasaka / Aoi Kujira / Azychika</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6963,10 +6968,10 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J89" t="n">
         <v>2</v>
@@ -6981,21 +6986,16 @@
         <v>2</v>
       </c>
       <c r="N89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O89" t="n">
-        <v>2.35</v>
+        <v>2.25</v>
       </c>
       <c r="P89" t="n">
-        <v>6.7875</v>
+        <v>6.5625</v>
       </c>
       <c r="Q89" t="n">
         <v>6</v>
-      </c>
-      <c r="R89" t="inlineStr">
-        <is>
-          <t>ongoing/unresolved as of ch. 47 (Jul 2026); low-mid confidence given thin reception in most languages researched</t>
-        </is>
       </c>
     </row>
     <row r="90">
@@ -7009,17 +7009,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>The Stormlight Archive</t>
+          <t>Märchen Crown</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Brandon Sanderson</t>
+          <t>Aka Akasaka / Aoi Kujira / Azychika</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -7045,46 +7045,51 @@
         <v>3</v>
       </c>
       <c r="L90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M90" t="n">
         <v>2</v>
       </c>
       <c r="N90" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O90" t="n">
-        <v>2.4</v>
+        <v>2.35</v>
       </c>
       <c r="P90" t="n">
-        <v>6.9</v>
+        <v>6.7875</v>
       </c>
       <c r="Q90" t="n">
         <v>6</v>
       </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>ongoing/unresolved as of ch. 47 (Jul 2026); low-mid confidence given thin reception in most languages researched</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Extreme Dark Fantasy</t>
+          <t>Dark Fantasy</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Attack on Titan</t>
+          <t>The Stormlight Archive</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Manga, Anime</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Hajime Isayama</t>
+          <t>Brandon Sanderson</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -7098,13 +7103,13 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I91" t="n">
         <v>2</v>
       </c>
       <c r="J91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K91" t="n">
         <v>3</v>
@@ -7116,40 +7121,40 @@
         <v>2</v>
       </c>
       <c r="N91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O91" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="P91" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="Q91" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Grimdark</t>
+          <t>Extreme Dark Fantasy</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>Attack on Titan</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Manga, Anime, Films</t>
+          <t>Manga, Anime</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Kentaro Miura</t>
+          <t>Hajime Isayama</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -7166,36 +7171,31 @@
         <v>3</v>
       </c>
       <c r="I92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J92" t="n">
         <v>3</v>
       </c>
       <c r="K92" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L92" t="n">
         <v>3</v>
       </c>
       <c r="M92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N92" t="n">
         <v>4</v>
       </c>
       <c r="O92" t="n">
-        <v>2.95</v>
+        <v>2.8</v>
       </c>
       <c r="P92" t="n">
-        <v>8.137499999999999</v>
+        <v>7.8</v>
       </c>
       <c r="Q92" t="n">
-        <v>8</v>
-      </c>
-      <c r="R92" t="inlineStr">
-        <is>
-          <t>re-audited: no documented reasoning survived from the original score; Limited Heroism and Narrative Acceptance of Injustice revised up on distinct evidence, Structural Corruption held at 2 after checking against A Song of Ice and Fire's multi-institutional bar</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="93">
@@ -7209,17 +7209,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Dark Souls I–III</t>
+          <t>Berserk</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Video Games</t>
+          <t>Manga, Anime, Films</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki</t>
+          <t>Kentaro Miura</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -7242,7 +7242,7 @@
         <v>3</v>
       </c>
       <c r="K93" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L93" t="n">
         <v>3</v>
@@ -7251,20 +7251,20 @@
         <v>3</v>
       </c>
       <c r="N93" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O93" t="n">
-        <v>3</v>
+        <v>2.95</v>
       </c>
       <c r="P93" t="n">
-        <v>8.25</v>
+        <v>8.137499999999999</v>
       </c>
       <c r="Q93" t="n">
         <v>8</v>
       </c>
       <c r="R93" t="inlineStr">
         <is>
-          <t>re-audited: previously flagged inconsistency vs. Elden Ring, resolved</t>
+          <t>re-audited: no documented reasoning survived from the original score; Limited Heroism and Narrative Acceptance of Injustice revised up on distinct evidence, Structural Corruption held at 2 after checking against A Song of Ice and Fire's multi-institutional bar</t>
         </is>
       </c>
     </row>
@@ -7279,17 +7279,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>A Song of Ice and Fire</t>
+          <t>Dark Souls I–III</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Novels / TV</t>
+          <t>Video Games</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>George R. R. Martin</t>
+          <t>FromSoftware / Hidetaka Miyazaki</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -7321,16 +7321,21 @@
         <v>3</v>
       </c>
       <c r="N94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O94" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="P94" t="n">
-        <v>8.475</v>
+        <v>8.25</v>
       </c>
       <c r="Q94" t="n">
         <v>8</v>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>re-audited: previously flagged inconsistency vs. Elden Ring, resolved</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -7344,17 +7349,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Elden Ring</t>
+          <t>A Song of Ice and Fire</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Video Game</t>
+          <t>Novels / TV</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
+          <t>George R. R. Martin</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -7368,31 +7373,31 @@
         </is>
       </c>
       <c r="H95" t="n">
+        <v>3</v>
+      </c>
+      <c r="I95" t="n">
+        <v>3</v>
+      </c>
+      <c r="J95" t="n">
+        <v>3</v>
+      </c>
+      <c r="K95" t="n">
+        <v>3</v>
+      </c>
+      <c r="L95" t="n">
+        <v>3</v>
+      </c>
+      <c r="M95" t="n">
+        <v>3</v>
+      </c>
+      <c r="N95" t="n">
         <v>4</v>
       </c>
-      <c r="I95" t="n">
-        <v>3</v>
-      </c>
-      <c r="J95" t="n">
-        <v>3</v>
-      </c>
-      <c r="K95" t="n">
-        <v>3</v>
-      </c>
-      <c r="L95" t="n">
-        <v>3</v>
-      </c>
-      <c r="M95" t="n">
-        <v>3</v>
-      </c>
-      <c r="N95" t="n">
-        <v>3</v>
-      </c>
       <c r="O95" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="P95" t="n">
-        <v>8.5875</v>
+        <v>8.475</v>
       </c>
       <c r="Q95" t="n">
         <v>8</v>
@@ -7409,17 +7414,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Fire Punch</t>
+          <t>Elden Ring</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Video Game</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Tatsuki Fujimoto</t>
+          <t>FromSoftware / Hidetaka Miyazaki / George R. R. Martin</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -7433,13 +7438,13 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I96" t="n">
         <v>3</v>
       </c>
       <c r="J96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K96" t="n">
         <v>3</v>
@@ -7451,13 +7456,13 @@
         <v>3</v>
       </c>
       <c r="N96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O96" t="n">
-        <v>3.25</v>
+        <v>3.15</v>
       </c>
       <c r="P96" t="n">
-        <v>8.8125</v>
+        <v>8.5875</v>
       </c>
       <c r="Q96" t="n">
         <v>8</v>
@@ -7465,26 +7470,26 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Extreme Grimdark</t>
+          <t>Grimdark</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>The First Law</t>
+          <t>Fire Punch</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Novels</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Joe Abercrombie</t>
+          <t>Tatsuki Fujimoto</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -7498,16 +7503,16 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J97" t="n">
         <v>4</v>
       </c>
       <c r="K97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L97" t="n">
         <v>3</v>
@@ -7519,37 +7524,37 @@
         <v>4</v>
       </c>
       <c r="O97" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="P97" t="n">
-        <v>9.824999999999999</v>
+        <v>8.8125</v>
       </c>
       <c r="Q97" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Very Extreme Grimdark</t>
+          <t>Extreme Grimdark</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Warhammer 40,000</t>
+          <t>The First Law</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Tabletop / Novels / Games / Animation</t>
+          <t>Novels</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Joe Abercrombie</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -7575,21 +7580,86 @@
         <v>4</v>
       </c>
       <c r="L98" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M98" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N98" t="n">
         <v>4</v>
       </c>
       <c r="O98" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P98" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>10</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Very Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Warhammer 40,000</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Tabletop / Novels / Games / Animation</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Games Workshop</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H99" t="n">
         <v>4</v>
       </c>
-      <c r="P98" t="n">
+      <c r="I99" t="n">
+        <v>4</v>
+      </c>
+      <c r="J99" t="n">
+        <v>4</v>
+      </c>
+      <c r="K99" t="n">
+        <v>4</v>
+      </c>
+      <c r="L99" t="n">
+        <v>4</v>
+      </c>
+      <c r="M99" t="n">
+        <v>4</v>
+      </c>
+      <c r="N99" t="n">
+        <v>4</v>
+      </c>
+      <c r="O99" t="n">
+        <v>4</v>
+      </c>
+      <c r="P99" t="n">
         <v>10.5</v>
       </c>
-      <c r="Q98" t="n">
+      <c r="Q99" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7652,7 +7722,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -7762,7 +7832,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total scored: 97 of 97 works in the full catalog.</t>
+          <t>Total scored: 98 of 98 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-audit The Nightmare Before Christmas again: minor Moral Cynicism refinement
User asked directly whether "Bright Fantasy" (tier 2's post-relabel name)
is really the right fit. Tested pushing Redemption Difficulty and
Narrative Acceptance of Injustice up (Santa's real endangerment, the
traumatized children's unaddressed fate) -- would have crossed into
tier 3 -- and rejected both: this film is the specific citation
CRITERIA_THEORY.md uses to explain why Explicit Darkness is allowed to
diverge from the other six criteria, so a low structural profile with
high Explicit Darkness is its intended shape, not an inconsistency.

One smaller refinement applied: Moral Cynicism 0->1, since Sally's
warnings against Jack's plan are repeatedly dismissed until vindicated.
Tier 2 unchanged, score 2.5125 -> 2.85, now tied with Willow instead of
Legend.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -2009,17 +2009,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>The Nightmare Before Christmas</t>
+          <t>Harry Potter and the Chamber of Secrets</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Film</t>
+          <t>Novel / Film</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tim Burton / Henry Selick</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2042,26 +2042,27 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O15" t="n">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="P15" t="n">
-        <v>2.5125</v>
+        <v>2.625</v>
       </c>
       <c r="Q15" t="n">
         <v>2</v>
       </c>
+      <c r="R15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2074,17 +2075,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Harry Potter and the Chamber of Secrets</t>
+          <t>The Little Prince</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Novel / Film</t>
+          <t>Book</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>J. K. Rowling</t>
+          <t>Antoine de Saint-Exupéry</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2098,22 +2099,22 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>2</v>
@@ -2127,7 +2128,6 @@
       <c r="Q16" t="n">
         <v>2</v>
       </c>
-      <c r="R16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2140,17 +2140,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The Little Prince</t>
+          <t>A Conspiracy of Truths</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Book</t>
+          <t>Novel</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Antoine de Saint-Exupéry</t>
+          <t>Alexandra Rowland</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -2173,7 +2173,7 @@
         <v>1</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -2182,17 +2182,18 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O17" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="P17" t="n">
-        <v>2.625</v>
+        <v>2.7375</v>
       </c>
       <c r="Q17" t="n">
         <v>2</v>
       </c>
+      <c r="R17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2205,17 +2206,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A Conspiracy of Truths</t>
+          <t>Dungeons &amp; Dragons (1983)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Alexandra Rowland</t>
+          <t>Marvel Productions / TSR</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2225,26 +2226,26 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N18" t="n">
         <v>1</v>
@@ -2258,7 +2259,11 @@
       <c r="Q18" t="n">
         <v>2</v>
       </c>
-      <c r="R18" s="5" t="n"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1983 animated series</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2271,17 +2276,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dungeons &amp; Dragons (1983)</t>
+          <t>Willow</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Marvel Productions / TSR</t>
+          <t>Ron Howard / George Lucas</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2298,36 +2303,31 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O19" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="P19" t="n">
-        <v>2.7375</v>
+        <v>2.85</v>
       </c>
       <c r="Q19" t="n">
         <v>2</v>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>1983 animated series</t>
-        </is>
       </c>
     </row>
     <row r="20">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Willow</t>
+          <t>The Nightmare Before Christmas</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Ron Howard / George Lucas</t>
+          <t>Tim Burton / Henry Selick</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2371,10 +2371,10 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -2393,6 +2393,11 @@
       </c>
       <c r="Q20" t="n">
         <v>2</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>re-audited again: Moral Cynicism revised 0-&gt;1 for Sally's warnings being repeatedly dismissed until vindicated</t>
+        </is>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Note the HBO TV adaptation on the Dunk & Egg entry
Season 1 (The Hedge Knight) aired Jan-Feb 2026 as a faithful
adaptation per the showrunner's own stated approach, so it's folded
into the existing entry's medium rather than rescored separately.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1017,7 +1017,7 @@
     <t xml:space="preserve">A Knight of the Seven Kingdoms (Dunk &amp; Egg)</t>
   </si>
   <si>
-    <t xml:space="preserve">Novellas</t>
+    <t xml:space="preserve">Novellas, TV series</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -7244,7 +7244,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="n">
         <v>7</v>
       </c>
@@ -7297,7 +7297,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="n">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Add Once Upon a Time to tier 4
Scored the 7-season ABC series against the 7 criteria. Final Score
4.20, Tier 4 (Fantasy in Gray Tones), tying The NeverEnding Story.
Caught and corrected an initial identical-profile match against
Fullmetal Alchemist: Brotherhood during the neighbor-check pass,
landing on a genuinely differentiated shape instead.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="336">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1020,10 +1020,16 @@
     <t xml:space="preserve">Novellas, TV series</t>
   </si>
   <si>
+    <t xml:space="preserve">Once Upon a Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edward Kitsis &amp; Adam Horowitz</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 101 of 101 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 102 of 102 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1830,7 +1836,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R102"/>
+  <dimension ref="A1:R103"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7348,6 +7354,59 @@
       </c>
       <c r="Q102" s="1" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G103" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J103" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N103" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O103" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P103" s="1" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="Q103" s="1" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -7382,7 +7441,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7426,7 +7485,7 @@
         <v>84</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7497,7 +7556,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Shannara Chronicles to tier 4
Scored the 2-season MTV/Spike adaptation against the 7 criteria.
Final Score 4.875, Tier 4 (Fantasy in Gray Tones), tying Final
Fantasy IX/The Boy and the Heron/Ranking of Kings/FMA:Brotherhood via
distinct profiles. Notes the show's cancellation explicitly, since it
left the Crimson persecution thread genuinely unresolved rather than
by narrative choice.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="338">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1026,10 +1026,16 @@
     <t xml:space="preserve">Edward Kitsis &amp; Adam Horowitz</t>
   </si>
   <si>
+    <t xml:space="preserve">The Shannara Chronicles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terry Brooks</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 102 of 102 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 103 of 103 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1836,7 +1842,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R103"/>
+  <dimension ref="A1:R104"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7356,7 +7362,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="n">
         <v>4</v>
       </c>
@@ -7406,6 +7412,59 @@
         <v>4.2</v>
       </c>
       <c r="Q103" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G104" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H104" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I104" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J104" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K104" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L104" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M104" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N104" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O104" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P104" s="1" t="n">
+        <v>4.875</v>
+      </c>
+      <c r="Q104" s="1" t="n">
         <v>4</v>
       </c>
     </row>
@@ -7441,7 +7500,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7485,7 +7544,7 @@
         <v>84</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7556,7 +7615,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Dirk Gently's Holistic Detective Agency to tier 4
Scored across both Douglas Adams novels and both TV adaptations
(2010 BBC, 2016-2017 BBC America) as one entry, since the two shows
are divergent takes on the same premise rather than sequential
chapters. Final Score 4.5375, Tier 4, tying Harry Potter and the
Prisoner of Azkaban. Explicit Darkness and Structural Corruption are
set by the notably more violent 2016 adaptation (Project Blackwing,
an on-screen assassin) rather than defaulting to the gentler novels.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="340">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1032,10 +1032,16 @@
     <t xml:space="preserve">Terry Brooks</t>
   </si>
   <si>
+    <t xml:space="preserve">Dirk Gently's Holistic Detective Agency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Douglas Adams</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 103 of 103 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 104 of 104 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1842,7 +1848,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R104"/>
+  <dimension ref="A1:R105"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7415,7 +7421,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="n">
         <v>4</v>
       </c>
@@ -7465,6 +7471,59 @@
         <v>4.875</v>
       </c>
       <c r="Q104" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H105" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I105" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J105" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K105" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L105" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M105" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N105" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O105" s="1" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="P105" s="1" t="n">
+        <v>4.5375</v>
+      </c>
+      <c r="Q105" s="1" t="n">
         <v>4</v>
       </c>
     </row>
@@ -7500,7 +7559,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7544,7 +7603,7 @@
         <v>84</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7615,7 +7674,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Sandman to tier 6
Scored the complete 75-issue Vertigo comic and the Netflix adaptation
(which carries the story through the same ending) against the 7
criteria. Final Score 6.1125, Tier 6, tying Re:Zero and Clevatess via
distinct profiles. Redemption Difficulty (3) is the highest value
assigned to any tier-6 work so far, reflecting that Dream's arc costs
him his literal existence -- a specific, evidence-based outlier
rather than a default.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="343">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1038,10 +1038,19 @@
     <t xml:space="preserve">Douglas Adams</t>
   </si>
   <si>
+    <t xml:space="preserve">The Sandman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comics, TV series</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neil Gaiman</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 104 of 104 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 105 of 105 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1848,7 +1857,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R105"/>
+  <dimension ref="A1:R106"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7474,7 +7483,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="n">
         <v>4</v>
       </c>
@@ -7525,6 +7534,59 @@
       </c>
       <c r="Q105" s="1" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="E106" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H106" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I106" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J106" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K106" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L106" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="M106" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N106" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O106" s="1" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="P106" s="1" t="n">
+        <v>6.1125</v>
+      </c>
+      <c r="Q106" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -7559,7 +7621,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7625,7 +7687,7 @@
         <v>86</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7674,7 +7736,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Supernatural to tier 6
Scored the complete 15-season series against the 7 criteria. Final
Score 6.90, the new tier-6 ceiling. Structural Corruption (3) and
Moral Cynicism (3) reflect the season 11/15 revelation that God
himself orchestrated the Winchesters' suffering across the whole
series for his own entertainment -- a multi-institutional (Heaven +
Hell + God) corruption case. Caught and corrected an initial
identical-profile match against Claymore during the neighbor-check
pass.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="345">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1047,10 +1047,16 @@
     <t xml:space="preserve">Neil Gaiman</t>
   </si>
   <si>
+    <t xml:space="preserve">Supernatural</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eric Kripke</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 105 of 105 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 106 of 106 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1857,7 +1863,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R106"/>
+  <dimension ref="A1:R107"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7536,7 +7542,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="n">
         <v>6</v>
       </c>
@@ -7586,6 +7592,59 @@
         <v>6.1125</v>
       </c>
       <c r="Q106" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G107" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H107" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I107" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J107" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="K107" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L107" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M107" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N107" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O107" s="1" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P107" s="1" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="Q107" s="1" t="n">
         <v>6</v>
       </c>
     </row>
@@ -7621,7 +7680,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7687,7 +7746,7 @@
         <v>86</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7736,7 +7795,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Charmed to tier 4
Scored the original 1998-2006 series (not the 2018 reboot) against
the 7 criteria. Final Score 4.65, Tier 4, tying Earthsea/Avatar/
Final Fantasy XII/Grimgar via distinct profiles. Redemption
Difficulty and Narrative Acceptance of Injustice carry the entry's
real weight: Cole's failed redemption arc and Prue's permanent,
narratively unaddressed death in the Season 3 finale.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="347">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1053,10 +1053,16 @@
     <t xml:space="preserve">Eric Kripke</t>
   </si>
   <si>
+    <t xml:space="preserve">Charmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constance M. Burge</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 106 of 106 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 107 of 107 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1863,7 +1869,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R107"/>
+  <dimension ref="A1:R108"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7595,7 +7601,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="1" t="n">
         <v>6</v>
       </c>
@@ -7646,6 +7652,59 @@
       </c>
       <c r="Q107" s="1" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="E108" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G108" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H108" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I108" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J108" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K108" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L108" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M108" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N108" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O108" s="1" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="P108" s="1" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="Q108" s="1" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -7680,7 +7739,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7724,7 +7783,7 @@
         <v>84</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7795,7 +7854,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Dark Crystal (1982 film) to tier 4
Scored the film only (Age of Resistance is a separate queue item)
against the 7 criteria. Final Score 4.20, Tier 4, tying The
NeverEnding Story and Once Upon a Time via distinct profiles.
Structural Corruption (3) reflects that the Skeksis are Thra's only
shown ruling power and its thousand-year reign is genocide and
exploitation by design, while Limited Heroism and Moral Cynicism
both sit at the floor given the ending's unusually complete
restoration.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="349">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1059,10 +1059,16 @@
     <t xml:space="preserve">Constance M. Burge</t>
   </si>
   <si>
+    <t xml:space="preserve">The Dark Crystal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jim Henson &amp; Frank Oz</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 107 of 107 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 108 of 108 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1869,7 +1875,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R108"/>
+  <dimension ref="A1:R109"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7654,7 +7660,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="n">
         <v>4</v>
       </c>
@@ -7704,6 +7710,59 @@
         <v>4.65</v>
       </c>
       <c r="Q108" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E109" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H109" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I109" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J109" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K109" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L109" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N109" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O109" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P109" s="1" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="Q109" s="1" t="n">
         <v>4</v>
       </c>
     </row>
@@ -7739,7 +7798,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7783,7 +7842,7 @@
         <v>84</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7854,7 +7913,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Dark Crystal: Age of Resistance to tier 6
Scored the complete (cancelled after one season) 2019 Netflix
prequel against the 7 criteria. Final Score 6.7875, Tier 6, tying
Marchen Crown via a distinct profile -- notably darker than its own
parent film (Tier 4, 4.20) since the prequel's real Season 1 victory
is read against the known, doomed future the film already
establishes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="350">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1065,10 +1065,13 @@
     <t xml:space="preserve">Jim Henson &amp; Frank Oz</t>
   </si>
   <si>
+    <t xml:space="preserve">The Dark Crystal: Age of Resistance</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 108 of 108 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 109 of 109 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1875,7 +1878,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R109"/>
+  <dimension ref="A1:R110"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7713,7 +7716,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="1" t="n">
         <v>4</v>
       </c>
@@ -7764,6 +7767,59 @@
       </c>
       <c r="Q109" s="1" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H110" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I110" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J110" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K110" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L110" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M110" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="N110" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O110" s="1" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="P110" s="1" t="n">
+        <v>6.7875</v>
+      </c>
+      <c r="Q110" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -7798,7 +7854,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7864,7 +7920,7 @@
         <v>86</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7913,7 +7969,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add His Dark Materials to tier 7
Scored Philip Pullman's trilogy and its TV adaptation against the 7
criteria. Final Score 7.4625, the new tier-7 floor. Limited Heroism
and Narrative Acceptance of Injustice are both unusually high,
grounded directly in the ending's own text: Lord Asriel's crusade
against the Magisterium explicitly fails as a strategy, leaving the
institution's child-mutilation program (intercision) unresolved.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="352">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1068,10 +1068,16 @@
     <t xml:space="preserve">The Dark Crystal: Age of Resistance</t>
   </si>
   <si>
+    <t xml:space="preserve">His Dark Materials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Philip Pullman</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 109 of 109 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 110 of 110 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1878,7 +1884,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R110"/>
+  <dimension ref="A1:R111"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7769,7 +7775,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="n">
         <v>6</v>
       </c>
@@ -7820,6 +7826,59 @@
       </c>
       <c r="Q110" s="1" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H111" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I111" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="J111" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K111" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L111" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M111" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="N111" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O111" s="1" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="P111" s="1" t="n">
+        <v>7.4625</v>
+      </c>
+      <c r="Q111" s="1" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -7854,7 +7913,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7931,7 +7990,7 @@
         <v>87</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7969,7 +8028,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Dresden Files to tier 6
Scored the 18 currently-published novels (of a planned 25) and the
2007 TV adaptation against the 7 criteria. Final Score 6.1125, Tier
6, tying Re:Zero/Clevatess/The Sandman via distinct profiles. Moral
Cynicism reflects Changes' central moral compromise: Harry himself
triggers a bloodline curse wiping out the entire Red Court vampire
nation to save his daughter -- the protagonist committing a
magically genocidal act as the story's own resolution.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="354">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1074,10 +1074,16 @@
     <t xml:space="preserve">Philip Pullman</t>
   </si>
   <si>
+    <t xml:space="preserve">The Dresden Files</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jim Butcher</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 110 of 110 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 111 of 111 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1884,7 +1890,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R111"/>
+  <dimension ref="A1:R112"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7828,7 +7834,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="1" t="n">
         <v>7</v>
       </c>
@@ -7879,6 +7885,59 @@
       </c>
       <c r="Q111" s="1" t="n">
         <v>7</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H112" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I112" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J112" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K112" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L112" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M112" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N112" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O112" s="1" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="P112" s="1" t="n">
+        <v>6.1125</v>
+      </c>
+      <c r="Q112" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -7913,7 +7972,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7979,7 +8038,7 @@
         <v>86</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8028,7 +8087,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Grim Company to tier 7
Scored the complete trilogy against the 7 criteria. Final Score
7.125, the new tier-7 floor. Caught an initial identical-profile
match against Marchen Crown during the neighbor-check pass; the
correction (Redemption Difficulty 2 -> 3, grounded in Cole's
self-erosion arc and the near-total cast death by book 3) moved the
total into a new tier rather than just avoiding the collision
cosmetically.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="356">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1080,10 +1080,16 @@
     <t xml:space="preserve">Jim Butcher</t>
   </si>
   <si>
+    <t xml:space="preserve">The Grim Company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luke Scull</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 111 of 111 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 112 of 112 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1890,7 +1896,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R112"/>
+  <dimension ref="A1:R113"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7887,7 +7893,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="n">
         <v>6</v>
       </c>
@@ -7938,6 +7944,59 @@
       </c>
       <c r="Q112" s="1" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G113" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H113" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I113" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J113" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K113" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L113" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="M113" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N113" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O113" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P113" s="1" t="n">
+        <v>7.125</v>
+      </c>
+      <c r="Q113" s="1" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -7972,7 +8031,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8049,7 +8108,7 @@
         <v>87</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8087,7 +8146,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Dark Tower to tier 7
Scored the complete 8-book series against the 7 criteria. Final
Score 7.80, tying Attack on Titan and House of the Dragon via
distinct profiles. Limited Heroism and Narrative Acceptance of
Injustice carry the real bleakness: Roland reaches the Tower and
succeeds, only to be reset to the start of his quest, implying an
unresolved cycle -- while Structural Despair stops short of the
ceiling since the Tower itself is genuinely stabilized by the end.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="358">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1086,10 +1086,16 @@
     <t xml:space="preserve">Luke Scull</t>
   </si>
   <si>
+    <t xml:space="preserve">The Dark Tower</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stephen King</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 112 of 112 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 113 of 113 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1896,7 +1902,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R113"/>
+  <dimension ref="A1:R114"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7946,7 +7952,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="n">
         <v>7</v>
       </c>
@@ -7996,6 +8002,59 @@
         <v>7.125</v>
       </c>
       <c r="Q113" s="1" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H114" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I114" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="J114" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K114" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L114" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="M114" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="N114" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O114" s="1" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="P114" s="1" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Q114" s="1" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8031,7 +8090,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8108,7 +8167,7 @@
         <v>87</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8146,7 +8205,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct The Grim Company: revert to Tier 6
Prompted by a direct question about why the session's last three
additions had all landed in Tier 7. Re-audited and found the
Redemption Difficulty 2->3 revision (which moved the entry from
Tier 6 to Tier 7) was collision-motivated rather than
evidence-driven: it was made specifically to escape an exact
profile match with Marchen Crown, and neither cited piece of
evidence actually confirmed the claim RD3 requires. Reverted to
RD2, landing back at 6.7875 (Tier 6) -- an exact tie with Marchen
Crown that is itself legitimate, not a problem. His Dark Materials
and The Dark Tower were re-checked against the same standard and
hold up: their key axis values were derived from direct textual
evidence before any collision was found, not after.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -7954,10 +7954,10 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>352</v>
@@ -7987,7 +7987,7 @@
         <v>3</v>
       </c>
       <c r="L113" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M113" s="1" t="n">
         <v>2</v>
@@ -7996,16 +7996,16 @@
         <v>4</v>
       </c>
       <c r="O113" s="1" t="n">
-        <v>2.5</v>
+        <v>2.35</v>
       </c>
       <c r="P113" s="1" t="n">
-        <v>7.125</v>
+        <v>6.7875</v>
       </c>
       <c r="Q113" s="1" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="1" t="n">
         <v>7</v>
       </c>
@@ -8156,7 +8156,7 @@
         <v>86</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8167,7 +8167,7 @@
         <v>87</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Eragon (The Inheritance Cycle) to tier 5
Scored the complete 4-book main cycle plus the 2006 film against the
7 criteria. Final Score 5.2125, Tier 5. Explicitly decided to bundle
rather than split by book (unlike Harry Potter): the cycle lacks HP's
dramatic audience-shift escalation and individual-book cultural
fame, even though darkness does intensify across the series
(escalating on-page torture of named characters, flagged as "a
crutch" by critics). The film, unlike some other adaptations handled
this session, is tonally lighter than the books and doesn't move any
axis.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="361">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1092,10 +1092,19 @@
     <t xml:space="preserve">Stephen King</t>
   </si>
   <si>
+    <t xml:space="preserve">Eragon (The Inheritance Cycle)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novels, Film</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christopher Paolini</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 113 of 113 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 114 of 114 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1902,7 +1911,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R114"/>
+  <dimension ref="A1:R115"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -8056,6 +8065,59 @@
       </c>
       <c r="Q114" s="1" t="n">
         <v>7</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H115" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I115" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J115" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K115" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L115" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M115" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N115" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O115" s="1" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="P115" s="1" t="n">
+        <v>5.2125</v>
+      </c>
+      <c r="Q115" s="1" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -8090,7 +8152,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8145,7 +8207,7 @@
         <v>85</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8205,7 +8267,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Princess Bride to tier 2
Scored William Goldman's novel and the 1987 film against the 7
criteria. Final Score 2.9625, Tier 2, tying Narnia and The Legend of
Zelda via distinct profiles. Moral Cynicism and Narrative Acceptance
of Injustice sit at 1 (not 0) specifically because of Goldman's
"life isn't fair" framing thesis, a real meta-level complication of
just-world causality even though the actual told story is a full,
clean triumph.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="364">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1101,10 +1101,19 @@
     <t xml:space="preserve">Christopher Paolini</t>
   </si>
   <si>
+    <t xml:space="preserve">The Princess Bride</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novel, Film</t>
+  </si>
+  <si>
+    <t xml:space="preserve">William Goldman</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 114 of 114 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 115 of 115 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1911,7 +1920,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R115"/>
+  <dimension ref="A1:R116"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -8067,7 +8076,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="1" t="n">
         <v>5</v>
       </c>
@@ -8118,6 +8127,59 @@
       </c>
       <c r="Q115" s="1" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H116" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I116" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K116" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L116" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N116" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O116" s="1" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="P116" s="1" t="n">
+        <v>2.9625</v>
+      </c>
+      <c r="Q116" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -8152,7 +8214,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8174,7 +8236,7 @@
         <v>82</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8267,7 +8329,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Fourth Wing (The Empyrean) to tier 6
Scored the three published novels (of a planned 5) against the 7
criteria, bundled as one entry after confirming the darkness
escalates continuously rather than shifting register book-to-book.
Final Score 6.7875, Tier 6. This landed as an exact 3-way tie with
Marchen Crown and the just-corrected Grim Company; each axis was
re-scrutinized independently against the standing rule that
collision-avoidance must never drive a score, and the match holds
as a legitimate coincidence rather than a sign any entry was
under-examined.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="367">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1110,10 +1110,19 @@
     <t xml:space="preserve">William Goldman</t>
   </si>
   <si>
+    <t xml:space="preserve">Fourth Wing (The Empyrean)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rebecca Yarros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ongoing series, 3 of 5 planned books published as of this entry</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 115 of 115 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 116 of 116 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1920,7 +1929,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R116"/>
+  <dimension ref="A1:R117"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -8129,7 +8138,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="1" t="n">
         <v>2</v>
       </c>
@@ -8180,6 +8189,62 @@
       </c>
       <c r="Q116" s="1" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H117" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I117" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J117" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K117" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L117" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M117" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N117" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O117" s="1" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="P117" s="1" t="n">
+        <v>6.7875</v>
+      </c>
+      <c r="Q117" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="R117" s="1" t="s">
+        <v>364</v>
       </c>
     </row>
   </sheetData>
@@ -8214,7 +8279,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8280,7 +8345,7 @@
         <v>86</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8329,7 +8394,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Sweet Tooth to tier 7
Scored Jeff Lemire's complete Vertigo comic against the 7 criteria,
using it (not the notably gentler Netflix show) as the darker,
defining version. Final Score 7.80, tying Attack on Titan, House of
the Dragon, and The Dark Tower via distinct profiles. Structural
Despair and Limited Heroism both reflect the comic's own confirmed
ending: humanity goes fully extinct, succeeded by the hybrids, an
outcome no individual heroism prevents.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="369">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1119,10 +1119,16 @@
     <t xml:space="preserve">ongoing series, 3 of 5 planned books published as of this entry</t>
   </si>
   <si>
+    <t xml:space="preserve">Sweet Tooth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeff Lemire</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 116 of 116 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 117 of 117 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -1929,7 +1935,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R117"/>
+  <dimension ref="A1:R118"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -8191,7 +8197,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="1" t="n">
         <v>6</v>
       </c>
@@ -8245,6 +8251,59 @@
       </c>
       <c r="R117" s="1" t="s">
         <v>364</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G118" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H118" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I118" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="J118" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="K118" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L118" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M118" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N118" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O118" s="1" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="P118" s="1" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Q118" s="1" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -8279,7 +8338,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8356,7 +8415,7 @@
         <v>87</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8394,7 +8453,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Wizard of Oz to tier 2, queue Return to Oz separately
Scored the 1900 novel + 1939 film bundled (final score 2.625, a three-way
profile-distinct tie with Chamber of Secrets and The Little Prince).
Structural Corruption lands at 2 on the Winkies' confirmed on-page
enslavement, not just the Wizard's fraud.

Also added Return to Oz (1985) to the queue as its own item - it draws on
Baum's darker 2nd/3rd Oz novels and is widely cited as unusually
disturbing for a children's film, the same reasoning that already kept
Wicked separate from this entry.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R120"/>
+  <dimension ref="A1:R121"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -8998,6 +8998,76 @@
       <c r="R120" s="15" t="inlineStr">
         <is>
           <t>scored as the duology (Alice's Adventures in Wonderland + Through the Looking-Glass), as commonly published/read together under this title</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="15" customHeight="1" s="9">
+      <c r="A121" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B121" s="15" t="inlineStr">
+        <is>
+          <t>Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C121" s="15" t="inlineStr">
+        <is>
+          <t>The Wizard of Oz</t>
+        </is>
+      </c>
+      <c r="D121" s="15" t="inlineStr">
+        <is>
+          <t>Novel, Film</t>
+        </is>
+      </c>
+      <c r="E121" s="15" t="inlineStr">
+        <is>
+          <t>L. Frank Baum</t>
+        </is>
+      </c>
+      <c r="F121" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G121" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H121" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I121" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J121" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K121" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L121" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M121" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N121" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O121" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P121" s="15" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="Q121" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="R121" s="15" t="inlineStr">
+        <is>
+          <t>scored as the 1900 novel + the 1939 film (bundled, same story/intensity); later Baum sequel novels and the 1985 Return to Oz not consulted here</t>
         </is>
       </c>
     </row>
@@ -9062,7 +9132,7 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
@@ -9172,7 +9242,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 119 of 119 works in the full catalog.</t>
+          <t>Total scored: 120 of 120 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Wicked to tier 7
Scored via Gregory Maguire's novel (Dillamond's assassination, Elphaba's
unresolved tragic death, the actively worsening Animal-rights oppression).
Final score 7.575, an exact tie with The Stormlight Archive via a
different profile. The stage musical/films are confirmed much softer
(estimated ~Tier 4 on their own) and don't move this entry - same
pattern as Eragon's film or Sweet Tooth's show, not a split like Wicked's
own relationship to The Wizard of Oz.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R121"/>
+  <dimension ref="A1:R122"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9068,6 +9068,76 @@
       <c r="R121" s="15" t="inlineStr">
         <is>
           <t>scored as the 1900 novel + the 1939 film (bundled, same story/intensity); later Baum sequel novels and the 1985 Return to Oz not consulted here</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="15" customHeight="1" s="9">
+      <c r="A122" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B122" s="15" t="inlineStr">
+        <is>
+          <t>Extreme Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C122" s="15" t="inlineStr">
+        <is>
+          <t>Wicked</t>
+        </is>
+      </c>
+      <c r="D122" s="15" t="inlineStr">
+        <is>
+          <t>Novel</t>
+        </is>
+      </c>
+      <c r="E122" s="15" t="inlineStr">
+        <is>
+          <t>Gregory Maguire</t>
+        </is>
+      </c>
+      <c r="F122" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G122" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L122" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N122" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O122" s="15" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="P122" s="15" t="n">
+        <v>7.575</v>
+      </c>
+      <c r="Q122" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="R122" s="15" t="inlineStr">
+        <is>
+          <t>scored via the novel (the darker, definitive version); the stage musical and the 2024/2025 films follow the musical, which is confirmed significantly softer (Dillamond silenced rather than murdered, Elphaba fakes her death rather than dying, reconciliation instead of erasure) and estimated around Tier 4 on its own - doesn't move this entry, same pattern as Eragon's film or Sweet Tooth's show</t>
         </is>
       </c>
     </row>
@@ -9197,7 +9267,7 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="9">
@@ -9242,7 +9312,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 120 of 120 works in the full catalog.</t>
+          <t>Total scored: 121 of 121 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Arcane to tier 6
Scored both seasons together (final score 6.7875), an exact 7-axis
profile match with Fourth Wing and The Grim Company. Ran the full
direct-neighbor, non-adjacent, and label checks before locking it in,
including specifically re-examining Redemption Difficulty against the
precedent set by Grim Company's own tie-breaking correction.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R122"/>
+  <dimension ref="A1:R123"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9138,6 +9138,76 @@
       <c r="R122" s="15" t="inlineStr">
         <is>
           <t>scored via the novel (the darker, definitive version); the stage musical and the 2024/2025 films follow the musical, which is confirmed significantly softer (Dillamond silenced rather than murdered, Elphaba fakes her death rather than dying, reconciliation instead of erasure) and estimated around Tier 4 on its own - doesn't move this entry, same pattern as Eragon's film or Sweet Tooth's show</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="15" customHeight="1" s="9">
+      <c r="A123" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B123" s="15" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C123" s="15" t="inlineStr">
+        <is>
+          <t>Arcane</t>
+        </is>
+      </c>
+      <c r="D123" s="15" t="inlineStr">
+        <is>
+          <t>TV series</t>
+        </is>
+      </c>
+      <c r="E123" s="15" t="inlineStr">
+        <is>
+          <t>Riot Games</t>
+        </is>
+      </c>
+      <c r="F123" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G123" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H123" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="I123" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="J123" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K123" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L123" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M123" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="N123" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="O123" s="15" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="P123" s="15" t="n">
+        <v>6.7875</v>
+      </c>
+      <c r="Q123" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="R123" s="15" t="inlineStr">
+        <is>
+          <t>scored against both seasons (2021, 2024); an exact 7-axis profile match with Fourth Wing and The Grim Company, checked against precedent before locking</t>
         </is>
       </c>
     </row>
@@ -9254,7 +9324,7 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="9">
@@ -9312,7 +9382,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 121 of 121 works in the full catalog.</t>
+          <t>Total scored: 122 of 122 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Percy Jackson & the Olympians to tier 3
Scored the original 5-book series + Disney+ TV adaptation. Final score
3.6375, an exact tie with The Hobbit and Howl's Moving Castle via a
different profile. The ending's forced, pantheon-wide reform of how the
gods treat their demigod children drives Limited Heroism and Narrative
Acceptance of Injustice both to 0. Also logged to SCORING_RECORD.md to
keep it in sync going forward.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R123"/>
+  <dimension ref="A1:R124"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9208,6 +9208,76 @@
       <c r="R123" s="15" t="inlineStr">
         <is>
           <t>scored against both seasons (2021, 2024); an exact 7-axis profile match with Fourth Wing and The Grim Company, checked against precedent before locking</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="15" customHeight="1" s="9">
+      <c r="A124" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B124" s="15" t="inlineStr">
+        <is>
+          <t>Moderately Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C124" s="15" t="inlineStr">
+        <is>
+          <t>Percy Jackson &amp; the Olympians</t>
+        </is>
+      </c>
+      <c r="D124" s="15" t="inlineStr">
+        <is>
+          <t>Novels, TV series</t>
+        </is>
+      </c>
+      <c r="E124" s="15" t="inlineStr">
+        <is>
+          <t>Rick Riordan</t>
+        </is>
+      </c>
+      <c r="F124" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G124" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H124" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I124" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J124" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K124" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L124" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M124" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N124" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O124" s="15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="P124" s="15" t="n">
+        <v>3.6375</v>
+      </c>
+      <c r="Q124" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="R124" s="15" t="inlineStr">
+        <is>
+          <t>scored against the original 5-book series (The Lightning Thief - The Last Olympian) and the closely-following Disney+ TV adaptation; later series (Heroes of Olympus, Trials of Apollo) out of scope</t>
         </is>
       </c>
     </row>
@@ -9285,7 +9355,7 @@
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="9">
@@ -9382,7 +9452,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 122 of 122 works in the full catalog.</t>
+          <t>Total scored: 123 of 123 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Violence Jack (tier 8) and Devilman Lady (tier 6); add genre-scope gate
Both are Go Nagai works tied into the Devilman mythos, confirmed as
genuine dark fantasy (not sci-fi) before scoring. Devilman Crybaby's
medium/creator fields were also corrected to reflect it being bundled
with the original manga (Go Nagai), not scored as anime alone.

Added an explicit genre-eligibility check to ADDITIONS_LOG.md and
README.md: candidates must be genuinely fantasy or a real fantasy
hybrid, not "the Fantastique" or other adjacent non-fantasy genres.

Also fixed stale "117 fantasy books" meta descriptions (both languages)
and README's stale "100 catalog works" mentions - actual count is 126.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R124"/>
+  <dimension ref="A1:R127"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9278,6 +9278,216 @@
       <c r="R124" s="15" t="inlineStr">
         <is>
           <t>scored against the original 5-book series (The Lightning Thief - The Last Olympian) and the closely-following Disney+ TV adaptation; later series (Heroes of Olympus, Trials of Apollo) out of scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="15" customHeight="1" s="9">
+      <c r="A125" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B125" s="15" t="inlineStr">
+        <is>
+          <t>Extreme Grimdark</t>
+        </is>
+      </c>
+      <c r="C125" s="15" t="inlineStr">
+        <is>
+          <t>Devilman Crybaby</t>
+        </is>
+      </c>
+      <c r="D125" s="15" t="inlineStr">
+        <is>
+          <t>Manga, Anime</t>
+        </is>
+      </c>
+      <c r="E125" s="15" t="inlineStr">
+        <is>
+          <t>Go Nagai</t>
+        </is>
+      </c>
+      <c r="F125" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G125" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H125" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="I125" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="J125" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K125" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L125" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M125" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="N125" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="O125" s="15" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P125" s="15" t="n">
+        <v>9.824999999999999</v>
+      </c>
+      <c r="Q125" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="R125" s="15" t="inlineStr">
+        <is>
+          <t>bundled with the original manga (same story, same ending) since the 2018 anime is explicitly the first adaptation to bring the manga's own dark ending to screen; excludes the earlier, considerably softer 1970s TV anime</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="15" customHeight="1" s="9">
+      <c r="A126" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B126" s="15" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C126" s="15" t="inlineStr">
+        <is>
+          <t>Violence Jack</t>
+        </is>
+      </c>
+      <c r="D126" s="15" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="E126" s="15" t="inlineStr">
+        <is>
+          <t>Go Nagai</t>
+        </is>
+      </c>
+      <c r="F126" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G126" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L126" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M126" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="N126" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="O126" s="15" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="P126" s="15" t="n">
+        <v>8.137499999999999</v>
+      </c>
+      <c r="Q126" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="R126" s="15" t="inlineStr">
+        <is>
+          <t>post-apocalyptic dark fantasy, directly tied to the Devilman mythos (Jack is revealed to be a revived Akira Fudo; Satan/Ryo Asuka created the Slum King)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="15" customHeight="1" s="9">
+      <c r="A127" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B127" s="15" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C127" s="15" t="inlineStr">
+        <is>
+          <t>Devilman Lady</t>
+        </is>
+      </c>
+      <c r="D127" s="15" t="inlineStr">
+        <is>
+          <t>Manga</t>
+        </is>
+      </c>
+      <c r="E127" s="15" t="inlineStr">
+        <is>
+          <t>Go Nagai</t>
+        </is>
+      </c>
+      <c r="F127" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G127" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H127" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I127" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="J127" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K127" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L127" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M127" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N127" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="O127" s="15" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="P127" s="15" t="n">
+        <v>6.1125</v>
+      </c>
+      <c r="Q127" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="R127" s="15" t="inlineStr">
+        <is>
+          <t>scored against the manga (1997-2000), confirmed more violent/sexually explicit than its own anime adaptation</t>
         </is>
       </c>
     </row>
@@ -9394,7 +9604,7 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="9">
@@ -9420,7 +9630,7 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="9">
@@ -9433,7 +9643,7 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="9">
@@ -9452,7 +9662,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 123 of 123 works in the full catalog.</t>
+          <t>Total scored: 126 of 126 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add The Mighty Nein to tier 6
Scored against the complete, finished tabletop campaign (141 episodes),
not just Amazon's still-airing TV adaptation, matching the House of the
Dragon/A Knight of the Seven Kingdoms precedent. Final score 6.225, a
three-way tie with The Witcher and Final Fantasy XIV. Structural
Corruption 3 driven by the Cerberus Assembly's confirmed manipulation of
Caleb into killing his own parents.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R127"/>
+  <dimension ref="A1:R128"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9488,6 +9488,76 @@
       <c r="R127" s="15" t="inlineStr">
         <is>
           <t>scored against the manga (1997-2000), confirmed more violent/sexually explicit than its own anime adaptation</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="15" customHeight="1" s="9">
+      <c r="A128" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B128" s="15" t="inlineStr">
+        <is>
+          <t>Dark Fantasy</t>
+        </is>
+      </c>
+      <c r="C128" s="15" t="inlineStr">
+        <is>
+          <t>The Mighty Nein</t>
+        </is>
+      </c>
+      <c r="D128" s="15" t="inlineStr">
+        <is>
+          <t>TV series / D&amp;D actual-play</t>
+        </is>
+      </c>
+      <c r="E128" s="15" t="inlineStr">
+        <is>
+          <t>Critical Role</t>
+        </is>
+      </c>
+      <c r="F128" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G128" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H128" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I128" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="J128" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K128" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L128" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M128" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="N128" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O128" s="15" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="P128" s="15" t="n">
+        <v>6.225</v>
+      </c>
+      <c r="Q128" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="R128" s="15" t="inlineStr">
+        <is>
+          <t>scored against the complete, finished tabletop campaign (141 episodes, 2018-2021), not just the still-airing Amazon TV adaptation (Season 1, Nov 2025), matching the precedent used for House of the Dragon and A Knight of the Seven Kingdoms</t>
         </is>
       </c>
     </row>
@@ -9604,7 +9674,7 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="9">
@@ -9662,7 +9732,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 126 of 126 works in the full catalog.</t>
+          <t>Total scored: 127 of 127 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rescore The Legend of Vox Machina against the complete tabletop campaign
Prompted by the user pointing out the show has other media and is itself
still airing/incomplete. Rescored against the finished 115-episode
Campaign 1 actual-play instead, matching The Mighty Nein precedent.
Limited Heroism raised 1->2: the prior v2 rescore had dropped Vax'ildan's
permanent departure to serve the Raven Queen from its analysis entirely,
even though the original v1 entry had captured it. New score 4.875
(was 4.8375) - same tier, but now an exact tie with Fullmetal Alchemist:
Brotherhood instead of sitting between it and Final Fantasy XII.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -4362,7 +4362,7 @@
       </c>
       <c r="D51" s="15" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>TV series / D&amp;D actual-play</t>
         </is>
       </c>
       <c r="E51" s="15" t="inlineStr">
@@ -4384,7 +4384,7 @@
         <v>1</v>
       </c>
       <c r="I51" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J51" s="15" t="n">
         <v>1</v>
@@ -4402,13 +4402,18 @@
         <v>3</v>
       </c>
       <c r="O51" s="15" t="n">
-        <v>1.35</v>
+        <v>1.5</v>
       </c>
       <c r="P51" s="15" t="n">
-        <v>4.8375</v>
+        <v>4.875</v>
       </c>
       <c r="Q51" s="15" t="n">
         <v>4</v>
+      </c>
+      <c r="R51" s="15" t="inlineStr">
+        <is>
+          <t>rescored against the complete Campaign 1 tabletop actual-play (115 episodes, finished 2017), not just the still-airing TV adaptation; Limited Heroism raised 1-&gt;2 to reflect Vax'ildan's permanent departure to serve the Raven Queen, a structurally real cost the prior TV-based scoring never addressed</t>
+        </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="9">

</xml_diff>

<commit_message>
Add Goblins to tier 8
Final score 8.1375, a three-way exact tie with Berserk and Violence Jack
via different profiles. Checked and rejected a dark-comedy framing before
scoring (critics confirm tonal dissonance, not a harmonious blend; the
creator has said the extreme villains process real trauma) - Moral
Cynicism and Structural Corruption both driven by the paladin Kore's
sanctioned infanticide and the setting's adventurer economy treating
goblins as disposable prey.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R128"/>
+  <dimension ref="A1:R129"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9563,6 +9563,76 @@
       <c r="R128" s="15" t="inlineStr">
         <is>
           <t>scored against the complete, finished tabletop campaign (141 episodes, 2018-2021), not just the still-airing Amazon TV adaptation (Season 1, Nov 2025), matching the precedent used for House of the Dragon and A Knight of the Seven Kingdoms</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="15" customHeight="1" s="9">
+      <c r="A129" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B129" s="15" t="inlineStr">
+        <is>
+          <t>Grimdark</t>
+        </is>
+      </c>
+      <c r="C129" s="15" t="inlineStr">
+        <is>
+          <t>Goblins</t>
+        </is>
+      </c>
+      <c r="D129" s="15" t="inlineStr">
+        <is>
+          <t>Webcomic</t>
+        </is>
+      </c>
+      <c r="E129" s="15" t="inlineStr">
+        <is>
+          <t>Tarol Hunt</t>
+        </is>
+      </c>
+      <c r="F129" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G129" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H129" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="I129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M129" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N129" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="O129" s="15" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="P129" s="15" t="n">
+        <v>8.137499999999999</v>
+      </c>
+      <c r="Q129" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="R129" s="15" t="inlineStr">
+        <is>
+          <t>still ongoing/unresolved as of 2025-2026; genre-checked - dark comedy framing does not apply (tonal dissonance, not harmonious blend, confirmed by critics and creator statement)</t>
         </is>
       </c>
     </row>
@@ -9705,7 +9775,7 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="9">
@@ -9737,7 +9807,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 127 of 127 works in the full catalog.</t>
+          <t>Total scored: 128 of 128 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Twilight to tier 4
Scored all four novels + films. Final score 4.20, a four-way exact tie
with The NeverEnding Story, Once Upon a Time, and The Dark Crystal.
Structural Corruption 2 and Narrative Acceptance of Injustice 2 driven
by the Volturi's absolute, unreformed rule - deterred once in the
finale, never actually challenged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R129"/>
+  <dimension ref="A1:R130"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9633,6 +9633,76 @@
       <c r="R129" s="15" t="inlineStr">
         <is>
           <t>still ongoing/unresolved as of 2025-2026; genre-checked - dark comedy framing does not apply (tonal dissonance, not harmonious blend, confirmed by critics and creator statement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="15" customHeight="1" s="9">
+      <c r="A130" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B130" s="15" t="inlineStr">
+        <is>
+          <t>Fantasy in Gray Tones</t>
+        </is>
+      </c>
+      <c r="C130" s="15" t="inlineStr">
+        <is>
+          <t>Twilight</t>
+        </is>
+      </c>
+      <c r="D130" s="15" t="inlineStr">
+        <is>
+          <t>Novels, Films</t>
+        </is>
+      </c>
+      <c r="E130" s="15" t="inlineStr">
+        <is>
+          <t>Stephenie Meyer</t>
+        </is>
+      </c>
+      <c r="F130" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G130" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H130" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I130" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J130" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K130" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L130" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M130" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="N130" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O130" s="15" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P130" s="15" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="Q130" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="R130" s="15" t="inlineStr">
+        <is>
+          <t>scored against all four novels + the film series; the Breaking Dawn Part 2 film's battle sequence is Alice's vision of a possible future, not real events, but the imagery still counts toward Explicit Darkness</t>
         </is>
       </c>
     </row>
@@ -9723,7 +9793,7 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="9">
@@ -9807,7 +9877,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 128 of 128 works in the full catalog.</t>
+          <t>Total scored: 129 of 129 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Wednesday to tier 4
Scored seasons 1-2 (complete as of Sept 2025); season 3 confirmed but
unreleased, not factored in. Final score 4.9875, a three-way tie with
Adventure Time and Star vs. the Forces of Evil right at the tier's top
edge - checked directly against the Tier 5 floor given how close the
gap is, confirmed not a coin-flip.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R130"/>
+  <dimension ref="A1:R131"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9703,6 +9703,76 @@
       <c r="R130" s="15" t="inlineStr">
         <is>
           <t>scored against all four novels + the film series; the Breaking Dawn Part 2 film's battle sequence is Alice's vision of a possible future, not real events, but the imagery still counts toward Explicit Darkness</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="15" customHeight="1" s="9">
+      <c r="A131" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B131" s="15" t="inlineStr">
+        <is>
+          <t>Fantasy in Gray Tones</t>
+        </is>
+      </c>
+      <c r="C131" s="15" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D131" s="15" t="inlineStr">
+        <is>
+          <t>TV series</t>
+        </is>
+      </c>
+      <c r="E131" s="15" t="inlineStr">
+        <is>
+          <t>Alfred Gough &amp; Miles Millar</t>
+        </is>
+      </c>
+      <c r="F131" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G131" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H131" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I131" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="J131" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K131" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L131" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M131" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="N131" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O131" s="15" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="P131" s="15" t="n">
+        <v>4.9875</v>
+      </c>
+      <c r="Q131" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="R131" s="15" t="inlineStr">
+        <is>
+          <t>scored against seasons 1-2 (complete as of Sept 2025); season 3 confirmed but unreleased, not factored in - season 2 ends on real unresolved cliffhangers (Enid, Ophelia), not a clean resolution</t>
         </is>
       </c>
     </row>
@@ -9793,7 +9863,7 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="9">
@@ -9877,7 +9947,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 129 of 129 works in the full catalog.</t>
+          <t>Total scored: 130 of 130 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add The Addams Family (1964-1992) to tier 2
Bundled across the 1964 live-action original, 1973 animated series, and
1992 animated series. Revised twice from an initial pass: Explicit
Darkness raised 1->2 (recurring bombs/guillotine imagery), Moral
Cynicism raised 0->1 after checking the axis outside the family - the
Addamses' warmth is consistently met with fear and rejection from
neighbors. Final score 2.2875, tied with Castle in the Sky and
Labyrinth. Added a year range to the title to disambiguate from the
still-pending Films queue item and from Wednesday.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R131"/>
+  <dimension ref="A1:R132"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9773,6 +9773,76 @@
       <c r="R131" s="15" t="inlineStr">
         <is>
           <t>scored against seasons 1-2 (complete as of Sept 2025); season 3 confirmed but unreleased, not factored in - season 2 ends on real unresolved cliffhangers (Enid, Ophelia), not a clean resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="15" customHeight="1" s="9">
+      <c r="A132" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B132" s="15" t="inlineStr">
+        <is>
+          <t>Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C132" s="15" t="inlineStr">
+        <is>
+          <t>The Addams Family (1964-1992)</t>
+        </is>
+      </c>
+      <c r="D132" s="15" t="inlineStr">
+        <is>
+          <t>TV series</t>
+        </is>
+      </c>
+      <c r="E132" s="15" t="inlineStr">
+        <is>
+          <t>Charles Addams (creator)</t>
+        </is>
+      </c>
+      <c r="F132" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G132" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H132" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I132" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J132" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K132" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L132" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M132" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N132" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O132" s="15" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P132" s="15" t="n">
+        <v>2.2875</v>
+      </c>
+      <c r="Q132" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="R132" s="15" t="inlineStr">
+        <is>
+          <t>bundled across the 1964, 1973, and 1992 TV incarnations - confirmed consistent tone across all three; genre-checked (real, if lightly-played, supernatural content: Grandmama's potions/broom, Morticia's psychic premonitions, Fester's electric powers, Thing as a sentient disembodied hand)</t>
         </is>
       </c>
     </row>
@@ -9824,7 +9894,7 @@
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="9">
@@ -9837,7 +9907,7 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
@@ -9947,7 +10017,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 130 of 130 works in the full catalog.</t>
+          <t>Total scored: 131 of 131 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add The Addams Family (1991-1993) films to tier 2
Scored the Barry Sonnenfeld live-action films only; the 2019/2021
animated films are confirmed genuinely lighter by critics and excluded,
matching the Dark Sun CRPG-exclusion precedent. Kept separate from the
TV series entry since the films (a serial-killer nanny, an electrocution
device threatening a baby) are confirmed meaningfully more intense.
Final score 2.85, tied with Willow and The Nightmare Before Christmas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R132"/>
+  <dimension ref="A1:R133"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9843,6 +9843,76 @@
       <c r="R132" s="15" t="inlineStr">
         <is>
           <t>bundled across the 1964, 1973, and 1992 TV incarnations - confirmed consistent tone across all three; genre-checked (real, if lightly-played, supernatural content: Grandmama's potions/broom, Morticia's psychic premonitions, Fester's electric powers, Thing as a sentient disembodied hand)</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="15" customHeight="1" s="9">
+      <c r="A133" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B133" s="15" t="inlineStr">
+        <is>
+          <t>Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C133" s="15" t="inlineStr">
+        <is>
+          <t>The Addams Family (1991-1993)</t>
+        </is>
+      </c>
+      <c r="D133" s="15" t="inlineStr">
+        <is>
+          <t>Films</t>
+        </is>
+      </c>
+      <c r="E133" s="15" t="inlineStr">
+        <is>
+          <t>dir. Barry Sonnenfeld</t>
+        </is>
+      </c>
+      <c r="F133" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G133" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H133" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I133" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J133" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K133" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L133" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M133" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N133" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O133" s="15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="P133" s="15" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="Q133" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="R133" s="15" t="inlineStr">
+        <is>
+          <t>the Barry Sonnenfeld live-action films (The Addams Family 1991, Addams Family Values 1993) only - the 2019/2021 animated films are confirmed lighter/less distinct by critics and omitted, matching the Dark Sun CRPG-exclusion precedent</t>
         </is>
       </c>
     </row>
@@ -9907,7 +9977,7 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
@@ -10017,7 +10087,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 131 of 131 works in the full catalog.</t>
+          <t>Total scored: 132 of 132 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Chrono Trigger to tier 3
Scored the canonical ending. Final score 3.975, an exact tie with a
six-work cluster (LOTR, Frieren, Black Clover, Record of Lodoss War,
Final Fantasy II, Nausicaä). Ran a full boundary check against Tier 4
given how close the raw score sits to the 4.0 cutoff - confirmed against
both the actual Tier 4 floor cluster and TIER_GUIDE.md's own tier
definitions that Tier 3 is the right fit, not a coin-flip.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R133"/>
+  <dimension ref="A1:R134"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9913,6 +9913,76 @@
       <c r="R133" s="15" t="inlineStr">
         <is>
           <t>the Barry Sonnenfeld live-action films (The Addams Family 1991, Addams Family Values 1993) only - the 2019/2021 animated films are confirmed lighter/less distinct by critics and omitted, matching the Dark Sun CRPG-exclusion precedent</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="15" customHeight="1" s="9">
+      <c r="A134" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B134" s="15" t="inlineStr">
+        <is>
+          <t>Moderately Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C134" s="15" t="inlineStr">
+        <is>
+          <t>Chrono Trigger</t>
+        </is>
+      </c>
+      <c r="D134" s="15" t="inlineStr">
+        <is>
+          <t>Video Game</t>
+        </is>
+      </c>
+      <c r="E134" s="15" t="inlineStr">
+        <is>
+          <t>Square</t>
+        </is>
+      </c>
+      <c r="F134" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G134" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H134" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="I134" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J134" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K134" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L134" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M134" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N134" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O134" s="15" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="P134" s="15" t="n">
+        <v>3.975</v>
+      </c>
+      <c r="Q134" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="R134" s="15" t="inlineStr">
+        <is>
+          <t>scored against the canonical/main ending (defeating Lavos after full story progression); alternate/joke endings from New Game+ or early game-overs not factored in</t>
         </is>
       </c>
     </row>
@@ -9990,7 +10060,7 @@
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="9">
@@ -10087,7 +10157,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 132 of 132 works in the full catalog.</t>
+          <t>Total scored: 133 of 133 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Forgotten Realms (core setting) to tier 4
Scored the general setting/lore only, explicitly excluding Drizzt and
the Baldur's Gate games since both are already separate catalog
entries. Final score 4.65, tied with Grimgar, Avatar: The Last
Airbender, Earthsea, Final Fantasy XII, and Charmed. Redemption
Difficulty 3 grounded in Artemis Entreri's confirmed refusal of full
redemption when offered. Sits sensibly in the middle of its own
franchise's already-scored spread (above BG I/II, below BG III/Drizzt).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R134"/>
+  <dimension ref="A1:R135"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9983,6 +9983,76 @@
       <c r="R134" s="15" t="inlineStr">
         <is>
           <t>scored against the canonical/main ending (defeating Lavos after full story progression); alternate/joke endings from New Game+ or early game-overs not factored in</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="15" customHeight="1" s="9">
+      <c r="A135" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B135" s="15" t="inlineStr">
+        <is>
+          <t>Fantasy in Gray Tones</t>
+        </is>
+      </c>
+      <c r="C135" s="15" t="inlineStr">
+        <is>
+          <t>Forgotten Realms</t>
+        </is>
+      </c>
+      <c r="D135" s="15" t="inlineStr">
+        <is>
+          <t>Tabletop (D&amp;D campaign setting), Novels</t>
+        </is>
+      </c>
+      <c r="E135" s="15" t="inlineStr">
+        <is>
+          <t>TSR / Wizards of the Coast</t>
+        </is>
+      </c>
+      <c r="F135" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G135" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H135" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I135" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J135" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K135" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L135" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M135" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N135" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O135" s="15" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="P135" s="15" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="Q135" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="R135" s="15" t="inlineStr">
+        <is>
+          <t>scored against the core setting/general lore only - Drizzt novels and the Baldur's Gate games are already separate catalog entries and excluded here to avoid double-counting</t>
         </is>
       </c>
     </row>
@@ -10073,7 +10143,7 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="9">
@@ -10157,7 +10227,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 133 of 133 works in the full catalog.</t>
+          <t>Total scored: 134 of 134 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Alice in Wonderland (2010-2016) films to tier 2
Kept separate from the novels entry - both Burton films are original
stories, not retellings, matching the Wicked/Age of Resistance
"genuinely different story" pattern rather than a fold-in. Final score
2.625, an exact 7-axis profile match with The Wizard of Oz (both a
"villain runs a real, contained tyranny, corrected cleanly" case).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R135"/>
+  <dimension ref="A1:R136"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -10053,6 +10053,76 @@
       <c r="R135" s="15" t="inlineStr">
         <is>
           <t>scored against the core setting/general lore only - Drizzt novels and the Baldur's Gate games are already separate catalog entries and excluded here to avoid double-counting</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="15" customHeight="1" s="9">
+      <c r="A136" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B136" s="15" t="inlineStr">
+        <is>
+          <t>Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C136" s="15" t="inlineStr">
+        <is>
+          <t>Alice in Wonderland (2010-2016)</t>
+        </is>
+      </c>
+      <c r="D136" s="15" t="inlineStr">
+        <is>
+          <t>Films</t>
+        </is>
+      </c>
+      <c r="E136" s="15" t="inlineStr">
+        <is>
+          <t>dir. Tim Burton</t>
+        </is>
+      </c>
+      <c r="F136" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G136" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H136" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I136" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J136" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K136" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L136" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M136" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N136" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O136" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P136" s="15" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="Q136" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="R136" s="15" t="inlineStr">
+        <is>
+          <t>an original story, not a retelling of Carroll's plot - kept separate from the "Alice in Wonderland" novels entry (Tier 2) for the same reason Wicked stayed separate from The Wizard of Oz</t>
         </is>
       </c>
     </row>
@@ -10117,7 +10187,7 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
@@ -10227,7 +10297,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Total scored: 134 of 134 works in the full catalog.</t>
+          <t>Total scored: 135 of 135 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move American McGee's Alice / Madness Returns to tier 7
Structural Corruption and Narrative Acceptance of Injustice were
underscored on the first pass: Bumby's orphanage is the actual
operating front for a child-trafficking ring, not one predator
abusing an otherwise-legitimate role.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1296,7 +1296,7 @@
     <t xml:space="preserve">American McGee (creative director)</t>
   </si>
   <si>
-    <t xml:space="preserve">genre-gated as a confirmed 'third-person dark fantasy action-adventure' per contemporary critical/marketing classification, despite Wonderland being explicitly the protagonist's psychological retreat (per creator American McGee's own clarification) rather than a separately 'real' world -- resolved via classification check rather than assumed either way, same treatment as other ambiguous-supernatural cases; bundled the two games (2000, 2011) as one entry since Madness Returns is a direct narrative sequel following the same protagonist's single arc, not a reboot -- the severity gap between them (game 1 alone would land near Tier 5, game 2 alone near Tier 6) is far narrower than the Final Fantasy I/II/XII precedent that justified a split, so scored holistically across both; Structural Corruption held at 2 rather than 3 since the abuse (Dr. Bumby, a trusted orphanage physician revealed to be a serial child-trafficker who murdered Alice's family to cover up raping her sister) is one predator exploiting a legitimate institutional role, not the orphanage/asylum system itself being designed for exploitation; Redemption Difficulty scored on Alice's own arc (a decade of misplaced survivor's guilt over a fire she didn't cause, resolved only at real cost) rather than Bumby's, who is killed rather than offered any redemption; Narrative Acceptance of Injustice at 2 since Alice's own core injustice is resolved (Bumby dies, her guilt is lifted) but the wider trafficking pattern implied by 'as he has done with other children' is left unaddressed.</t>
+    <t xml:space="preserve">genre-gated as a confirmed 'third-person dark fantasy action-adventure' per contemporary critical/marketing classification, despite Wonderland being explicitly the protagonist's psychological retreat (per creator American McGee's own clarification) rather than a separately 'real' world -- resolved via classification check rather than assumed either way, same treatment as other ambiguous-supernatural cases; bundled the two games (2000, 2011) as one entry since Madness Returns is a direct narrative sequel following the same protagonist's single arc, not a reboot -- the severity gap between them (game 1 alone would land near Tier 5, game 2 alone near Tier 6) is far narrower than the Final Fantasy I/II/XII precedent that justified a split, so scored holistically across both; Structural Corruption raised to 3 on review -- Dr. Bumby's orphanage guardianship isn't an isolated abuse of a legitimate role but the actual operating front for a child sex-trafficking ring serving 'many of London's perverts and pedophiles,' with victims mentally broken and numbered for distribution -- the institution's real function, not an anomaly within it; Redemption Difficulty scored on Alice's own arc (a decade of misplaced survivor's guilt over a fire she didn't cause, resolved only at real cost) rather than Bumby's, who is killed rather than offered any redemption; Narrative Acceptance of Injustice raised to 3 on review -- Alice kills Bumby and resolves her own case, but the buyer network and demand side of the trafficking operation are never addressed or dismantled by the story, closer to a structural condition the narrative doesn't attempt to fully erase than a genuinely ambivalent half-resolution.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -9491,12 +9491,12 @@
         <v>421</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C137" s="1" t="s">
         <v>422</v>
@@ -9523,25 +9523,25 @@
         <v>3</v>
       </c>
       <c r="K137" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L137" s="1" t="n">
         <v>2</v>
       </c>
       <c r="M137" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N137" s="1" t="n">
         <v>3</v>
       </c>
       <c r="O137" s="1" t="n">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
       <c r="P137" s="1" t="n">
-        <v>6.9</v>
+        <v>7.575</v>
       </c>
       <c r="Q137" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R137" s="1" t="s">
         <v>424</v>
@@ -9645,7 +9645,7 @@
         <v>86</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9656,7 +9656,7 @@
         <v>87</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add Return to Oz to tier 3
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="430">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1299,10 +1299,19 @@
     <t xml:space="preserve">genre-gated as a confirmed 'third-person dark fantasy action-adventure' per contemporary critical/marketing classification, despite Wonderland being explicitly the protagonist's psychological retreat (per creator American McGee's own clarification) rather than a separately 'real' world -- resolved via classification check rather than assumed either way, same treatment as other ambiguous-supernatural cases; bundled the two games (2000, 2011) as one entry since Madness Returns is a direct narrative sequel following the same protagonist's single arc, not a reboot -- the severity gap between them (game 1 alone would land near Tier 5, game 2 alone near Tier 6) is far narrower than the Final Fantasy I/II/XII precedent that justified a split, so scored holistically across both; Structural Corruption raised to 3 on review -- Dr. Bumby's orphanage guardianship isn't an isolated abuse of a legitimate role but the actual operating front for a child sex-trafficking ring serving 'many of London's perverts and pedophiles,' with victims mentally broken and numbered for distribution -- the institution's real function, not an anomaly within it; Redemption Difficulty scored on Alice's own arc (a decade of misplaced survivor's guilt over a fire she didn't cause, resolved only at real cost) rather than Bumby's, who is killed rather than offered any redemption; Narrative Acceptance of Injustice raised to 3 on review -- Alice kills Bumby and resolves her own case, but the buyer network and demand side of the trafficking operation are never addressed or dismantled by the story, closer to a structural condition the narrative doesn't attempt to fully erase than a genuinely ambivalent half-resolution.</t>
   </si>
   <si>
+    <t xml:space="preserve">Return to Oz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dir. Walter Murch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">based on Baum's 2nd/3rd Oz novels (The Marvelous Land of Oz, Ozma of Oz), not the first book -- kept separate from The Wizard of Oz entry (Tier 2) for the same reason Wicked stayed separate from it; Structural Despair, Limited Heroism, Redemption Difficulty, and Narrative Acceptance of Injustice all bottom out at 0 since both the Oz plot (the Nome King's conquest, Emerald City's citizens turned to stone) and the frame story (Dorothy's abusive sanitarium) resolve completely and durably -- Oz and its people are fully restored, the sanitarium burns down, the abusive Dr. Worley dies, his nurse-accomplice is arrested, and Ozma confirms Dorothy's experiences were real, not delusion; Moral Cynicism (1) since Dorothy's honesty about Oz is initially met with forced institutionalization and a scheduled electroshock 'cure' rather than being believed -- the same 'sincerity dismissed until vindicated' pattern already on record for The Nightmare Before Christmas's MC1 (Sally's warnings), here more severe (institutionalized and nearly tortured, not just ignored) before vindication; Structural Corruption (2) matches the same 'one real, contained tyranny, corrected cleanly' shape already scored for The Wizard of Oz's Wicked Witch and Alice in Wonderland (2010-2016)'s Red Queen -- the sanitarium subplot was weighed as a second corrupt institution but kept out of Structural Corruption's count since Dr. Worley's electrotherapy reads as era-appropriate- but-brutal malpractice by one reckless doctor, not an institution built to perpetuate harm (unlike American McGee's Alice's Bumby, where the orphanage was literally a trafficking front); Explicit Darkness (4) -- Mombi's wall of living, swappable severed heads is genuine recurring body horror (not just atmospheric dread), on top of the electroshock opening, the Wheelers, and a near-cannibalism scene, matching the 'horror corporal... central y recurrente' anchor that separates this from the ED3 ceiling of its closer genre-siblings (Nightmare Before Christmas, Willow, Dark Crystal, The NeverEnding Story); multiple contemporary retrospectives call it 'the most terrifying Disney movie ever made.'</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 136 of 136 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 137 of 137 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -2109,7 +2118,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R137"/>
+  <dimension ref="A1:R138"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -9545,6 +9554,62 @@
       </c>
       <c r="R137" s="1" t="s">
         <v>424</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="D138" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E138" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="F138" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G138" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H138" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I138" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J138" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K138" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L138" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M138" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N138" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O138" s="1" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P138" s="1" t="n">
+        <v>3.4125</v>
+      </c>
+      <c r="Q138" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="R138" s="1" t="s">
+        <v>427</v>
       </c>
     </row>
   </sheetData>
@@ -9579,7 +9644,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9612,7 +9677,7 @@
         <v>83</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9694,7 +9759,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Ravenloft to tier 9
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="432">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1308,10 +1308,16 @@
     <t xml:space="preserve">based on Baum's 2nd/3rd Oz novels (The Marvelous Land of Oz, Ozma of Oz), not the first book -- kept separate from The Wizard of Oz entry (Tier 2) for the same reason Wicked stayed separate from it; Structural Despair, Limited Heroism, Redemption Difficulty, and Narrative Acceptance of Injustice all bottom out at 0 since both the Oz plot (the Nome King's conquest, Emerald City's citizens turned to stone) and the frame story (Dorothy's abusive sanitarium) resolve completely and durably -- Oz and its people are fully restored, the sanitarium burns down, the abusive Dr. Worley dies, his nurse-accomplice is arrested, and Ozma confirms Dorothy's experiences were real, not delusion; Moral Cynicism (1) since Dorothy's honesty about Oz is initially met with forced institutionalization and a scheduled electroshock 'cure' rather than being believed -- the same 'sincerity dismissed until vindicated' pattern already on record for The Nightmare Before Christmas's MC1 (Sally's warnings), here more severe (institutionalized and nearly tortured, not just ignored) before vindication; Structural Corruption (2) matches the same 'one real, contained tyranny, corrected cleanly' shape already scored for The Wizard of Oz's Wicked Witch and Alice in Wonderland (2010-2016)'s Red Queen -- the sanitarium subplot was weighed as a second corrupt institution but kept out of Structural Corruption's count since Dr. Worley's electrotherapy reads as era-appropriate- but-brutal malpractice by one reckless doctor, not an institution built to perpetuate harm (unlike American McGee's Alice's Bumby, where the orphanage was literally a trafficking front); Explicit Darkness (4) -- Mombi's wall of living, swappable severed heads is genuine recurring body horror (not just atmospheric dread), on top of the electroshock opening, the Wheelers, and a near-cannibalism scene, matching the 'horror corporal... central y recurrente' anchor that separates this from the ED3 ceiling of its closer genre-siblings (Nightmare Before Christmas, Willow, Dark Crystal, The NeverEnding Story); multiple contemporary retrospectives call it 'the most terrifying Disney movie ever made.'</t>
   </si>
   <si>
+    <t xml:space="preserve">Ravenloft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scored via the core AD&amp;D/D&amp;D gothic horror campaign setting (the Demiplane of Dread, its Darklords, and the Dark Powers) plus the flagship novel line (Vampire of the Mists / I, Strahd) as co-primary sources, matching the Dark Sun precedent (setting + Prism Pentad novels); Structural Despair (4) and Structural Corruption (4) since the demiplane's entire premise is a structurally condemned prison-world where every domain is, by design, ruled by a corrupt Darklord as both throne and prison, not an incidental flaw; Limited Heroism (3) since parties genuinely can and regularly do defeat individual Darklords in actual play (real, if domain-local, victories), keeping this below Warhammer 40,000's total-futility 4; Moral Cynicism (2) since the Dark Powers read as amoral and capricious rather than actively rewarding cruelty -- innocents get trapped in the mists same as the guilty, but villainy isn't specifically rewarded either, distinguishing this from Dark Sun's might-makes-right MC3; Redemption Difficulty (4) and Narrative Acceptance of Injustice (4) held higher than Dark Sun's RD3/NAI3 specifically because Dark Sun's co-primary source (the Prism Pentad) has a definitive ending showing real redemption and real progress, while Ravenloft's flagship figure (Strahd) has never once escaped his curse across the setting's ~40-year history -- only two Darklords ever have, both via metaphysical loopholes (godhood, total domain abandonment) rather than genuine moral repair, and the demiplane is explicitly designed to never resolve at the meta level, generating new Darklords and trapped victims indefinitely; Explicit Darkness (4) for played-straight Poe/Shelley/ Stoker-style gothic horror (vampiric assault, body horror, notoriously disturbing set-pieces like Curse of Strahd's 'Death House' opener).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 137 of 137 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 138 of 138 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -2118,7 +2124,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R138"/>
+  <dimension ref="A1:R139"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -9556,7 +9562,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="1" t="n">
         <v>3</v>
       </c>
@@ -9610,6 +9616,62 @@
       </c>
       <c r="R138" s="1" t="s">
         <v>427</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B139" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="D139" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="E139" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="F139" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G139" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H139" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="I139" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="J139" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K139" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="L139" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="M139" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="N139" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O139" s="1" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="P139" s="1" t="n">
+        <v>9.4875</v>
+      </c>
+      <c r="Q139" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="R139" s="1" t="s">
+        <v>429</v>
       </c>
     </row>
   </sheetData>
@@ -9644,7 +9706,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9743,7 +9805,7 @@
         <v>89</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9759,7 +9821,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Shadowrun to tier 8
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="436">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1314,10 +1314,22 @@
     <t xml:space="preserve">scored via the core AD&amp;D/D&amp;D gothic horror campaign setting (the Demiplane of Dread, its Darklords, and the Dark Powers) plus the flagship novel line (Vampire of the Mists / I, Strahd) as co-primary sources, matching the Dark Sun precedent (setting + Prism Pentad novels); Structural Despair (4) and Structural Corruption (4) since the demiplane's entire premise is a structurally condemned prison-world where every domain is, by design, ruled by a corrupt Darklord as both throne and prison, not an incidental flaw; Limited Heroism (3) since parties genuinely can and regularly do defeat individual Darklords in actual play (real, if domain-local, victories), keeping this below Warhammer 40,000's total-futility 4; Moral Cynicism (2) since the Dark Powers read as amoral and capricious rather than actively rewarding cruelty -- innocents get trapped in the mists same as the guilty, but villainy isn't specifically rewarded either, distinguishing this from Dark Sun's might-makes-right MC3; Redemption Difficulty (4) and Narrative Acceptance of Injustice (4) held higher than Dark Sun's RD3/NAI3 specifically because Dark Sun's co-primary source (the Prism Pentad) has a definitive ending showing real redemption and real progress, while Ravenloft's flagship figure (Strahd) has never once escaped his curse across the setting's ~40-year history -- only two Darklords ever have, both via metaphysical loopholes (godhood, total domain abandonment) rather than genuine moral repair, and the demiplane is explicitly designed to never resolve at the meta level, generating new Darklords and trapped victims indefinitely; Explicit Darkness (4) for played-straight Poe/Shelley/ Stoker-style gothic horror (vampiric assault, body horror, notoriously disturbing set-pieces like Curse of Strahd's 'Death House' opener).</t>
   </si>
   <si>
+    <t xml:space="preserve">Shadowrun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabletop, Novels, Video Games</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FASA / Catalyst Game Labs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">genre-checked in the queue item itself: a genuine cyberpunk/urban-fantasy hybrid, not sci-fi with fantasy garnish -- magic is a co-equal design pillar post-Awakening (2011), and sapient dragons literally run megacorporations, a load-bearing mythic-political element; matches the precedent already set by Warhammer 40,000's inclusion. Media scope: tabletop + novels + the Harebrained Schemes trilogy (Shadowrun Returns, Dragonfall, Hong Kong), excluding the earlier SNES/Genesis/ Mega-CD games and the 2007 FPS as lower-notability, matching the Dark Sun CRPG-exclusion precedent. Structural Corruption (4) since megacorporations hold extraterritorial status, exempt from law, effectively sovereign entities built specifically to escape accountability -- matches the 'institutions exist, in practice, to sustain exploitation' anchor almost exactly; Limited Heroism (3) is directly textually confirmed by Dragonfall's own ending, described by critics as 'you defeat the villain and realize the status quo sucks and you just helped preserve it' -- local threats (a genocide-virus plot) are genuinely stopped, but the broader corporate system is explicitly, narratively unchanged; Moral Cynicism (3) since corporate executives are 'utterly amoral' and thrive on it, though held below 4 since genuine moral stances are shown as rare-but-real (Lofwyr's surprise at a shadowrunner's moral refusal to use the virus, rather than treating morality as nonexistent); Redemption Difficulty (2) since moral action is shown as possible at real cost, with no stronger textual signal of redemption-denial than that; Narrative Acceptance of Injustice (4) is the genre's own defining convention, confirmed directly by Dragonfall's ending -- the core injustice (corporate rule) is never addressed by design, not just left open; Explicit Darkness (4) for organ-legging (including forced-breeding operations using kidnapped women 'as machines to produce fetuses'), BTL chip addiction, and genocide plotting, presented as recurring black-market features of the setting, not one-off shock content.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 138 of 138 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 139 of 139 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -2124,7 +2136,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R139"/>
+  <dimension ref="A1:R140"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -9618,7 +9630,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="1" t="n">
         <v>9</v>
       </c>
@@ -9672,6 +9684,62 @@
       </c>
       <c r="R139" s="1" t="s">
         <v>429</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B140" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="D140" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="E140" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="F140" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G140" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H140" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I140" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="J140" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="K140" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="L140" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M140" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="N140" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O140" s="1" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="P140" s="1" t="n">
+        <v>8.8125</v>
+      </c>
+      <c r="Q140" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="R140" s="1" t="s">
+        <v>433</v>
       </c>
     </row>
   </sheetData>
@@ -9706,7 +9774,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9794,7 +9862,7 @@
         <v>88</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9821,7 +9889,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Legend of the Five Rings to tier 7; queue Journey to the West
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="440">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1326,10 +1326,22 @@
     <t xml:space="preserve">genre-checked in the queue item itself: a genuine cyberpunk/urban-fantasy hybrid, not sci-fi with fantasy garnish -- magic is a co-equal design pillar post-Awakening (2011), and sapient dragons literally run megacorporations, a load-bearing mythic-political element; matches the precedent already set by Warhammer 40,000's inclusion. Media scope: tabletop + novels + the Harebrained Schemes trilogy (Shadowrun Returns, Dragonfall, Hong Kong), excluding the earlier SNES/Genesis/ Mega-CD games and the 2007 FPS as lower-notability, matching the Dark Sun CRPG-exclusion precedent. Structural Corruption (4) since megacorporations hold extraterritorial status, exempt from law, effectively sovereign entities built specifically to escape accountability -- matches the 'institutions exist, in practice, to sustain exploitation' anchor almost exactly; Limited Heroism (3) is directly textually confirmed by Dragonfall's own ending, described by critics as 'you defeat the villain and realize the status quo sucks and you just helped preserve it' -- local threats (a genocide-virus plot) are genuinely stopped, but the broader corporate system is explicitly, narratively unchanged; Moral Cynicism (3) since corporate executives are 'utterly amoral' and thrive on it, though held below 4 since genuine moral stances are shown as rare-but-real (Lofwyr's surprise at a shadowrunner's moral refusal to use the virus, rather than treating morality as nonexistent); Redemption Difficulty (2) since moral action is shown as possible at real cost, with no stronger textual signal of redemption-denial than that; Narrative Acceptance of Injustice (4) is the genre's own defining convention, confirmed directly by Dragonfall's ending -- the core injustice (corporate rule) is never addressed by design, not just left open; Explicit Darkness (4) for organ-legging (including forced-breeding operations using kidnapped women 'as machines to produce fetuses'), BTL chip addiction, and genocide plotting, presented as recurring black-market features of the setting, not one-off shock content.</t>
   </si>
   <si>
+    <t xml:space="preserve">Legend of the Five Rings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabletop, Novels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AEG / Fantasy Flight Games</t>
+  </si>
+  <si>
+    <t xml:space="preserve">genre gate trivial -- Jigoku (the Realm of Evil), a fallen Kami's demonic corruption, and the Shadowlands Taint are all load-bearing cosmic-horror fantasy elements, not decoration. Scope: bundled the core Rokugan tabletop setting with its extensive storyline/novel material as co-primary sources (the two aren't really separable here the way Drizzt's novels are separable from generic Forgotten Realms lore -- L5R's ~20-year metaplot was told largely through the card game's own narrative sets plus tie-in fiction as one continuous story), matching the Dark Sun precedent over the Forgotten Realms 'core lore only' approach. Structural Despair (2) and Limited Heroism (2) reflect a cyclical pattern -- major existential threats (Fu Leng's First War, the Scorpion Clan Coup that successfully assassinated an Emperor, the Destroyer War) are genuinely defeated each time at real cost, but the underlying instability (a chronically fragile, often-heirless imperial line, endemic clan rivalry) never actually resolves between crises -- scored conservatively rather than pushed to 3 despite a real case for it (flagged explicitly and left as the user's call: Tier 7 confirmed over the alternative Tier 8 reading). Moral Cynicism (2) similarly conservative -- the Scorpion Clan's entire institutional role is sanctioned deception/blackmail as a legitimate parallel path to power, not a punished one, which argues for 3, but bushido's nominal framework does still operate as the setting's stated and often-honored moral compass. Structural Corruption (3) since the honor system institutionalizes lethal punishment (seppuku) for often-minor dishonor as a permanent structural feature, and a major clan's entire function is sanctioned deception -- genuinely rooted in central institutions, though the Empire isn't irrecoverable. Redemption Difficulty (3) since the setting's primary answer to moral failure is frequently death (seppuku) rather than reform-and-forgiveness; Taint-corruption redemption exists via Kuni Witch Hunters but is rare and often too late. Narrative Acceptance of Injustice (3) since specific wars get resolved but the deeper tragic structural conditions (honor-vs-love, endemic rivalry) are explicitly never solved -- Rokugan's own stated genre convention is that 'love will conflict with duty and thus lead to tragedy,' a recurring pattern, not an occasional lapse. Explicit Darkness (4) for ritualized self-disembowelment as a normalized, recurring institutional practice, plus visceral Shadowlands body-horror corruption and genocide-scale content (the Destroyer War: nine-tenths of a population sacrificed, souls imprisoned in metal shells to build an undead army).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 139 of 139 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 140 of 140 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -2136,7 +2148,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R140"/>
+  <dimension ref="A1:R141"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -9686,7 +9698,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="1" t="n">
         <v>8</v>
       </c>
@@ -9740,6 +9752,62 @@
       </c>
       <c r="R140" s="1" t="s">
         <v>433</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B141" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="D141" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="E141" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="F141" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G141" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H141" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I141" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J141" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K141" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L141" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="M141" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="N141" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O141" s="1" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="P141" s="1" t="n">
+        <v>7.4625</v>
+      </c>
+      <c r="Q141" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="R141" s="1" t="s">
+        <v>437</v>
       </c>
     </row>
   </sheetData>
@@ -9774,7 +9842,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9851,7 +9919,7 @@
         <v>87</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9889,7 +9957,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Self-audit corrections: Return to Oz, Ravenloft, Shadowrun
- Return to Oz: revert Explicit Darkness 4->3 (3.41->3.19), the
  earlier revision didn't hold up against its genre-sibling
  comparison set on re-examination. Tier 3 placement unchanged.
- Ravenloft: fix a source citation (Vampire of the Mists and I,
  Strahd are two separate novels, not one), and ground Structural
  Despair / Narrative Acceptance of Injustice in I, Strahd's own
  verified ending rather than a looser meta-IP claim. No score
  change, same conclusion on firmer footing.
- Shadowrun: strengthen Redemption Difficulty's rationale with a
  concrete example (Hong Kong's reconciliation arc) instead of an
  absence-of-counter-evidence inference. No score change.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1305,13 +1305,13 @@
     <t xml:space="preserve">dir. Walter Murch</t>
   </si>
   <si>
-    <t xml:space="preserve">based on Baum's 2nd/3rd Oz novels (The Marvelous Land of Oz, Ozma of Oz), not the first book -- kept separate from The Wizard of Oz entry (Tier 2) for the same reason Wicked stayed separate from it; Structural Despair, Limited Heroism, Redemption Difficulty, and Narrative Acceptance of Injustice all bottom out at 0 since both the Oz plot (the Nome King's conquest, Emerald City's citizens turned to stone) and the frame story (Dorothy's abusive sanitarium) resolve completely and durably -- Oz and its people are fully restored, the sanitarium burns down, the abusive Dr. Worley dies, his nurse-accomplice is arrested, and Ozma confirms Dorothy's experiences were real, not delusion; Moral Cynicism (1) since Dorothy's honesty about Oz is initially met with forced institutionalization and a scheduled electroshock 'cure' rather than being believed -- the same 'sincerity dismissed until vindicated' pattern already on record for The Nightmare Before Christmas's MC1 (Sally's warnings), here more severe (institutionalized and nearly tortured, not just ignored) before vindication; Structural Corruption (2) matches the same 'one real, contained tyranny, corrected cleanly' shape already scored for The Wizard of Oz's Wicked Witch and Alice in Wonderland (2010-2016)'s Red Queen -- the sanitarium subplot was weighed as a second corrupt institution but kept out of Structural Corruption's count since Dr. Worley's electrotherapy reads as era-appropriate- but-brutal malpractice by one reckless doctor, not an institution built to perpetuate harm (unlike American McGee's Alice's Bumby, where the orphanage was literally a trafficking front); Explicit Darkness (4) -- Mombi's wall of living, swappable severed heads is genuine recurring body horror (not just atmospheric dread), on top of the electroshock opening, the Wheelers, and a near-cannibalism scene, matching the 'horror corporal... central y recurrente' anchor that separates this from the ED3 ceiling of its closer genre-siblings (Nightmare Before Christmas, Willow, Dark Crystal, The NeverEnding Story); multiple contemporary retrospectives call it 'the most terrifying Disney movie ever made.'</t>
+    <t xml:space="preserve">based on Baum's 2nd/3rd Oz novels (The Marvelous Land of Oz, Ozma of Oz), not the first book -- kept separate from The Wizard of Oz entry (Tier 2) for the same reason Wicked stayed separate from it; Structural Despair, Limited Heroism, Redemption Difficulty, and Narrative Acceptance of Injustice all bottom out at 0 since both the Oz plot (the Nome King's conquest, Emerald City's citizens turned to stone) and the frame story (Dorothy's abusive sanitarium) resolve completely and durably -- Oz and its people are fully restored, the sanitarium burns down, the abusive Dr. Worley dies, his nurse-accomplice is arrested, and Ozma confirms Dorothy's experiences were real, not delusion; Moral Cynicism (1) since Dorothy's honesty about Oz is initially met with forced institutionalization and a scheduled electroshock 'cure' rather than being believed -- the same 'sincerity dismissed until vindicated' pattern already on record for The Nightmare Before Christmas's MC1 (Sally's warnings), here more severe (institutionalized and nearly tortured, not just ignored) before vindication; Structural Corruption (2) matches the same 'one real, contained tyranny, corrected cleanly' shape already scored for The Wizard of Oz's Wicked Witch and Alice in Wonderland (2010-2016)'s Red Queen -- the sanitarium subplot was weighed as a second corrupt institution but kept out of Structural Corruption's count since Dr. Worley's electrotherapy reads as era-appropriate- but-brutal malpractice by one reckless doctor, not an institution built to perpetuate harm; Explicit Darkness (3) -- calibrated against this catalog's own precedent for 'visually disturbing but thematically light' family-dark-fantasy (Nightmare Before Christmas, Willow, Dark Crystal, The NeverEnding Story, all ED3): Mombi's wall of living severed heads and the electroshock opening are unsettling in concept, but nothing in the source material indicates graphic on-screen depiction beyond that genre-sibling register -- an earlier pass revised this to 4 during the same discussion where a Tier 3 lean had just been stated, and on later self-audit (prompted by the user directly asking whether any score carried doubt) that revision didn't hold up on its own textual merits and was reverted; multiple contemporary retrospectives calling this 'the most terrifying Disney movie ever made' support real atmospheric intensity, not confirmed graphic depiction.</t>
   </si>
   <si>
     <t xml:space="preserve">Ravenloft</t>
   </si>
   <si>
-    <t xml:space="preserve">scored via the core AD&amp;D/D&amp;D gothic horror campaign setting (the Demiplane of Dread, its Darklords, and the Dark Powers) plus the flagship novel line (Vampire of the Mists / I, Strahd) as co-primary sources, matching the Dark Sun precedent (setting + Prism Pentad novels); Structural Despair (4) and Structural Corruption (4) since the demiplane's entire premise is a structurally condemned prison-world where every domain is, by design, ruled by a corrupt Darklord as both throne and prison, not an incidental flaw; Limited Heroism (3) since parties genuinely can and regularly do defeat individual Darklords in actual play (real, if domain-local, victories), keeping this below Warhammer 40,000's total-futility 4; Moral Cynicism (2) since the Dark Powers read as amoral and capricious rather than actively rewarding cruelty -- innocents get trapped in the mists same as the guilty, but villainy isn't specifically rewarded either, distinguishing this from Dark Sun's might-makes-right MC3; Redemption Difficulty (4) and Narrative Acceptance of Injustice (4) held higher than Dark Sun's RD3/NAI3 specifically because Dark Sun's co-primary source (the Prism Pentad) has a definitive ending showing real redemption and real progress, while Ravenloft's flagship figure (Strahd) has never once escaped his curse across the setting's ~40-year history -- only two Darklords ever have, both via metaphysical loopholes (godhood, total domain abandonment) rather than genuine moral repair, and the demiplane is explicitly designed to never resolve at the meta level, generating new Darklords and trapped victims indefinitely; Explicit Darkness (4) for played-straight Poe/Shelley/ Stoker-style gothic horror (vampiric assault, body horror, notoriously disturbing set-pieces like Curse of Strahd's 'Death House' opener).</t>
+    <t xml:space="preserve">scored via the core AD&amp;D/D&amp;D gothic horror campaign setting (the Demiplane of Dread, its Darklords, and the Dark Powers) plus 'I, Strahd: The Memoirs of a Vampire' (P.N. Elrod, 1993) as co-primary sources, matching the Dark Sun precedent (setting + Prism Pentad novels); Structural Despair (4) and Narrative Acceptance of Injustice (4) are grounded directly in that novel's own ending, verified on self-audit rather than inferred from the wider ~40-year product line: Strahd loses Tatyana (she breaks his enchantment and falls to her death), and the novel's own closing material explicitly establishes the curse as eternal and cyclical -- Tatyana reincarnating across the centuries, 'each incarnation bringing joy but their relationships always ending in tragedy' -- not a looser meta-claim about the franchise never resolving; Structural Corruption (4) since every domain is, by design, ruled by a corrupt Darklord as both throne and prison, not an incidental flaw; Limited Heroism (3) since parties genuinely can and regularly do defeat individual Darklords in actual play (real, if domain-local, victories), keeping this below Warhammer 40,000's total-futility 4; Moral Cynicism (2) since the Dark Powers read as amoral and capricious rather than actively rewarding cruelty -- innocents get trapped in the mists same as the guilty, but villainy isn't specifically rewarded either, distinguishing this from Dark Sun's might-makes-right MC3; Redemption Difficulty (4) held higher than Dark Sun's RD3 since Strahd, the setting's flagship figure, has never once escaped his curse across the setting's history -- only two Darklords ever have, both via metaphysical loopholes (godhood, total domain abandonment) rather than genuine moral repair; Explicit Darkness (4) for played-straight Poe/Shelley/Stoker-style gothic horror (vampiric assault, body horror, notoriously disturbing set-pieces like Curse of Strahd's 'Death House' opener).</t>
   </si>
   <si>
     <t xml:space="preserve">Shadowrun</t>
@@ -1323,7 +1323,7 @@
     <t xml:space="preserve">FASA / Catalyst Game Labs</t>
   </si>
   <si>
-    <t xml:space="preserve">genre-checked in the queue item itself: a genuine cyberpunk/urban-fantasy hybrid, not sci-fi with fantasy garnish -- magic is a co-equal design pillar post-Awakening (2011), and sapient dragons literally run megacorporations, a load-bearing mythic-political element; matches the precedent already set by Warhammer 40,000's inclusion. Media scope: tabletop + novels + the Harebrained Schemes trilogy (Shadowrun Returns, Dragonfall, Hong Kong), excluding the earlier SNES/Genesis/ Mega-CD games and the 2007 FPS as lower-notability, matching the Dark Sun CRPG-exclusion precedent. Structural Corruption (4) since megacorporations hold extraterritorial status, exempt from law, effectively sovereign entities built specifically to escape accountability -- matches the 'institutions exist, in practice, to sustain exploitation' anchor almost exactly; Limited Heroism (3) is directly textually confirmed by Dragonfall's own ending, described by critics as 'you defeat the villain and realize the status quo sucks and you just helped preserve it' -- local threats (a genocide-virus plot) are genuinely stopped, but the broader corporate system is explicitly, narratively unchanged; Moral Cynicism (3) since corporate executives are 'utterly amoral' and thrive on it, though held below 4 since genuine moral stances are shown as rare-but-real (Lofwyr's surprise at a shadowrunner's moral refusal to use the virus, rather than treating morality as nonexistent); Redemption Difficulty (2) since moral action is shown as possible at real cost, with no stronger textual signal of redemption-denial than that; Narrative Acceptance of Injustice (4) is the genre's own defining convention, confirmed directly by Dragonfall's ending -- the core injustice (corporate rule) is never addressed by design, not just left open; Explicit Darkness (4) for organ-legging (including forced-breeding operations using kidnapped women 'as machines to produce fetuses'), BTL chip addiction, and genocide plotting, presented as recurring black-market features of the setting, not one-off shock content.</t>
+    <t xml:space="preserve">genre-checked in the queue item itself: a genuine cyberpunk/urban-fantasy hybrid, not sci-fi with fantasy garnish -- magic is a co-equal design pillar post-Awakening (2011), and sapient dragons literally run megacorporations, a load-bearing mythic-political element; matches the precedent already set by Warhammer 40,000's inclusion. Media scope: tabletop + novels + the Harebrained Schemes trilogy (Shadowrun Returns, Dragonfall, Hong Kong), excluding the earlier SNES/Genesis/ Mega-CD games and the 2007 FPS as lower-notability, matching the Dark Sun CRPG-exclusion precedent. Structural Corruption (4) since megacorporations hold extraterritorial status, exempt from law, effectively sovereign entities built specifically to escape accountability -- matches the 'institutions exist, in practice, to sustain exploitation' anchor almost exactly; Limited Heroism (3) is directly textually confirmed by Dragonfall's own ending, described by critics as 'you defeat the villain and realize the status quo sucks and you just helped preserve it' -- local threats (a genocide-virus plot) are genuinely stopped, but the broader corporate system is explicitly, narratively unchanged; Moral Cynicism (3) since corporate executives are 'utterly amoral' and thrive on it, though held below 4 since genuine moral stances are shown as rare-but-real (Lofwyr's surprise at a shadowrunner's moral refusal to use the virus, rather than treating morality as nonexistent); Redemption Difficulty (2) since moral action is shown as possible at real cost, most concretely in Shadowrun: Hong Kong's protagonist, whose central arc is reconciling with an estranged foster father and brother after years of prison-caused separation; Narrative Acceptance of Injustice (4) is the genre's own defining convention, confirmed directly by Dragonfall's ending -- the core injustice (corporate rule) is never addressed by design, not just left open; Explicit Darkness (4) for organ-legging (including forced-breeding operations using kidnapped women 'as machines to produce fetuses'), BTL chip addiction, and genocide plotting, presented as recurring black-market features of the setting, not one-off shock content.</t>
   </si>
   <si>
     <t xml:space="preserve">Legend of the Five Rings</t>
@@ -9627,13 +9627,13 @@
         <v>0</v>
       </c>
       <c r="N138" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O138" s="1" t="n">
-        <v>0.85</v>
+        <v>0.75</v>
       </c>
       <c r="P138" s="1" t="n">
-        <v>3.4125</v>
+        <v>3.1875</v>
       </c>
       <c r="Q138" s="1" t="n">
         <v>3</v>
@@ -9754,7 +9754,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="1" t="n">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Add Black Myth: Wukong to tier 7
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="443">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1338,10 +1338,19 @@
     <t xml:space="preserve">genre gate trivial -- Jigoku (the Realm of Evil), a fallen Kami's demonic corruption, and the Shadowlands Taint are all load-bearing cosmic-horror fantasy elements, not decoration. Scope: bundled the core Rokugan tabletop setting with its extensive storyline/novel material as co-primary sources (the two aren't really separable here the way Drizzt's novels are separable from generic Forgotten Realms lore -- L5R's ~20-year metaplot was told largely through the card game's own narrative sets plus tie-in fiction as one continuous story), matching the Dark Sun precedent over the Forgotten Realms 'core lore only' approach. Structural Despair (2) and Limited Heroism (2) reflect a cyclical pattern -- major existential threats (Fu Leng's First War, the Scorpion Clan Coup that successfully assassinated an Emperor, the Destroyer War) are genuinely defeated each time at real cost, but the underlying instability (a chronically fragile, often-heirless imperial line, endemic clan rivalry) never actually resolves between crises -- scored conservatively rather than pushed to 3 despite a real case for it (flagged explicitly and left as the user's call: Tier 7 confirmed over the alternative Tier 8 reading). Moral Cynicism (2) similarly conservative -- the Scorpion Clan's entire institutional role is sanctioned deception/blackmail as a legitimate parallel path to power, not a punished one, which argues for 3, but bushido's nominal framework does still operate as the setting's stated and often-honored moral compass. Structural Corruption (3) since the honor system institutionalizes lethal punishment (seppuku) for often-minor dishonor as a permanent structural feature, and a major clan's entire function is sanctioned deception -- genuinely rooted in central institutions, though the Empire isn't irrecoverable. Redemption Difficulty (3) since the setting's primary answer to moral failure is frequently death (seppuku) rather than reform-and-forgiveness; Taint-corruption redemption exists via Kuni Witch Hunters but is rare and often too late. Narrative Acceptance of Injustice (3) since specific wars get resolved but the deeper tragic structural conditions (honor-vs-love, endemic rivalry) are explicitly never solved -- Rokugan's own stated genre convention is that 'love will conflict with duty and thus lead to tragedy,' a recurring pattern, not an occasional lapse. Explicit Darkness (4) for ritualized self-disembowelment as a normalized, recurring institutional practice, plus visceral Shadowlands body-horror corruption and genocide-scale content (the Destroyer War: nine-tenths of a population sacrificed, souls imprisoned in metal shells to build an undead army).</t>
   </si>
   <si>
+    <t xml:space="preserve">Black Myth: Wukong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Game Science</t>
+  </si>
+  <si>
+    <t xml:space="preserve">genre-checked in the queue item itself: an action RPG retelling episodes of Journey to the West through the 'Destined One,' with real mythological stakes (gods, demons, Buddhist/Taoist cosmology). The game picks up after Sun Wukong achieves Buddhahood and rejects it, is defeated by the god Erlang, and resealed in stone; several boss-demons are framed as tragic figures, several destroyed by Heaven's own manipulation. Both endings keep some version of the cycle running (re-imprisonment as the new Monkey King under a controlling headband, or a 'true' ending that still inherits the same power structure rather than escaping it). Structural Despair (3), Limited Heroism (3), Moral Cynicism (3), and Narrative Acceptance of Injustice (3) reflect this: Heaven's control never actually breaks in either ending, even the greatest rebel in the mythology (Wukong himself) ultimately lost despite trying every path to legitimacy, and Heaven's own justice is unreliable (Wukong's legitimately earned Buddhahood didn't protect him). Structural Corruption (2) and Redemption Difficulty (2) were revised down from an initial 3/3 on self-audit, benchmarked more carefully: 'gods and Buddhas who CAN mutiny or lose their hearts' signals an exception, not the systemic default (Bodhisattva Lingji's mercy toward Yellow Wind Sage shows Heaven isn't uniformly corrupt, unlike Shadowrun's every-megacorp or Ravenloft's every-domain design) -- matches 'notorious corruption in one institution, others still legitimate' rather than 'central institutions exist to sustain exploitation'; the Yellow Wind Sage tragedy (good intentions curdling into catastrophe) is a weaker match for Redemption Difficulty's specific construct (a character who did wrong failing to achieve moral repair) than for general tragic tone. Explicit Darkness (3), also revised down from 4 on self-audit: benchmarked directly against Dark Souls I-III (already ED3 in this catalog), the closest genre-sibling -- 'Blood and Gore' is the same ESRB descriptor Dark Souls carries, and nothing found shows this game's violence is more graphic than its nearest comparison, so it doesn't clear a full step above that ceiling.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 140 of 140 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 141 of 141 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -2148,7 +2157,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R141"/>
+  <dimension ref="A1:R142"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -9808,6 +9817,62 @@
       </c>
       <c r="R141" s="1" t="s">
         <v>437</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="D142" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E142" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="F142" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G142" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H142" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I142" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="J142" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="K142" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L142" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M142" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="N142" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O142" s="1" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="P142" s="1" t="n">
+        <v>7.575</v>
+      </c>
+      <c r="Q142" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="R142" s="1" t="s">
+        <v>440</v>
       </c>
     </row>
   </sheetData>
@@ -9842,7 +9907,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9919,7 +9984,7 @@
         <v>87</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9957,7 +10022,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rescore Dark Sun to tier 9
Structural Despair and Narrative Acceptance of Injustice raised
3->4: the Prism Pentad's partial victory (2-3 of ~9-10
sorcerer-kings fall) is an exceptional story arc, not the
setting's own default/preferred state -- TSR's later design
explicitly treated that resolution as undermining the setting,
and 4th Edition wound the timeline back to recapture the
pre-resolution baseline. Now ties Ravenloft exactly.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -1140,7 +1140,7 @@
     <t xml:space="preserve">TSR / Wizards of the Coast</t>
   </si>
   <si>
-    <t xml:space="preserve">scored via the AD&amp;D 2nd Edition campaign setting + the Prism Pentad novels (Troy Denning) as co-primary/definitive sources; the 4th Edition (2010) revival and the Shattered Lands/Wake of the Ravager CRPGs were checked as supporting context but don't move any axis, so excluded from separate scoring; unofficial 3rd-edition/d20 material and the unreleased 2027 5th-edition books are out of scope</t>
+    <t xml:space="preserve">scored via the AD&amp;D 2nd Edition campaign setting + the Prism Pentad novels (Troy Denning) as co-primary/definitive sources; the 4th Edition (2010) revival and the Shattered Lands/Wake of the Ravager CRPGs were checked as supporting context but don't move any axis, so excluded from separate scoring; unofficial 3rd-edition/d20 material and the unreleased 2027 5th-edition books are out of scope. Structural Despair and Narrative Acceptance of Injustice revised 3-&gt;4 on rescore (prompted by the user, supplied with community/design-history context): the Prism Pentad's ending shows real but partial progress (2-3 of roughly 9-10 sorcerer-kings fall, tentative ecological revival), but that resolution is an exceptional story arc, not the setting's own default/preferred state -- TSR's later design explicitly treated the Pentad's resolution as undermining the setting ('the great appeal... was the overwhelming sense of oppression and brutality as everyday facts of life; killing off the sorcerer-kings undermined the setting'), and 4th Edition deliberately wound the timeline back to just after the first novel to recapture the pre-resolution baseline. Scored against that baseline (all sorcerer-kings unchallenged, oppression permanent and unattempted) rather than the Pentad's partial, exceptional victory, Structural Despair and Narrative Acceptance of Injustice both match their '4' anchors. Limited Heroism, Moral Cynicism, and Redemption Difficulty were left unrevised -- these measure what happens when protagonists actually act, and the Pentad remains the only substantial long-form narrative testing those constructs, with no equally strong evidence pointing elsewhere. Checked against Ravenloft (also 9.4875 after this revision, tied): no equivalent baseline-vs-narrative divergence exists there, since Ravenloft's flagship novel (I, Strahd) and its base tabletop premise have always told the same story (permanent, unresolved tragedy), unlike Dark Sun's Pentad, which diverges from the setting's own preferred baseline.</t>
   </si>
   <si>
     <t xml:space="preserve">Alice in Wonderland</t>
@@ -8533,10 +8533,10 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>369</v>
@@ -8554,7 +8554,7 @@
         <v>104</v>
       </c>
       <c r="H119" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I119" s="1" t="n">
         <v>3</v>
@@ -8569,19 +8569,19 @@
         <v>3</v>
       </c>
       <c r="M119" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N119" s="1" t="n">
         <v>4</v>
       </c>
       <c r="O119" s="1" t="n">
-        <v>3.25</v>
+        <v>3.55</v>
       </c>
       <c r="P119" s="1" t="n">
-        <v>8.8125</v>
+        <v>9.4875</v>
       </c>
       <c r="Q119" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R119" s="1" t="s">
         <v>372</v>
@@ -9819,7 +9819,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="1" t="n">
         <v>7</v>
       </c>
@@ -9995,7 +9995,7 @@
         <v>88</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10006,7 +10006,7 @@
         <v>89</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add KPop Demon Hunters to tier 3
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1032" uniqueCount="446">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1347,10 +1347,19 @@
     <t xml:space="preserve">genre-checked in the queue item itself: an action RPG retelling episodes of Journey to the West through the 'Destined One,' with real mythological stakes (gods, demons, Buddhist/Taoist cosmology). The game picks up after Sun Wukong achieves Buddhahood and rejects it, is defeated by the god Erlang, and resealed in stone; several boss-demons are framed as tragic figures, several destroyed by Heaven's own manipulation. Both endings keep some version of the cycle running (re-imprisonment as the new Monkey King under a controlling headband, or a 'true' ending that still inherits the same power structure rather than escaping it). Structural Despair (3), Limited Heroism (3), Moral Cynicism (3), and Narrative Acceptance of Injustice (3) reflect this: Heaven's control never actually breaks in either ending, even the greatest rebel in the mythology (Wukong himself) ultimately lost despite trying every path to legitimacy, and Heaven's own justice is unreliable (Wukong's legitimately earned Buddhahood didn't protect him). Structural Corruption (2) and Redemption Difficulty (2) were revised down from an initial 3/3 on self-audit, benchmarked more carefully: 'gods and Buddhas who CAN mutiny or lose their hearts' signals an exception, not the systemic default (Bodhisattva Lingji's mercy toward Yellow Wind Sage shows Heaven isn't uniformly corrupt, unlike Shadowrun's every-megacorp or Ravenloft's every-domain design) -- matches 'notorious corruption in one institution, others still legitimate' rather than 'central institutions exist to sustain exploitation'; the Yellow Wind Sage tragedy (good intentions curdling into catastrophe) is a weaker match for Redemption Difficulty's specific construct (a character who did wrong failing to achieve moral repair) than for general tragic tone. Explicit Darkness (3), also revised down from 4 on self-audit: benchmarked directly against Dark Souls I-III (already ED3 in this catalog), the closest genre-sibling -- 'Blood and Gore' is the same ESRB descriptor Dark Souls carries, and nothing found shows this game's violence is more graphic than its nearest comparison, so it doesn't clear a full step above that ceiling.</t>
   </si>
   <si>
+    <t xml:space="preserve">KPop Demon Hunters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dir. Maggie Kang &amp; Chris Appelhans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">genre-checked before scoring per the newly-formalized relevance/fit step: real demon mythology (Gwi-Ma, the Saja Boys, the Golden Honmoon barrier) is the story's structural core from the premise onward, not incidental dressing on a different mode -- clears easily, unlike Charlie the Unicorn (researched and left off the queue for the same check). Structural Despair (1) and Limited Heroism (1) reflect real, durable improvement -- centuries of demon predation meaningfully checked, Gwi-Ma defeated -- tempered only by the rebuilt Honmoon's explicit imperfection ('still prone to demons passing through'), a minor coda detail rather than a load-bearing 'nothing changed' beat. Moral Cynicism (0) since the film's explicit thesis (per co-director Maggie Kang, 'overcoming your inner demons,' not merely accepting them) directly rewards courage/self-acceptance. Structural Corruption (1) since Gwi-Ma and the Saja Boys are a specific infiltrating threat, not a systemically corrupt institution -- the K-pop industry itself isn't indicted. Redemption Difficulty (2) rests on Jinu: a demon who genuinely redeems himself, but only by sacrificing his own life to save Rumi -- real redemption, real cost. Narrative Acceptance of Injustice (1) since the core conflict resolves with real hope, though centuries of past soul-loss are never undone and the new barrier stays imperfect. Explicit Darkness (2) for real, visible demonic danger and body-marking (Rumi's 'patterns') without confirmed graphic content, matching a broad-audience Netflix animated actioner.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 141 of 141 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 142 of 142 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -2157,7 +2166,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R142"/>
+  <dimension ref="A1:R143"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -9873,6 +9882,62 @@
       </c>
       <c r="R142" s="1" t="s">
         <v>440</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B143" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="D143" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E143" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="F143" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G143" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="H143" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I143" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J143" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K143" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L143" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M143" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N143" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O143" s="1" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="P143" s="1" t="n">
+        <v>3.975</v>
+      </c>
+      <c r="Q143" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="R143" s="1" t="s">
+        <v>443</v>
       </c>
     </row>
   </sheetData>
@@ -9907,7 +9972,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9940,7 +10005,7 @@
         <v>83</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10022,7 +10087,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Chaotic Good Barbarian to tier 2
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1032" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="450">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1356,10 +1356,22 @@
     <t xml:space="preserve">genre-checked before scoring per the newly-formalized relevance/fit step: real demon mythology (Gwi-Ma, the Saja Boys, the Golden Honmoon barrier) is the story's structural core from the premise onward, not incidental dressing on a different mode -- clears easily, unlike Charlie the Unicorn (researched and left off the queue for the same check). Structural Despair (1) and Limited Heroism (1) reflect real, durable improvement -- centuries of demon predation meaningfully checked, Gwi-Ma defeated -- tempered only by the rebuilt Honmoon's explicit imperfection ('still prone to demons passing through'), a minor coda detail rather than a load-bearing 'nothing changed' beat. Moral Cynicism (0) since the film's explicit thesis (per co-director Maggie Kang, 'overcoming your inner demons,' not merely accepting them) directly rewards courage/self-acceptance. Structural Corruption (1) since Gwi-Ma and the Saja Boys are a specific infiltrating threat, not a systemically corrupt institution -- the K-pop industry itself isn't indicted. Redemption Difficulty (2) rests on Jinu: a demon who genuinely redeems himself, but only by sacrificing his own life to save Rumi -- real redemption, real cost. Narrative Acceptance of Injustice (1) since the core conflict resolves with real hope, though centuries of past soul-loss are never undone and the new barrier stays imperfect. Explicit Darkness (2) for real, visible demonic danger and body-marking (Rumi's 'patterns') without confirmed graphic content, matching a broad-audience Netflix animated actioner.</t>
   </si>
   <si>
+    <t xml:space="preserve">Chaotic Good Barbarian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web animation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dungeon Soup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D&amp;D-parody web series (Dungeon Soup); relevance/fit check run before scoring: comedy here is genre-specific D&amp;D-trope parody (liches, phylacteries, monster-slaying tropes used as the actual comedic mechanism, not swappable decoration), closer to Goblins' relationship to its D&amp;D setting than to Charlie the Unicorn's genre-agnostic absurdism -- clears the gate. Dark-comedy check (against the same checklist used for Goblins, per the queue item's own framing): matches the Nightmare Before Christmas pattern, not Goblins' -- no tonal-dissonance criticism, fan reactions are amused/surprised rather than genuinely saddened (no 'IMSAD'-style response), no creator statement of sincere intent, and the show stays in 'played for absurdist laughs' register throughout rather than transitioning into sustained tragedy. Structural Despair/Limited Heroism/Structural Corruption/Redemption Difficulty/Narrative Acceptance of Injustice all bottom out at 0: episodic monster-of-the-week format, the Barbarian's victories are always total and immediate, no institution is ever examined, no redemption arc exists, no injustice is explored (monsters' fates are framed as deserved). Moral Cynicism (1) reflects a real ironic beat the show itself includes -- even other sadistic creatures (Liches, Vampires, Gorgons, Orcs) are disturbed by the nominally 'good'-aligned Barbarian's methods, the same 'sanctioned goodness enables real monstrosity' observation Goblins builds its Moral Cynicism 3 on via the paladin Kore -- but played as a punchline the show never dwells on or lets cost the Barbarian anything, rather than Goblins' sustained, sincere structural argument, so scored well below Goblins' level rather than matched to it. Explicit Darkness (4) for genuinely graphic, detailed, recurring body-horror content that is the show's literal central structure every episode (a Banshee turned into a bagpipe, a Dragon into a pinata, a still-screaming Dryad's transfigured body eaten for breakfast), not an occasional shock beat -- diverging completely from the all-zero thematic profile, matching the theoretical pattern CRITERIA_THEORY.md describes for Explicit Darkness.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 142 of 142 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 143 of 143 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -2166,7 +2178,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R143"/>
+  <dimension ref="A1:R144"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -9884,7 +9896,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="n">
         <v>3</v>
       </c>
@@ -9938,6 +9950,62 @@
       </c>
       <c r="R143" s="1" t="s">
         <v>443</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B144" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="D144" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="E144" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="F144" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G144" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H144" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I144" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J144" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K144" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L144" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M144" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N144" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O144" s="1" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="P144" s="1" t="n">
+        <v>2.7375</v>
+      </c>
+      <c r="Q144" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R144" s="1" t="s">
+        <v>447</v>
       </c>
     </row>
   </sheetData>
@@ -9972,7 +10040,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9994,7 +10062,7 @@
         <v>82</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10087,7 +10155,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Primal to tier 5
Also fixes a duplicate row and a stale Summary sheet tier-1 count
found while adding this entry -- recomputed all tier counts
directly from the Evaluations data instead of trusting prior
incremental edits.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="453">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1368,10 +1368,19 @@
     <t xml:space="preserve">D&amp;D-parody web series (Dungeon Soup); relevance/fit check run before scoring: comedy here is genre-specific D&amp;D-trope parody (liches, phylacteries, monster-slaying tropes used as the actual comedic mechanism, not swappable decoration), closer to Goblins' relationship to its D&amp;D setting than to Charlie the Unicorn's genre-agnostic absurdism -- clears the gate. Dark-comedy check (against the same checklist used for Goblins, per the queue item's own framing): matches the Nightmare Before Christmas pattern, not Goblins' -- no tonal-dissonance criticism, fan reactions are amused/surprised rather than genuinely saddened (no 'IMSAD'-style response), no creator statement of sincere intent, and the show stays in 'played for absurdist laughs' register throughout rather than transitioning into sustained tragedy. Structural Despair/Limited Heroism/Structural Corruption/Redemption Difficulty/Narrative Acceptance of Injustice all bottom out at 0: episodic monster-of-the-week format, the Barbarian's victories are always total and immediate, no institution is ever examined, no redemption arc exists, no injustice is explored (monsters' fates are framed as deserved). Moral Cynicism (1) reflects a real ironic beat the show itself includes -- even other sadistic creatures (Liches, Vampires, Gorgons, Orcs) are disturbed by the nominally 'good'-aligned Barbarian's methods, the same 'sanctioned goodness enables real monstrosity' observation Goblins builds its Moral Cynicism 3 on via the paladin Kore -- but played as a punchline the show never dwells on or lets cost the Barbarian anything, rather than Goblins' sustained, sincere structural argument, so scored well below Goblins' level rather than matched to it. Explicit Darkness (4) for genuinely graphic, detailed, recurring body-horror content that is the show's literal central structure every episode (a Banshee turned into a bagpipe, a Dragon into a pinata, a still-screaming Dryad's transfigured body eaten for breakfast), not an occasional shock beat -- diverging completely from the all-zero thematic profile, matching the theoretical pattern CRITERIA_THEORY.md describes for Explicit Darkness.</t>
   </si>
   <si>
+    <t xml:space="preserve">Primal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genndy Tartakovsky</t>
+  </si>
+  <si>
+    <t xml:space="preserve">genre-checked: not pure prehistoric-survival realism -- Season 2 (a full third of the show's run) introduces sustained supernatural content (a 'Coven of the Damned' performing human sacrifice, real magic entering the show's own mythology, a horned 'demi-god of Hell' styled on Norse myth/Surtur), explicitly discussed by critics and the creator as sword-and-sorcery in the Robert E. Howard tradition -- clears the relevance/fit check comfortably, unlike Charlie the Unicorn's late-arriving, brief fantasy coda. Spear (a mute Neanderthal) loses his wife and children to predators in the opening; Fang (a T-Rex) loses her hatchlings the same day; grief bonds them into found-family. Season 3 has Spear undergo an undead/corrupted transformation he must fight to overcome. Ends genuinely hopefully: Spear reunites with a new partner, child, and Fang, returns to peace, and a coda shows his daughter thriving years later. Structural Despair (2) since Spear's personal arc trends toward real healing, but the wider prehistoric/supernatural world stays harsh and dangerous as its baseline nature throughout. Limited Heroism (1) since Spear's actions produce a real, durable personal victory by the finale. Moral Cynicism (1) since virtue (loyalty, perseverance, love) is ultimately rewarded, though real, permanent losses occur along the way. Structural Corruption (1) since the Coven and similar threats are organized evil cults, not a world-spanning institution. Redemption Difficulty (2) since Spear's undead/corrupted-self arc is a real struggle, resolved only at real cost. Narrative Acceptance of Injustice (1) since the original losses are never undone, but the story's own posture is one of successfully overcoming grief, not leaving it unaddressed. Explicit Darkness (4) for 'unrelenting bloodshed' as the show's constant, wordless, central visual mode across its entire run -- critics consistently note real narrative consequence to each violent act, not gratuitous shock, but the sheer frequency/intensity is the show's defining register throughout. Hopepunk tag researched and rejected: no source discusses this work in Hopepunk terms; critics' leading descriptors are 'bleak,' 'ferocious,' 'eat or be eaten,' with emotional connection as a secondary, moderating layer rather than the organizing throughline the tag requires.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total scored: 143 of 143 works in the full catalog.</t>
+    <t xml:space="preserve">Total scored: 144 of 144 works in the full catalog.</t>
   </si>
 </sst>
 </file>
@@ -2178,7 +2187,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R144"/>
+  <dimension ref="A1:R145"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -9952,7 +9961,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="1" t="n">
         <v>2</v>
       </c>
@@ -10006,6 +10015,62 @@
       </c>
       <c r="R144" s="1" t="s">
         <v>447</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="D145" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="E145" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="F145" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G145" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H145" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I145" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J145" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K145" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L145" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M145" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N145" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O145" s="1" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="P145" s="1" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="Q145" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="R145" s="1" t="s">
+        <v>450</v>
       </c>
     </row>
   </sheetData>
@@ -10040,7 +10105,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10051,7 +10116,7 @@
         <v>81</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10095,7 +10160,7 @@
         <v>85</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10155,7 +10220,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Heavy Metal (1981) to tier 3; exclude Heavy Metal 2000
Heavy Metal 2000 fails the genre gate on its own -- its "magic"
is explicitly classified as advanced alien technology, not real
mythology, and it shares no characters/setting/story with the
1981 film beyond a title and the Loc-Nar framing device.
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -985,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R146"/>
+  <dimension ref="A1:R147"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="8" min="1" max="1"/>
@@ -10820,6 +10820,76 @@
       <c r="R146" s="8" t="inlineStr">
         <is>
           <t>genre gate trivial -- one of China's Four Great Classical Novels, real Buddhist/Taoist cosmology (Heaven, the Underworld, Buddha, the Jade Emperor) throughout. Tang Sanzang travels to India for sacred scriptures with three disciples -- Sun Wukong, Zhu Bajie, Sha Wujing -- all celestial beings being punished for past transgressions (Wukong stole the peaches of immortality and rebelled against Heaven; Buddha sealed him under a mountain for 500 years); the pilgrimage and its 81 tribulations against demons are explicitly Heaven's own redemption mechanism, and all five pilgrims succeed completely, achieving enlightenment. Structural Despair (1) and Limited Heroism (0) reflect the pilgrimage's total, durable success -- every trial ultimately overcome. Moral Cynicism (0) since this is close to a pure 'just world' narrative: wrongdoing brings punishment, genuine virtue brings real redemption. Structural Corruption (1) since Heaven/Buddha are fundamentally legitimate (Wukong's punishment is just, the redemption path real), though many individual episodes involve corrupt local human courts along the way. Redemption Difficulty (1) since it's genuinely difficult (81 hardships, ~14 years) but universal -- every disciple who sincerely pursues it succeeds. Narrative Acceptance of Injustice (0) since every central injustice is fully, explicitly resolved by the ending. Explicit Darkness (2) for real, frequent danger (many demons' recurring goal is to eat the monk's flesh for immortality) without extreme graphic detail, matching the source's classical literary register. Compared explicitly against Black Myth: Wukong (Tier 7, 7.575), the modern reinterpretation of this same mythology per the queue item's own framing: a 5-tier gap, not an inconsistency but the game deliberately inverting the novel's moral framework axis by axis -- the novel's pilgrimage succeeds completely and Heaven's justice is affirmed; the game's own thesis is that even Wukong's total rebellion ultimately failed and Heaven's control is never actually resolved by either ending. Same shape as Wizard of Oz (Tier 2) vs. Wicked (Tier 7): a beloved source text vs. a modern, deliberately subversive reinterpretation of the same events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="15" customHeight="1" s="9">
+      <c r="A147" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B147" s="8" t="inlineStr">
+        <is>
+          <t>Moderately Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C147" s="8" t="inlineStr">
+        <is>
+          <t>Heavy Metal</t>
+        </is>
+      </c>
+      <c r="D147" s="8" t="inlineStr">
+        <is>
+          <t>Film</t>
+        </is>
+      </c>
+      <c r="E147" s="8" t="inlineStr">
+        <is>
+          <t>dir. Gerald Potterton</t>
+        </is>
+      </c>
+      <c r="F147" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G147" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H147" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I147" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J147" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K147" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L147" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M147" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N147" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="O147" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P147" s="8" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="Q147" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="R147" s="8" t="inlineStr">
+        <is>
+          <t>1981 R-rated adult animated sci-fi/fantasy anthology, framed by the Loc-Nar, an ancient evil orb corrupting everyone it touches; genre-mixed by nature, scored as the full released film (frame + all segments) rather than isolated fantasy-coded segments only, since the Loc-Nar throughline and the climactic Taarna segment give the whole film a genuine fantasy backbone. Relevance/fit check passed comfortably on the strength of 'Taarna' (the film's most iconic segment: a mute warrior of an ancient protector race sacrifices herself to permanently destroy the Loc-Nar, reincarnating into a new host) and 'Den' (set in the explicit fantasy world Neverwhere) -- real sword-and-sorcery, not decoration. Heavy Metal 2000, queued alongside this entry, was researched separately and excluded from the catalog entirely: critics and plot analysis explicitly classify it as 'primarily science fiction with fantasy trappings... the magic (immortality serum, the crystal's power) functions as advanced alien technology rather than true magic or mythology' -- fails the genre gate on its own terms, and shares no characters/setting/story with the 1981 film to anchor it, only the Loc-Nar framing device and a title. Structural Despair (1) and Limited Heroism (0) reflect Taarna's sacrifice permanently and completely destroying the Loc-Nar. Moral Cynicism (1) and Structural Corruption (1) both rest on the Captain Sternn segment: an actual murderer/pirate/rapist escapes justice entirely via courtroom chaos the Loc-Nar causes, played for dark comedy -- an isolated institutional failure, not systemic. Redemption Difficulty (0) since no character arc centers on atoning for wrongdoing. Narrative Acceptance of Injustice (1) since Sternn's escape is a real, if comedically-framed, injustice the film never revisits. Explicit Darkness (4) for R-rated content explicitly remembered and marketed for its intensity ('laden with sex, violence'), graphic and frequent across most segments (zombie horror in 'B-17,' sexual content in 'So Beautiful, So Dangerous' and 'Den,' Taarna's climactic battle).</t>
         </is>
       </c>
     </row>
@@ -10897,7 +10967,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="9">
@@ -10994,7 +11064,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Total scored: 145 of 145 works in the full catalog.</t>
+          <t>Total scored: 146 of 146 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Hercules to tier 2
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -985,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R147"/>
+  <dimension ref="A1:R148"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="8" min="1" max="1"/>
@@ -10890,6 +10890,76 @@
       <c r="R147" s="8" t="inlineStr">
         <is>
           <t>1981 R-rated adult animated sci-fi/fantasy anthology, framed by the Loc-Nar, an ancient evil orb corrupting everyone it touches; genre-mixed by nature, scored as the full released film (frame + all segments) rather than isolated fantasy-coded segments only, since the Loc-Nar throughline and the climactic Taarna segment give the whole film a genuine fantasy backbone. Relevance/fit check passed comfortably on the strength of 'Taarna' (the film's most iconic segment: a mute warrior of an ancient protector race sacrifices herself to permanently destroy the Loc-Nar, reincarnating into a new host) and 'Den' (set in the explicit fantasy world Neverwhere) -- real sword-and-sorcery, not decoration. Heavy Metal 2000, queued alongside this entry, was researched separately and excluded from the catalog entirely: critics and plot analysis explicitly classify it as 'primarily science fiction with fantasy trappings... the magic (immortality serum, the crystal's power) functions as advanced alien technology rather than true magic or mythology' -- fails the genre gate on its own terms, and shares no characters/setting/story with the 1981 film to anchor it, only the Loc-Nar framing device and a title. Structural Despair (1) and Limited Heroism (0) reflect Taarna's sacrifice permanently and completely destroying the Loc-Nar. Moral Cynicism (1) and Structural Corruption (1) both rest on the Captain Sternn segment: an actual murderer/pirate/rapist escapes justice entirely via courtroom chaos the Loc-Nar causes, played for dark comedy -- an isolated institutional failure, not systemic. Redemption Difficulty (0) since no character arc centers on atoning for wrongdoing. Narrative Acceptance of Injustice (1) since Sternn's escape is a real, if comedically-framed, injustice the film never revisits. Explicit Darkness (4) for R-rated content explicitly remembered and marketed for its intensity ('laden with sex, violence'), graphic and frequent across most segments (zombie horror in 'B-17,' sexual content in 'So Beautiful, So Dangerous' and 'Den,' Taarna's climactic battle).</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="15" customHeight="1" s="9">
+      <c r="A148" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B148" s="8" t="inlineStr">
+        <is>
+          <t>Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C148" s="8" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="D148" s="8" t="inlineStr">
+        <is>
+          <t>Film</t>
+        </is>
+      </c>
+      <c r="E148" s="8" t="inlineStr">
+        <is>
+          <t>Disney</t>
+        </is>
+      </c>
+      <c r="F148" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G148" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H148" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I148" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J148" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K148" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L148" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M148" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N148" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O148" s="8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P148" s="8" t="n">
+        <v>2.2875</v>
+      </c>
+      <c r="Q148" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="R148" s="8" t="inlineStr">
+        <is>
+          <t>genre gate trivial -- real Greek gods, Hades as an actual deity-antagonist plotting to overthrow Zeus and Olympus, the Fates, the imprisoned Titans. Structural Despair (0), Limited Heroism (0), Structural Corruption (0), and Narrative Acceptance of Injustice (0) all bottom out since the central conflict (Hades' coup) resolves completely and cleanly -- Olympus itself is legitimate, Hades is a jealous individual schemer, not evidence of systemic rot. Moral Cynicism (0) since the film's entire thesis is that self-sacrifice and love define true heroism, directly and explicitly rewarded -- it's literally the mechanism of Hercules' apotheosis (the Fates grant him immortality specifically because he willingly dies to save Meg). Redemption Difficulty (1) rests on Meg: a cynical, self-protective woman secretly indebted to Hades who genuinely grows into self-sacrificial love, nearly dying for it before Hercules saves her. Explicit Darkness (2) for real creature-threat danger (the Hydra, Cerberus, the Titans, the River Styx's souls of the dead) without graphic detail, consistent with a 'mostly lighthearted musical comedy' register.</t>
         </is>
       </c>
     </row>
@@ -10954,7 +11024,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
@@ -11064,7 +11134,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Total scored: 146 of 146 works in the full catalog.</t>
+          <t>Total scored: 147 of 147 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Frozen (2013) to tier 2
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -985,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R148"/>
+  <dimension ref="A1:R149"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="8" min="1" max="1"/>
@@ -10960,6 +10960,76 @@
       <c r="R148" s="8" t="inlineStr">
         <is>
           <t>genre gate trivial -- real Greek gods, Hades as an actual deity-antagonist plotting to overthrow Zeus and Olympus, the Fates, the imprisoned Titans. Structural Despair (0), Limited Heroism (0), Structural Corruption (0), and Narrative Acceptance of Injustice (0) all bottom out since the central conflict (Hades' coup) resolves completely and cleanly -- Olympus itself is legitimate, Hades is a jealous individual schemer, not evidence of systemic rot. Moral Cynicism (0) since the film's entire thesis is that self-sacrifice and love define true heroism, directly and explicitly rewarded -- it's literally the mechanism of Hercules' apotheosis (the Fates grant him immortality specifically because he willingly dies to save Meg). Redemption Difficulty (1) rests on Meg: a cynical, self-protective woman secretly indebted to Hades who genuinely grows into self-sacrificial love, nearly dying for it before Hercules saves her. Explicit Darkness (2) for real creature-threat danger (the Hydra, Cerberus, the Titans, the River Styx's souls of the dead) without graphic detail, consistent with a 'mostly lighthearted musical comedy' register.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="15" customHeight="1" s="9">
+      <c r="A149" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B149" s="8" t="inlineStr">
+        <is>
+          <t>Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t>Frozen</t>
+        </is>
+      </c>
+      <c r="D149" s="8" t="inlineStr">
+        <is>
+          <t>Film</t>
+        </is>
+      </c>
+      <c r="E149" s="8" t="inlineStr">
+        <is>
+          <t>Disney</t>
+        </is>
+      </c>
+      <c r="F149" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G149" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H149" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I149" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J149" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K149" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L149" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M149" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N149" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O149" s="8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P149" s="8" t="n">
+        <v>2.2875</v>
+      </c>
+      <c r="Q149" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="R149" s="8" t="inlineStr">
+        <is>
+          <t>genre gate trivial -- Elsa's ice magic is a real, central power with real consequences (the eternal winter), trolls are a genuine magical species. Scope: scored via the 2013 film only, matching the queue item's own year-specific naming -- Frozen II (2019) is confirmed 'notably darker in tone... heavier focus on action, death, and intense imagery' by critics, different enough that bundling would blur both scores; flagged as a candidate for a future separate entry rather than assumed either way. Structural Despair (0), Limited Heroism (0), Structural Corruption (0), and Narrative Acceptance of Injustice (0) all bottom out since the winter crisis resolves completely and cleanly via Anna's sacrifice, and Arendelle's monarchy is legitimate (Hans is an individual outside schemer, not evidence of systemic rot). Moral Cynicism (1) reflects the Hans twist -- a seemingly genuine love interest revealed as a calculating manipulator willing to let Anna die for the throne -- a real cynicism beat, though he's fully defeated and exposed by the end. Redemption Difficulty (0) since no character arc centers on atoning for real wrongdoing; Elsa's arc is self-acceptance, not redemption. Explicit Darkness (2) for real, visible peril (Anna's heart freezing, Hans's attempted killing blow) without graphic depiction, consistent with family-fantasy register.</t>
         </is>
       </c>
     </row>
@@ -11024,7 +11094,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
@@ -11134,7 +11204,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Total scored: 147 of 147 works in the full catalog.</t>
+          <t>Total scored: 148 of 148 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Moana to tier 2
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -985,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R149"/>
+  <dimension ref="A1:R150"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="8" min="1" max="1"/>
@@ -11030,6 +11030,76 @@
       <c r="R149" s="8" t="inlineStr">
         <is>
           <t>genre gate trivial -- Elsa's ice magic is a real, central power with real consequences (the eternal winter), trolls are a genuine magical species. Scope: scored via the 2013 film only, matching the queue item's own year-specific naming -- Frozen II (2019) is confirmed 'notably darker in tone... heavier focus on action, death, and intense imagery' by critics, different enough that bundling would blur both scores; flagged as a candidate for a future separate entry rather than assumed either way. Structural Despair (0), Limited Heroism (0), Structural Corruption (0), and Narrative Acceptance of Injustice (0) all bottom out since the winter crisis resolves completely and cleanly via Anna's sacrifice, and Arendelle's monarchy is legitimate (Hans is an individual outside schemer, not evidence of systemic rot). Moral Cynicism (1) reflects the Hans twist -- a seemingly genuine love interest revealed as a calculating manipulator willing to let Anna die for the throne -- a real cynicism beat, though he's fully defeated and exposed by the end. Redemption Difficulty (0) since no character arc centers on atoning for real wrongdoing; Elsa's arc is self-acceptance, not redemption. Explicit Darkness (2) for real, visible peril (Anna's heart freezing, Hans's attempted killing blow) without graphic depiction, consistent with family-fantasy register.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="15" customHeight="1" s="9">
+      <c r="A150" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B150" s="8" t="inlineStr">
+        <is>
+          <t>Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t>Moana</t>
+        </is>
+      </c>
+      <c r="D150" s="8" t="inlineStr">
+        <is>
+          <t>Film</t>
+        </is>
+      </c>
+      <c r="E150" s="8" t="inlineStr">
+        <is>
+          <t>Disney</t>
+        </is>
+      </c>
+      <c r="F150" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G150" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H150" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I150" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J150" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K150" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L150" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M150" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N150" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O150" s="8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P150" s="8" t="n">
+        <v>2.2875</v>
+      </c>
+      <c r="Q150" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="R150" s="8" t="inlineStr">
+        <is>
+          <t>genre gate trivial -- a real demigod (Maui), a real ocean deity (Te Fiti), real Polynesian mythological stakes driving the entire plot. Structural Despair (0), Limited Heroism (0), Structural Corruption (0), and Narrative Acceptance of Injustice (0) all bottom out since the blight crisis (Te Fiti's stolen heart) is real and vividly shown but fully, cleanly reversed by the end, matching this catalog's consistent pattern for 'real crisis, completely resolved'; Motunui's own leadership is legitimate, and Gramma Tala's death is framed spiritually/gracefully within the story's own cultural framework (she returns as a manta-ray spirit guide), not an unresolved wound. Moral Cynicism (0) since the film's explicit thesis -- that compassion and self-awareness define true heroism -- is directly rewarded (Moana approaches Te Ka with compassion rather than combat to resolve the climax). Redemption Difficulty (1) rests on Maui: a demigod whose theft of the heart came from a genuine wound (abandoned by his human parents as a baby, seeking validation through 'great deeds' ever since) who genuinely grows and apologizes by the end. Explicit Darkness (2) for real, visible danger (Te Ka's frightening lava-monster design, the Kakamora pirate attack, storms) without graphic detail, consistent with family-fantasy register.</t>
         </is>
       </c>
     </row>
@@ -11094,7 +11164,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
@@ -11204,7 +11274,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Total scored: 148 of 148 works in the full catalog.</t>
+          <t>Total scored: 149 of 149 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Encanto to tier 3
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -985,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R150"/>
+  <dimension ref="A1:R151"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="8" min="1" max="1"/>
@@ -11100,6 +11100,76 @@
       <c r="R150" s="8" t="inlineStr">
         <is>
           <t>genre gate trivial -- a real demigod (Maui), a real ocean deity (Te Fiti), real Polynesian mythological stakes driving the entire plot. Structural Despair (0), Limited Heroism (0), Structural Corruption (0), and Narrative Acceptance of Injustice (0) all bottom out since the blight crisis (Te Fiti's stolen heart) is real and vividly shown but fully, cleanly reversed by the end, matching this catalog's consistent pattern for 'real crisis, completely resolved'; Motunui's own leadership is legitimate, and Gramma Tala's death is framed spiritually/gracefully within the story's own cultural framework (she returns as a manta-ray spirit guide), not an unresolved wound. Moral Cynicism (0) since the film's explicit thesis -- that compassion and self-awareness define true heroism -- is directly rewarded (Moana approaches Te Ka with compassion rather than combat to resolve the climax). Redemption Difficulty (1) rests on Maui: a demigod whose theft of the heart came from a genuine wound (abandoned by his human parents as a baby, seeking validation through 'great deeds' ever since) who genuinely grows and apologizes by the end. Explicit Darkness (2) for real, visible danger (Te Ka's frightening lava-monster design, the Kakamora pirate attack, storms) without graphic detail, consistent with family-fantasy register.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="15" customHeight="1" s="9">
+      <c r="A151" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B151" s="8" t="inlineStr">
+        <is>
+          <t>Moderately Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C151" s="8" t="inlineStr">
+        <is>
+          <t>Encanto</t>
+        </is>
+      </c>
+      <c r="D151" s="8" t="inlineStr">
+        <is>
+          <t>Film</t>
+        </is>
+      </c>
+      <c r="E151" s="8" t="inlineStr">
+        <is>
+          <t>Disney</t>
+        </is>
+      </c>
+      <c r="F151" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G151" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H151" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I151" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J151" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K151" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L151" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M151" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N151" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O151" s="8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="P151" s="8" t="n">
+        <v>3.6375</v>
+      </c>
+      <c r="Q151" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="R151" s="8" t="inlineStr">
+        <is>
+          <t>genre gate trivial -- a real magic house and real bestowed magical gifts are the plot's central mechanism. Structural Despair (0) and Limited Heroism (0) since the magic crisis fully collapses (the house, the candle) but is completely restored by the end through Mirabel's actions. Moral Cynicism (0) since vulnerability and honesty are directly, explicitly rewarded. Structural Corruption (1) -- the village of Encanto was literally founded and protected by the Madrigal magic (the family functions as the town's de facto magical governance/protection institution, not just a private family), and Alma's distortion of that structure around gift-based usefulness is a real corruption of it, not an isolated family quirk. Redemption Difficulty (2), revised up from an initial 1 on self-audit prompted by the user -- Alma's reckoning isn't just an emotional apology; it's preceded by the complete, total loss of the magic and house (50 years of safety she'd clung to since her husband's death) directly caused by her own controlling behavior, a real severed cost connected to the redemption, not incidental. Narrative Acceptance of Injustice (2), revised up from 0 -- prompted by the user flagging the opening armed-conflict/displacement sequence as a specific allusion to Colombia's Guerra de los Mil Dias and its broader decades-spanning history of internal armed conflict and displacement, not generic fairy-tale villain backstory; Pedro's death is never revisited, resolved, or avenged within the plot even as the present-day family conflict resolves completely -- an 'ambivalent, some injustices resolve while others persist without explanation' pattern. Explicit Darkness (2) for the real violent opening (armed marauders, Pedro's death) and the house's dramatic collapse, without graphic depiction.</t>
         </is>
       </c>
     </row>
@@ -11177,7 +11247,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="9">
@@ -11274,7 +11344,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Total scored: 149 of 149 works in the full catalog.</t>
+          <t>Total scored: 150 of 150 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Onward to tier 2
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -985,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R151"/>
+  <dimension ref="A1:R152"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="8" min="1" max="1"/>
@@ -11170,6 +11170,76 @@
       <c r="R151" s="8" t="inlineStr">
         <is>
           <t>genre gate trivial -- a real magic house and real bestowed magical gifts are the plot's central mechanism. Structural Despair (0) and Limited Heroism (0) since the magic crisis fully collapses (the house, the candle) but is completely restored by the end through Mirabel's actions. Moral Cynicism (0) since vulnerability and honesty are directly, explicitly rewarded. Structural Corruption (1) -- the village of Encanto was literally founded and protected by the Madrigal magic (the family functions as the town's de facto magical governance/protection institution, not just a private family), and Alma's distortion of that structure around gift-based usefulness is a real corruption of it, not an isolated family quirk. Redemption Difficulty (2), revised up from an initial 1 on self-audit prompted by the user -- Alma's reckoning isn't just an emotional apology; it's preceded by the complete, total loss of the magic and house (50 years of safety she'd clung to since her husband's death) directly caused by her own controlling behavior, a real severed cost connected to the redemption, not incidental. Narrative Acceptance of Injustice (2), revised up from 0 -- prompted by the user flagging the opening armed-conflict/displacement sequence as a specific allusion to Colombia's Guerra de los Mil Dias and its broader decades-spanning history of internal armed conflict and displacement, not generic fairy-tale villain backstory; Pedro's death is never revisited, resolved, or avenged within the plot even as the present-day family conflict resolves completely -- an 'ambivalent, some injustices resolve while others persist without explanation' pattern. Explicit Darkness (2) for the real violent opening (armed marauders, Pedro's death) and the house's dramatic collapse, without graphic depiction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="15" customHeight="1" s="9">
+      <c r="A152" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B152" s="8" t="inlineStr">
+        <is>
+          <t>Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t>Onward</t>
+        </is>
+      </c>
+      <c r="D152" s="8" t="inlineStr">
+        <is>
+          <t>Film</t>
+        </is>
+      </c>
+      <c r="E152" s="8" t="inlineStr">
+        <is>
+          <t>Pixar</t>
+        </is>
+      </c>
+      <c r="F152" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G152" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H152" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I152" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J152" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K152" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L152" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M152" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N152" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O152" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P152" s="8" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="Q152" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="R152" s="8" t="inlineStr">
+        <is>
+          <t>genre gate trivial -- an explicit fantasy world of elves, wizards, dragons, and unicorns, real magic as the plot's central mechanism. Structural Despair (0) since the boys' personal quest reawakens real magic and connection in their lives by the end. Limited Heroism (1) since the broader quest (the beast defeated, magic proven real) succeeds completely, but Ian's own specific goal -- actually meeting his father -- is never achieved, a real if minor unresolved detail (only Barley, who actually remembers their dad, gets a real goodbye). Moral Cynicism (0) and Structural Corruption (0) since there's no cynical-world content or institution examined. Redemption Difficulty (0) since Ian's arc (embarrassment softening into appreciation of Barley) is coming-of-age, not atonement for real wrongdoing. Narrative Acceptance of Injustice (1) since Ian's specific loss (never getting to meet his father) is permanent and never undone, but the narrative frames it as something he can genuinely move past (realizing Barley has been his father figure all along), not a wound it leaves untouched. Explicit Darkness (2) for real but contained danger (a curse, a dragon-beast battle, chase sequences) without graphic content, consistent with family-fantasy register.</t>
         </is>
       </c>
     </row>
@@ -11234,7 +11304,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
@@ -11344,7 +11414,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Total scored: 150 of 150 works in the full catalog.</t>
+          <t>Total scored: 151 of 151 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Rise of the Guardians to tier 3
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -985,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R152"/>
+  <dimension ref="A1:R153"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="8" min="1" max="1"/>
@@ -11240,6 +11240,76 @@
       <c r="R152" s="8" t="inlineStr">
         <is>
           <t>genre gate trivial -- an explicit fantasy world of elves, wizards, dragons, and unicorns, real magic as the plot's central mechanism. Structural Despair (0) since the boys' personal quest reawakens real magic and connection in their lives by the end. Limited Heroism (1) since the broader quest (the beast defeated, magic proven real) succeeds completely, but Ian's own specific goal -- actually meeting his father -- is never achieved, a real if minor unresolved detail (only Barley, who actually remembers their dad, gets a real goodbye). Moral Cynicism (0) and Structural Corruption (0) since there's no cynical-world content or institution examined. Redemption Difficulty (0) since Ian's arc (embarrassment softening into appreciation of Barley) is coming-of-age, not atonement for real wrongdoing. Narrative Acceptance of Injustice (1) since Ian's specific loss (never getting to meet his father) is permanent and never undone, but the narrative frames it as something he can genuinely move past (realizing Barley has been his father figure all along), not a wound it leaves untouched. Explicit Darkness (2) for real but contained danger (a curse, a dragon-beast battle, chase sequences) without graphic content, consistent with family-fantasy register.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="15" customHeight="1" s="9">
+      <c r="A153" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B153" s="8" t="inlineStr">
+        <is>
+          <t>Moderately Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C153" s="8" t="inlineStr">
+        <is>
+          <t>Rise of the Guardians</t>
+        </is>
+      </c>
+      <c r="D153" s="8" t="inlineStr">
+        <is>
+          <t>Film</t>
+        </is>
+      </c>
+      <c r="E153" s="8" t="inlineStr">
+        <is>
+          <t>DreamWorks</t>
+        </is>
+      </c>
+      <c r="F153" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G153" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H153" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I153" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J153" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K153" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L153" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M153" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N153" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="O153" s="8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="P153" s="8" t="n">
+        <v>3.525</v>
+      </c>
+      <c r="Q153" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="R153" s="8" t="inlineStr">
+        <is>
+          <t>genre gate established at queue time -- Santa, the Tooth Fairy, the Sandman, Jack Frost, and the Easter Bunny as real magical beings with real powers, fighting an embodied evil (Pitch Black), not holiday theming. Structural Despair (1) since the underlying premise is a permanent, cyclical tension between belief and fear that's never fully resolved, even though this specific crisis resolves clearly. Limited Heroism (2) since the victory depends on the children's collective belief as much as the Guardians' own actions, and Pitch survives (dragged back to his lair by his own nightmare creatures, not destroyed) -- resolves the immediate threat, leaves the conditions that generated it intact. Moral Cynicism (0) and Structural Corruption (0) since belief/goodness is directly rewarded and Pitch is an individual embodiment of fear, not a corrupt institution. Redemption Difficulty (0) since Jack Frost's arc is about self-acceptance and finding purpose (centuries of isolation from being unseen/unbelieved in), not atonement for wrongdoing. Narrative Acceptance of Injustice (1) since Pitch's survival is a real loose end, but the film's own posture is confidently triumphant, not dwelling on it as an open wound. Explicit Darkness (3) for a real, visible character death (Sandy, overwhelmed and killed by black nightmare sand before being resurrected by children's renewed belief), genuinely frightening nightmare-creature designs, and Jack's centuries of ghost-like isolation -- notably darker register than this batch's other entries, matching this film's critical reputation for being surprisingly intense for younger children.</t>
         </is>
       </c>
     </row>
@@ -11317,7 +11387,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="9">
@@ -11414,7 +11484,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Total scored: 151 of 151 works in the full catalog.</t>
+          <t>Total scored: 152 of 152 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Shrek, Puss in Boots, and Puss in Boots: The Last Wish
Split into three entries rather than one bundle: the mainline
Shrek quadrilogy (tier 3), Puss in Boots 2011 (tier 2), and
Puss in Boots: The Last Wish 2022 (tier 3, confirmed meaningfully
darker than the rest of the franchise by critics).
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -985,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R153"/>
+  <dimension ref="A1:R156"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="8" min="1" max="1"/>
@@ -11310,6 +11310,216 @@
       <c r="R153" s="8" t="inlineStr">
         <is>
           <t>genre gate established at queue time -- Santa, the Tooth Fairy, the Sandman, Jack Frost, and the Easter Bunny as real magical beings with real powers, fighting an embodied evil (Pitch Black), not holiday theming. Structural Despair (1) since the underlying premise is a permanent, cyclical tension between belief and fear that's never fully resolved, even though this specific crisis resolves clearly. Limited Heroism (2) since the victory depends on the children's collective belief as much as the Guardians' own actions, and Pitch survives (dragged back to his lair by his own nightmare creatures, not destroyed) -- resolves the immediate threat, leaves the conditions that generated it intact. Moral Cynicism (0) and Structural Corruption (0) since belief/goodness is directly rewarded and Pitch is an individual embodiment of fear, not a corrupt institution. Redemption Difficulty (0) since Jack Frost's arc is about self-acceptance and finding purpose (centuries of isolation from being unseen/unbelieved in), not atonement for wrongdoing. Narrative Acceptance of Injustice (1) since Pitch's survival is a real loose end, but the film's own posture is confidently triumphant, not dwelling on it as an open wound. Explicit Darkness (3) for a real, visible character death (Sandy, overwhelmed and killed by black nightmare sand before being resurrected by children's renewed belief), genuinely frightening nightmare-creature designs, and Jack's centuries of ghost-like isolation -- notably darker register than this batch's other entries, matching this film's critical reputation for being surprisingly intense for younger children.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="15" customHeight="1" s="9">
+      <c r="A154" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B154" s="8" t="inlineStr">
+        <is>
+          <t>Moderately Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C154" s="8" t="inlineStr">
+        <is>
+          <t>Shrek</t>
+        </is>
+      </c>
+      <c r="D154" s="8" t="inlineStr">
+        <is>
+          <t>Films</t>
+        </is>
+      </c>
+      <c r="E154" s="8" t="inlineStr">
+        <is>
+          <t>DreamWorks</t>
+        </is>
+      </c>
+      <c r="F154" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G154" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H154" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I154" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J154" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K154" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L154" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N154" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="O154" s="8" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="P154" s="8" t="n">
+        <v>3.8625</v>
+      </c>
+      <c r="Q154" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="R154" s="8" t="inlineStr">
+        <is>
+          <t>genre gate trivial -- real curses, real transformation magic (the True Love's Kiss curse is the entire plot engine of film 1), genuine fairy-tale creatures as a functioning world. Scope: scored via the mainline quadrilogy (Shrek, Shrek 2, Shrek the Third, Shrek Forever After) only -- Puss in Boots (2011) and Puss in Boots: The Last Wish (2022) are scored as their own separate entries, matching the Legend of Vox Machina / Mighty Nein precedent for different-protagonist spinoffs within the same shared universe, and specifically because The Last Wish is confirmed meaningfully darker than the rest of the franchise. Structural Despair (1) and Structural Corruption (2) are grounded in Shrek Forever After's alternate timeline: Shrek is erased from history via a Rumpelstiltskin deal, who then rules Far Far Away as a dictator -- ogres enslaved and whipped for hard labor, hunted by bounty hunters, Fiona leading an armed resistance -- genuinely dark, vivid imagery, fully undone (retroactively erased, not just resolved) by the ending's true-love's-kiss reset. Limited Heroism (1) since resolution across the bundle relies partly on this kind of external/magical reset rather than pure direct heroic triumph. Moral Cynicism (1) for the recurring trickster-dealmaker fraud pattern (Rumpelstiltskin's soul-trading contract). Redemption Difficulty (0) since no character arc within the mainline four films alone centers on atoning for real wrongdoing -- Shrek's own arc is self-acceptance, not redemption (the only redemption-difficulty content in the franchise, Humpty Dumpty and Puss's, belongs to the separately-scored Puss in Boots entries). Narrative Acceptance of Injustice (0) since every conflict resolves completely, and the alternate-timeline dystopia isn't just resolved, it's retroactively un-happened. Explicit Darkness (3) for the enslavement/whipping imagery specifically, on top of recurring villain peril elsewhere (Farquaad, the Fairy Godmother, Prince Charming).</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="15" customHeight="1" s="9">
+      <c r="A155" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B155" s="8" t="inlineStr">
+        <is>
+          <t>Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>Puss in Boots</t>
+        </is>
+      </c>
+      <c r="D155" s="8" t="inlineStr">
+        <is>
+          <t>Film</t>
+        </is>
+      </c>
+      <c r="E155" s="8" t="inlineStr">
+        <is>
+          <t>DreamWorks</t>
+        </is>
+      </c>
+      <c r="F155" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G155" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H155" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I155" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J155" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K155" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L155" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M155" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N155" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O155" s="8" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="P155" s="8" t="n">
+        <v>2.9625</v>
+      </c>
+      <c r="Q155" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="R155" s="8" t="inlineStr">
+        <is>
+          <t>scored as its own entry, separate from the mainline Shrek quadrilogy, per the Vox Machina / Mighty Nein precedent for different-protagonist spinoffs sharing a universe. Puss and his childhood friend Humpty Dumpty had a falling out after a botched heist Humpty orchestrated left Puss framed as an outlaw; years later Humpty lures Puss into a scheme to steal a golden goose using magic beans, which turns out to be an elaborate act of revenge luring the goose's giant mother back to destroy Puss's hometown. Puss appeals to the good still in Humpty, who redeems himself with a genuine heroic sacrifice to save the goose and the town. Structural Despair (0) and Limited Heroism (0) since the crisis resolves completely and durably. Moral Cynicism (1) for the real betrayal-by-a-trusted-friend beat (twice -- as children and again as adults), though ultimately resolved positively. Structural Corruption (0) since this is a personal betrayal/heist story, no institution examined. Redemption Difficulty (2) since Humpty's arc is genuine and costly: real wrongdoing (an elaborate revenge plot to destroy his former friend's hometown) redeemed through an actual heroic self-sacrifice. Narrative Acceptance of Injustice (0) since full reconciliation is achieved by the end. Explicit Darkness (2) for real but comedic-registered peril (chase sequences, a giant-creature threat) without graphic content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="15" customHeight="1" s="9">
+      <c r="A156" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B156" s="8" t="inlineStr">
+        <is>
+          <t>Moderately Bright Fantasy</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="inlineStr">
+        <is>
+          <t>Puss in Boots: The Last Wish</t>
+        </is>
+      </c>
+      <c r="D156" s="8" t="inlineStr">
+        <is>
+          <t>Film</t>
+        </is>
+      </c>
+      <c r="E156" s="8" t="inlineStr">
+        <is>
+          <t>DreamWorks</t>
+        </is>
+      </c>
+      <c r="F156" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G156" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H156" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I156" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J156" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K156" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L156" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M156" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N156" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="O156" s="8" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="P156" s="8" t="n">
+        <v>3.075</v>
+      </c>
+      <c r="Q156" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="R156" s="8" t="inlineStr">
+        <is>
+          <t>scored separately from both the Shrek quadrilogy and Puss in Boots (2011) given a confirmed, deliberate tonal shift -- critics consistently describe this as 'definitely darker' than the rest of the franchise, with Death itself (embodied as the Big Bad Wolf) stalking Puss with 'a personal but genuine vendetta' for wasting his lives; encounters are repeatedly compared to slasher-film pacing and tension. Puss, down to his last of nine lives, ultimately destroys the wishing star and forfeits his wish entirely, accepting mortality rather than chasing immortality; Jack Horner (consumed by greed) falls to his death after over-consuming magic. Structural Despair, Limited Heroism, Moral Cynicism, and Structural Corruption all bottom out at 0 since the personal-scale conflict resolves completely and cleanly. Redemption Difficulty (2) since Puss must genuinely reckon with his own recklessness toward his own life, at real cost (forfeiting his last wish, confronting real fear/vulnerability for the first time). Narrative Acceptance of Injustice (0) since full resolution is achieved. Explicit Darkness (4) since Death's stalking presence is a central, recurring, genuinely horror-registered threat throughout the film, not an occasional dark beat -- the director has said he deliberately drew on the darker Brothers Grimm cautionary-tale tradition rather than the franchise's usual register.</t>
         </is>
       </c>
     </row>
@@ -11374,7 +11584,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
@@ -11387,7 +11597,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="9">
@@ -11484,7 +11694,7 @@
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Total scored: 152 of 152 works in the full catalog.</t>
+          <t>Total scored: 155 of 155 works in the full catalog.</t>
         </is>
       </c>
     </row>

</xml_diff>